<commit_message>
Atualização automática: tpjl (10/07/2026 10:12)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -13038,7 +13038,7 @@
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -13105,7 +13105,7 @@
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -13172,7 +13172,7 @@
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -13239,7 +13239,7 @@
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -13306,7 +13306,7 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -13373,7 +13373,7 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -13440,7 +13440,7 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -13507,7 +13507,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -13574,7 +13574,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -13641,7 +13641,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -13773,7 +13773,7 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -13840,7 +13840,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -13907,7 +13907,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -13974,7 +13974,7 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -14041,7 +14041,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -14108,7 +14108,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -14175,7 +14175,7 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -14242,7 +14242,7 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -14309,7 +14309,7 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -14376,7 +14376,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -14443,7 +14443,7 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -14510,7 +14510,7 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -14577,7 +14577,7 @@
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -14644,7 +14644,7 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -14711,7 +14711,7 @@
         </is>
       </c>
       <c r="M27" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -14778,7 +14778,7 @@
         </is>
       </c>
       <c r="M28" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -14845,7 +14845,7 @@
         </is>
       </c>
       <c r="M29" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -14912,7 +14912,7 @@
         </is>
       </c>
       <c r="M30" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -14979,7 +14979,7 @@
         </is>
       </c>
       <c r="M31" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -15046,7 +15046,7 @@
         </is>
       </c>
       <c r="M32" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -15113,7 +15113,7 @@
         </is>
       </c>
       <c r="M33" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -15180,7 +15180,7 @@
         </is>
       </c>
       <c r="M34" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -15247,7 +15247,7 @@
         </is>
       </c>
       <c r="M35" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -15314,7 +15314,7 @@
         </is>
       </c>
       <c r="M36" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -15381,7 +15381,7 @@
         </is>
       </c>
       <c r="M37" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -15448,7 +15448,7 @@
         </is>
       </c>
       <c r="M38" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -15515,7 +15515,7 @@
         </is>
       </c>
       <c r="M39" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -15582,7 +15582,7 @@
         </is>
       </c>
       <c r="M40" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática: tpjl (10/07/2026 17:32)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,87 +422,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -582,7 +570,7 @@
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -649,7 +637,7 @@
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" s="2" t="n">
+      <c r="P3" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -716,7 +704,7 @@
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" s="2" t="n">
+      <c r="P4" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -913,7 +901,7 @@
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -980,7 +968,7 @@
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" s="2" t="n">
+      <c r="P8" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1047,7 +1035,7 @@
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1118,7 +1106,7 @@
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" s="2" t="n">
+      <c r="P10" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1311,7 +1299,7 @@
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" s="2" t="n">
+      <c r="P13" s="1" t="n">
         <v>46037</v>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -1378,7 +1366,7 @@
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" s="2" t="n">
+      <c r="P14" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -1445,7 +1433,7 @@
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" s="2" t="n">
+      <c r="P15" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -1512,7 +1500,7 @@
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" s="2" t="n">
+      <c r="P16" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1583,7 +1571,7 @@
         </is>
       </c>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" s="2" t="n">
+      <c r="P17" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -1650,7 +1638,7 @@
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" s="2" t="n">
+      <c r="P18" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -1847,7 +1835,7 @@
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" s="2" t="n">
+      <c r="P21" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -1914,7 +1902,7 @@
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" s="2" t="n">
+      <c r="P22" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -2046,7 +2034,7 @@
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" s="2" t="n">
+      <c r="P24" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2117,7 +2105,7 @@
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" s="2" t="n">
+      <c r="P25" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2188,7 +2176,7 @@
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" s="2" t="n">
+      <c r="P26" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -2255,7 +2243,7 @@
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" s="2" t="n">
+      <c r="P27" s="1" t="n">
         <v>45964</v>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -2322,7 +2310,7 @@
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" s="2" t="n">
+      <c r="P28" s="1" t="n">
         <v>45984</v>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -2454,7 +2442,7 @@
         </is>
       </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" s="2" t="n">
+      <c r="P30" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q30" t="inlineStr"/>
@@ -2586,7 +2574,7 @@
         </is>
       </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" s="2" t="n">
+      <c r="P32" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2657,7 +2645,7 @@
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" s="2" t="n">
+      <c r="P33" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -2724,7 +2712,7 @@
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
-      <c r="P34" s="2" t="n">
+      <c r="P34" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -2791,7 +2779,7 @@
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" s="2" t="n">
+      <c r="P35" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -2923,7 +2911,7 @@
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" s="2" t="n">
+      <c r="P37" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -2990,7 +2978,7 @@
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" s="2" t="n">
+      <c r="P38" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -3057,7 +3045,7 @@
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" s="2" t="n">
+      <c r="P39" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q39" t="inlineStr"/>
@@ -3189,7 +3177,7 @@
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" s="2" t="n">
+      <c r="P41" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q41" t="inlineStr"/>
@@ -3256,7 +3244,7 @@
         </is>
       </c>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" s="2" t="n">
+      <c r="P42" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -3323,7 +3311,7 @@
         </is>
       </c>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" s="2" t="n">
+      <c r="P43" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -3390,7 +3378,7 @@
         </is>
       </c>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" s="2" t="n">
+      <c r="P44" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -3652,7 +3640,7 @@
         </is>
       </c>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" s="2" t="n">
+      <c r="P48" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -3719,7 +3707,7 @@
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" s="2" t="n">
+      <c r="P49" s="1" t="n">
         <v>45955</v>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -3786,7 +3774,7 @@
         </is>
       </c>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" s="2" t="n">
+      <c r="P50" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -3853,7 +3841,7 @@
         </is>
       </c>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" s="2" t="n">
+      <c r="P51" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q51" t="inlineStr">
@@ -3924,7 +3912,7 @@
         </is>
       </c>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" s="2" t="n">
+      <c r="P52" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -3991,7 +3979,7 @@
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" s="2" t="n">
+      <c r="P53" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -4119,7 +4107,7 @@
         </is>
       </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" s="2" t="n">
+      <c r="P55" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -4186,7 +4174,7 @@
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" s="2" t="n">
+      <c r="P56" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -4322,7 +4310,7 @@
         </is>
       </c>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" s="2" t="n">
+      <c r="P58" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -4389,7 +4377,7 @@
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" s="2" t="n">
+      <c r="P59" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q59" t="inlineStr">
@@ -4460,7 +4448,7 @@
         </is>
       </c>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" s="2" t="n">
+      <c r="P60" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -4527,7 +4515,7 @@
         </is>
       </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" s="2" t="n">
+      <c r="P61" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q61" t="inlineStr"/>
@@ -4594,7 +4582,7 @@
         </is>
       </c>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" s="2" t="n">
+      <c r="P62" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q62" t="inlineStr"/>
@@ -4661,7 +4649,7 @@
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" s="2" t="n">
+      <c r="P63" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q63" t="inlineStr"/>
@@ -4728,7 +4716,7 @@
         </is>
       </c>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" s="2" t="n">
+      <c r="P64" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q64" t="inlineStr">
@@ -4799,7 +4787,7 @@
         </is>
       </c>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" s="2" t="n">
+      <c r="P65" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q65" t="inlineStr"/>
@@ -4866,7 +4854,7 @@
         </is>
       </c>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" s="2" t="n">
+      <c r="P66" s="1" t="n">
         <v>45946</v>
       </c>
       <c r="Q66" t="inlineStr">
@@ -4937,7 +4925,7 @@
         </is>
       </c>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" s="2" t="n">
+      <c r="P67" s="1" t="n">
         <v>45916</v>
       </c>
       <c r="Q67" t="inlineStr"/>
@@ -5004,7 +4992,7 @@
         </is>
       </c>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" s="2" t="n">
+      <c r="P68" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5075,7 +5063,7 @@
         </is>
       </c>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" s="2" t="n">
+      <c r="P69" s="1" t="n">
         <v>45989</v>
       </c>
       <c r="Q69" t="inlineStr">
@@ -5211,7 +5199,7 @@
         </is>
       </c>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" s="2" t="n">
+      <c r="P71" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -5278,7 +5266,7 @@
         </is>
       </c>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" s="2" t="n">
+      <c r="P72" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q72" t="inlineStr"/>
@@ -5345,7 +5333,7 @@
         </is>
       </c>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" s="2" t="n">
+      <c r="P73" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q73" t="inlineStr"/>
@@ -5412,7 +5400,7 @@
         </is>
       </c>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" s="2" t="n">
+      <c r="P74" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q74" t="inlineStr"/>
@@ -5479,7 +5467,7 @@
         </is>
       </c>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" s="2" t="n">
+      <c r="P75" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q75" t="inlineStr"/>
@@ -5546,7 +5534,7 @@
         </is>
       </c>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" s="2" t="n">
+      <c r="P76" s="1" t="n">
         <v>46130</v>
       </c>
       <c r="Q76" t="inlineStr"/>
@@ -5678,7 +5666,7 @@
         </is>
       </c>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" s="2" t="n">
+      <c r="P78" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q78" t="inlineStr"/>
@@ -5745,7 +5733,7 @@
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
-      <c r="P79" s="2" t="n">
+      <c r="P79" s="1" t="n">
         <v>46140</v>
       </c>
       <c r="Q79" t="inlineStr"/>
@@ -5812,7 +5800,7 @@
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" s="2" t="n">
+      <c r="P80" s="1" t="n">
         <v>46095</v>
       </c>
       <c r="Q80" t="inlineStr"/>
@@ -5879,7 +5867,7 @@
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" s="2" t="n">
+      <c r="P81" s="1" t="n">
         <v>46040</v>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -5946,7 +5934,7 @@
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" s="2" t="n">
+      <c r="P82" s="1" t="n">
         <v>46060</v>
       </c>
       <c r="Q82" t="inlineStr"/>
@@ -6013,7 +6001,7 @@
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" s="2" t="n">
+      <c r="P83" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -6080,7 +6068,7 @@
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" s="2" t="n">
+      <c r="P84" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q84" t="inlineStr"/>
@@ -6147,7 +6135,7 @@
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
-      <c r="P85" s="2" t="n">
+      <c r="P85" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6218,7 +6206,7 @@
         </is>
       </c>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" s="2" t="n">
+      <c r="P86" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q86" t="inlineStr"/>
@@ -6285,7 +6273,7 @@
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" s="2" t="n">
+      <c r="P87" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q87" t="inlineStr"/>
@@ -6352,7 +6340,7 @@
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" s="2" t="n">
+      <c r="P88" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q88" t="inlineStr"/>
@@ -6419,7 +6407,7 @@
         </is>
       </c>
       <c r="O89" t="inlineStr"/>
-      <c r="P89" s="2" t="n">
+      <c r="P89" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q89" t="inlineStr"/>
@@ -6486,7 +6474,7 @@
         </is>
       </c>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" s="2" t="n">
+      <c r="P90" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q90" t="inlineStr"/>
@@ -6553,7 +6541,7 @@
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
-      <c r="P91" s="2" t="n">
+      <c r="P91" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="Q91" t="inlineStr"/>
@@ -6620,7 +6608,7 @@
         </is>
       </c>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" s="2" t="n">
+      <c r="P92" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="Q92" t="inlineStr"/>
@@ -6687,7 +6675,7 @@
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" s="2" t="n">
+      <c r="P93" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q93" t="inlineStr"/>
@@ -6754,7 +6742,7 @@
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" s="2" t="n">
+      <c r="P94" s="1" t="n">
         <v>46037</v>
       </c>
       <c r="Q94" t="inlineStr"/>
@@ -6890,7 +6878,7 @@
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
-      <c r="P96" s="2" t="n">
+      <c r="P96" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q96" t="inlineStr"/>
@@ -6957,7 +6945,7 @@
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
-      <c r="P97" s="2" t="n">
+      <c r="P97" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q97" t="inlineStr"/>
@@ -7154,7 +7142,7 @@
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
-      <c r="P100" s="2" t="n">
+      <c r="P100" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q100" t="inlineStr"/>
@@ -7221,7 +7209,7 @@
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
-      <c r="P101" s="2" t="n">
+      <c r="P101" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q101" t="inlineStr"/>
@@ -7288,7 +7276,7 @@
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
-      <c r="P102" s="2" t="n">
+      <c r="P102" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q102" t="inlineStr"/>
@@ -7355,7 +7343,7 @@
         </is>
       </c>
       <c r="O103" t="inlineStr"/>
-      <c r="P103" s="2" t="n">
+      <c r="P103" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q103" t="inlineStr"/>
@@ -7483,7 +7471,7 @@
         </is>
       </c>
       <c r="O105" t="inlineStr"/>
-      <c r="P105" s="2" t="n">
+      <c r="P105" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q105" t="inlineStr"/>
@@ -7550,7 +7538,7 @@
         </is>
       </c>
       <c r="O106" t="inlineStr"/>
-      <c r="P106" s="2" t="n">
+      <c r="P106" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q106" t="inlineStr">
@@ -7621,7 +7609,7 @@
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
-      <c r="P107" s="2" t="n">
+      <c r="P107" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -7688,7 +7676,7 @@
         </is>
       </c>
       <c r="O108" t="inlineStr"/>
-      <c r="P108" s="2" t="n">
+      <c r="P108" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -7885,7 +7873,7 @@
         </is>
       </c>
       <c r="O111" t="inlineStr"/>
-      <c r="P111" s="2" t="n">
+      <c r="P111" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -7952,7 +7940,7 @@
         </is>
       </c>
       <c r="O112" t="inlineStr"/>
-      <c r="P112" s="2" t="n">
+      <c r="P112" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -8084,7 +8072,7 @@
         </is>
       </c>
       <c r="O114" t="inlineStr"/>
-      <c r="P114" s="2" t="n">
+      <c r="P114" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q114" t="inlineStr"/>
@@ -8151,7 +8139,7 @@
         </is>
       </c>
       <c r="O115" t="inlineStr"/>
-      <c r="P115" s="2" t="n">
+      <c r="P115" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -8218,7 +8206,7 @@
         </is>
       </c>
       <c r="O116" t="inlineStr"/>
-      <c r="P116" s="2" t="n">
+      <c r="P116" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q116" t="inlineStr"/>
@@ -8285,7 +8273,7 @@
         </is>
       </c>
       <c r="O117" t="inlineStr"/>
-      <c r="P117" s="2" t="n">
+      <c r="P117" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="Q117" t="inlineStr"/>
@@ -8352,7 +8340,7 @@
         </is>
       </c>
       <c r="O118" t="inlineStr"/>
-      <c r="P118" s="2" t="n">
+      <c r="P118" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -8419,7 +8407,7 @@
         </is>
       </c>
       <c r="O119" t="inlineStr"/>
-      <c r="P119" s="2" t="n">
+      <c r="P119" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q119" t="inlineStr"/>
@@ -8486,7 +8474,7 @@
         </is>
       </c>
       <c r="O120" t="inlineStr"/>
-      <c r="P120" s="2" t="n">
+      <c r="P120" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q120" t="inlineStr"/>
@@ -8553,7 +8541,7 @@
         </is>
       </c>
       <c r="O121" t="inlineStr"/>
-      <c r="P121" s="2" t="n">
+      <c r="P121" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -8685,7 +8673,7 @@
         </is>
       </c>
       <c r="O123" t="inlineStr"/>
-      <c r="P123" s="2" t="n">
+      <c r="P123" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q123" t="inlineStr"/>
@@ -8947,7 +8935,7 @@
         </is>
       </c>
       <c r="O127" t="inlineStr"/>
-      <c r="P127" s="2" t="n">
+      <c r="P127" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q127" t="inlineStr"/>
@@ -9014,7 +9002,7 @@
         </is>
       </c>
       <c r="O128" t="inlineStr"/>
-      <c r="P128" s="2" t="n">
+      <c r="P128" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q128" t="inlineStr"/>
@@ -9081,7 +9069,7 @@
         </is>
       </c>
       <c r="O129" t="inlineStr"/>
-      <c r="P129" s="2" t="n">
+      <c r="P129" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q129" t="inlineStr"/>
@@ -9148,7 +9136,7 @@
         </is>
       </c>
       <c r="O130" t="inlineStr"/>
-      <c r="P130" s="2" t="n">
+      <c r="P130" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q130" t="inlineStr"/>
@@ -9215,7 +9203,7 @@
         </is>
       </c>
       <c r="O131" t="inlineStr"/>
-      <c r="P131" s="2" t="n">
+      <c r="P131" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -9282,7 +9270,7 @@
         </is>
       </c>
       <c r="O132" t="inlineStr"/>
-      <c r="P132" s="2" t="n">
+      <c r="P132" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -9349,7 +9337,7 @@
         </is>
       </c>
       <c r="O133" t="inlineStr"/>
-      <c r="P133" s="2" t="n">
+      <c r="P133" s="1" t="n">
         <v>46130</v>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -9481,7 +9469,7 @@
         </is>
       </c>
       <c r="O135" t="inlineStr"/>
-      <c r="P135" s="2" t="n">
+      <c r="P135" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q135" t="inlineStr"/>
@@ -9548,7 +9536,7 @@
         </is>
       </c>
       <c r="O136" t="inlineStr"/>
-      <c r="P136" s="2" t="n">
+      <c r="P136" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q136" t="inlineStr"/>
@@ -9680,7 +9668,7 @@
         </is>
       </c>
       <c r="O138" t="inlineStr"/>
-      <c r="P138" s="2" t="n">
+      <c r="P138" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q138" t="inlineStr"/>
@@ -9877,7 +9865,7 @@
         </is>
       </c>
       <c r="O141" t="inlineStr"/>
-      <c r="P141" s="2" t="n">
+      <c r="P141" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q141" t="inlineStr"/>
@@ -9944,7 +9932,7 @@
         </is>
       </c>
       <c r="O142" t="inlineStr"/>
-      <c r="P142" s="2" t="n">
+      <c r="P142" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q142" t="inlineStr"/>
@@ -10076,7 +10064,7 @@
         </is>
       </c>
       <c r="O144" t="inlineStr"/>
-      <c r="P144" s="2" t="n">
+      <c r="P144" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q144" t="inlineStr"/>
@@ -10143,7 +10131,7 @@
         </is>
       </c>
       <c r="O145" t="inlineStr"/>
-      <c r="P145" s="2" t="n">
+      <c r="P145" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q145" t="inlineStr"/>
@@ -10210,7 +10198,7 @@
         </is>
       </c>
       <c r="O146" t="inlineStr"/>
-      <c r="P146" s="2" t="n">
+      <c r="P146" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q146" t="inlineStr"/>
@@ -10277,7 +10265,7 @@
         </is>
       </c>
       <c r="O147" t="inlineStr"/>
-      <c r="P147" s="2" t="n">
+      <c r="P147" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="Q147" t="inlineStr"/>
@@ -10344,7 +10332,7 @@
         </is>
       </c>
       <c r="O148" t="inlineStr"/>
-      <c r="P148" s="2" t="n">
+      <c r="P148" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q148" t="inlineStr"/>
@@ -10411,7 +10399,7 @@
         </is>
       </c>
       <c r="O149" t="inlineStr"/>
-      <c r="P149" s="2" t="n">
+      <c r="P149" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q149" t="inlineStr"/>
@@ -10478,7 +10466,7 @@
         </is>
       </c>
       <c r="O150" t="inlineStr"/>
-      <c r="P150" s="2" t="n">
+      <c r="P150" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q150" t="inlineStr"/>
@@ -10545,7 +10533,7 @@
         </is>
       </c>
       <c r="O151" t="inlineStr"/>
-      <c r="P151" s="2" t="n">
+      <c r="P151" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q151" t="inlineStr"/>
@@ -10677,7 +10665,7 @@
         </is>
       </c>
       <c r="O153" t="inlineStr"/>
-      <c r="P153" s="2" t="n">
+      <c r="P153" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q153" t="inlineStr"/>
@@ -10939,7 +10927,7 @@
         </is>
       </c>
       <c r="O157" t="inlineStr"/>
-      <c r="P157" s="2" t="n">
+      <c r="P157" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q157" t="inlineStr"/>
@@ -11006,7 +10994,7 @@
         </is>
       </c>
       <c r="O158" t="inlineStr"/>
-      <c r="P158" s="2" t="n">
+      <c r="P158" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q158" t="inlineStr"/>
@@ -11073,7 +11061,7 @@
         </is>
       </c>
       <c r="O159" t="inlineStr"/>
-      <c r="P159" s="2" t="n">
+      <c r="P159" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q159" t="inlineStr"/>
@@ -11140,7 +11128,7 @@
         </is>
       </c>
       <c r="O160" t="inlineStr"/>
-      <c r="P160" s="2" t="n">
+      <c r="P160" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q160" t="inlineStr"/>
@@ -11272,7 +11260,7 @@
         </is>
       </c>
       <c r="O162" t="inlineStr"/>
-      <c r="P162" s="2" t="n">
+      <c r="P162" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q162" t="inlineStr"/>
@@ -11339,7 +11327,7 @@
         </is>
       </c>
       <c r="O163" t="inlineStr"/>
-      <c r="P163" s="2" t="n">
+      <c r="P163" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q163" t="inlineStr"/>
@@ -11406,7 +11394,7 @@
         </is>
       </c>
       <c r="O164" t="inlineStr"/>
-      <c r="P164" s="2" t="n">
+      <c r="P164" s="1" t="n">
         <v>45984</v>
       </c>
       <c r="Q164" t="inlineStr"/>
@@ -11473,7 +11461,7 @@
         </is>
       </c>
       <c r="O165" t="inlineStr"/>
-      <c r="P165" s="2" t="n">
+      <c r="P165" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q165" t="inlineStr"/>
@@ -11540,7 +11528,7 @@
         </is>
       </c>
       <c r="O166" t="inlineStr"/>
-      <c r="P166" s="2" t="n">
+      <c r="P166" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q166" t="inlineStr"/>
@@ -11607,7 +11595,7 @@
         </is>
       </c>
       <c r="O167" t="inlineStr"/>
-      <c r="P167" s="2" t="n">
+      <c r="P167" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q167" t="inlineStr"/>
@@ -11674,7 +11662,7 @@
         </is>
       </c>
       <c r="O168" t="inlineStr"/>
-      <c r="P168" s="2" t="n">
+      <c r="P168" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q168" t="inlineStr"/>
@@ -11741,7 +11729,7 @@
         </is>
       </c>
       <c r="O169" t="inlineStr"/>
-      <c r="P169" s="2" t="n">
+      <c r="P169" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q169" t="inlineStr"/>
@@ -11808,7 +11796,7 @@
         </is>
       </c>
       <c r="O170" t="inlineStr"/>
-      <c r="P170" s="2" t="n">
+      <c r="P170" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q170" t="inlineStr"/>
@@ -11875,7 +11863,7 @@
         </is>
       </c>
       <c r="O171" t="inlineStr"/>
-      <c r="P171" s="2" t="n">
+      <c r="P171" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q171" t="inlineStr"/>
@@ -11942,7 +11930,7 @@
         </is>
       </c>
       <c r="O172" t="inlineStr"/>
-      <c r="P172" s="2" t="n">
+      <c r="P172" s="1" t="n">
         <v>45954</v>
       </c>
       <c r="Q172" t="inlineStr"/>
@@ -12009,7 +11997,7 @@
         </is>
       </c>
       <c r="O173" t="inlineStr"/>
-      <c r="P173" s="2" t="n">
+      <c r="P173" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q173" t="inlineStr"/>
@@ -12076,7 +12064,7 @@
         </is>
       </c>
       <c r="O174" t="inlineStr"/>
-      <c r="P174" s="2" t="n">
+      <c r="P174" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q174" t="inlineStr"/>
@@ -12143,7 +12131,7 @@
         </is>
       </c>
       <c r="O175" t="inlineStr"/>
-      <c r="P175" s="2" t="n">
+      <c r="P175" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q175" t="inlineStr"/>
@@ -12210,7 +12198,7 @@
         </is>
       </c>
       <c r="O176" t="inlineStr"/>
-      <c r="P176" s="2" t="n">
+      <c r="P176" s="1" t="n">
         <v>45835</v>
       </c>
       <c r="Q176" t="inlineStr"/>
@@ -12277,7 +12265,7 @@
         </is>
       </c>
       <c r="O177" t="inlineStr"/>
-      <c r="P177" s="2" t="n">
+      <c r="P177" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q177" t="inlineStr"/>
@@ -12344,7 +12332,7 @@
         </is>
       </c>
       <c r="O178" t="inlineStr"/>
-      <c r="P178" s="2" t="n">
+      <c r="P178" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q178" t="inlineStr"/>
@@ -12411,7 +12399,7 @@
         </is>
       </c>
       <c r="O179" t="inlineStr"/>
-      <c r="P179" s="2" t="n">
+      <c r="P179" s="1" t="n">
         <v>45835</v>
       </c>
       <c r="Q179" t="inlineStr"/>
@@ -12478,7 +12466,7 @@
         </is>
       </c>
       <c r="O180" t="inlineStr"/>
-      <c r="P180" s="2" t="n">
+      <c r="P180" s="1" t="n">
         <v>46025</v>
       </c>
       <c r="Q180" t="inlineStr"/>
@@ -12545,7 +12533,7 @@
         </is>
       </c>
       <c r="O181" t="inlineStr"/>
-      <c r="P181" s="2" t="n">
+      <c r="P181" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q181" t="inlineStr"/>
@@ -12612,7 +12600,7 @@
         </is>
       </c>
       <c r="O182" t="inlineStr"/>
-      <c r="P182" s="2" t="n">
+      <c r="P182" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q182" t="inlineStr"/>
@@ -12744,7 +12732,7 @@
         </is>
       </c>
       <c r="O184" t="inlineStr"/>
-      <c r="P184" s="2" t="n">
+      <c r="P184" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q184" t="inlineStr"/>
@@ -12876,7 +12864,7 @@
         </is>
       </c>
       <c r="O186" t="inlineStr"/>
-      <c r="P186" s="2" t="n">
+      <c r="P186" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q186" t="inlineStr"/>
@@ -12896,87 +12884,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -13037,7 +13025,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="M2" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N2" t="inlineStr">
@@ -13104,7 +13092,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="M3" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N3" t="inlineStr">
@@ -13171,7 +13159,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="M4" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -13238,7 +13226,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="M5" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N5" t="inlineStr">
@@ -13305,7 +13293,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N6" t="inlineStr">
@@ -13372,7 +13360,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -13439,7 +13427,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="M8" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N8" t="inlineStr">
@@ -13506,7 +13494,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N9" t="inlineStr">
@@ -13573,7 +13561,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -13640,7 +13628,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="M11" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -13772,7 +13760,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M13" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N13" t="inlineStr">
@@ -13839,7 +13827,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="M14" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N14" t="inlineStr">
@@ -13906,7 +13894,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="M15" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N15" t="inlineStr">
@@ -13973,7 +13961,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="M16" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N16" t="inlineStr">
@@ -14040,7 +14028,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M17" s="2" t="n">
+      <c r="M17" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N17" t="inlineStr">
@@ -14107,7 +14095,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="M18" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N18" t="inlineStr">
@@ -14174,7 +14162,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="M19" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N19" t="inlineStr">
@@ -14241,7 +14229,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M20" s="2" t="n">
+      <c r="M20" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N20" t="inlineStr">
@@ -14308,7 +14296,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="M21" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N21" t="inlineStr">
@@ -14375,7 +14363,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="M22" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N22" t="inlineStr">
@@ -14442,7 +14430,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M23" s="2" t="n">
+      <c r="M23" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N23" t="inlineStr">
@@ -14509,7 +14497,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="M24" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N24" t="inlineStr">
@@ -14576,7 +14564,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="M25" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N25" t="inlineStr">
@@ -14643,7 +14631,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="M26" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N26" t="inlineStr">
@@ -14710,7 +14698,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="M27" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N27" t="inlineStr">
@@ -14777,7 +14765,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="M28" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N28" t="inlineStr">
@@ -14844,7 +14832,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M29" s="2" t="n">
+      <c r="M29" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N29" t="inlineStr">
@@ -14911,7 +14899,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="M30" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N30" t="inlineStr">
@@ -14978,7 +14966,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="M31" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N31" t="inlineStr">
@@ -15045,7 +15033,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M32" s="2" t="n">
+      <c r="M32" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N32" t="inlineStr">
@@ -15112,7 +15100,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="M33" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N33" t="inlineStr">
@@ -15179,7 +15167,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M34" s="2" t="n">
+      <c r="M34" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N34" t="inlineStr">
@@ -15246,7 +15234,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M35" s="2" t="n">
+      <c r="M35" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N35" t="inlineStr">
@@ -15313,7 +15301,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M36" s="2" t="n">
+      <c r="M36" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N36" t="inlineStr">
@@ -15380,7 +15368,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="M37" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N37" t="inlineStr">
@@ -15447,7 +15435,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="M38" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N38" t="inlineStr">
@@ -15514,7 +15502,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M39" s="2" t="n">
+      <c r="M39" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N39" t="inlineStr">
@@ -15581,7 +15569,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M40" s="2" t="n">
+      <c r="M40" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N40" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: tpjl (10/07/2026 16:01)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +49,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -422,87 +434,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -570,7 +582,7 @@
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" s="1" t="n">
+      <c r="P2" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -637,7 +649,7 @@
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" s="1" t="n">
+      <c r="P3" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -704,7 +716,7 @@
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" s="1" t="n">
+      <c r="P4" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -901,7 +913,7 @@
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" s="1" t="n">
+      <c r="P7" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -968,7 +980,7 @@
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" s="1" t="n">
+      <c r="P8" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1035,7 +1047,7 @@
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" s="1" t="n">
+      <c r="P9" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1106,7 +1118,7 @@
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" s="1" t="n">
+      <c r="P10" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1299,7 +1311,7 @@
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" s="1" t="n">
+      <c r="P13" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -1366,7 +1378,7 @@
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" s="1" t="n">
+      <c r="P14" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -1433,7 +1445,7 @@
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" s="1" t="n">
+      <c r="P15" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -1500,7 +1512,7 @@
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" s="1" t="n">
+      <c r="P16" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1571,7 +1583,7 @@
         </is>
       </c>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" s="1" t="n">
+      <c r="P17" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -1638,7 +1650,7 @@
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" s="1" t="n">
+      <c r="P18" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -1835,7 +1847,7 @@
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" s="1" t="n">
+      <c r="P21" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -1902,7 +1914,7 @@
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" s="1" t="n">
+      <c r="P22" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -2034,7 +2046,7 @@
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" s="1" t="n">
+      <c r="P24" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2105,7 +2117,7 @@
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" s="1" t="n">
+      <c r="P25" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2176,7 +2188,7 @@
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" s="1" t="n">
+      <c r="P26" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -2243,7 +2255,7 @@
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" s="1" t="n">
+      <c r="P27" s="2" t="n">
         <v>45964</v>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -2310,7 +2322,7 @@
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" s="1" t="n">
+      <c r="P28" s="2" t="n">
         <v>45984</v>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -2442,7 +2454,7 @@
         </is>
       </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" s="1" t="n">
+      <c r="P30" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q30" t="inlineStr"/>
@@ -2574,7 +2586,7 @@
         </is>
       </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" s="1" t="n">
+      <c r="P32" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2645,7 +2657,7 @@
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" s="1" t="n">
+      <c r="P33" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -2712,7 +2724,7 @@
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
-      <c r="P34" s="1" t="n">
+      <c r="P34" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -2779,7 +2791,7 @@
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" s="1" t="n">
+      <c r="P35" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -2911,7 +2923,7 @@
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" s="1" t="n">
+      <c r="P37" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -2978,7 +2990,7 @@
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" s="1" t="n">
+      <c r="P38" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -3045,7 +3057,7 @@
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" s="1" t="n">
+      <c r="P39" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q39" t="inlineStr"/>
@@ -3177,7 +3189,7 @@
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" s="1" t="n">
+      <c r="P41" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q41" t="inlineStr"/>
@@ -3244,7 +3256,7 @@
         </is>
       </c>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" s="1" t="n">
+      <c r="P42" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -3311,7 +3323,7 @@
         </is>
       </c>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" s="1" t="n">
+      <c r="P43" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -3378,7 +3390,7 @@
         </is>
       </c>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" s="1" t="n">
+      <c r="P44" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -3640,7 +3652,7 @@
         </is>
       </c>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" s="1" t="n">
+      <c r="P48" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -3707,7 +3719,7 @@
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" s="1" t="n">
+      <c r="P49" s="2" t="n">
         <v>45955</v>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -3774,7 +3786,7 @@
         </is>
       </c>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" s="1" t="n">
+      <c r="P50" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -3841,7 +3853,7 @@
         </is>
       </c>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" s="1" t="n">
+      <c r="P51" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q51" t="inlineStr">
@@ -3912,7 +3924,7 @@
         </is>
       </c>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" s="1" t="n">
+      <c r="P52" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -3979,7 +3991,7 @@
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" s="1" t="n">
+      <c r="P53" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -4107,7 +4119,7 @@
         </is>
       </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" s="1" t="n">
+      <c r="P55" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -4174,7 +4186,7 @@
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" s="1" t="n">
+      <c r="P56" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -4310,7 +4322,7 @@
         </is>
       </c>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" s="1" t="n">
+      <c r="P58" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -4377,7 +4389,7 @@
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" s="1" t="n">
+      <c r="P59" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q59" t="inlineStr">
@@ -4448,7 +4460,7 @@
         </is>
       </c>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" s="1" t="n">
+      <c r="P60" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -4515,7 +4527,7 @@
         </is>
       </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" s="1" t="n">
+      <c r="P61" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q61" t="inlineStr"/>
@@ -4582,7 +4594,7 @@
         </is>
       </c>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" s="1" t="n">
+      <c r="P62" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q62" t="inlineStr"/>
@@ -4649,7 +4661,7 @@
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" s="1" t="n">
+      <c r="P63" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q63" t="inlineStr"/>
@@ -4716,7 +4728,7 @@
         </is>
       </c>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" s="1" t="n">
+      <c r="P64" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q64" t="inlineStr">
@@ -4787,7 +4799,7 @@
         </is>
       </c>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" s="1" t="n">
+      <c r="P65" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q65" t="inlineStr"/>
@@ -4854,7 +4866,7 @@
         </is>
       </c>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" s="1" t="n">
+      <c r="P66" s="2" t="n">
         <v>45946</v>
       </c>
       <c r="Q66" t="inlineStr">
@@ -4925,7 +4937,7 @@
         </is>
       </c>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" s="1" t="n">
+      <c r="P67" s="2" t="n">
         <v>45916</v>
       </c>
       <c r="Q67" t="inlineStr"/>
@@ -4992,7 +5004,7 @@
         </is>
       </c>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" s="1" t="n">
+      <c r="P68" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5063,7 +5075,7 @@
         </is>
       </c>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" s="1" t="n">
+      <c r="P69" s="2" t="n">
         <v>45989</v>
       </c>
       <c r="Q69" t="inlineStr">
@@ -5199,7 +5211,7 @@
         </is>
       </c>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" s="1" t="n">
+      <c r="P71" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -5266,7 +5278,7 @@
         </is>
       </c>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" s="1" t="n">
+      <c r="P72" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q72" t="inlineStr"/>
@@ -5333,7 +5345,7 @@
         </is>
       </c>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" s="1" t="n">
+      <c r="P73" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q73" t="inlineStr"/>
@@ -5400,7 +5412,7 @@
         </is>
       </c>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" s="1" t="n">
+      <c r="P74" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q74" t="inlineStr"/>
@@ -5467,7 +5479,7 @@
         </is>
       </c>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" s="1" t="n">
+      <c r="P75" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q75" t="inlineStr"/>
@@ -5534,7 +5546,7 @@
         </is>
       </c>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" s="1" t="n">
+      <c r="P76" s="2" t="n">
         <v>46130</v>
       </c>
       <c r="Q76" t="inlineStr"/>
@@ -5666,7 +5678,7 @@
         </is>
       </c>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" s="1" t="n">
+      <c r="P78" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q78" t="inlineStr"/>
@@ -5733,7 +5745,7 @@
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
-      <c r="P79" s="1" t="n">
+      <c r="P79" s="2" t="n">
         <v>46140</v>
       </c>
       <c r="Q79" t="inlineStr"/>
@@ -5800,7 +5812,7 @@
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" s="1" t="n">
+      <c r="P80" s="2" t="n">
         <v>46095</v>
       </c>
       <c r="Q80" t="inlineStr"/>
@@ -5867,7 +5879,7 @@
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" s="1" t="n">
+      <c r="P81" s="2" t="n">
         <v>46040</v>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -5934,7 +5946,7 @@
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" s="1" t="n">
+      <c r="P82" s="2" t="n">
         <v>46060</v>
       </c>
       <c r="Q82" t="inlineStr"/>
@@ -6001,7 +6013,7 @@
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" s="1" t="n">
+      <c r="P83" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -6068,7 +6080,7 @@
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" s="1" t="n">
+      <c r="P84" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q84" t="inlineStr"/>
@@ -6135,7 +6147,7 @@
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
-      <c r="P85" s="1" t="n">
+      <c r="P85" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6206,7 +6218,7 @@
         </is>
       </c>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" s="1" t="n">
+      <c r="P86" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q86" t="inlineStr"/>
@@ -6273,7 +6285,7 @@
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" s="1" t="n">
+      <c r="P87" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q87" t="inlineStr"/>
@@ -6340,7 +6352,7 @@
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" s="1" t="n">
+      <c r="P88" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q88" t="inlineStr"/>
@@ -6407,7 +6419,7 @@
         </is>
       </c>
       <c r="O89" t="inlineStr"/>
-      <c r="P89" s="1" t="n">
+      <c r="P89" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q89" t="inlineStr"/>
@@ -6474,7 +6486,7 @@
         </is>
       </c>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" s="1" t="n">
+      <c r="P90" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q90" t="inlineStr"/>
@@ -6541,7 +6553,7 @@
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
-      <c r="P91" s="1" t="n">
+      <c r="P91" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="Q91" t="inlineStr"/>
@@ -6608,7 +6620,7 @@
         </is>
       </c>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" s="1" t="n">
+      <c r="P92" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="Q92" t="inlineStr"/>
@@ -6675,7 +6687,7 @@
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" s="1" t="n">
+      <c r="P93" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q93" t="inlineStr"/>
@@ -6742,7 +6754,7 @@
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" s="1" t="n">
+      <c r="P94" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="Q94" t="inlineStr"/>
@@ -6878,7 +6890,7 @@
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
-      <c r="P96" s="1" t="n">
+      <c r="P96" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q96" t="inlineStr"/>
@@ -6945,7 +6957,7 @@
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
-      <c r="P97" s="1" t="n">
+      <c r="P97" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q97" t="inlineStr"/>
@@ -7142,7 +7154,7 @@
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
-      <c r="P100" s="1" t="n">
+      <c r="P100" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q100" t="inlineStr"/>
@@ -7209,7 +7221,7 @@
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
-      <c r="P101" s="1" t="n">
+      <c r="P101" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q101" t="inlineStr"/>
@@ -7276,7 +7288,7 @@
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
-      <c r="P102" s="1" t="n">
+      <c r="P102" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q102" t="inlineStr"/>
@@ -7343,7 +7355,7 @@
         </is>
       </c>
       <c r="O103" t="inlineStr"/>
-      <c r="P103" s="1" t="n">
+      <c r="P103" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q103" t="inlineStr"/>
@@ -7471,7 +7483,7 @@
         </is>
       </c>
       <c r="O105" t="inlineStr"/>
-      <c r="P105" s="1" t="n">
+      <c r="P105" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="Q105" t="inlineStr"/>
@@ -7538,7 +7550,7 @@
         </is>
       </c>
       <c r="O106" t="inlineStr"/>
-      <c r="P106" s="1" t="n">
+      <c r="P106" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q106" t="inlineStr">
@@ -7609,7 +7621,7 @@
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
-      <c r="P107" s="1" t="n">
+      <c r="P107" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -7676,7 +7688,7 @@
         </is>
       </c>
       <c r="O108" t="inlineStr"/>
-      <c r="P108" s="1" t="n">
+      <c r="P108" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -7873,7 +7885,7 @@
         </is>
       </c>
       <c r="O111" t="inlineStr"/>
-      <c r="P111" s="1" t="n">
+      <c r="P111" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -7940,7 +7952,7 @@
         </is>
       </c>
       <c r="O112" t="inlineStr"/>
-      <c r="P112" s="1" t="n">
+      <c r="P112" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -8072,7 +8084,7 @@
         </is>
       </c>
       <c r="O114" t="inlineStr"/>
-      <c r="P114" s="1" t="n">
+      <c r="P114" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="Q114" t="inlineStr"/>
@@ -8139,7 +8151,7 @@
         </is>
       </c>
       <c r="O115" t="inlineStr"/>
-      <c r="P115" s="1" t="n">
+      <c r="P115" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -8206,7 +8218,7 @@
         </is>
       </c>
       <c r="O116" t="inlineStr"/>
-      <c r="P116" s="1" t="n">
+      <c r="P116" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q116" t="inlineStr"/>
@@ -8273,7 +8285,7 @@
         </is>
       </c>
       <c r="O117" t="inlineStr"/>
-      <c r="P117" s="1" t="n">
+      <c r="P117" s="2" t="n">
         <v>46081</v>
       </c>
       <c r="Q117" t="inlineStr"/>
@@ -8340,7 +8352,7 @@
         </is>
       </c>
       <c r="O118" t="inlineStr"/>
-      <c r="P118" s="1" t="n">
+      <c r="P118" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -8407,7 +8419,7 @@
         </is>
       </c>
       <c r="O119" t="inlineStr"/>
-      <c r="P119" s="1" t="n">
+      <c r="P119" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q119" t="inlineStr"/>
@@ -8474,7 +8486,7 @@
         </is>
       </c>
       <c r="O120" t="inlineStr"/>
-      <c r="P120" s="1" t="n">
+      <c r="P120" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q120" t="inlineStr"/>
@@ -8541,7 +8553,7 @@
         </is>
       </c>
       <c r="O121" t="inlineStr"/>
-      <c r="P121" s="1" t="n">
+      <c r="P121" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -8673,7 +8685,7 @@
         </is>
       </c>
       <c r="O123" t="inlineStr"/>
-      <c r="P123" s="1" t="n">
+      <c r="P123" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q123" t="inlineStr"/>
@@ -8935,7 +8947,7 @@
         </is>
       </c>
       <c r="O127" t="inlineStr"/>
-      <c r="P127" s="1" t="n">
+      <c r="P127" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="Q127" t="inlineStr"/>
@@ -9002,7 +9014,7 @@
         </is>
       </c>
       <c r="O128" t="inlineStr"/>
-      <c r="P128" s="1" t="n">
+      <c r="P128" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q128" t="inlineStr"/>
@@ -9069,7 +9081,7 @@
         </is>
       </c>
       <c r="O129" t="inlineStr"/>
-      <c r="P129" s="1" t="n">
+      <c r="P129" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q129" t="inlineStr"/>
@@ -9136,7 +9148,7 @@
         </is>
       </c>
       <c r="O130" t="inlineStr"/>
-      <c r="P130" s="1" t="n">
+      <c r="P130" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q130" t="inlineStr"/>
@@ -9203,7 +9215,7 @@
         </is>
       </c>
       <c r="O131" t="inlineStr"/>
-      <c r="P131" s="1" t="n">
+      <c r="P131" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -9270,7 +9282,7 @@
         </is>
       </c>
       <c r="O132" t="inlineStr"/>
-      <c r="P132" s="1" t="n">
+      <c r="P132" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -9337,7 +9349,7 @@
         </is>
       </c>
       <c r="O133" t="inlineStr"/>
-      <c r="P133" s="1" t="n">
+      <c r="P133" s="2" t="n">
         <v>46130</v>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -9469,7 +9481,7 @@
         </is>
       </c>
       <c r="O135" t="inlineStr"/>
-      <c r="P135" s="1" t="n">
+      <c r="P135" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q135" t="inlineStr"/>
@@ -9536,7 +9548,7 @@
         </is>
       </c>
       <c r="O136" t="inlineStr"/>
-      <c r="P136" s="1" t="n">
+      <c r="P136" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q136" t="inlineStr"/>
@@ -9668,7 +9680,7 @@
         </is>
       </c>
       <c r="O138" t="inlineStr"/>
-      <c r="P138" s="1" t="n">
+      <c r="P138" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q138" t="inlineStr"/>
@@ -9865,7 +9877,7 @@
         </is>
       </c>
       <c r="O141" t="inlineStr"/>
-      <c r="P141" s="1" t="n">
+      <c r="P141" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q141" t="inlineStr"/>
@@ -9932,7 +9944,7 @@
         </is>
       </c>
       <c r="O142" t="inlineStr"/>
-      <c r="P142" s="1" t="n">
+      <c r="P142" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q142" t="inlineStr"/>
@@ -10064,7 +10076,7 @@
         </is>
       </c>
       <c r="O144" t="inlineStr"/>
-      <c r="P144" s="1" t="n">
+      <c r="P144" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="Q144" t="inlineStr"/>
@@ -10131,7 +10143,7 @@
         </is>
       </c>
       <c r="O145" t="inlineStr"/>
-      <c r="P145" s="1" t="n">
+      <c r="P145" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q145" t="inlineStr"/>
@@ -10198,7 +10210,7 @@
         </is>
       </c>
       <c r="O146" t="inlineStr"/>
-      <c r="P146" s="1" t="n">
+      <c r="P146" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q146" t="inlineStr"/>
@@ -10265,7 +10277,7 @@
         </is>
       </c>
       <c r="O147" t="inlineStr"/>
-      <c r="P147" s="1" t="n">
+      <c r="P147" s="2" t="n">
         <v>46081</v>
       </c>
       <c r="Q147" t="inlineStr"/>
@@ -10332,7 +10344,7 @@
         </is>
       </c>
       <c r="O148" t="inlineStr"/>
-      <c r="P148" s="1" t="n">
+      <c r="P148" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q148" t="inlineStr"/>
@@ -10399,7 +10411,7 @@
         </is>
       </c>
       <c r="O149" t="inlineStr"/>
-      <c r="P149" s="1" t="n">
+      <c r="P149" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q149" t="inlineStr"/>
@@ -10466,7 +10478,7 @@
         </is>
       </c>
       <c r="O150" t="inlineStr"/>
-      <c r="P150" s="1" t="n">
+      <c r="P150" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q150" t="inlineStr"/>
@@ -10533,7 +10545,7 @@
         </is>
       </c>
       <c r="O151" t="inlineStr"/>
-      <c r="P151" s="1" t="n">
+      <c r="P151" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q151" t="inlineStr"/>
@@ -10665,7 +10677,7 @@
         </is>
       </c>
       <c r="O153" t="inlineStr"/>
-      <c r="P153" s="1" t="n">
+      <c r="P153" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q153" t="inlineStr"/>
@@ -10927,7 +10939,7 @@
         </is>
       </c>
       <c r="O157" t="inlineStr"/>
-      <c r="P157" s="1" t="n">
+      <c r="P157" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="Q157" t="inlineStr"/>
@@ -10994,7 +11006,7 @@
         </is>
       </c>
       <c r="O158" t="inlineStr"/>
-      <c r="P158" s="1" t="n">
+      <c r="P158" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q158" t="inlineStr"/>
@@ -11061,7 +11073,7 @@
         </is>
       </c>
       <c r="O159" t="inlineStr"/>
-      <c r="P159" s="1" t="n">
+      <c r="P159" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q159" t="inlineStr"/>
@@ -11128,7 +11140,7 @@
         </is>
       </c>
       <c r="O160" t="inlineStr"/>
-      <c r="P160" s="1" t="n">
+      <c r="P160" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q160" t="inlineStr"/>
@@ -11260,7 +11272,7 @@
         </is>
       </c>
       <c r="O162" t="inlineStr"/>
-      <c r="P162" s="1" t="n">
+      <c r="P162" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q162" t="inlineStr"/>
@@ -11327,7 +11339,7 @@
         </is>
       </c>
       <c r="O163" t="inlineStr"/>
-      <c r="P163" s="1" t="n">
+      <c r="P163" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q163" t="inlineStr"/>
@@ -11394,7 +11406,7 @@
         </is>
       </c>
       <c r="O164" t="inlineStr"/>
-      <c r="P164" s="1" t="n">
+      <c r="P164" s="2" t="n">
         <v>45984</v>
       </c>
       <c r="Q164" t="inlineStr"/>
@@ -11461,7 +11473,7 @@
         </is>
       </c>
       <c r="O165" t="inlineStr"/>
-      <c r="P165" s="1" t="n">
+      <c r="P165" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q165" t="inlineStr"/>
@@ -11528,7 +11540,7 @@
         </is>
       </c>
       <c r="O166" t="inlineStr"/>
-      <c r="P166" s="1" t="n">
+      <c r="P166" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q166" t="inlineStr"/>
@@ -11595,7 +11607,7 @@
         </is>
       </c>
       <c r="O167" t="inlineStr"/>
-      <c r="P167" s="1" t="n">
+      <c r="P167" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q167" t="inlineStr"/>
@@ -11662,7 +11674,7 @@
         </is>
       </c>
       <c r="O168" t="inlineStr"/>
-      <c r="P168" s="1" t="n">
+      <c r="P168" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q168" t="inlineStr"/>
@@ -11729,7 +11741,7 @@
         </is>
       </c>
       <c r="O169" t="inlineStr"/>
-      <c r="P169" s="1" t="n">
+      <c r="P169" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q169" t="inlineStr"/>
@@ -11796,7 +11808,7 @@
         </is>
       </c>
       <c r="O170" t="inlineStr"/>
-      <c r="P170" s="1" t="n">
+      <c r="P170" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q170" t="inlineStr"/>
@@ -11863,7 +11875,7 @@
         </is>
       </c>
       <c r="O171" t="inlineStr"/>
-      <c r="P171" s="1" t="n">
+      <c r="P171" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q171" t="inlineStr"/>
@@ -11930,7 +11942,7 @@
         </is>
       </c>
       <c r="O172" t="inlineStr"/>
-      <c r="P172" s="1" t="n">
+      <c r="P172" s="2" t="n">
         <v>45954</v>
       </c>
       <c r="Q172" t="inlineStr"/>
@@ -11997,7 +12009,7 @@
         </is>
       </c>
       <c r="O173" t="inlineStr"/>
-      <c r="P173" s="1" t="n">
+      <c r="P173" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q173" t="inlineStr"/>
@@ -12064,7 +12076,7 @@
         </is>
       </c>
       <c r="O174" t="inlineStr"/>
-      <c r="P174" s="1" t="n">
+      <c r="P174" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q174" t="inlineStr"/>
@@ -12131,7 +12143,7 @@
         </is>
       </c>
       <c r="O175" t="inlineStr"/>
-      <c r="P175" s="1" t="n">
+      <c r="P175" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q175" t="inlineStr"/>
@@ -12198,7 +12210,7 @@
         </is>
       </c>
       <c r="O176" t="inlineStr"/>
-      <c r="P176" s="1" t="n">
+      <c r="P176" s="2" t="n">
         <v>45835</v>
       </c>
       <c r="Q176" t="inlineStr"/>
@@ -12265,7 +12277,7 @@
         </is>
       </c>
       <c r="O177" t="inlineStr"/>
-      <c r="P177" s="1" t="n">
+      <c r="P177" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q177" t="inlineStr"/>
@@ -12332,7 +12344,7 @@
         </is>
       </c>
       <c r="O178" t="inlineStr"/>
-      <c r="P178" s="1" t="n">
+      <c r="P178" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q178" t="inlineStr"/>
@@ -12399,7 +12411,7 @@
         </is>
       </c>
       <c r="O179" t="inlineStr"/>
-      <c r="P179" s="1" t="n">
+      <c r="P179" s="2" t="n">
         <v>45835</v>
       </c>
       <c r="Q179" t="inlineStr"/>
@@ -12466,7 +12478,7 @@
         </is>
       </c>
       <c r="O180" t="inlineStr"/>
-      <c r="P180" s="1" t="n">
+      <c r="P180" s="2" t="n">
         <v>46025</v>
       </c>
       <c r="Q180" t="inlineStr"/>
@@ -12533,7 +12545,7 @@
         </is>
       </c>
       <c r="O181" t="inlineStr"/>
-      <c r="P181" s="1" t="n">
+      <c r="P181" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q181" t="inlineStr"/>
@@ -12600,7 +12612,7 @@
         </is>
       </c>
       <c r="O182" t="inlineStr"/>
-      <c r="P182" s="1" t="n">
+      <c r="P182" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q182" t="inlineStr"/>
@@ -12732,7 +12744,7 @@
         </is>
       </c>
       <c r="O184" t="inlineStr"/>
-      <c r="P184" s="1" t="n">
+      <c r="P184" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q184" t="inlineStr"/>
@@ -12864,7 +12876,7 @@
         </is>
       </c>
       <c r="O186" t="inlineStr"/>
-      <c r="P186" s="1" t="n">
+      <c r="P186" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q186" t="inlineStr"/>
@@ -12884,87 +12896,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -13025,7 +13037,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M2" s="1" t="n">
+      <c r="M2" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N2" t="inlineStr">
@@ -13092,7 +13104,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M3" s="1" t="n">
+      <c r="M3" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N3" t="inlineStr">
@@ -13159,7 +13171,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M4" s="1" t="n">
+      <c r="M4" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -13226,7 +13238,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M5" s="1" t="n">
+      <c r="M5" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N5" t="inlineStr">
@@ -13293,7 +13305,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M6" s="1" t="n">
+      <c r="M6" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N6" t="inlineStr">
@@ -13360,7 +13372,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M7" s="1" t="n">
+      <c r="M7" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -13427,7 +13439,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M8" s="1" t="n">
+      <c r="M8" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N8" t="inlineStr">
@@ -13494,7 +13506,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M9" s="1" t="n">
+      <c r="M9" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N9" t="inlineStr">
@@ -13561,7 +13573,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M10" s="1" t="n">
+      <c r="M10" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -13628,7 +13640,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M11" s="1" t="n">
+      <c r="M11" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -13760,7 +13772,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M13" s="1" t="n">
+      <c r="M13" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N13" t="inlineStr">
@@ -13827,7 +13839,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M14" s="1" t="n">
+      <c r="M14" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N14" t="inlineStr">
@@ -13894,7 +13906,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M15" s="1" t="n">
+      <c r="M15" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N15" t="inlineStr">
@@ -13961,7 +13973,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M16" s="1" t="n">
+      <c r="M16" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N16" t="inlineStr">
@@ -14028,7 +14040,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M17" s="1" t="n">
+      <c r="M17" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N17" t="inlineStr">
@@ -14095,7 +14107,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M18" s="1" t="n">
+      <c r="M18" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N18" t="inlineStr">
@@ -14162,7 +14174,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M19" s="1" t="n">
+      <c r="M19" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N19" t="inlineStr">
@@ -14229,7 +14241,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M20" s="1" t="n">
+      <c r="M20" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N20" t="inlineStr">
@@ -14296,7 +14308,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M21" s="1" t="n">
+      <c r="M21" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N21" t="inlineStr">
@@ -14363,7 +14375,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M22" s="1" t="n">
+      <c r="M22" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N22" t="inlineStr">
@@ -14430,7 +14442,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M23" s="1" t="n">
+      <c r="M23" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N23" t="inlineStr">
@@ -14497,7 +14509,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M24" s="1" t="n">
+      <c r="M24" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N24" t="inlineStr">
@@ -14564,7 +14576,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M25" s="1" t="n">
+      <c r="M25" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N25" t="inlineStr">
@@ -14631,7 +14643,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M26" s="1" t="n">
+      <c r="M26" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N26" t="inlineStr">
@@ -14698,7 +14710,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M27" s="1" t="n">
+      <c r="M27" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N27" t="inlineStr">
@@ -14765,7 +14777,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M28" s="1" t="n">
+      <c r="M28" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N28" t="inlineStr">
@@ -14832,7 +14844,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M29" s="1" t="n">
+      <c r="M29" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N29" t="inlineStr">
@@ -14899,7 +14911,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M30" s="1" t="n">
+      <c r="M30" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N30" t="inlineStr">
@@ -14966,7 +14978,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M31" s="1" t="n">
+      <c r="M31" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N31" t="inlineStr">
@@ -15033,7 +15045,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M32" s="1" t="n">
+      <c r="M32" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N32" t="inlineStr">
@@ -15100,7 +15112,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M33" s="1" t="n">
+      <c r="M33" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N33" t="inlineStr">
@@ -15167,7 +15179,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M34" s="1" t="n">
+      <c r="M34" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N34" t="inlineStr">
@@ -15234,7 +15246,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M35" s="1" t="n">
+      <c r="M35" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N35" t="inlineStr">
@@ -15301,7 +15313,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M36" s="1" t="n">
+      <c r="M36" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N36" t="inlineStr">
@@ -15368,7 +15380,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M37" s="1" t="n">
+      <c r="M37" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N37" t="inlineStr">
@@ -15435,7 +15447,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M38" s="1" t="n">
+      <c r="M38" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N38" t="inlineStr">
@@ -15502,7 +15514,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M39" s="1" t="n">
+      <c r="M39" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N39" t="inlineStr">
@@ -15569,7 +15581,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M40" s="1" t="n">
+      <c r="M40" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N40" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: tpjl (10/07/2026 22:39)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,87 +422,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -582,7 +570,7 @@
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -649,7 +637,7 @@
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" s="2" t="n">
+      <c r="P3" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -716,7 +704,7 @@
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" s="2" t="n">
+      <c r="P4" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -913,7 +901,7 @@
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -980,7 +968,7 @@
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" s="2" t="n">
+      <c r="P8" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1047,7 +1035,7 @@
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1118,7 +1106,7 @@
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" s="2" t="n">
+      <c r="P10" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1311,7 +1299,7 @@
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" s="2" t="n">
+      <c r="P13" s="1" t="n">
         <v>46037</v>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -1378,7 +1366,7 @@
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" s="2" t="n">
+      <c r="P14" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -1445,7 +1433,7 @@
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" s="2" t="n">
+      <c r="P15" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -1512,7 +1500,7 @@
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" s="2" t="n">
+      <c r="P16" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1583,7 +1571,7 @@
         </is>
       </c>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" s="2" t="n">
+      <c r="P17" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -1650,7 +1638,7 @@
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" s="2" t="n">
+      <c r="P18" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -1847,7 +1835,7 @@
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" s="2" t="n">
+      <c r="P21" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -1914,7 +1902,7 @@
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" s="2" t="n">
+      <c r="P22" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -2046,7 +2034,7 @@
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" s="2" t="n">
+      <c r="P24" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2117,7 +2105,7 @@
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" s="2" t="n">
+      <c r="P25" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2188,7 +2176,7 @@
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" s="2" t="n">
+      <c r="P26" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -2255,7 +2243,7 @@
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" s="2" t="n">
+      <c r="P27" s="1" t="n">
         <v>45964</v>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -2322,7 +2310,7 @@
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" s="2" t="n">
+      <c r="P28" s="1" t="n">
         <v>45984</v>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -2454,7 +2442,7 @@
         </is>
       </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" s="2" t="n">
+      <c r="P30" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q30" t="inlineStr"/>
@@ -2586,7 +2574,7 @@
         </is>
       </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" s="2" t="n">
+      <c r="P32" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2657,7 +2645,7 @@
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" s="2" t="n">
+      <c r="P33" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -2724,7 +2712,7 @@
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
-      <c r="P34" s="2" t="n">
+      <c r="P34" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -2791,7 +2779,7 @@
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" s="2" t="n">
+      <c r="P35" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -2923,7 +2911,7 @@
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" s="2" t="n">
+      <c r="P37" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -2990,7 +2978,7 @@
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" s="2" t="n">
+      <c r="P38" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -3057,7 +3045,7 @@
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" s="2" t="n">
+      <c r="P39" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q39" t="inlineStr"/>
@@ -3189,7 +3177,7 @@
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" s="2" t="n">
+      <c r="P41" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q41" t="inlineStr"/>
@@ -3256,7 +3244,7 @@
         </is>
       </c>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" s="2" t="n">
+      <c r="P42" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -3323,7 +3311,7 @@
         </is>
       </c>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" s="2" t="n">
+      <c r="P43" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -3390,7 +3378,7 @@
         </is>
       </c>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" s="2" t="n">
+      <c r="P44" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -3652,7 +3640,7 @@
         </is>
       </c>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" s="2" t="n">
+      <c r="P48" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -3719,7 +3707,7 @@
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" s="2" t="n">
+      <c r="P49" s="1" t="n">
         <v>45955</v>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -3786,7 +3774,7 @@
         </is>
       </c>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" s="2" t="n">
+      <c r="P50" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -3853,7 +3841,7 @@
         </is>
       </c>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" s="2" t="n">
+      <c r="P51" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q51" t="inlineStr">
@@ -3924,7 +3912,7 @@
         </is>
       </c>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" s="2" t="n">
+      <c r="P52" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -3991,7 +3979,7 @@
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" s="2" t="n">
+      <c r="P53" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -4119,7 +4107,7 @@
         </is>
       </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" s="2" t="n">
+      <c r="P55" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -4186,7 +4174,7 @@
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" s="2" t="n">
+      <c r="P56" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -4322,7 +4310,7 @@
         </is>
       </c>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" s="2" t="n">
+      <c r="P58" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -4389,7 +4377,7 @@
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" s="2" t="n">
+      <c r="P59" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q59" t="inlineStr">
@@ -4460,7 +4448,7 @@
         </is>
       </c>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" s="2" t="n">
+      <c r="P60" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -4527,7 +4515,7 @@
         </is>
       </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" s="2" t="n">
+      <c r="P61" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q61" t="inlineStr"/>
@@ -4594,7 +4582,7 @@
         </is>
       </c>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" s="2" t="n">
+      <c r="P62" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q62" t="inlineStr"/>
@@ -4661,7 +4649,7 @@
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" s="2" t="n">
+      <c r="P63" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q63" t="inlineStr"/>
@@ -4728,7 +4716,7 @@
         </is>
       </c>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" s="2" t="n">
+      <c r="P64" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q64" t="inlineStr">
@@ -4799,7 +4787,7 @@
         </is>
       </c>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" s="2" t="n">
+      <c r="P65" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q65" t="inlineStr"/>
@@ -4866,7 +4854,7 @@
         </is>
       </c>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" s="2" t="n">
+      <c r="P66" s="1" t="n">
         <v>45946</v>
       </c>
       <c r="Q66" t="inlineStr">
@@ -4937,7 +4925,7 @@
         </is>
       </c>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" s="2" t="n">
+      <c r="P67" s="1" t="n">
         <v>45916</v>
       </c>
       <c r="Q67" t="inlineStr"/>
@@ -5004,7 +4992,7 @@
         </is>
       </c>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" s="2" t="n">
+      <c r="P68" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5075,7 +5063,7 @@
         </is>
       </c>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" s="2" t="n">
+      <c r="P69" s="1" t="n">
         <v>45989</v>
       </c>
       <c r="Q69" t="inlineStr">
@@ -5211,7 +5199,7 @@
         </is>
       </c>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" s="2" t="n">
+      <c r="P71" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -5278,7 +5266,7 @@
         </is>
       </c>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" s="2" t="n">
+      <c r="P72" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q72" t="inlineStr"/>
@@ -5345,7 +5333,7 @@
         </is>
       </c>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" s="2" t="n">
+      <c r="P73" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q73" t="inlineStr"/>
@@ -5412,7 +5400,7 @@
         </is>
       </c>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" s="2" t="n">
+      <c r="P74" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q74" t="inlineStr"/>
@@ -5479,7 +5467,7 @@
         </is>
       </c>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" s="2" t="n">
+      <c r="P75" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q75" t="inlineStr"/>
@@ -5546,7 +5534,7 @@
         </is>
       </c>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" s="2" t="n">
+      <c r="P76" s="1" t="n">
         <v>46130</v>
       </c>
       <c r="Q76" t="inlineStr"/>
@@ -5678,7 +5666,7 @@
         </is>
       </c>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" s="2" t="n">
+      <c r="P78" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q78" t="inlineStr"/>
@@ -5745,7 +5733,7 @@
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
-      <c r="P79" s="2" t="n">
+      <c r="P79" s="1" t="n">
         <v>46140</v>
       </c>
       <c r="Q79" t="inlineStr"/>
@@ -5812,7 +5800,7 @@
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" s="2" t="n">
+      <c r="P80" s="1" t="n">
         <v>46095</v>
       </c>
       <c r="Q80" t="inlineStr"/>
@@ -5879,7 +5867,7 @@
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" s="2" t="n">
+      <c r="P81" s="1" t="n">
         <v>46040</v>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -5946,7 +5934,7 @@
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" s="2" t="n">
+      <c r="P82" s="1" t="n">
         <v>46060</v>
       </c>
       <c r="Q82" t="inlineStr"/>
@@ -6013,7 +6001,7 @@
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" s="2" t="n">
+      <c r="P83" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -6080,7 +6068,7 @@
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" s="2" t="n">
+      <c r="P84" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q84" t="inlineStr"/>
@@ -6147,7 +6135,7 @@
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
-      <c r="P85" s="2" t="n">
+      <c r="P85" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6218,7 +6206,7 @@
         </is>
       </c>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" s="2" t="n">
+      <c r="P86" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q86" t="inlineStr"/>
@@ -6285,7 +6273,7 @@
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" s="2" t="n">
+      <c r="P87" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q87" t="inlineStr"/>
@@ -6352,7 +6340,7 @@
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" s="2" t="n">
+      <c r="P88" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q88" t="inlineStr"/>
@@ -6419,7 +6407,7 @@
         </is>
       </c>
       <c r="O89" t="inlineStr"/>
-      <c r="P89" s="2" t="n">
+      <c r="P89" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q89" t="inlineStr"/>
@@ -6486,7 +6474,7 @@
         </is>
       </c>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" s="2" t="n">
+      <c r="P90" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q90" t="inlineStr"/>
@@ -6553,7 +6541,7 @@
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
-      <c r="P91" s="2" t="n">
+      <c r="P91" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="Q91" t="inlineStr"/>
@@ -6620,7 +6608,7 @@
         </is>
       </c>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" s="2" t="n">
+      <c r="P92" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="Q92" t="inlineStr"/>
@@ -6687,7 +6675,7 @@
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" s="2" t="n">
+      <c r="P93" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q93" t="inlineStr"/>
@@ -6754,7 +6742,7 @@
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" s="2" t="n">
+      <c r="P94" s="1" t="n">
         <v>46037</v>
       </c>
       <c r="Q94" t="inlineStr"/>
@@ -6890,7 +6878,7 @@
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
-      <c r="P96" s="2" t="n">
+      <c r="P96" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q96" t="inlineStr"/>
@@ -6957,7 +6945,7 @@
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
-      <c r="P97" s="2" t="n">
+      <c r="P97" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q97" t="inlineStr"/>
@@ -7154,7 +7142,7 @@
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
-      <c r="P100" s="2" t="n">
+      <c r="P100" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q100" t="inlineStr"/>
@@ -7221,7 +7209,7 @@
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
-      <c r="P101" s="2" t="n">
+      <c r="P101" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q101" t="inlineStr"/>
@@ -7288,7 +7276,7 @@
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
-      <c r="P102" s="2" t="n">
+      <c r="P102" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q102" t="inlineStr"/>
@@ -7355,7 +7343,7 @@
         </is>
       </c>
       <c r="O103" t="inlineStr"/>
-      <c r="P103" s="2" t="n">
+      <c r="P103" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q103" t="inlineStr"/>
@@ -7483,7 +7471,7 @@
         </is>
       </c>
       <c r="O105" t="inlineStr"/>
-      <c r="P105" s="2" t="n">
+      <c r="P105" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q105" t="inlineStr"/>
@@ -7550,7 +7538,7 @@
         </is>
       </c>
       <c r="O106" t="inlineStr"/>
-      <c r="P106" s="2" t="n">
+      <c r="P106" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q106" t="inlineStr">
@@ -7621,7 +7609,7 @@
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
-      <c r="P107" s="2" t="n">
+      <c r="P107" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -7688,7 +7676,7 @@
         </is>
       </c>
       <c r="O108" t="inlineStr"/>
-      <c r="P108" s="2" t="n">
+      <c r="P108" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -7885,7 +7873,7 @@
         </is>
       </c>
       <c r="O111" t="inlineStr"/>
-      <c r="P111" s="2" t="n">
+      <c r="P111" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -7952,7 +7940,7 @@
         </is>
       </c>
       <c r="O112" t="inlineStr"/>
-      <c r="P112" s="2" t="n">
+      <c r="P112" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -8084,7 +8072,7 @@
         </is>
       </c>
       <c r="O114" t="inlineStr"/>
-      <c r="P114" s="2" t="n">
+      <c r="P114" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q114" t="inlineStr"/>
@@ -8151,7 +8139,7 @@
         </is>
       </c>
       <c r="O115" t="inlineStr"/>
-      <c r="P115" s="2" t="n">
+      <c r="P115" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -8218,7 +8206,7 @@
         </is>
       </c>
       <c r="O116" t="inlineStr"/>
-      <c r="P116" s="2" t="n">
+      <c r="P116" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q116" t="inlineStr"/>
@@ -8285,7 +8273,7 @@
         </is>
       </c>
       <c r="O117" t="inlineStr"/>
-      <c r="P117" s="2" t="n">
+      <c r="P117" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="Q117" t="inlineStr"/>
@@ -8352,7 +8340,7 @@
         </is>
       </c>
       <c r="O118" t="inlineStr"/>
-      <c r="P118" s="2" t="n">
+      <c r="P118" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -8419,7 +8407,7 @@
         </is>
       </c>
       <c r="O119" t="inlineStr"/>
-      <c r="P119" s="2" t="n">
+      <c r="P119" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q119" t="inlineStr"/>
@@ -8486,7 +8474,7 @@
         </is>
       </c>
       <c r="O120" t="inlineStr"/>
-      <c r="P120" s="2" t="n">
+      <c r="P120" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q120" t="inlineStr"/>
@@ -8553,7 +8541,7 @@
         </is>
       </c>
       <c r="O121" t="inlineStr"/>
-      <c r="P121" s="2" t="n">
+      <c r="P121" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -8685,7 +8673,7 @@
         </is>
       </c>
       <c r="O123" t="inlineStr"/>
-      <c r="P123" s="2" t="n">
+      <c r="P123" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q123" t="inlineStr"/>
@@ -8947,7 +8935,7 @@
         </is>
       </c>
       <c r="O127" t="inlineStr"/>
-      <c r="P127" s="2" t="n">
+      <c r="P127" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q127" t="inlineStr"/>
@@ -9014,7 +9002,7 @@
         </is>
       </c>
       <c r="O128" t="inlineStr"/>
-      <c r="P128" s="2" t="n">
+      <c r="P128" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q128" t="inlineStr"/>
@@ -9081,7 +9069,7 @@
         </is>
       </c>
       <c r="O129" t="inlineStr"/>
-      <c r="P129" s="2" t="n">
+      <c r="P129" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q129" t="inlineStr"/>
@@ -9148,7 +9136,7 @@
         </is>
       </c>
       <c r="O130" t="inlineStr"/>
-      <c r="P130" s="2" t="n">
+      <c r="P130" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q130" t="inlineStr"/>
@@ -9215,7 +9203,7 @@
         </is>
       </c>
       <c r="O131" t="inlineStr"/>
-      <c r="P131" s="2" t="n">
+      <c r="P131" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -9282,7 +9270,7 @@
         </is>
       </c>
       <c r="O132" t="inlineStr"/>
-      <c r="P132" s="2" t="n">
+      <c r="P132" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -9349,7 +9337,7 @@
         </is>
       </c>
       <c r="O133" t="inlineStr"/>
-      <c r="P133" s="2" t="n">
+      <c r="P133" s="1" t="n">
         <v>46130</v>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -9481,7 +9469,7 @@
         </is>
       </c>
       <c r="O135" t="inlineStr"/>
-      <c r="P135" s="2" t="n">
+      <c r="P135" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q135" t="inlineStr"/>
@@ -9548,7 +9536,7 @@
         </is>
       </c>
       <c r="O136" t="inlineStr"/>
-      <c r="P136" s="2" t="n">
+      <c r="P136" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q136" t="inlineStr"/>
@@ -9680,7 +9668,7 @@
         </is>
       </c>
       <c r="O138" t="inlineStr"/>
-      <c r="P138" s="2" t="n">
+      <c r="P138" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q138" t="inlineStr"/>
@@ -9877,7 +9865,7 @@
         </is>
       </c>
       <c r="O141" t="inlineStr"/>
-      <c r="P141" s="2" t="n">
+      <c r="P141" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q141" t="inlineStr"/>
@@ -9944,7 +9932,7 @@
         </is>
       </c>
       <c r="O142" t="inlineStr"/>
-      <c r="P142" s="2" t="n">
+      <c r="P142" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q142" t="inlineStr"/>
@@ -10076,7 +10064,7 @@
         </is>
       </c>
       <c r="O144" t="inlineStr"/>
-      <c r="P144" s="2" t="n">
+      <c r="P144" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q144" t="inlineStr"/>
@@ -10143,7 +10131,7 @@
         </is>
       </c>
       <c r="O145" t="inlineStr"/>
-      <c r="P145" s="2" t="n">
+      <c r="P145" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q145" t="inlineStr"/>
@@ -10210,7 +10198,7 @@
         </is>
       </c>
       <c r="O146" t="inlineStr"/>
-      <c r="P146" s="2" t="n">
+      <c r="P146" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q146" t="inlineStr"/>
@@ -10277,7 +10265,7 @@
         </is>
       </c>
       <c r="O147" t="inlineStr"/>
-      <c r="P147" s="2" t="n">
+      <c r="P147" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="Q147" t="inlineStr"/>
@@ -10344,7 +10332,7 @@
         </is>
       </c>
       <c r="O148" t="inlineStr"/>
-      <c r="P148" s="2" t="n">
+      <c r="P148" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q148" t="inlineStr"/>
@@ -10411,7 +10399,7 @@
         </is>
       </c>
       <c r="O149" t="inlineStr"/>
-      <c r="P149" s="2" t="n">
+      <c r="P149" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q149" t="inlineStr"/>
@@ -10478,7 +10466,7 @@
         </is>
       </c>
       <c r="O150" t="inlineStr"/>
-      <c r="P150" s="2" t="n">
+      <c r="P150" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q150" t="inlineStr"/>
@@ -10545,7 +10533,7 @@
         </is>
       </c>
       <c r="O151" t="inlineStr"/>
-      <c r="P151" s="2" t="n">
+      <c r="P151" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q151" t="inlineStr"/>
@@ -10677,7 +10665,7 @@
         </is>
       </c>
       <c r="O153" t="inlineStr"/>
-      <c r="P153" s="2" t="n">
+      <c r="P153" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q153" t="inlineStr"/>
@@ -10939,7 +10927,7 @@
         </is>
       </c>
       <c r="O157" t="inlineStr"/>
-      <c r="P157" s="2" t="n">
+      <c r="P157" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q157" t="inlineStr"/>
@@ -11006,7 +10994,7 @@
         </is>
       </c>
       <c r="O158" t="inlineStr"/>
-      <c r="P158" s="2" t="n">
+      <c r="P158" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q158" t="inlineStr"/>
@@ -11073,7 +11061,7 @@
         </is>
       </c>
       <c r="O159" t="inlineStr"/>
-      <c r="P159" s="2" t="n">
+      <c r="P159" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q159" t="inlineStr"/>
@@ -11140,7 +11128,7 @@
         </is>
       </c>
       <c r="O160" t="inlineStr"/>
-      <c r="P160" s="2" t="n">
+      <c r="P160" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q160" t="inlineStr"/>
@@ -11272,7 +11260,7 @@
         </is>
       </c>
       <c r="O162" t="inlineStr"/>
-      <c r="P162" s="2" t="n">
+      <c r="P162" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q162" t="inlineStr"/>
@@ -11339,7 +11327,7 @@
         </is>
       </c>
       <c r="O163" t="inlineStr"/>
-      <c r="P163" s="2" t="n">
+      <c r="P163" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q163" t="inlineStr"/>
@@ -11406,7 +11394,7 @@
         </is>
       </c>
       <c r="O164" t="inlineStr"/>
-      <c r="P164" s="2" t="n">
+      <c r="P164" s="1" t="n">
         <v>45984</v>
       </c>
       <c r="Q164" t="inlineStr"/>
@@ -11473,7 +11461,7 @@
         </is>
       </c>
       <c r="O165" t="inlineStr"/>
-      <c r="P165" s="2" t="n">
+      <c r="P165" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q165" t="inlineStr"/>
@@ -11540,7 +11528,7 @@
         </is>
       </c>
       <c r="O166" t="inlineStr"/>
-      <c r="P166" s="2" t="n">
+      <c r="P166" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q166" t="inlineStr"/>
@@ -11607,7 +11595,7 @@
         </is>
       </c>
       <c r="O167" t="inlineStr"/>
-      <c r="P167" s="2" t="n">
+      <c r="P167" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q167" t="inlineStr"/>
@@ -11674,7 +11662,7 @@
         </is>
       </c>
       <c r="O168" t="inlineStr"/>
-      <c r="P168" s="2" t="n">
+      <c r="P168" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q168" t="inlineStr"/>
@@ -11741,7 +11729,7 @@
         </is>
       </c>
       <c r="O169" t="inlineStr"/>
-      <c r="P169" s="2" t="n">
+      <c r="P169" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q169" t="inlineStr"/>
@@ -11808,7 +11796,7 @@
         </is>
       </c>
       <c r="O170" t="inlineStr"/>
-      <c r="P170" s="2" t="n">
+      <c r="P170" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q170" t="inlineStr"/>
@@ -11875,7 +11863,7 @@
         </is>
       </c>
       <c r="O171" t="inlineStr"/>
-      <c r="P171" s="2" t="n">
+      <c r="P171" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q171" t="inlineStr"/>
@@ -11942,7 +11930,7 @@
         </is>
       </c>
       <c r="O172" t="inlineStr"/>
-      <c r="P172" s="2" t="n">
+      <c r="P172" s="1" t="n">
         <v>45954</v>
       </c>
       <c r="Q172" t="inlineStr"/>
@@ -12009,7 +11997,7 @@
         </is>
       </c>
       <c r="O173" t="inlineStr"/>
-      <c r="P173" s="2" t="n">
+      <c r="P173" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q173" t="inlineStr"/>
@@ -12076,7 +12064,7 @@
         </is>
       </c>
       <c r="O174" t="inlineStr"/>
-      <c r="P174" s="2" t="n">
+      <c r="P174" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q174" t="inlineStr"/>
@@ -12143,7 +12131,7 @@
         </is>
       </c>
       <c r="O175" t="inlineStr"/>
-      <c r="P175" s="2" t="n">
+      <c r="P175" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q175" t="inlineStr"/>
@@ -12210,7 +12198,7 @@
         </is>
       </c>
       <c r="O176" t="inlineStr"/>
-      <c r="P176" s="2" t="n">
+      <c r="P176" s="1" t="n">
         <v>45835</v>
       </c>
       <c r="Q176" t="inlineStr"/>
@@ -12277,7 +12265,7 @@
         </is>
       </c>
       <c r="O177" t="inlineStr"/>
-      <c r="P177" s="2" t="n">
+      <c r="P177" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q177" t="inlineStr"/>
@@ -12344,7 +12332,7 @@
         </is>
       </c>
       <c r="O178" t="inlineStr"/>
-      <c r="P178" s="2" t="n">
+      <c r="P178" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q178" t="inlineStr"/>
@@ -12411,7 +12399,7 @@
         </is>
       </c>
       <c r="O179" t="inlineStr"/>
-      <c r="P179" s="2" t="n">
+      <c r="P179" s="1" t="n">
         <v>45835</v>
       </c>
       <c r="Q179" t="inlineStr"/>
@@ -12478,7 +12466,7 @@
         </is>
       </c>
       <c r="O180" t="inlineStr"/>
-      <c r="P180" s="2" t="n">
+      <c r="P180" s="1" t="n">
         <v>46025</v>
       </c>
       <c r="Q180" t="inlineStr"/>
@@ -12545,7 +12533,7 @@
         </is>
       </c>
       <c r="O181" t="inlineStr"/>
-      <c r="P181" s="2" t="n">
+      <c r="P181" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q181" t="inlineStr"/>
@@ -12612,7 +12600,7 @@
         </is>
       </c>
       <c r="O182" t="inlineStr"/>
-      <c r="P182" s="2" t="n">
+      <c r="P182" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q182" t="inlineStr"/>
@@ -12744,7 +12732,7 @@
         </is>
       </c>
       <c r="O184" t="inlineStr"/>
-      <c r="P184" s="2" t="n">
+      <c r="P184" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q184" t="inlineStr"/>
@@ -12876,7 +12864,7 @@
         </is>
       </c>
       <c r="O186" t="inlineStr"/>
-      <c r="P186" s="2" t="n">
+      <c r="P186" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q186" t="inlineStr"/>
@@ -12896,87 +12884,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -13037,7 +13025,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="M2" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N2" t="inlineStr">
@@ -13104,7 +13092,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="M3" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N3" t="inlineStr">
@@ -13171,7 +13159,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="M4" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -13238,7 +13226,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="M5" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N5" t="inlineStr">
@@ -13305,7 +13293,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N6" t="inlineStr">
@@ -13372,7 +13360,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -13439,7 +13427,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="M8" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N8" t="inlineStr">
@@ -13506,7 +13494,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N9" t="inlineStr">
@@ -13573,7 +13561,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -13640,7 +13628,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="M11" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -13772,7 +13760,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M13" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N13" t="inlineStr">
@@ -13839,7 +13827,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="M14" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N14" t="inlineStr">
@@ -13906,7 +13894,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="M15" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N15" t="inlineStr">
@@ -13973,7 +13961,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="M16" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N16" t="inlineStr">
@@ -14040,7 +14028,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M17" s="2" t="n">
+      <c r="M17" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N17" t="inlineStr">
@@ -14107,7 +14095,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="M18" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N18" t="inlineStr">
@@ -14174,7 +14162,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="M19" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N19" t="inlineStr">
@@ -14241,7 +14229,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M20" s="2" t="n">
+      <c r="M20" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N20" t="inlineStr">
@@ -14308,7 +14296,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="M21" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N21" t="inlineStr">
@@ -14375,7 +14363,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="M22" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N22" t="inlineStr">
@@ -14442,7 +14430,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M23" s="2" t="n">
+      <c r="M23" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N23" t="inlineStr">
@@ -14509,7 +14497,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="M24" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N24" t="inlineStr">
@@ -14576,7 +14564,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="M25" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N25" t="inlineStr">
@@ -14643,7 +14631,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="M26" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="N26" t="inlineStr">
@@ -14710,7 +14698,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="M27" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N27" t="inlineStr">
@@ -14777,7 +14765,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="M28" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N28" t="inlineStr">
@@ -14844,7 +14832,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M29" s="2" t="n">
+      <c r="M29" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N29" t="inlineStr">
@@ -14911,7 +14899,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="M30" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N30" t="inlineStr">
@@ -14978,7 +14966,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="M31" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N31" t="inlineStr">
@@ -15045,7 +15033,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M32" s="2" t="n">
+      <c r="M32" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N32" t="inlineStr">
@@ -15112,7 +15100,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="M33" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N33" t="inlineStr">
@@ -15179,7 +15167,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M34" s="2" t="n">
+      <c r="M34" s="1" t="n">
         <v>46288</v>
       </c>
       <c r="N34" t="inlineStr">
@@ -15246,7 +15234,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M35" s="2" t="n">
+      <c r="M35" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N35" t="inlineStr">
@@ -15313,7 +15301,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M36" s="2" t="n">
+      <c r="M36" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N36" t="inlineStr">
@@ -15380,7 +15368,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="M37" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N37" t="inlineStr">
@@ -15447,7 +15435,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="M38" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N38" t="inlineStr">
@@ -15514,7 +15502,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M39" s="2" t="n">
+      <c r="M39" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N39" t="inlineStr">
@@ -15581,7 +15569,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M40" s="2" t="n">
+      <c r="M40" s="1" t="n">
         <v>46303</v>
       </c>
       <c r="N40" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: tpjl (10/07/2026 20:01)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,12 +49,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -422,87 +434,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -570,7 +582,7 @@
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" s="1" t="n">
+      <c r="P2" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -637,7 +649,7 @@
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" s="1" t="n">
+      <c r="P3" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -704,7 +716,7 @@
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" s="1" t="n">
+      <c r="P4" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -901,7 +913,7 @@
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" s="1" t="n">
+      <c r="P7" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -968,7 +980,7 @@
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" s="1" t="n">
+      <c r="P8" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1035,7 +1047,7 @@
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" s="1" t="n">
+      <c r="P9" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1106,7 +1118,7 @@
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" s="1" t="n">
+      <c r="P10" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1299,7 +1311,7 @@
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" s="1" t="n">
+      <c r="P13" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -1366,7 +1378,7 @@
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" s="1" t="n">
+      <c r="P14" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -1433,7 +1445,7 @@
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" s="1" t="n">
+      <c r="P15" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -1500,7 +1512,7 @@
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" s="1" t="n">
+      <c r="P16" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1571,7 +1583,7 @@
         </is>
       </c>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" s="1" t="n">
+      <c r="P17" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -1638,7 +1650,7 @@
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" s="1" t="n">
+      <c r="P18" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -1835,7 +1847,7 @@
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" s="1" t="n">
+      <c r="P21" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -1902,7 +1914,7 @@
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" s="1" t="n">
+      <c r="P22" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -2034,7 +2046,7 @@
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" s="1" t="n">
+      <c r="P24" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2105,7 +2117,7 @@
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" s="1" t="n">
+      <c r="P25" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2176,7 +2188,7 @@
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" s="1" t="n">
+      <c r="P26" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -2243,7 +2255,7 @@
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" s="1" t="n">
+      <c r="P27" s="2" t="n">
         <v>45964</v>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -2310,7 +2322,7 @@
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" s="1" t="n">
+      <c r="P28" s="2" t="n">
         <v>45984</v>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -2442,7 +2454,7 @@
         </is>
       </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" s="1" t="n">
+      <c r="P30" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q30" t="inlineStr"/>
@@ -2574,7 +2586,7 @@
         </is>
       </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" s="1" t="n">
+      <c r="P32" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2645,7 +2657,7 @@
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" s="1" t="n">
+      <c r="P33" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -2712,7 +2724,7 @@
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
-      <c r="P34" s="1" t="n">
+      <c r="P34" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -2779,7 +2791,7 @@
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" s="1" t="n">
+      <c r="P35" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -2911,7 +2923,7 @@
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" s="1" t="n">
+      <c r="P37" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -2978,7 +2990,7 @@
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" s="1" t="n">
+      <c r="P38" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -3045,7 +3057,7 @@
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" s="1" t="n">
+      <c r="P39" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q39" t="inlineStr"/>
@@ -3177,7 +3189,7 @@
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" s="1" t="n">
+      <c r="P41" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q41" t="inlineStr"/>
@@ -3244,7 +3256,7 @@
         </is>
       </c>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" s="1" t="n">
+      <c r="P42" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -3311,7 +3323,7 @@
         </is>
       </c>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" s="1" t="n">
+      <c r="P43" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -3378,7 +3390,7 @@
         </is>
       </c>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" s="1" t="n">
+      <c r="P44" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -3640,7 +3652,7 @@
         </is>
       </c>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" s="1" t="n">
+      <c r="P48" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -3707,7 +3719,7 @@
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" s="1" t="n">
+      <c r="P49" s="2" t="n">
         <v>45955</v>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -3774,7 +3786,7 @@
         </is>
       </c>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" s="1" t="n">
+      <c r="P50" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -3841,7 +3853,7 @@
         </is>
       </c>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" s="1" t="n">
+      <c r="P51" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q51" t="inlineStr">
@@ -3912,7 +3924,7 @@
         </is>
       </c>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" s="1" t="n">
+      <c r="P52" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -3979,7 +3991,7 @@
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" s="1" t="n">
+      <c r="P53" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -4107,7 +4119,7 @@
         </is>
       </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" s="1" t="n">
+      <c r="P55" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -4174,7 +4186,7 @@
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" s="1" t="n">
+      <c r="P56" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -4310,7 +4322,7 @@
         </is>
       </c>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" s="1" t="n">
+      <c r="P58" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -4377,7 +4389,7 @@
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" s="1" t="n">
+      <c r="P59" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="Q59" t="inlineStr">
@@ -4448,7 +4460,7 @@
         </is>
       </c>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" s="1" t="n">
+      <c r="P60" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -4515,7 +4527,7 @@
         </is>
       </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" s="1" t="n">
+      <c r="P61" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q61" t="inlineStr"/>
@@ -4582,7 +4594,7 @@
         </is>
       </c>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" s="1" t="n">
+      <c r="P62" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q62" t="inlineStr"/>
@@ -4649,7 +4661,7 @@
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" s="1" t="n">
+      <c r="P63" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q63" t="inlineStr"/>
@@ -4716,7 +4728,7 @@
         </is>
       </c>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" s="1" t="n">
+      <c r="P64" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q64" t="inlineStr">
@@ -4787,7 +4799,7 @@
         </is>
       </c>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" s="1" t="n">
+      <c r="P65" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q65" t="inlineStr"/>
@@ -4854,7 +4866,7 @@
         </is>
       </c>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" s="1" t="n">
+      <c r="P66" s="2" t="n">
         <v>45946</v>
       </c>
       <c r="Q66" t="inlineStr">
@@ -4925,7 +4937,7 @@
         </is>
       </c>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" s="1" t="n">
+      <c r="P67" s="2" t="n">
         <v>45916</v>
       </c>
       <c r="Q67" t="inlineStr"/>
@@ -4992,7 +5004,7 @@
         </is>
       </c>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" s="1" t="n">
+      <c r="P68" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5063,7 +5075,7 @@
         </is>
       </c>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" s="1" t="n">
+      <c r="P69" s="2" t="n">
         <v>45989</v>
       </c>
       <c r="Q69" t="inlineStr">
@@ -5199,7 +5211,7 @@
         </is>
       </c>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" s="1" t="n">
+      <c r="P71" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -5266,7 +5278,7 @@
         </is>
       </c>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" s="1" t="n">
+      <c r="P72" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q72" t="inlineStr"/>
@@ -5333,7 +5345,7 @@
         </is>
       </c>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" s="1" t="n">
+      <c r="P73" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q73" t="inlineStr"/>
@@ -5400,7 +5412,7 @@
         </is>
       </c>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" s="1" t="n">
+      <c r="P74" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q74" t="inlineStr"/>
@@ -5467,7 +5479,7 @@
         </is>
       </c>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" s="1" t="n">
+      <c r="P75" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q75" t="inlineStr"/>
@@ -5534,7 +5546,7 @@
         </is>
       </c>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" s="1" t="n">
+      <c r="P76" s="2" t="n">
         <v>46130</v>
       </c>
       <c r="Q76" t="inlineStr"/>
@@ -5666,7 +5678,7 @@
         </is>
       </c>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" s="1" t="n">
+      <c r="P78" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q78" t="inlineStr"/>
@@ -5733,7 +5745,7 @@
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
-      <c r="P79" s="1" t="n">
+      <c r="P79" s="2" t="n">
         <v>46140</v>
       </c>
       <c r="Q79" t="inlineStr"/>
@@ -5800,7 +5812,7 @@
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" s="1" t="n">
+      <c r="P80" s="2" t="n">
         <v>46095</v>
       </c>
       <c r="Q80" t="inlineStr"/>
@@ -5867,7 +5879,7 @@
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" s="1" t="n">
+      <c r="P81" s="2" t="n">
         <v>46040</v>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -5934,7 +5946,7 @@
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" s="1" t="n">
+      <c r="P82" s="2" t="n">
         <v>46060</v>
       </c>
       <c r="Q82" t="inlineStr"/>
@@ -6001,7 +6013,7 @@
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" s="1" t="n">
+      <c r="P83" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -6068,7 +6080,7 @@
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" s="1" t="n">
+      <c r="P84" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q84" t="inlineStr"/>
@@ -6135,7 +6147,7 @@
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
-      <c r="P85" s="1" t="n">
+      <c r="P85" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6206,7 +6218,7 @@
         </is>
       </c>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" s="1" t="n">
+      <c r="P86" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q86" t="inlineStr"/>
@@ -6273,7 +6285,7 @@
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" s="1" t="n">
+      <c r="P87" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q87" t="inlineStr"/>
@@ -6340,7 +6352,7 @@
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" s="1" t="n">
+      <c r="P88" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q88" t="inlineStr"/>
@@ -6407,7 +6419,7 @@
         </is>
       </c>
       <c r="O89" t="inlineStr"/>
-      <c r="P89" s="1" t="n">
+      <c r="P89" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q89" t="inlineStr"/>
@@ -6474,7 +6486,7 @@
         </is>
       </c>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" s="1" t="n">
+      <c r="P90" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q90" t="inlineStr"/>
@@ -6541,7 +6553,7 @@
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
-      <c r="P91" s="1" t="n">
+      <c r="P91" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="Q91" t="inlineStr"/>
@@ -6608,7 +6620,7 @@
         </is>
       </c>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" s="1" t="n">
+      <c r="P92" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="Q92" t="inlineStr"/>
@@ -6675,7 +6687,7 @@
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" s="1" t="n">
+      <c r="P93" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q93" t="inlineStr"/>
@@ -6742,7 +6754,7 @@
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" s="1" t="n">
+      <c r="P94" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="Q94" t="inlineStr"/>
@@ -6878,7 +6890,7 @@
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
-      <c r="P96" s="1" t="n">
+      <c r="P96" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q96" t="inlineStr"/>
@@ -6945,7 +6957,7 @@
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
-      <c r="P97" s="1" t="n">
+      <c r="P97" s="2" t="n">
         <v>46032</v>
       </c>
       <c r="Q97" t="inlineStr"/>
@@ -7142,7 +7154,7 @@
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
-      <c r="P100" s="1" t="n">
+      <c r="P100" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q100" t="inlineStr"/>
@@ -7209,7 +7221,7 @@
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
-      <c r="P101" s="1" t="n">
+      <c r="P101" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q101" t="inlineStr"/>
@@ -7276,7 +7288,7 @@
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
-      <c r="P102" s="1" t="n">
+      <c r="P102" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q102" t="inlineStr"/>
@@ -7343,7 +7355,7 @@
         </is>
       </c>
       <c r="O103" t="inlineStr"/>
-      <c r="P103" s="1" t="n">
+      <c r="P103" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q103" t="inlineStr"/>
@@ -7471,7 +7483,7 @@
         </is>
       </c>
       <c r="O105" t="inlineStr"/>
-      <c r="P105" s="1" t="n">
+      <c r="P105" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="Q105" t="inlineStr"/>
@@ -7538,7 +7550,7 @@
         </is>
       </c>
       <c r="O106" t="inlineStr"/>
-      <c r="P106" s="1" t="n">
+      <c r="P106" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q106" t="inlineStr">
@@ -7609,7 +7621,7 @@
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
-      <c r="P107" s="1" t="n">
+      <c r="P107" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -7676,7 +7688,7 @@
         </is>
       </c>
       <c r="O108" t="inlineStr"/>
-      <c r="P108" s="1" t="n">
+      <c r="P108" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -7873,7 +7885,7 @@
         </is>
       </c>
       <c r="O111" t="inlineStr"/>
-      <c r="P111" s="1" t="n">
+      <c r="P111" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -7940,7 +7952,7 @@
         </is>
       </c>
       <c r="O112" t="inlineStr"/>
-      <c r="P112" s="1" t="n">
+      <c r="P112" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -8072,7 +8084,7 @@
         </is>
       </c>
       <c r="O114" t="inlineStr"/>
-      <c r="P114" s="1" t="n">
+      <c r="P114" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="Q114" t="inlineStr"/>
@@ -8139,7 +8151,7 @@
         </is>
       </c>
       <c r="O115" t="inlineStr"/>
-      <c r="P115" s="1" t="n">
+      <c r="P115" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -8206,7 +8218,7 @@
         </is>
       </c>
       <c r="O116" t="inlineStr"/>
-      <c r="P116" s="1" t="n">
+      <c r="P116" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q116" t="inlineStr"/>
@@ -8273,7 +8285,7 @@
         </is>
       </c>
       <c r="O117" t="inlineStr"/>
-      <c r="P117" s="1" t="n">
+      <c r="P117" s="2" t="n">
         <v>46081</v>
       </c>
       <c r="Q117" t="inlineStr"/>
@@ -8340,7 +8352,7 @@
         </is>
       </c>
       <c r="O118" t="inlineStr"/>
-      <c r="P118" s="1" t="n">
+      <c r="P118" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -8407,7 +8419,7 @@
         </is>
       </c>
       <c r="O119" t="inlineStr"/>
-      <c r="P119" s="1" t="n">
+      <c r="P119" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q119" t="inlineStr"/>
@@ -8474,7 +8486,7 @@
         </is>
       </c>
       <c r="O120" t="inlineStr"/>
-      <c r="P120" s="1" t="n">
+      <c r="P120" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q120" t="inlineStr"/>
@@ -8541,7 +8553,7 @@
         </is>
       </c>
       <c r="O121" t="inlineStr"/>
-      <c r="P121" s="1" t="n">
+      <c r="P121" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -8673,7 +8685,7 @@
         </is>
       </c>
       <c r="O123" t="inlineStr"/>
-      <c r="P123" s="1" t="n">
+      <c r="P123" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q123" t="inlineStr"/>
@@ -8935,7 +8947,7 @@
         </is>
       </c>
       <c r="O127" t="inlineStr"/>
-      <c r="P127" s="1" t="n">
+      <c r="P127" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="Q127" t="inlineStr"/>
@@ -9002,7 +9014,7 @@
         </is>
       </c>
       <c r="O128" t="inlineStr"/>
-      <c r="P128" s="1" t="n">
+      <c r="P128" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q128" t="inlineStr"/>
@@ -9069,7 +9081,7 @@
         </is>
       </c>
       <c r="O129" t="inlineStr"/>
-      <c r="P129" s="1" t="n">
+      <c r="P129" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q129" t="inlineStr"/>
@@ -9136,7 +9148,7 @@
         </is>
       </c>
       <c r="O130" t="inlineStr"/>
-      <c r="P130" s="1" t="n">
+      <c r="P130" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q130" t="inlineStr"/>
@@ -9203,7 +9215,7 @@
         </is>
       </c>
       <c r="O131" t="inlineStr"/>
-      <c r="P131" s="1" t="n">
+      <c r="P131" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -9270,7 +9282,7 @@
         </is>
       </c>
       <c r="O132" t="inlineStr"/>
-      <c r="P132" s="1" t="n">
+      <c r="P132" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -9337,7 +9349,7 @@
         </is>
       </c>
       <c r="O133" t="inlineStr"/>
-      <c r="P133" s="1" t="n">
+      <c r="P133" s="2" t="n">
         <v>46130</v>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -9469,7 +9481,7 @@
         </is>
       </c>
       <c r="O135" t="inlineStr"/>
-      <c r="P135" s="1" t="n">
+      <c r="P135" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q135" t="inlineStr"/>
@@ -9536,7 +9548,7 @@
         </is>
       </c>
       <c r="O136" t="inlineStr"/>
-      <c r="P136" s="1" t="n">
+      <c r="P136" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q136" t="inlineStr"/>
@@ -9668,7 +9680,7 @@
         </is>
       </c>
       <c r="O138" t="inlineStr"/>
-      <c r="P138" s="1" t="n">
+      <c r="P138" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q138" t="inlineStr"/>
@@ -9865,7 +9877,7 @@
         </is>
       </c>
       <c r="O141" t="inlineStr"/>
-      <c r="P141" s="1" t="n">
+      <c r="P141" s="2" t="n">
         <v>46160</v>
       </c>
       <c r="Q141" t="inlineStr"/>
@@ -9932,7 +9944,7 @@
         </is>
       </c>
       <c r="O142" t="inlineStr"/>
-      <c r="P142" s="1" t="n">
+      <c r="P142" s="2" t="n">
         <v>46123</v>
       </c>
       <c r="Q142" t="inlineStr"/>
@@ -10064,7 +10076,7 @@
         </is>
       </c>
       <c r="O144" t="inlineStr"/>
-      <c r="P144" s="1" t="n">
+      <c r="P144" s="2" t="n">
         <v>46167</v>
       </c>
       <c r="Q144" t="inlineStr"/>
@@ -10131,7 +10143,7 @@
         </is>
       </c>
       <c r="O145" t="inlineStr"/>
-      <c r="P145" s="1" t="n">
+      <c r="P145" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q145" t="inlineStr"/>
@@ -10198,7 +10210,7 @@
         </is>
       </c>
       <c r="O146" t="inlineStr"/>
-      <c r="P146" s="1" t="n">
+      <c r="P146" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="Q146" t="inlineStr"/>
@@ -10265,7 +10277,7 @@
         </is>
       </c>
       <c r="O147" t="inlineStr"/>
-      <c r="P147" s="1" t="n">
+      <c r="P147" s="2" t="n">
         <v>46081</v>
       </c>
       <c r="Q147" t="inlineStr"/>
@@ -10332,7 +10344,7 @@
         </is>
       </c>
       <c r="O148" t="inlineStr"/>
-      <c r="P148" s="1" t="n">
+      <c r="P148" s="2" t="n">
         <v>45976</v>
       </c>
       <c r="Q148" t="inlineStr"/>
@@ -10399,7 +10411,7 @@
         </is>
       </c>
       <c r="O149" t="inlineStr"/>
-      <c r="P149" s="1" t="n">
+      <c r="P149" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q149" t="inlineStr"/>
@@ -10466,7 +10478,7 @@
         </is>
       </c>
       <c r="O150" t="inlineStr"/>
-      <c r="P150" s="1" t="n">
+      <c r="P150" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q150" t="inlineStr"/>
@@ -10533,7 +10545,7 @@
         </is>
       </c>
       <c r="O151" t="inlineStr"/>
-      <c r="P151" s="1" t="n">
+      <c r="P151" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="Q151" t="inlineStr"/>
@@ -10665,7 +10677,7 @@
         </is>
       </c>
       <c r="O153" t="inlineStr"/>
-      <c r="P153" s="1" t="n">
+      <c r="P153" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q153" t="inlineStr"/>
@@ -10927,7 +10939,7 @@
         </is>
       </c>
       <c r="O157" t="inlineStr"/>
-      <c r="P157" s="1" t="n">
+      <c r="P157" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="Q157" t="inlineStr"/>
@@ -10994,7 +11006,7 @@
         </is>
       </c>
       <c r="O158" t="inlineStr"/>
-      <c r="P158" s="1" t="n">
+      <c r="P158" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q158" t="inlineStr"/>
@@ -11061,7 +11073,7 @@
         </is>
       </c>
       <c r="O159" t="inlineStr"/>
-      <c r="P159" s="1" t="n">
+      <c r="P159" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q159" t="inlineStr"/>
@@ -11128,7 +11140,7 @@
         </is>
       </c>
       <c r="O160" t="inlineStr"/>
-      <c r="P160" s="1" t="n">
+      <c r="P160" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q160" t="inlineStr"/>
@@ -11260,7 +11272,7 @@
         </is>
       </c>
       <c r="O162" t="inlineStr"/>
-      <c r="P162" s="1" t="n">
+      <c r="P162" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q162" t="inlineStr"/>
@@ -11327,7 +11339,7 @@
         </is>
       </c>
       <c r="O163" t="inlineStr"/>
-      <c r="P163" s="1" t="n">
+      <c r="P163" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q163" t="inlineStr"/>
@@ -11394,7 +11406,7 @@
         </is>
       </c>
       <c r="O164" t="inlineStr"/>
-      <c r="P164" s="1" t="n">
+      <c r="P164" s="2" t="n">
         <v>45984</v>
       </c>
       <c r="Q164" t="inlineStr"/>
@@ -11461,7 +11473,7 @@
         </is>
       </c>
       <c r="O165" t="inlineStr"/>
-      <c r="P165" s="1" t="n">
+      <c r="P165" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q165" t="inlineStr"/>
@@ -11528,7 +11540,7 @@
         </is>
       </c>
       <c r="O166" t="inlineStr"/>
-      <c r="P166" s="1" t="n">
+      <c r="P166" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q166" t="inlineStr"/>
@@ -11595,7 +11607,7 @@
         </is>
       </c>
       <c r="O167" t="inlineStr"/>
-      <c r="P167" s="1" t="n">
+      <c r="P167" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q167" t="inlineStr"/>
@@ -11662,7 +11674,7 @@
         </is>
       </c>
       <c r="O168" t="inlineStr"/>
-      <c r="P168" s="1" t="n">
+      <c r="P168" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="Q168" t="inlineStr"/>
@@ -11729,7 +11741,7 @@
         </is>
       </c>
       <c r="O169" t="inlineStr"/>
-      <c r="P169" s="1" t="n">
+      <c r="P169" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q169" t="inlineStr"/>
@@ -11796,7 +11808,7 @@
         </is>
       </c>
       <c r="O170" t="inlineStr"/>
-      <c r="P170" s="1" t="n">
+      <c r="P170" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q170" t="inlineStr"/>
@@ -11863,7 +11875,7 @@
         </is>
       </c>
       <c r="O171" t="inlineStr"/>
-      <c r="P171" s="1" t="n">
+      <c r="P171" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q171" t="inlineStr"/>
@@ -11930,7 +11942,7 @@
         </is>
       </c>
       <c r="O172" t="inlineStr"/>
-      <c r="P172" s="1" t="n">
+      <c r="P172" s="2" t="n">
         <v>45954</v>
       </c>
       <c r="Q172" t="inlineStr"/>
@@ -11997,7 +12009,7 @@
         </is>
       </c>
       <c r="O173" t="inlineStr"/>
-      <c r="P173" s="1" t="n">
+      <c r="P173" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q173" t="inlineStr"/>
@@ -12064,7 +12076,7 @@
         </is>
       </c>
       <c r="O174" t="inlineStr"/>
-      <c r="P174" s="1" t="n">
+      <c r="P174" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q174" t="inlineStr"/>
@@ -12131,7 +12143,7 @@
         </is>
       </c>
       <c r="O175" t="inlineStr"/>
-      <c r="P175" s="1" t="n">
+      <c r="P175" s="2" t="n">
         <v>45911</v>
       </c>
       <c r="Q175" t="inlineStr"/>
@@ -12198,7 +12210,7 @@
         </is>
       </c>
       <c r="O176" t="inlineStr"/>
-      <c r="P176" s="1" t="n">
+      <c r="P176" s="2" t="n">
         <v>45835</v>
       </c>
       <c r="Q176" t="inlineStr"/>
@@ -12265,7 +12277,7 @@
         </is>
       </c>
       <c r="O177" t="inlineStr"/>
-      <c r="P177" s="1" t="n">
+      <c r="P177" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q177" t="inlineStr"/>
@@ -12332,7 +12344,7 @@
         </is>
       </c>
       <c r="O178" t="inlineStr"/>
-      <c r="P178" s="1" t="n">
+      <c r="P178" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="Q178" t="inlineStr"/>
@@ -12399,7 +12411,7 @@
         </is>
       </c>
       <c r="O179" t="inlineStr"/>
-      <c r="P179" s="1" t="n">
+      <c r="P179" s="2" t="n">
         <v>45835</v>
       </c>
       <c r="Q179" t="inlineStr"/>
@@ -12466,7 +12478,7 @@
         </is>
       </c>
       <c r="O180" t="inlineStr"/>
-      <c r="P180" s="1" t="n">
+      <c r="P180" s="2" t="n">
         <v>46025</v>
       </c>
       <c r="Q180" t="inlineStr"/>
@@ -12533,7 +12545,7 @@
         </is>
       </c>
       <c r="O181" t="inlineStr"/>
-      <c r="P181" s="1" t="n">
+      <c r="P181" s="2" t="n">
         <v>46024</v>
       </c>
       <c r="Q181" t="inlineStr"/>
@@ -12600,7 +12612,7 @@
         </is>
       </c>
       <c r="O182" t="inlineStr"/>
-      <c r="P182" s="1" t="n">
+      <c r="P182" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q182" t="inlineStr"/>
@@ -12732,7 +12744,7 @@
         </is>
       </c>
       <c r="O184" t="inlineStr"/>
-      <c r="P184" s="1" t="n">
+      <c r="P184" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q184" t="inlineStr"/>
@@ -12864,7 +12876,7 @@
         </is>
       </c>
       <c r="O186" t="inlineStr"/>
-      <c r="P186" s="1" t="n">
+      <c r="P186" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="Q186" t="inlineStr"/>
@@ -12884,87 +12896,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -13025,7 +13037,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M2" s="1" t="n">
+      <c r="M2" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N2" t="inlineStr">
@@ -13092,7 +13104,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M3" s="1" t="n">
+      <c r="M3" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N3" t="inlineStr">
@@ -13159,7 +13171,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M4" s="1" t="n">
+      <c r="M4" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -13226,7 +13238,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M5" s="1" t="n">
+      <c r="M5" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N5" t="inlineStr">
@@ -13293,7 +13305,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M6" s="1" t="n">
+      <c r="M6" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N6" t="inlineStr">
@@ -13360,7 +13372,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M7" s="1" t="n">
+      <c r="M7" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -13427,7 +13439,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M8" s="1" t="n">
+      <c r="M8" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N8" t="inlineStr">
@@ -13494,7 +13506,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M9" s="1" t="n">
+      <c r="M9" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N9" t="inlineStr">
@@ -13561,7 +13573,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M10" s="1" t="n">
+      <c r="M10" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -13628,7 +13640,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M11" s="1" t="n">
+      <c r="M11" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -13760,7 +13772,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M13" s="1" t="n">
+      <c r="M13" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N13" t="inlineStr">
@@ -13827,7 +13839,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M14" s="1" t="n">
+      <c r="M14" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N14" t="inlineStr">
@@ -13894,7 +13906,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M15" s="1" t="n">
+      <c r="M15" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N15" t="inlineStr">
@@ -13961,7 +13973,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M16" s="1" t="n">
+      <c r="M16" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N16" t="inlineStr">
@@ -14028,7 +14040,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M17" s="1" t="n">
+      <c r="M17" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N17" t="inlineStr">
@@ -14095,7 +14107,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M18" s="1" t="n">
+      <c r="M18" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N18" t="inlineStr">
@@ -14162,7 +14174,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M19" s="1" t="n">
+      <c r="M19" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N19" t="inlineStr">
@@ -14229,7 +14241,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M20" s="1" t="n">
+      <c r="M20" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N20" t="inlineStr">
@@ -14296,7 +14308,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M21" s="1" t="n">
+      <c r="M21" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N21" t="inlineStr">
@@ -14363,7 +14375,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M22" s="1" t="n">
+      <c r="M22" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N22" t="inlineStr">
@@ -14430,7 +14442,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M23" s="1" t="n">
+      <c r="M23" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N23" t="inlineStr">
@@ -14497,7 +14509,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M24" s="1" t="n">
+      <c r="M24" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N24" t="inlineStr">
@@ -14564,7 +14576,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M25" s="1" t="n">
+      <c r="M25" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N25" t="inlineStr">
@@ -14631,7 +14643,7 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M26" s="1" t="n">
+      <c r="M26" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="N26" t="inlineStr">
@@ -14698,7 +14710,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M27" s="1" t="n">
+      <c r="M27" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N27" t="inlineStr">
@@ -14765,7 +14777,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M28" s="1" t="n">
+      <c r="M28" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N28" t="inlineStr">
@@ -14832,7 +14844,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M29" s="1" t="n">
+      <c r="M29" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N29" t="inlineStr">
@@ -14899,7 +14911,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M30" s="1" t="n">
+      <c r="M30" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N30" t="inlineStr">
@@ -14966,7 +14978,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M31" s="1" t="n">
+      <c r="M31" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N31" t="inlineStr">
@@ -15033,7 +15045,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M32" s="1" t="n">
+      <c r="M32" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N32" t="inlineStr">
@@ -15100,7 +15112,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M33" s="1" t="n">
+      <c r="M33" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N33" t="inlineStr">
@@ -15167,7 +15179,7 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M34" s="1" t="n">
+      <c r="M34" s="2" t="n">
         <v>46288</v>
       </c>
       <c r="N34" t="inlineStr">
@@ -15234,7 +15246,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M35" s="1" t="n">
+      <c r="M35" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N35" t="inlineStr">
@@ -15301,7 +15313,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M36" s="1" t="n">
+      <c r="M36" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N36" t="inlineStr">
@@ -15368,7 +15380,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M37" s="1" t="n">
+      <c r="M37" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N37" t="inlineStr">
@@ -15435,7 +15447,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M38" s="1" t="n">
+      <c r="M38" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N38" t="inlineStr">
@@ -15502,7 +15514,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M39" s="1" t="n">
+      <c r="M39" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N39" t="inlineStr">
@@ -15569,7 +15581,7 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M40" s="1" t="n">
+      <c r="M40" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="N40" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: tpjl (11/07/2026 07:20)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,87 +422,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -582,7 +570,7 @@
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -649,7 +637,7 @@
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" s="2" t="n">
+      <c r="P3" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -716,7 +704,7 @@
         </is>
       </c>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" s="2" t="n">
+      <c r="P4" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -913,7 +901,7 @@
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -980,7 +968,7 @@
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" s="2" t="n">
+      <c r="P8" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -1047,7 +1035,7 @@
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1118,7 +1106,7 @@
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" s="2" t="n">
+      <c r="P10" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1311,7 +1299,7 @@
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" s="2" t="n">
+      <c r="P13" s="1" t="n">
         <v>46037</v>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -1378,7 +1366,7 @@
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" s="2" t="n">
+      <c r="P14" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -1445,7 +1433,7 @@
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" s="2" t="n">
+      <c r="P15" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -1512,7 +1500,7 @@
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" s="2" t="n">
+      <c r="P16" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1583,7 +1571,7 @@
         </is>
       </c>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" s="2" t="n">
+      <c r="P17" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -1650,7 +1638,7 @@
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" s="2" t="n">
+      <c r="P18" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -1847,7 +1835,7 @@
         </is>
       </c>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" s="2" t="n">
+      <c r="P21" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -1914,7 +1902,7 @@
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" s="2" t="n">
+      <c r="P22" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -2046,7 +2034,7 @@
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" s="2" t="n">
+      <c r="P24" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q24" t="inlineStr">
@@ -2117,7 +2105,7 @@
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" s="2" t="n">
+      <c r="P25" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q25" t="inlineStr">
@@ -2188,7 +2176,7 @@
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" s="2" t="n">
+      <c r="P26" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -2255,7 +2243,7 @@
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" s="2" t="n">
+      <c r="P27" s="1" t="n">
         <v>45964</v>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -2322,7 +2310,7 @@
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" s="2" t="n">
+      <c r="P28" s="1" t="n">
         <v>45984</v>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -2454,7 +2442,7 @@
         </is>
       </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" s="2" t="n">
+      <c r="P30" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q30" t="inlineStr"/>
@@ -2586,7 +2574,7 @@
         </is>
       </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" s="2" t="n">
+      <c r="P32" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2657,7 +2645,7 @@
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" s="2" t="n">
+      <c r="P33" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -2724,7 +2712,7 @@
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
-      <c r="P34" s="2" t="n">
+      <c r="P34" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -2791,7 +2779,7 @@
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" s="2" t="n">
+      <c r="P35" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -2923,7 +2911,7 @@
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" s="2" t="n">
+      <c r="P37" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -2990,7 +2978,7 @@
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" s="2" t="n">
+      <c r="P38" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -3057,7 +3045,7 @@
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" s="2" t="n">
+      <c r="P39" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q39" t="inlineStr"/>
@@ -3189,7 +3177,7 @@
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" s="2" t="n">
+      <c r="P41" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q41" t="inlineStr"/>
@@ -3256,7 +3244,7 @@
         </is>
       </c>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" s="2" t="n">
+      <c r="P42" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -3323,7 +3311,7 @@
         </is>
       </c>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" s="2" t="n">
+      <c r="P43" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -3390,7 +3378,7 @@
         </is>
       </c>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" s="2" t="n">
+      <c r="P44" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -3652,7 +3640,7 @@
         </is>
       </c>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" s="2" t="n">
+      <c r="P48" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -3719,7 +3707,7 @@
         </is>
       </c>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" s="2" t="n">
+      <c r="P49" s="1" t="n">
         <v>45955</v>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -3786,7 +3774,7 @@
         </is>
       </c>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" s="2" t="n">
+      <c r="P50" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -3853,7 +3841,7 @@
         </is>
       </c>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" s="2" t="n">
+      <c r="P51" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q51" t="inlineStr">
@@ -3924,7 +3912,7 @@
         </is>
       </c>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" s="2" t="n">
+      <c r="P52" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -3991,7 +3979,7 @@
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" s="2" t="n">
+      <c r="P53" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -4119,7 +4107,7 @@
         </is>
       </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" s="2" t="n">
+      <c r="P55" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -4186,7 +4174,7 @@
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" s="2" t="n">
+      <c r="P56" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -4322,7 +4310,7 @@
         </is>
       </c>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" s="2" t="n">
+      <c r="P58" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -4389,7 +4377,7 @@
         </is>
       </c>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" s="2" t="n">
+      <c r="P59" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="Q59" t="inlineStr">
@@ -4460,7 +4448,7 @@
         </is>
       </c>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" s="2" t="n">
+      <c r="P60" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -4527,7 +4515,7 @@
         </is>
       </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" s="2" t="n">
+      <c r="P61" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q61" t="inlineStr"/>
@@ -4594,7 +4582,7 @@
         </is>
       </c>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" s="2" t="n">
+      <c r="P62" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q62" t="inlineStr"/>
@@ -4661,7 +4649,7 @@
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" s="2" t="n">
+      <c r="P63" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q63" t="inlineStr"/>
@@ -4728,7 +4716,7 @@
         </is>
       </c>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" s="2" t="n">
+      <c r="P64" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q64" t="inlineStr">
@@ -4799,7 +4787,7 @@
         </is>
       </c>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" s="2" t="n">
+      <c r="P65" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q65" t="inlineStr"/>
@@ -4866,7 +4854,7 @@
         </is>
       </c>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" s="2" t="n">
+      <c r="P66" s="1" t="n">
         <v>45946</v>
       </c>
       <c r="Q66" t="inlineStr">
@@ -4937,7 +4925,7 @@
         </is>
       </c>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" s="2" t="n">
+      <c r="P67" s="1" t="n">
         <v>45916</v>
       </c>
       <c r="Q67" t="inlineStr"/>
@@ -5004,7 +4992,7 @@
         </is>
       </c>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" s="2" t="n">
+      <c r="P68" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5075,7 +5063,7 @@
         </is>
       </c>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" s="2" t="n">
+      <c r="P69" s="1" t="n">
         <v>45989</v>
       </c>
       <c r="Q69" t="inlineStr">
@@ -5211,7 +5199,7 @@
         </is>
       </c>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" s="2" t="n">
+      <c r="P71" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -5278,7 +5266,7 @@
         </is>
       </c>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" s="2" t="n">
+      <c r="P72" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q72" t="inlineStr"/>
@@ -5345,7 +5333,7 @@
         </is>
       </c>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" s="2" t="n">
+      <c r="P73" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q73" t="inlineStr"/>
@@ -5412,7 +5400,7 @@
         </is>
       </c>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" s="2" t="n">
+      <c r="P74" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q74" t="inlineStr"/>
@@ -5479,7 +5467,7 @@
         </is>
       </c>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" s="2" t="n">
+      <c r="P75" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q75" t="inlineStr"/>
@@ -5546,7 +5534,7 @@
         </is>
       </c>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" s="2" t="n">
+      <c r="P76" s="1" t="n">
         <v>46130</v>
       </c>
       <c r="Q76" t="inlineStr"/>
@@ -5678,7 +5666,7 @@
         </is>
       </c>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" s="2" t="n">
+      <c r="P78" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q78" t="inlineStr"/>
@@ -5745,7 +5733,7 @@
         </is>
       </c>
       <c r="O79" t="inlineStr"/>
-      <c r="P79" s="2" t="n">
+      <c r="P79" s="1" t="n">
         <v>46140</v>
       </c>
       <c r="Q79" t="inlineStr"/>
@@ -5812,7 +5800,7 @@
         </is>
       </c>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" s="2" t="n">
+      <c r="P80" s="1" t="n">
         <v>46095</v>
       </c>
       <c r="Q80" t="inlineStr"/>
@@ -5879,7 +5867,7 @@
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" s="2" t="n">
+      <c r="P81" s="1" t="n">
         <v>46040</v>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -5946,7 +5934,7 @@
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" s="2" t="n">
+      <c r="P82" s="1" t="n">
         <v>46060</v>
       </c>
       <c r="Q82" t="inlineStr"/>
@@ -6013,7 +6001,7 @@
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" s="2" t="n">
+      <c r="P83" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -6080,7 +6068,7 @@
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" s="2" t="n">
+      <c r="P84" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q84" t="inlineStr"/>
@@ -6147,7 +6135,7 @@
         </is>
       </c>
       <c r="O85" t="inlineStr"/>
-      <c r="P85" s="2" t="n">
+      <c r="P85" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6218,7 +6206,7 @@
         </is>
       </c>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" s="2" t="n">
+      <c r="P86" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q86" t="inlineStr"/>
@@ -6285,7 +6273,7 @@
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" s="2" t="n">
+      <c r="P87" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q87" t="inlineStr"/>
@@ -6352,7 +6340,7 @@
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" s="2" t="n">
+      <c r="P88" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q88" t="inlineStr"/>
@@ -6419,7 +6407,7 @@
         </is>
       </c>
       <c r="O89" t="inlineStr"/>
-      <c r="P89" s="2" t="n">
+      <c r="P89" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q89" t="inlineStr"/>
@@ -6486,7 +6474,7 @@
         </is>
       </c>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" s="2" t="n">
+      <c r="P90" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q90" t="inlineStr"/>
@@ -6553,7 +6541,7 @@
         </is>
       </c>
       <c r="O91" t="inlineStr"/>
-      <c r="P91" s="2" t="n">
+      <c r="P91" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="Q91" t="inlineStr"/>
@@ -6620,7 +6608,7 @@
         </is>
       </c>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" s="2" t="n">
+      <c r="P92" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="Q92" t="inlineStr"/>
@@ -6687,7 +6675,7 @@
         </is>
       </c>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" s="2" t="n">
+      <c r="P93" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q93" t="inlineStr"/>
@@ -6754,7 +6742,7 @@
         </is>
       </c>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" s="2" t="n">
+      <c r="P94" s="1" t="n">
         <v>46037</v>
       </c>
       <c r="Q94" t="inlineStr"/>
@@ -6890,7 +6878,7 @@
         </is>
       </c>
       <c r="O96" t="inlineStr"/>
-      <c r="P96" s="2" t="n">
+      <c r="P96" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q96" t="inlineStr"/>
@@ -6957,7 +6945,7 @@
         </is>
       </c>
       <c r="O97" t="inlineStr"/>
-      <c r="P97" s="2" t="n">
+      <c r="P97" s="1" t="n">
         <v>46032</v>
       </c>
       <c r="Q97" t="inlineStr"/>
@@ -7154,7 +7142,7 @@
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
-      <c r="P100" s="2" t="n">
+      <c r="P100" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q100" t="inlineStr"/>
@@ -7221,7 +7209,7 @@
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
-      <c r="P101" s="2" t="n">
+      <c r="P101" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q101" t="inlineStr"/>
@@ -7288,7 +7276,7 @@
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
-      <c r="P102" s="2" t="n">
+      <c r="P102" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q102" t="inlineStr"/>
@@ -7355,7 +7343,7 @@
         </is>
       </c>
       <c r="O103" t="inlineStr"/>
-      <c r="P103" s="2" t="n">
+      <c r="P103" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q103" t="inlineStr"/>
@@ -7483,7 +7471,7 @@
         </is>
       </c>
       <c r="O105" t="inlineStr"/>
-      <c r="P105" s="2" t="n">
+      <c r="P105" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q105" t="inlineStr"/>
@@ -7550,7 +7538,7 @@
         </is>
       </c>
       <c r="O106" t="inlineStr"/>
-      <c r="P106" s="2" t="n">
+      <c r="P106" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q106" t="inlineStr">
@@ -7621,7 +7609,7 @@
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
-      <c r="P107" s="2" t="n">
+      <c r="P107" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -7688,7 +7676,7 @@
         </is>
       </c>
       <c r="O108" t="inlineStr"/>
-      <c r="P108" s="2" t="n">
+      <c r="P108" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -7885,7 +7873,7 @@
         </is>
       </c>
       <c r="O111" t="inlineStr"/>
-      <c r="P111" s="2" t="n">
+      <c r="P111" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -7952,7 +7940,7 @@
         </is>
       </c>
       <c r="O112" t="inlineStr"/>
-      <c r="P112" s="2" t="n">
+      <c r="P112" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -8084,7 +8072,7 @@
         </is>
       </c>
       <c r="O114" t="inlineStr"/>
-      <c r="P114" s="2" t="n">
+      <c r="P114" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q114" t="inlineStr"/>
@@ -8151,7 +8139,7 @@
         </is>
       </c>
       <c r="O115" t="inlineStr"/>
-      <c r="P115" s="2" t="n">
+      <c r="P115" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -8218,7 +8206,7 @@
         </is>
       </c>
       <c r="O116" t="inlineStr"/>
-      <c r="P116" s="2" t="n">
+      <c r="P116" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q116" t="inlineStr"/>
@@ -8285,7 +8273,7 @@
         </is>
       </c>
       <c r="O117" t="inlineStr"/>
-      <c r="P117" s="2" t="n">
+      <c r="P117" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="Q117" t="inlineStr"/>
@@ -8352,7 +8340,7 @@
         </is>
       </c>
       <c r="O118" t="inlineStr"/>
-      <c r="P118" s="2" t="n">
+      <c r="P118" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -8419,7 +8407,7 @@
         </is>
       </c>
       <c r="O119" t="inlineStr"/>
-      <c r="P119" s="2" t="n">
+      <c r="P119" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q119" t="inlineStr"/>
@@ -8486,7 +8474,7 @@
         </is>
       </c>
       <c r="O120" t="inlineStr"/>
-      <c r="P120" s="2" t="n">
+      <c r="P120" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q120" t="inlineStr"/>
@@ -8553,7 +8541,7 @@
         </is>
       </c>
       <c r="O121" t="inlineStr"/>
-      <c r="P121" s="2" t="n">
+      <c r="P121" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -8685,7 +8673,7 @@
         </is>
       </c>
       <c r="O123" t="inlineStr"/>
-      <c r="P123" s="2" t="n">
+      <c r="P123" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q123" t="inlineStr"/>
@@ -8947,7 +8935,7 @@
         </is>
       </c>
       <c r="O127" t="inlineStr"/>
-      <c r="P127" s="2" t="n">
+      <c r="P127" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q127" t="inlineStr"/>
@@ -9014,7 +9002,7 @@
         </is>
       </c>
       <c r="O128" t="inlineStr"/>
-      <c r="P128" s="2" t="n">
+      <c r="P128" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q128" t="inlineStr"/>
@@ -9081,7 +9069,7 @@
         </is>
       </c>
       <c r="O129" t="inlineStr"/>
-      <c r="P129" s="2" t="n">
+      <c r="P129" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q129" t="inlineStr"/>
@@ -9148,7 +9136,7 @@
         </is>
       </c>
       <c r="O130" t="inlineStr"/>
-      <c r="P130" s="2" t="n">
+      <c r="P130" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q130" t="inlineStr"/>
@@ -9215,7 +9203,7 @@
         </is>
       </c>
       <c r="O131" t="inlineStr"/>
-      <c r="P131" s="2" t="n">
+      <c r="P131" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -9282,7 +9270,7 @@
         </is>
       </c>
       <c r="O132" t="inlineStr"/>
-      <c r="P132" s="2" t="n">
+      <c r="P132" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -9349,7 +9337,7 @@
         </is>
       </c>
       <c r="O133" t="inlineStr"/>
-      <c r="P133" s="2" t="n">
+      <c r="P133" s="1" t="n">
         <v>46130</v>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -9481,7 +9469,7 @@
         </is>
       </c>
       <c r="O135" t="inlineStr"/>
-      <c r="P135" s="2" t="n">
+      <c r="P135" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q135" t="inlineStr"/>
@@ -9548,7 +9536,7 @@
         </is>
       </c>
       <c r="O136" t="inlineStr"/>
-      <c r="P136" s="2" t="n">
+      <c r="P136" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q136" t="inlineStr"/>
@@ -9680,7 +9668,7 @@
         </is>
       </c>
       <c r="O138" t="inlineStr"/>
-      <c r="P138" s="2" t="n">
+      <c r="P138" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q138" t="inlineStr"/>
@@ -9877,7 +9865,7 @@
         </is>
       </c>
       <c r="O141" t="inlineStr"/>
-      <c r="P141" s="2" t="n">
+      <c r="P141" s="1" t="n">
         <v>46160</v>
       </c>
       <c r="Q141" t="inlineStr"/>
@@ -9944,7 +9932,7 @@
         </is>
       </c>
       <c r="O142" t="inlineStr"/>
-      <c r="P142" s="2" t="n">
+      <c r="P142" s="1" t="n">
         <v>46123</v>
       </c>
       <c r="Q142" t="inlineStr"/>
@@ -10076,7 +10064,7 @@
         </is>
       </c>
       <c r="O144" t="inlineStr"/>
-      <c r="P144" s="2" t="n">
+      <c r="P144" s="1" t="n">
         <v>46167</v>
       </c>
       <c r="Q144" t="inlineStr"/>
@@ -10143,7 +10131,7 @@
         </is>
       </c>
       <c r="O145" t="inlineStr"/>
-      <c r="P145" s="2" t="n">
+      <c r="P145" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q145" t="inlineStr"/>
@@ -10210,7 +10198,7 @@
         </is>
       </c>
       <c r="O146" t="inlineStr"/>
-      <c r="P146" s="2" t="n">
+      <c r="P146" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="Q146" t="inlineStr"/>
@@ -10277,7 +10265,7 @@
         </is>
       </c>
       <c r="O147" t="inlineStr"/>
-      <c r="P147" s="2" t="n">
+      <c r="P147" s="1" t="n">
         <v>46081</v>
       </c>
       <c r="Q147" t="inlineStr"/>
@@ -10344,7 +10332,7 @@
         </is>
       </c>
       <c r="O148" t="inlineStr"/>
-      <c r="P148" s="2" t="n">
+      <c r="P148" s="1" t="n">
         <v>45976</v>
       </c>
       <c r="Q148" t="inlineStr"/>
@@ -10411,7 +10399,7 @@
         </is>
       </c>
       <c r="O149" t="inlineStr"/>
-      <c r="P149" s="2" t="n">
+      <c r="P149" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q149" t="inlineStr"/>
@@ -10478,7 +10466,7 @@
         </is>
       </c>
       <c r="O150" t="inlineStr"/>
-      <c r="P150" s="2" t="n">
+      <c r="P150" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q150" t="inlineStr"/>
@@ -10545,7 +10533,7 @@
         </is>
       </c>
       <c r="O151" t="inlineStr"/>
-      <c r="P151" s="2" t="n">
+      <c r="P151" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="Q151" t="inlineStr"/>
@@ -10677,7 +10665,7 @@
         </is>
       </c>
       <c r="O153" t="inlineStr"/>
-      <c r="P153" s="2" t="n">
+      <c r="P153" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q153" t="inlineStr"/>
@@ -10939,7 +10927,7 @@
         </is>
       </c>
       <c r="O157" t="inlineStr"/>
-      <c r="P157" s="2" t="n">
+      <c r="P157" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="Q157" t="inlineStr"/>
@@ -11006,7 +10994,7 @@
         </is>
       </c>
       <c r="O158" t="inlineStr"/>
-      <c r="P158" s="2" t="n">
+      <c r="P158" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q158" t="inlineStr"/>
@@ -11073,7 +11061,7 @@
         </is>
       </c>
       <c r="O159" t="inlineStr"/>
-      <c r="P159" s="2" t="n">
+      <c r="P159" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q159" t="inlineStr"/>
@@ -11140,7 +11128,7 @@
         </is>
       </c>
       <c r="O160" t="inlineStr"/>
-      <c r="P160" s="2" t="n">
+      <c r="P160" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q160" t="inlineStr"/>
@@ -11272,7 +11260,7 @@
         </is>
       </c>
       <c r="O162" t="inlineStr"/>
-      <c r="P162" s="2" t="n">
+      <c r="P162" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q162" t="inlineStr"/>
@@ -11339,7 +11327,7 @@
         </is>
       </c>
       <c r="O163" t="inlineStr"/>
-      <c r="P163" s="2" t="n">
+      <c r="P163" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q163" t="inlineStr"/>
@@ -11406,7 +11394,7 @@
         </is>
       </c>
       <c r="O164" t="inlineStr"/>
-      <c r="P164" s="2" t="n">
+      <c r="P164" s="1" t="n">
         <v>45984</v>
       </c>
       <c r="Q164" t="inlineStr"/>
@@ -11473,7 +11461,7 @@
         </is>
       </c>
       <c r="O165" t="inlineStr"/>
-      <c r="P165" s="2" t="n">
+      <c r="P165" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q165" t="inlineStr"/>
@@ -11540,7 +11528,7 @@
         </is>
       </c>
       <c r="O166" t="inlineStr"/>
-      <c r="P166" s="2" t="n">
+      <c r="P166" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q166" t="inlineStr"/>
@@ -11607,7 +11595,7 @@
         </is>
       </c>
       <c r="O167" t="inlineStr"/>
-      <c r="P167" s="2" t="n">
+      <c r="P167" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q167" t="inlineStr"/>
@@ -11674,7 +11662,7 @@
         </is>
       </c>
       <c r="O168" t="inlineStr"/>
-      <c r="P168" s="2" t="n">
+      <c r="P168" s="1" t="n">
         <v>45994</v>
       </c>
       <c r="Q168" t="inlineStr"/>
@@ -11741,7 +11729,7 @@
         </is>
       </c>
       <c r="O169" t="inlineStr"/>
-      <c r="P169" s="2" t="n">
+      <c r="P169" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q169" t="inlineStr"/>
@@ -11808,7 +11796,7 @@
         </is>
       </c>
       <c r="O170" t="inlineStr"/>
-      <c r="P170" s="2" t="n">
+      <c r="P170" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q170" t="inlineStr"/>
@@ -11875,7 +11863,7 @@
         </is>
       </c>
       <c r="O171" t="inlineStr"/>
-      <c r="P171" s="2" t="n">
+      <c r="P171" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q171" t="inlineStr"/>
@@ -11942,7 +11930,7 @@
         </is>
       </c>
       <c r="O172" t="inlineStr"/>
-      <c r="P172" s="2" t="n">
+      <c r="P172" s="1" t="n">
         <v>45954</v>
       </c>
       <c r="Q172" t="inlineStr"/>
@@ -12009,7 +11997,7 @@
         </is>
       </c>
       <c r="O173" t="inlineStr"/>
-      <c r="P173" s="2" t="n">
+      <c r="P173" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q173" t="inlineStr"/>
@@ -12076,7 +12064,7 @@
         </is>
       </c>
       <c r="O174" t="inlineStr"/>
-      <c r="P174" s="2" t="n">
+      <c r="P174" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q174" t="inlineStr"/>
@@ -12143,7 +12131,7 @@
         </is>
       </c>
       <c r="O175" t="inlineStr"/>
-      <c r="P175" s="2" t="n">
+      <c r="P175" s="1" t="n">
         <v>45911</v>
       </c>
       <c r="Q175" t="inlineStr"/>
@@ -12210,7 +12198,7 @@
         </is>
       </c>
       <c r="O176" t="inlineStr"/>
-      <c r="P176" s="2" t="n">
+      <c r="P176" s="1" t="n">
         <v>45835</v>
       </c>
       <c r="Q176" t="inlineStr"/>
@@ -12277,7 +12265,7 @@
         </is>
       </c>
       <c r="O177" t="inlineStr"/>
-      <c r="P177" s="2" t="n">
+      <c r="P177" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q177" t="inlineStr"/>
@@ -12344,7 +12332,7 @@
         </is>
       </c>
       <c r="O178" t="inlineStr"/>
-      <c r="P178" s="2" t="n">
+      <c r="P178" s="1" t="n">
         <v>45908</v>
       </c>
       <c r="Q178" t="inlineStr"/>
@@ -12411,7 +12399,7 @@
         </is>
       </c>
       <c r="O179" t="inlineStr"/>
-      <c r="P179" s="2" t="n">
+      <c r="P179" s="1" t="n">
         <v>45835</v>
       </c>
       <c r="Q179" t="inlineStr"/>
@@ -12478,7 +12466,7 @@
         </is>
       </c>
       <c r="O180" t="inlineStr"/>
-      <c r="P180" s="2" t="n">
+      <c r="P180" s="1" t="n">
         <v>46025</v>
       </c>
       <c r="Q180" t="inlineStr"/>
@@ -12545,7 +12533,7 @@
         </is>
       </c>
       <c r="O181" t="inlineStr"/>
-      <c r="P181" s="2" t="n">
+      <c r="P181" s="1" t="n">
         <v>46024</v>
       </c>
       <c r="Q181" t="inlineStr"/>
@@ -12612,7 +12600,7 @@
         </is>
       </c>
       <c r="O182" t="inlineStr"/>
-      <c r="P182" s="2" t="n">
+      <c r="P182" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q182" t="inlineStr"/>
@@ -12744,7 +12732,7 @@
         </is>
       </c>
       <c r="O184" t="inlineStr"/>
-      <c r="P184" s="2" t="n">
+      <c r="P184" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q184" t="inlineStr"/>
@@ -12876,7 +12864,7 @@
         </is>
       </c>
       <c r="O186" t="inlineStr"/>
-      <c r="P186" s="2" t="n">
+      <c r="P186" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="Q186" t="inlineStr"/>
@@ -12896,87 +12884,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_requisicao</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pjt</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pn</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>qtd</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_unit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>status_comprar</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>status_11g</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>status_atual</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>previsao_empenho</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao_previsao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dias_atraso</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dpe</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>observacao_coordenadores</t>
         </is>
@@ -13037,8 +13025,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n">
-        <v>46223</v>
+      <c r="M2" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -13104,8 +13092,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M3" s="2" t="n">
-        <v>46223</v>
+      <c r="M3" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -13171,8 +13159,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>46223</v>
+      <c r="M4" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -13238,8 +13226,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
-        <v>46223</v>
+      <c r="M5" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -13305,8 +13293,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
-        <v>46223</v>
+      <c r="M6" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -13372,8 +13360,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
-        <v>46223</v>
+      <c r="M7" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -13439,8 +13427,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M8" s="2" t="n">
-        <v>46288</v>
+      <c r="M8" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -13506,8 +13494,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n">
-        <v>46223</v>
+      <c r="M9" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -13573,8 +13561,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n">
-        <v>46288</v>
+      <c r="M10" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -13640,8 +13628,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M11" s="2" t="n">
-        <v>46288</v>
+      <c r="M11" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -13772,8 +13760,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M13" s="2" t="n">
-        <v>46223</v>
+      <c r="M13" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -13839,8 +13827,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M14" s="2" t="n">
-        <v>46223</v>
+      <c r="M14" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -13906,8 +13894,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M15" s="2" t="n">
-        <v>46303</v>
+      <c r="M15" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -13973,8 +13961,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M16" s="2" t="n">
-        <v>46288</v>
+      <c r="M16" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -14040,8 +14028,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M17" s="2" t="n">
-        <v>46303</v>
+      <c r="M17" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -14107,8 +14095,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M18" s="2" t="n">
-        <v>46288</v>
+      <c r="M18" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -14174,8 +14162,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M19" s="2" t="n">
-        <v>46288</v>
+      <c r="M19" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -14241,8 +14229,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M20" s="2" t="n">
-        <v>46288</v>
+      <c r="M20" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -14308,8 +14296,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M21" s="2" t="n">
-        <v>46288</v>
+      <c r="M21" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -14375,8 +14363,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M22" s="2" t="n">
-        <v>46223</v>
+      <c r="M22" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -14442,8 +14430,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M23" s="2" t="n">
-        <v>46223</v>
+      <c r="M23" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -14509,8 +14497,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M24" s="2" t="n">
-        <v>46223</v>
+      <c r="M24" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -14576,8 +14564,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n">
-        <v>46303</v>
+      <c r="M25" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -14643,8 +14631,8 @@
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="M26" s="2" t="n">
-        <v>46223</v>
+      <c r="M26" s="1" t="n">
+        <v>46224</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -14710,8 +14698,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M27" s="2" t="n">
-        <v>46288</v>
+      <c r="M27" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -14777,8 +14765,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M28" s="2" t="n">
-        <v>46288</v>
+      <c r="M28" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -14844,8 +14832,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M29" s="2" t="n">
-        <v>46288</v>
+      <c r="M29" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -14911,8 +14899,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M30" s="2" t="n">
-        <v>46288</v>
+      <c r="M30" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -14978,8 +14966,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M31" s="2" t="n">
-        <v>46303</v>
+      <c r="M31" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -15045,8 +15033,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M32" s="2" t="n">
-        <v>46303</v>
+      <c r="M32" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -15112,8 +15100,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M33" s="2" t="n">
-        <v>46303</v>
+      <c r="M33" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -15179,8 +15167,8 @@
           <t>Validada</t>
         </is>
       </c>
-      <c r="M34" s="2" t="n">
-        <v>46288</v>
+      <c r="M34" s="1" t="n">
+        <v>46289</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -15246,8 +15234,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M35" s="2" t="n">
-        <v>46303</v>
+      <c r="M35" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -15313,8 +15301,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M36" s="2" t="n">
-        <v>46303</v>
+      <c r="M36" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -15380,8 +15368,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M37" s="2" t="n">
-        <v>46303</v>
+      <c r="M37" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -15447,8 +15435,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M38" s="2" t="n">
-        <v>46303</v>
+      <c r="M38" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -15514,8 +15502,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M39" s="2" t="n">
-        <v>46303</v>
+      <c r="M39" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -15581,8 +15569,8 @@
           <t>Análise do Pedido</t>
         </is>
       </c>
-      <c r="M40" s="2" t="n">
-        <v>46303</v>
+      <c r="M40" s="1" t="n">
+        <v>46304</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática: tpjl (14/07/2026 06:40)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -12880,7 +12880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13007,26 +13007,26 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Mapa Aprovado</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M2" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -13074,7 +13074,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Aguardando Intenção de Recurso</t>
+          <t>Mapa Aprovado</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -13093,7 +13093,7 @@
         </is>
       </c>
       <c r="M3" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -13141,26 +13141,26 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Mapa Aprovado</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M4" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -13227,7 +13227,7 @@
         </is>
       </c>
       <c r="M5" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -13275,7 +13275,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Aguardando Intenção de Recurso</t>
+          <t>Mapa Aprovado</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -13294,7 +13294,7 @@
         </is>
       </c>
       <c r="M6" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -13342,7 +13342,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Aguardando Intenção de Recurso</t>
+          <t>Mapa Aprovado</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -13361,7 +13361,7 @@
         </is>
       </c>
       <c r="M7" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -13428,7 +13428,7 @@
         </is>
       </c>
       <c r="M8" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -13476,7 +13476,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Aguardando Intenção de Recurso</t>
+          <t>Mapa Aprovado</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -13495,7 +13495,7 @@
         </is>
       </c>
       <c r="M9" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -13562,7 +13562,7 @@
         </is>
       </c>
       <c r="M10" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -13629,7 +13629,7 @@
         </is>
       </c>
       <c r="M11" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -13742,26 +13742,26 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>Aguardando Conferência do ACI</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M13" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -13809,26 +13809,26 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>Mapa Aprovado</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M14" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -13895,7 +13895,7 @@
         </is>
       </c>
       <c r="M15" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -13962,7 +13962,7 @@
         </is>
       </c>
       <c r="M16" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -14029,7 +14029,7 @@
         </is>
       </c>
       <c r="M17" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -14096,7 +14096,7 @@
         </is>
       </c>
       <c r="M18" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -14163,7 +14163,7 @@
         </is>
       </c>
       <c r="M19" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -14230,7 +14230,7 @@
         </is>
       </c>
       <c r="M20" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -14297,7 +14297,7 @@
         </is>
       </c>
       <c r="M21" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -14345,26 +14345,26 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>Mapa Aprovado</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M22" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -14412,26 +14412,26 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>Mapa Aprovado</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M23" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -14479,26 +14479,26 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>Mapa Aprovado</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M24" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -14565,7 +14565,7 @@
         </is>
       </c>
       <c r="M25" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -14613,26 +14613,26 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>Mapa Aprovado</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>Mapa Gerado</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Mapa Gerado</t>
-        </is>
-      </c>
       <c r="M26" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -14699,7 +14699,7 @@
         </is>
       </c>
       <c r="M27" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -14766,7 +14766,7 @@
         </is>
       </c>
       <c r="M28" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -14833,7 +14833,7 @@
         </is>
       </c>
       <c r="M29" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -14900,7 +14900,7 @@
         </is>
       </c>
       <c r="M30" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -14967,7 +14967,7 @@
         </is>
       </c>
       <c r="M31" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -15034,7 +15034,7 @@
         </is>
       </c>
       <c r="M32" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -15101,7 +15101,7 @@
         </is>
       </c>
       <c r="M33" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -15168,7 +15168,7 @@
         </is>
       </c>
       <c r="M34" s="1" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -15235,7 +15235,7 @@
         </is>
       </c>
       <c r="M35" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -15283,7 +15283,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Aguardando Validação</t>
+          <t>Análise do Pedido</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -15302,7 +15302,7 @@
         </is>
       </c>
       <c r="M36" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -15350,7 +15350,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Aguardando Validação</t>
+          <t>Análise do Pedido</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -15369,7 +15369,7 @@
         </is>
       </c>
       <c r="M37" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -15417,7 +15417,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Aguardando Validação</t>
+          <t>Análise do Pedido</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -15436,7 +15436,7 @@
         </is>
       </c>
       <c r="M38" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -15503,7 +15503,7 @@
         </is>
       </c>
       <c r="M39" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -15551,7 +15551,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Aguardando Validação</t>
+          <t>Análise do Pedido</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -15570,7 +15570,7 @@
         </is>
       </c>
       <c r="M40" s="1" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -15580,6 +15580,195 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LST187002U8</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2601188-204</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>COMPRESSOR DRIVE ASSY</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>7603</v>
+      </c>
+      <c r="H41" t="n">
+        <v>7603</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Aguardando Validação</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Aguardando Validação</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Aguardando Validação</t>
+        </is>
+      </c>
+      <c r="M41" s="1" t="n">
+        <v>46297</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>No prazo</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LST190003U8</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P7036368-01</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PROPELLER ASSEMBLY</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" t="n">
+        <v>42076.37</v>
+      </c>
+      <c r="H42" t="n">
+        <v>210381.85</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Análise do Pedido</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Análise do Pedido</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Análise do Pedido</t>
+        </is>
+      </c>
+      <c r="M42" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>No prazo</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LST191002U8</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>30994-001</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BATTERY-MARATHON TSP410 NICAD</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H43" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Análise do Pedido</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Análise do Pedido</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Análise do Pedido</t>
+        </is>
+      </c>
+      <c r="M43" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>No prazo</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualização automática: tpjl (15/07/2026 16:11)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10117,7 +10117,7 @@
         <v>514</v>
       </c>
       <c r="M2" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N2" t="s">
         <v>518</v>
@@ -10161,7 +10161,7 @@
         <v>514</v>
       </c>
       <c r="M3" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N3" t="s">
         <v>518</v>
@@ -10205,7 +10205,7 @@
         <v>514</v>
       </c>
       <c r="M4" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N4" t="s">
         <v>518</v>
@@ -10249,7 +10249,7 @@
         <v>514</v>
       </c>
       <c r="M5" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N5" t="s">
         <v>518</v>
@@ -10293,7 +10293,7 @@
         <v>514</v>
       </c>
       <c r="M6" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N6" t="s">
         <v>518</v>
@@ -10337,7 +10337,7 @@
         <v>514</v>
       </c>
       <c r="M7" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N7" t="s">
         <v>518</v>
@@ -10381,7 +10381,7 @@
         <v>515</v>
       </c>
       <c r="M8" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N8" t="s">
         <v>518</v>
@@ -10425,7 +10425,7 @@
         <v>514</v>
       </c>
       <c r="M9" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N9" t="s">
         <v>518</v>
@@ -10469,7 +10469,7 @@
         <v>515</v>
       </c>
       <c r="M10" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N10" t="s">
         <v>518</v>
@@ -10513,7 +10513,7 @@
         <v>515</v>
       </c>
       <c r="M11" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N11" t="s">
         <v>518</v>
@@ -10598,7 +10598,7 @@
         <v>514</v>
       </c>
       <c r="M13" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N13" t="s">
         <v>518</v>
@@ -10642,7 +10642,7 @@
         <v>514</v>
       </c>
       <c r="M14" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N14" t="s">
         <v>518</v>
@@ -10686,7 +10686,7 @@
         <v>517</v>
       </c>
       <c r="M15" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N15" t="s">
         <v>518</v>
@@ -10730,7 +10730,7 @@
         <v>515</v>
       </c>
       <c r="M16" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N16" t="s">
         <v>518</v>
@@ -10774,7 +10774,7 @@
         <v>517</v>
       </c>
       <c r="M17" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N17" t="s">
         <v>518</v>
@@ -10818,7 +10818,7 @@
         <v>515</v>
       </c>
       <c r="M18" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N18" t="s">
         <v>518</v>
@@ -10862,7 +10862,7 @@
         <v>515</v>
       </c>
       <c r="M19" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N19" t="s">
         <v>518</v>
@@ -10906,7 +10906,7 @@
         <v>515</v>
       </c>
       <c r="M20" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N20" t="s">
         <v>518</v>
@@ -10950,7 +10950,7 @@
         <v>515</v>
       </c>
       <c r="M21" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N21" t="s">
         <v>518</v>
@@ -10994,7 +10994,7 @@
         <v>514</v>
       </c>
       <c r="M22" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N22" t="s">
         <v>518</v>
@@ -11038,7 +11038,7 @@
         <v>514</v>
       </c>
       <c r="M23" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N23" t="s">
         <v>518</v>
@@ -11082,7 +11082,7 @@
         <v>514</v>
       </c>
       <c r="M24" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N24" t="s">
         <v>518</v>
@@ -11126,7 +11126,7 @@
         <v>517</v>
       </c>
       <c r="M25" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N25" t="s">
         <v>518</v>
@@ -11170,7 +11170,7 @@
         <v>514</v>
       </c>
       <c r="M26" s="1">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="N26" t="s">
         <v>518</v>
@@ -11214,7 +11214,7 @@
         <v>515</v>
       </c>
       <c r="M27" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N27" t="s">
         <v>518</v>
@@ -11258,7 +11258,7 @@
         <v>515</v>
       </c>
       <c r="M28" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N28" t="s">
         <v>518</v>
@@ -11302,7 +11302,7 @@
         <v>515</v>
       </c>
       <c r="M29" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N29" t="s">
         <v>518</v>
@@ -11346,7 +11346,7 @@
         <v>515</v>
       </c>
       <c r="M30" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N30" t="s">
         <v>518</v>
@@ -11390,7 +11390,7 @@
         <v>517</v>
       </c>
       <c r="M31" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N31" t="s">
         <v>518</v>
@@ -11434,7 +11434,7 @@
         <v>517</v>
       </c>
       <c r="M32" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N32" t="s">
         <v>518</v>
@@ -11478,7 +11478,7 @@
         <v>517</v>
       </c>
       <c r="M33" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N33" t="s">
         <v>518</v>
@@ -11522,7 +11522,7 @@
         <v>515</v>
       </c>
       <c r="M34" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N34" t="s">
         <v>518</v>
@@ -11566,7 +11566,7 @@
         <v>517</v>
       </c>
       <c r="M35" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N35" t="s">
         <v>518</v>
@@ -11610,7 +11610,7 @@
         <v>517</v>
       </c>
       <c r="M36" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N36" t="s">
         <v>518</v>
@@ -11654,7 +11654,7 @@
         <v>517</v>
       </c>
       <c r="M37" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N37" t="s">
         <v>518</v>
@@ -11698,7 +11698,7 @@
         <v>517</v>
       </c>
       <c r="M38" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N38" t="s">
         <v>518</v>
@@ -11742,7 +11742,7 @@
         <v>517</v>
       </c>
       <c r="M39" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N39" t="s">
         <v>518</v>
@@ -11786,7 +11786,7 @@
         <v>517</v>
       </c>
       <c r="M40" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N40" t="s">
         <v>518</v>
@@ -11827,7 +11827,7 @@
         <v>382</v>
       </c>
       <c r="M41" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N41" t="s">
         <v>518</v>
@@ -11868,7 +11868,7 @@
         <v>517</v>
       </c>
       <c r="M42" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N42" t="s">
         <v>518</v>
@@ -11909,7 +11909,7 @@
         <v>517</v>
       </c>
       <c r="M43" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N43" t="s">
         <v>518</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (16/07/2026 16:04)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10117,7 +10117,7 @@
         <v>514</v>
       </c>
       <c r="M2" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N2" t="s">
         <v>518</v>
@@ -10161,7 +10161,7 @@
         <v>514</v>
       </c>
       <c r="M3" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N3" t="s">
         <v>518</v>
@@ -10205,7 +10205,7 @@
         <v>514</v>
       </c>
       <c r="M4" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N4" t="s">
         <v>518</v>
@@ -10249,7 +10249,7 @@
         <v>514</v>
       </c>
       <c r="M5" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N5" t="s">
         <v>518</v>
@@ -10293,7 +10293,7 @@
         <v>514</v>
       </c>
       <c r="M6" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N6" t="s">
         <v>518</v>
@@ -10337,7 +10337,7 @@
         <v>514</v>
       </c>
       <c r="M7" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N7" t="s">
         <v>518</v>
@@ -10381,7 +10381,7 @@
         <v>515</v>
       </c>
       <c r="M8" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N8" t="s">
         <v>518</v>
@@ -10425,7 +10425,7 @@
         <v>514</v>
       </c>
       <c r="M9" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N9" t="s">
         <v>518</v>
@@ -10469,7 +10469,7 @@
         <v>515</v>
       </c>
       <c r="M10" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N10" t="s">
         <v>518</v>
@@ -10513,7 +10513,7 @@
         <v>515</v>
       </c>
       <c r="M11" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N11" t="s">
         <v>518</v>
@@ -10598,7 +10598,7 @@
         <v>514</v>
       </c>
       <c r="M13" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N13" t="s">
         <v>518</v>
@@ -10642,7 +10642,7 @@
         <v>514</v>
       </c>
       <c r="M14" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N14" t="s">
         <v>518</v>
@@ -10686,7 +10686,7 @@
         <v>517</v>
       </c>
       <c r="M15" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N15" t="s">
         <v>518</v>
@@ -10730,7 +10730,7 @@
         <v>515</v>
       </c>
       <c r="M16" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N16" t="s">
         <v>518</v>
@@ -10774,7 +10774,7 @@
         <v>517</v>
       </c>
       <c r="M17" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N17" t="s">
         <v>518</v>
@@ -10818,7 +10818,7 @@
         <v>515</v>
       </c>
       <c r="M18" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N18" t="s">
         <v>518</v>
@@ -10862,7 +10862,7 @@
         <v>515</v>
       </c>
       <c r="M19" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N19" t="s">
         <v>518</v>
@@ -10906,7 +10906,7 @@
         <v>515</v>
       </c>
       <c r="M20" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N20" t="s">
         <v>518</v>
@@ -10950,7 +10950,7 @@
         <v>515</v>
       </c>
       <c r="M21" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N21" t="s">
         <v>518</v>
@@ -10994,7 +10994,7 @@
         <v>514</v>
       </c>
       <c r="M22" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N22" t="s">
         <v>518</v>
@@ -11038,7 +11038,7 @@
         <v>514</v>
       </c>
       <c r="M23" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N23" t="s">
         <v>518</v>
@@ -11082,7 +11082,7 @@
         <v>514</v>
       </c>
       <c r="M24" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N24" t="s">
         <v>518</v>
@@ -11126,7 +11126,7 @@
         <v>517</v>
       </c>
       <c r="M25" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N25" t="s">
         <v>518</v>
@@ -11170,7 +11170,7 @@
         <v>514</v>
       </c>
       <c r="M26" s="1">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="N26" t="s">
         <v>518</v>
@@ -11214,7 +11214,7 @@
         <v>515</v>
       </c>
       <c r="M27" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N27" t="s">
         <v>518</v>
@@ -11258,7 +11258,7 @@
         <v>515</v>
       </c>
       <c r="M28" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N28" t="s">
         <v>518</v>
@@ -11302,7 +11302,7 @@
         <v>515</v>
       </c>
       <c r="M29" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N29" t="s">
         <v>518</v>
@@ -11346,7 +11346,7 @@
         <v>515</v>
       </c>
       <c r="M30" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N30" t="s">
         <v>518</v>
@@ -11390,7 +11390,7 @@
         <v>517</v>
       </c>
       <c r="M31" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N31" t="s">
         <v>518</v>
@@ -11434,7 +11434,7 @@
         <v>517</v>
       </c>
       <c r="M32" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N32" t="s">
         <v>518</v>
@@ -11478,7 +11478,7 @@
         <v>517</v>
       </c>
       <c r="M33" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N33" t="s">
         <v>518</v>
@@ -11522,7 +11522,7 @@
         <v>515</v>
       </c>
       <c r="M34" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N34" t="s">
         <v>518</v>
@@ -11566,7 +11566,7 @@
         <v>517</v>
       </c>
       <c r="M35" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N35" t="s">
         <v>518</v>
@@ -11610,7 +11610,7 @@
         <v>517</v>
       </c>
       <c r="M36" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N36" t="s">
         <v>518</v>
@@ -11654,7 +11654,7 @@
         <v>517</v>
       </c>
       <c r="M37" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N37" t="s">
         <v>518</v>
@@ -11698,7 +11698,7 @@
         <v>517</v>
       </c>
       <c r="M38" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N38" t="s">
         <v>518</v>
@@ -11742,7 +11742,7 @@
         <v>517</v>
       </c>
       <c r="M39" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N39" t="s">
         <v>518</v>
@@ -11786,7 +11786,7 @@
         <v>517</v>
       </c>
       <c r="M40" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N40" t="s">
         <v>518</v>
@@ -11827,7 +11827,7 @@
         <v>382</v>
       </c>
       <c r="M41" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N41" t="s">
         <v>518</v>
@@ -11868,7 +11868,7 @@
         <v>517</v>
       </c>
       <c r="M42" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N42" t="s">
         <v>518</v>
@@ -11909,7 +11909,7 @@
         <v>517</v>
       </c>
       <c r="M43" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N43" t="s">
         <v>518</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (17/07/2026 16:04)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2313" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2403" uniqueCount="548">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1361,6 +1361,36 @@
     <t>LST191002U8</t>
   </si>
   <si>
+    <t>LST196002U8</t>
+  </si>
+  <si>
+    <t>LST196003U8</t>
+  </si>
+  <si>
+    <t>LST196004U8</t>
+  </si>
+  <si>
+    <t>LST196005U8</t>
+  </si>
+  <si>
+    <t>LST197001U8</t>
+  </si>
+  <si>
+    <t>LST197002U8</t>
+  </si>
+  <si>
+    <t>LST197003U8</t>
+  </si>
+  <si>
+    <t>LST197004U8</t>
+  </si>
+  <si>
+    <t>LST197005U8</t>
+  </si>
+  <si>
+    <t>LST197006U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1466,6 +1496,36 @@
     <t>30994-001</t>
   </si>
   <si>
+    <t>723908</t>
+  </si>
+  <si>
+    <t>S3465-2-0112</t>
+  </si>
+  <si>
+    <t>2613439-1</t>
+  </si>
+  <si>
+    <t>2617015-22</t>
+  </si>
+  <si>
+    <t>2617015-18</t>
+  </si>
+  <si>
+    <t>E6391</t>
+  </si>
+  <si>
+    <t>011-01020-10</t>
+  </si>
+  <si>
+    <t>PM-57</t>
+  </si>
+  <si>
+    <t>5319026-1</t>
+  </si>
+  <si>
+    <t>2615011-2</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1557,6 +1617,33 @@
   </si>
   <si>
     <t>BATTERY-MARATHON TSP410 NICAD</t>
+  </si>
+  <si>
+    <t>HOSE ASSY TEE</t>
+  </si>
+  <si>
+    <t>SHIELD</t>
+  </si>
+  <si>
+    <t>HINGE DOOR LH</t>
+  </si>
+  <si>
+    <t>BULKHEAD ASSY</t>
+  </si>
+  <si>
+    <t>AFCS MODE CONTROLLER GMC 710</t>
+  </si>
+  <si>
+    <t>RADOME BOOT</t>
+  </si>
+  <si>
+    <t>HANDLE,DOOR</t>
+  </si>
+  <si>
+    <t>WINDOW MOLDING</t>
+  </si>
+  <si>
+    <t>Empenho Solicitado</t>
   </si>
   <si>
     <t>Mapa Gerado</t>
@@ -10023,7 +10110,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q43"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10105,22 +10192,22 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J2" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K2" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L2" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M2" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N2" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -10149,22 +10236,22 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J3" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K3" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L3" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M3" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N3" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -10178,7 +10265,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10193,22 +10280,22 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J4" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K4" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L4" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M4" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N4" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -10222,10 +10309,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>449</v>
+        <v>459</v>
       </c>
       <c r="E5" t="s">
-        <v>483</v>
+        <v>503</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10237,22 +10324,22 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="J5" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K5" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L5" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M5" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N5" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -10281,22 +10368,22 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J6" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K6" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L6" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M6" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N6" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -10325,22 +10412,22 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J7" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K7" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L7" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M7" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N7" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -10369,22 +10456,22 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="J8" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K8" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L8" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M8" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N8" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10398,7 +10485,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10413,22 +10500,22 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J9" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K9" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L9" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M9" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N9" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -10442,10 +10529,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>451</v>
+        <v>461</v>
       </c>
       <c r="E10" t="s">
-        <v>484</v>
+        <v>504</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10460,19 +10547,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K10" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L10" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M10" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N10" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10486,7 +10573,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10504,19 +10591,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K11" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L11" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M11" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N11" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10530,10 +10617,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="E12" t="s">
-        <v>485</v>
+        <v>505</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -10586,22 +10673,22 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>516</v>
+        <v>545</v>
       </c>
       <c r="J13" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K13" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L13" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M13" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N13" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -10615,10 +10702,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
       <c r="E14" t="s">
-        <v>486</v>
+        <v>506</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -10630,22 +10717,22 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J14" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K14" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L14" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M14" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N14" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -10659,10 +10746,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="E15" t="s">
-        <v>487</v>
+        <v>507</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -10674,22 +10761,22 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J15" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K15" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L15" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M15" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N15" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10703,10 +10790,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>456</v>
+        <v>466</v>
       </c>
       <c r="E16" t="s">
-        <v>488</v>
+        <v>508</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -10721,19 +10808,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K16" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L16" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M16" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N16" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10747,10 +10834,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
       <c r="E17" t="s">
-        <v>489</v>
+        <v>509</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -10762,22 +10849,22 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J17" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K17" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L17" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M17" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N17" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10791,10 +10878,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>458</v>
+        <v>468</v>
       </c>
       <c r="E18" t="s">
-        <v>490</v>
+        <v>510</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -10809,19 +10896,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K18" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L18" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M18" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N18" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10835,10 +10922,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="E19" t="s">
-        <v>491</v>
+        <v>511</v>
       </c>
       <c r="F19">
         <v>4</v>
@@ -10853,19 +10940,19 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K19" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L19" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M19" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N19" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -10879,10 +10966,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="E20" t="s">
-        <v>492</v>
+        <v>512</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -10897,19 +10984,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K20" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L20" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M20" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N20" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -10923,10 +11010,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="E21" t="s">
-        <v>493</v>
+        <v>513</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -10941,19 +11028,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K21" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L21" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M21" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N21" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -10967,10 +11054,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>462</v>
+        <v>472</v>
       </c>
       <c r="E22" t="s">
-        <v>494</v>
+        <v>514</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -10982,22 +11069,22 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J22" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K22" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L22" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M22" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N22" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="23" spans="1:14">
@@ -11011,10 +11098,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>463</v>
+        <v>473</v>
       </c>
       <c r="E23" t="s">
-        <v>495</v>
+        <v>515</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11026,22 +11113,22 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J23" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K23" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L23" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M23" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N23" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -11055,7 +11142,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>464</v>
+        <v>474</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11070,22 +11157,22 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J24" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K24" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L24" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M24" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N24" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -11099,10 +11186,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="E25" t="s">
-        <v>496</v>
+        <v>516</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11114,22 +11201,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J25" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K25" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L25" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M25" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N25" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11143,10 +11230,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
       <c r="E26" t="s">
-        <v>497</v>
+        <v>517</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11158,22 +11245,22 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>380</v>
+        <v>542</v>
       </c>
       <c r="J26" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="K26" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="L26" t="s">
-        <v>514</v>
+        <v>543</v>
       </c>
       <c r="M26" s="1">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="N26" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="27" spans="1:14">
@@ -11187,10 +11274,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>467</v>
+        <v>477</v>
       </c>
       <c r="E27" t="s">
-        <v>498</v>
+        <v>518</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11202,22 +11289,22 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="J27" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K27" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L27" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M27" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N27" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11231,10 +11318,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>468</v>
+        <v>478</v>
       </c>
       <c r="E28" t="s">
-        <v>499</v>
+        <v>519</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11249,19 +11336,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K28" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L28" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M28" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N28" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11275,10 +11362,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>469</v>
+        <v>479</v>
       </c>
       <c r="E29" t="s">
-        <v>500</v>
+        <v>520</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11290,22 +11377,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J29" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K29" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L29" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M29" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N29" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11319,10 +11406,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>470</v>
+        <v>480</v>
       </c>
       <c r="E30" t="s">
-        <v>501</v>
+        <v>521</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11337,19 +11424,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K30" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L30" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M30" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N30" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11363,10 +11450,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>471</v>
+        <v>481</v>
       </c>
       <c r="E31" t="s">
-        <v>502</v>
+        <v>522</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11378,22 +11465,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J31" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K31" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L31" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M31" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N31" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11407,10 +11494,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>472</v>
+        <v>482</v>
       </c>
       <c r="E32" t="s">
-        <v>503</v>
+        <v>523</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11422,22 +11509,22 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J32" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K32" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L32" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M32" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N32" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11451,10 +11538,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>473</v>
+        <v>483</v>
       </c>
       <c r="E33" t="s">
-        <v>504</v>
+        <v>524</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11466,22 +11553,22 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J33" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K33" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L33" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M33" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N33" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11495,10 +11582,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="E34" t="s">
-        <v>505</v>
+        <v>525</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11510,22 +11597,22 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J34" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="K34" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="L34" t="s">
-        <v>515</v>
+        <v>544</v>
       </c>
       <c r="M34" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N34" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11539,10 +11626,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>475</v>
+        <v>485</v>
       </c>
       <c r="E35" t="s">
-        <v>506</v>
+        <v>526</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11554,22 +11641,22 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J35" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K35" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L35" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M35" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N35" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11583,10 +11670,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="E36" t="s">
-        <v>507</v>
+        <v>527</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -11598,22 +11685,22 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="J36" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K36" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L36" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M36" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N36" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11627,10 +11714,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="E37" t="s">
-        <v>508</v>
+        <v>528</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -11642,22 +11729,22 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="J37" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K37" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L37" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M37" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N37" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11671,10 +11758,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>478</v>
+        <v>488</v>
       </c>
       <c r="E38" t="s">
-        <v>509</v>
+        <v>529</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -11686,22 +11773,22 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="J38" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K38" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L38" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M38" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N38" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11715,10 +11802,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>479</v>
+        <v>489</v>
       </c>
       <c r="E39" t="s">
-        <v>510</v>
+        <v>530</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -11730,22 +11817,22 @@
         <v>312.36</v>
       </c>
       <c r="I39" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="J39" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K39" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L39" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M39" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N39" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11759,10 +11846,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="E40" t="s">
-        <v>511</v>
+        <v>531</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -11774,22 +11861,22 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="J40" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K40" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L40" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M40" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N40" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11803,10 +11890,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
       <c r="E41" t="s">
-        <v>512</v>
+        <v>532</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -11827,10 +11914,10 @@
         <v>382</v>
       </c>
       <c r="M41" s="1">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="N41" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11859,19 +11946,19 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="K42" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="L42" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="M42" s="1">
-        <v>46309</v>
+        <v>46295</v>
       </c>
       <c r="N42" t="s">
-        <v>518</v>
+        <v>547</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -11885,10 +11972,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="E43" t="s">
-        <v>513</v>
+        <v>533</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -11900,19 +11987,429 @@
         <v>5000</v>
       </c>
       <c r="I43" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="K43" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="L43" t="s">
-        <v>517</v>
+        <v>546</v>
       </c>
       <c r="M43" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="N43" t="s">
-        <v>518</v>
+        <v>547</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
+      <c r="A44" t="s">
+        <v>448</v>
+      </c>
+      <c r="B44" t="s">
+        <v>172</v>
+      </c>
+      <c r="C44" t="s">
+        <v>173</v>
+      </c>
+      <c r="D44" t="s">
+        <v>493</v>
+      </c>
+      <c r="E44" t="s">
+        <v>296</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <v>163.13</v>
+      </c>
+      <c r="H44">
+        <v>163.13</v>
+      </c>
+      <c r="I44" t="s">
+        <v>382</v>
+      </c>
+      <c r="K44" t="s">
+        <v>382</v>
+      </c>
+      <c r="L44" t="s">
+        <v>382</v>
+      </c>
+      <c r="M44" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N44" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
+      <c r="A45" t="s">
+        <v>449</v>
+      </c>
+      <c r="B45" t="s">
+        <v>172</v>
+      </c>
+      <c r="C45" t="s">
+        <v>173</v>
+      </c>
+      <c r="D45" t="s">
+        <v>494</v>
+      </c>
+      <c r="E45" t="s">
+        <v>534</v>
+      </c>
+      <c r="F45">
+        <v>2</v>
+      </c>
+      <c r="G45">
+        <v>188.31</v>
+      </c>
+      <c r="H45">
+        <v>376.62</v>
+      </c>
+      <c r="I45" t="s">
+        <v>382</v>
+      </c>
+      <c r="K45" t="s">
+        <v>382</v>
+      </c>
+      <c r="L45" t="s">
+        <v>382</v>
+      </c>
+      <c r="M45" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N45" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
+      <c r="A46" t="s">
+        <v>450</v>
+      </c>
+      <c r="B46" t="s">
+        <v>172</v>
+      </c>
+      <c r="C46" t="s">
+        <v>173</v>
+      </c>
+      <c r="D46" t="s">
+        <v>495</v>
+      </c>
+      <c r="E46" t="s">
+        <v>535</v>
+      </c>
+      <c r="F46">
+        <v>2</v>
+      </c>
+      <c r="G46">
+        <v>860.76</v>
+      </c>
+      <c r="H46">
+        <v>1721.52</v>
+      </c>
+      <c r="I46" t="s">
+        <v>544</v>
+      </c>
+      <c r="K46" t="s">
+        <v>544</v>
+      </c>
+      <c r="L46" t="s">
+        <v>544</v>
+      </c>
+      <c r="M46" s="1">
+        <v>46295</v>
+      </c>
+      <c r="N46" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
+      <c r="A47" t="s">
+        <v>451</v>
+      </c>
+      <c r="B47" t="s">
+        <v>172</v>
+      </c>
+      <c r="C47" t="s">
+        <v>173</v>
+      </c>
+      <c r="D47" t="s">
+        <v>496</v>
+      </c>
+      <c r="E47" t="s">
+        <v>536</v>
+      </c>
+      <c r="F47">
+        <v>2</v>
+      </c>
+      <c r="G47">
+        <v>1288.97</v>
+      </c>
+      <c r="H47">
+        <v>2577.94</v>
+      </c>
+      <c r="I47" t="s">
+        <v>544</v>
+      </c>
+      <c r="K47" t="s">
+        <v>544</v>
+      </c>
+      <c r="L47" t="s">
+        <v>544</v>
+      </c>
+      <c r="M47" s="1">
+        <v>46295</v>
+      </c>
+      <c r="N47" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
+      <c r="A48" t="s">
+        <v>452</v>
+      </c>
+      <c r="B48" t="s">
+        <v>172</v>
+      </c>
+      <c r="C48" t="s">
+        <v>173</v>
+      </c>
+      <c r="D48" t="s">
+        <v>497</v>
+      </c>
+      <c r="E48" t="s">
+        <v>536</v>
+      </c>
+      <c r="F48">
+        <v>2</v>
+      </c>
+      <c r="G48">
+        <v>1729.85</v>
+      </c>
+      <c r="H48">
+        <v>3459.7</v>
+      </c>
+      <c r="I48" t="s">
+        <v>382</v>
+      </c>
+      <c r="K48" t="s">
+        <v>382</v>
+      </c>
+      <c r="L48" t="s">
+        <v>382</v>
+      </c>
+      <c r="M48" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N48" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14">
+      <c r="A49" t="s">
+        <v>453</v>
+      </c>
+      <c r="B49" t="s">
+        <v>172</v>
+      </c>
+      <c r="C49" t="s">
+        <v>173</v>
+      </c>
+      <c r="D49" t="s">
+        <v>498</v>
+      </c>
+      <c r="E49" t="s">
+        <v>537</v>
+      </c>
+      <c r="F49">
+        <v>9</v>
+      </c>
+      <c r="G49">
+        <v>1528.6</v>
+      </c>
+      <c r="H49">
+        <v>13757.4</v>
+      </c>
+      <c r="I49" t="s">
+        <v>382</v>
+      </c>
+      <c r="K49" t="s">
+        <v>382</v>
+      </c>
+      <c r="L49" t="s">
+        <v>382</v>
+      </c>
+      <c r="M49" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N49" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14">
+      <c r="A50" t="s">
+        <v>454</v>
+      </c>
+      <c r="B50" t="s">
+        <v>172</v>
+      </c>
+      <c r="C50" t="s">
+        <v>173</v>
+      </c>
+      <c r="D50" t="s">
+        <v>499</v>
+      </c>
+      <c r="E50" t="s">
+        <v>538</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50">
+        <v>4208.01</v>
+      </c>
+      <c r="H50">
+        <v>4208.01</v>
+      </c>
+      <c r="I50" t="s">
+        <v>382</v>
+      </c>
+      <c r="K50" t="s">
+        <v>382</v>
+      </c>
+      <c r="L50" t="s">
+        <v>382</v>
+      </c>
+      <c r="M50" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N50" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14">
+      <c r="A51" t="s">
+        <v>455</v>
+      </c>
+      <c r="B51" t="s">
+        <v>172</v>
+      </c>
+      <c r="C51" t="s">
+        <v>173</v>
+      </c>
+      <c r="D51" t="s">
+        <v>500</v>
+      </c>
+      <c r="E51" t="s">
+        <v>539</v>
+      </c>
+      <c r="F51">
+        <v>4</v>
+      </c>
+      <c r="G51">
+        <v>241.09</v>
+      </c>
+      <c r="H51">
+        <v>964.36</v>
+      </c>
+      <c r="I51" t="s">
+        <v>382</v>
+      </c>
+      <c r="K51" t="s">
+        <v>382</v>
+      </c>
+      <c r="L51" t="s">
+        <v>382</v>
+      </c>
+      <c r="M51" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N51" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14">
+      <c r="A52" t="s">
+        <v>456</v>
+      </c>
+      <c r="B52" t="s">
+        <v>172</v>
+      </c>
+      <c r="C52" t="s">
+        <v>173</v>
+      </c>
+      <c r="D52" t="s">
+        <v>501</v>
+      </c>
+      <c r="E52" t="s">
+        <v>540</v>
+      </c>
+      <c r="F52">
+        <v>1</v>
+      </c>
+      <c r="G52">
+        <v>674.64</v>
+      </c>
+      <c r="H52">
+        <v>674.64</v>
+      </c>
+      <c r="I52" t="s">
+        <v>382</v>
+      </c>
+      <c r="K52" t="s">
+        <v>382</v>
+      </c>
+      <c r="L52" t="s">
+        <v>382</v>
+      </c>
+      <c r="M52" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N52" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14">
+      <c r="A53" t="s">
+        <v>457</v>
+      </c>
+      <c r="B53" t="s">
+        <v>172</v>
+      </c>
+      <c r="C53" t="s">
+        <v>173</v>
+      </c>
+      <c r="D53" t="s">
+        <v>502</v>
+      </c>
+      <c r="E53" t="s">
+        <v>541</v>
+      </c>
+      <c r="F53">
+        <v>2</v>
+      </c>
+      <c r="G53">
+        <v>422.53</v>
+      </c>
+      <c r="H53">
+        <v>845.0599999999999</v>
+      </c>
+      <c r="I53" t="s">
+        <v>382</v>
+      </c>
+      <c r="K53" t="s">
+        <v>382</v>
+      </c>
+      <c r="L53" t="s">
+        <v>382</v>
+      </c>
+      <c r="M53" s="1">
+        <v>46300</v>
+      </c>
+      <c r="N53" t="s">
+        <v>547</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (20/07/2026 16:20)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10204,7 +10204,7 @@
         <v>543</v>
       </c>
       <c r="M2" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N2" t="s">
         <v>547</v>
@@ -10248,7 +10248,7 @@
         <v>543</v>
       </c>
       <c r="M3" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N3" t="s">
         <v>547</v>
@@ -10292,7 +10292,7 @@
         <v>543</v>
       </c>
       <c r="M4" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N4" t="s">
         <v>547</v>
@@ -10336,7 +10336,7 @@
         <v>543</v>
       </c>
       <c r="M5" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N5" t="s">
         <v>547</v>
@@ -10380,7 +10380,7 @@
         <v>543</v>
       </c>
       <c r="M6" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N6" t="s">
         <v>547</v>
@@ -10424,7 +10424,7 @@
         <v>543</v>
       </c>
       <c r="M7" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N7" t="s">
         <v>547</v>
@@ -10468,7 +10468,7 @@
         <v>544</v>
       </c>
       <c r="M8" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N8" t="s">
         <v>547</v>
@@ -10512,7 +10512,7 @@
         <v>543</v>
       </c>
       <c r="M9" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N9" t="s">
         <v>547</v>
@@ -10556,7 +10556,7 @@
         <v>544</v>
       </c>
       <c r="M10" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N10" t="s">
         <v>547</v>
@@ -10600,7 +10600,7 @@
         <v>544</v>
       </c>
       <c r="M11" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N11" t="s">
         <v>547</v>
@@ -10685,7 +10685,7 @@
         <v>543</v>
       </c>
       <c r="M13" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N13" t="s">
         <v>547</v>
@@ -10729,7 +10729,7 @@
         <v>543</v>
       </c>
       <c r="M14" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N14" t="s">
         <v>547</v>
@@ -10773,7 +10773,7 @@
         <v>546</v>
       </c>
       <c r="M15" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N15" t="s">
         <v>547</v>
@@ -10817,7 +10817,7 @@
         <v>544</v>
       </c>
       <c r="M16" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N16" t="s">
         <v>547</v>
@@ -10861,7 +10861,7 @@
         <v>546</v>
       </c>
       <c r="M17" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N17" t="s">
         <v>547</v>
@@ -10905,7 +10905,7 @@
         <v>544</v>
       </c>
       <c r="M18" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N18" t="s">
         <v>547</v>
@@ -10949,7 +10949,7 @@
         <v>544</v>
       </c>
       <c r="M19" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N19" t="s">
         <v>547</v>
@@ -10993,7 +10993,7 @@
         <v>544</v>
       </c>
       <c r="M20" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N20" t="s">
         <v>547</v>
@@ -11037,7 +11037,7 @@
         <v>544</v>
       </c>
       <c r="M21" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N21" t="s">
         <v>547</v>
@@ -11081,7 +11081,7 @@
         <v>543</v>
       </c>
       <c r="M22" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N22" t="s">
         <v>547</v>
@@ -11125,7 +11125,7 @@
         <v>543</v>
       </c>
       <c r="M23" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N23" t="s">
         <v>547</v>
@@ -11169,7 +11169,7 @@
         <v>543</v>
       </c>
       <c r="M24" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N24" t="s">
         <v>547</v>
@@ -11213,7 +11213,7 @@
         <v>546</v>
       </c>
       <c r="M25" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N25" t="s">
         <v>547</v>
@@ -11257,7 +11257,7 @@
         <v>543</v>
       </c>
       <c r="M26" s="1">
-        <v>46230</v>
+        <v>46233</v>
       </c>
       <c r="N26" t="s">
         <v>547</v>
@@ -11301,7 +11301,7 @@
         <v>544</v>
       </c>
       <c r="M27" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N27" t="s">
         <v>547</v>
@@ -11345,7 +11345,7 @@
         <v>544</v>
       </c>
       <c r="M28" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N28" t="s">
         <v>547</v>
@@ -11389,7 +11389,7 @@
         <v>544</v>
       </c>
       <c r="M29" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N29" t="s">
         <v>547</v>
@@ -11433,7 +11433,7 @@
         <v>544</v>
       </c>
       <c r="M30" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N30" t="s">
         <v>547</v>
@@ -11477,7 +11477,7 @@
         <v>546</v>
       </c>
       <c r="M31" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N31" t="s">
         <v>547</v>
@@ -11521,7 +11521,7 @@
         <v>546</v>
       </c>
       <c r="M32" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N32" t="s">
         <v>547</v>
@@ -11565,7 +11565,7 @@
         <v>546</v>
       </c>
       <c r="M33" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N33" t="s">
         <v>547</v>
@@ -11609,7 +11609,7 @@
         <v>544</v>
       </c>
       <c r="M34" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N34" t="s">
         <v>547</v>
@@ -11653,7 +11653,7 @@
         <v>546</v>
       </c>
       <c r="M35" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N35" t="s">
         <v>547</v>
@@ -11697,7 +11697,7 @@
         <v>546</v>
       </c>
       <c r="M36" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N36" t="s">
         <v>547</v>
@@ -11741,7 +11741,7 @@
         <v>546</v>
       </c>
       <c r="M37" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N37" t="s">
         <v>547</v>
@@ -11785,7 +11785,7 @@
         <v>546</v>
       </c>
       <c r="M38" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N38" t="s">
         <v>547</v>
@@ -11829,7 +11829,7 @@
         <v>546</v>
       </c>
       <c r="M39" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N39" t="s">
         <v>547</v>
@@ -11873,7 +11873,7 @@
         <v>546</v>
       </c>
       <c r="M40" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N40" t="s">
         <v>547</v>
@@ -11914,7 +11914,7 @@
         <v>382</v>
       </c>
       <c r="M41" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N41" t="s">
         <v>547</v>
@@ -11955,7 +11955,7 @@
         <v>544</v>
       </c>
       <c r="M42" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N42" t="s">
         <v>547</v>
@@ -11996,7 +11996,7 @@
         <v>546</v>
       </c>
       <c r="M43" s="1">
-        <v>46310</v>
+        <v>46313</v>
       </c>
       <c r="N43" t="s">
         <v>547</v>
@@ -12037,7 +12037,7 @@
         <v>382</v>
       </c>
       <c r="M44" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N44" t="s">
         <v>547</v>
@@ -12078,7 +12078,7 @@
         <v>382</v>
       </c>
       <c r="M45" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N45" t="s">
         <v>547</v>
@@ -12119,7 +12119,7 @@
         <v>544</v>
       </c>
       <c r="M46" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N46" t="s">
         <v>547</v>
@@ -12160,7 +12160,7 @@
         <v>544</v>
       </c>
       <c r="M47" s="1">
-        <v>46295</v>
+        <v>46298</v>
       </c>
       <c r="N47" t="s">
         <v>547</v>
@@ -12201,7 +12201,7 @@
         <v>382</v>
       </c>
       <c r="M48" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N48" t="s">
         <v>547</v>
@@ -12242,7 +12242,7 @@
         <v>382</v>
       </c>
       <c r="M49" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N49" t="s">
         <v>547</v>
@@ -12283,7 +12283,7 @@
         <v>382</v>
       </c>
       <c r="M50" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N50" t="s">
         <v>547</v>
@@ -12324,7 +12324,7 @@
         <v>382</v>
       </c>
       <c r="M51" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N51" t="s">
         <v>547</v>
@@ -12365,7 +12365,7 @@
         <v>382</v>
       </c>
       <c r="M52" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N52" t="s">
         <v>547</v>
@@ -12406,7 +12406,7 @@
         <v>382</v>
       </c>
       <c r="M53" s="1">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="N53" t="s">
         <v>547</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/07/2026 16:09)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2403" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2412" uniqueCount="551">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1391,6 +1391,9 @@
     <t>LST197006U8</t>
   </si>
   <si>
+    <t>LST202001U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1526,6 +1529,9 @@
     <t>2615011-2</t>
   </si>
   <si>
+    <t>2611137-7</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1643,19 +1649,22 @@
     <t>WINDOW MOLDING</t>
   </si>
   <si>
+    <t>CAP MAIN LAND</t>
+  </si>
+  <si>
     <t>Empenho Solicitado</t>
   </si>
   <si>
     <t>Mapa Gerado</t>
   </si>
   <si>
+    <t>Selecionada em Plano</t>
+  </si>
+  <si>
+    <t>Análise do Pedido</t>
+  </si>
+  <si>
     <t>Validada</t>
-  </si>
-  <si>
-    <t>Aguardando Conferência do ACI</t>
-  </si>
-  <si>
-    <t>Análise do Pedido</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10110,7 +10119,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10192,22 +10201,22 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J2" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K2" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L2" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M2" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N2" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -10236,22 +10245,22 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J3" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K3" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L3" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M3" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N3" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -10265,7 +10274,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10280,22 +10289,22 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J4" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K4" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L4" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M4" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N4" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -10309,10 +10318,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E5" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10324,22 +10333,22 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="J5" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K5" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L5" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M5" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N5" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -10368,22 +10377,22 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J6" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K6" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L6" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M6" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N6" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -10412,22 +10421,22 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J7" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K7" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L7" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M7" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N7" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -10456,22 +10465,22 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J8" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K8" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L8" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M8" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N8" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10485,7 +10494,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10500,22 +10509,22 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J9" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K9" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L9" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M9" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N9" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -10529,10 +10538,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E10" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10547,19 +10556,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K10" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L10" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M10" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N10" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10573,7 +10582,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10591,19 +10600,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K11" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L11" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M11" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N11" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10617,10 +10626,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E12" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -10673,22 +10682,22 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>545</v>
+        <v>380</v>
       </c>
       <c r="J13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M13" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N13" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -10702,10 +10711,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E14" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -10717,22 +10726,22 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J14" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K14" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L14" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M14" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N14" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -10746,10 +10755,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E15" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -10761,22 +10770,22 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J15" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K15" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L15" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M15" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N15" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10790,10 +10799,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E16" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -10808,19 +10817,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K16" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L16" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M16" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N16" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10834,10 +10843,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E17" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -10849,22 +10858,22 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J17" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K17" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L17" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M17" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N17" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10878,10 +10887,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E18" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -10896,19 +10905,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K18" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L18" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M18" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N18" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10922,10 +10931,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E19" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="F19">
         <v>4</v>
@@ -10940,19 +10949,19 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K19" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L19" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M19" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N19" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -10966,10 +10975,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E20" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -10984,19 +10993,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K20" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L20" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M20" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N20" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11010,10 +11019,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E21" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11028,19 +11037,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K21" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L21" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M21" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N21" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11054,10 +11063,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E22" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11069,22 +11078,22 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J22" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K22" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L22" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M22" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N22" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="23" spans="1:14">
@@ -11098,10 +11107,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E23" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11113,22 +11122,22 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J23" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K23" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L23" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M23" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N23" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -11142,7 +11151,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11157,22 +11166,22 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J24" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K24" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L24" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M24" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N24" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -11186,10 +11195,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E25" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11201,22 +11210,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M25" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N25" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11230,10 +11239,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E26" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11245,22 +11254,22 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J26" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K26" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="L26" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="M26" s="1">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="N26" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="27" spans="1:14">
@@ -11274,10 +11283,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E27" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11289,22 +11298,22 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J27" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K27" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L27" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M27" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N27" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11318,10 +11327,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E28" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11336,19 +11345,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K28" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L28" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M28" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N28" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11362,10 +11371,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E29" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11377,22 +11386,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J29" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K29" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L29" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M29" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N29" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11406,10 +11415,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E30" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11424,19 +11433,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K30" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L30" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M30" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N30" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11450,10 +11459,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E31" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11465,22 +11474,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J31" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K31" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L31" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M31" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N31" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11494,10 +11503,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E32" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11509,22 +11518,22 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J32" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K32" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L32" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M32" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N32" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11538,10 +11547,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E33" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11553,22 +11562,22 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J33" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K33" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L33" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M33" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N33" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11582,10 +11591,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E34" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11597,22 +11606,22 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J34" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="K34" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="L34" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="M34" s="1">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N34" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11626,10 +11635,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E35" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11641,22 +11650,22 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J35" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K35" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L35" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M35" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N35" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11670,10 +11679,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E36" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -11685,22 +11694,22 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J36" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K36" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L36" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M36" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N36" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11714,10 +11723,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E37" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -11729,22 +11738,22 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J37" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K37" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L37" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M37" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N37" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11758,10 +11767,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E38" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -11773,22 +11782,22 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J38" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K38" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L38" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M38" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N38" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11802,10 +11811,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E39" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -11817,22 +11826,22 @@
         <v>312.36</v>
       </c>
       <c r="I39" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="J39" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K39" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L39" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M39" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N39" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11846,10 +11855,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E40" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -11861,22 +11870,22 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J40" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K40" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L40" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M40" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N40" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11890,10 +11899,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E41" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -11914,10 +11923,10 @@
         <v>382</v>
       </c>
       <c r="M41" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N41" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11946,19 +11955,19 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="K42" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="L42" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="M42" s="1">
-        <v>46298</v>
+        <v>46289</v>
       </c>
       <c r="N42" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -11972,10 +11981,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E43" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -11987,19 +11996,19 @@
         <v>5000</v>
       </c>
       <c r="I43" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K43" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L43" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="M43" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N43" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12013,7 +12022,7 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
@@ -12037,10 +12046,10 @@
         <v>382</v>
       </c>
       <c r="M44" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N44" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12054,10 +12063,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E45" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12078,10 +12087,10 @@
         <v>382</v>
       </c>
       <c r="M45" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N45" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12095,10 +12104,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E46" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12110,19 +12119,19 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="K46" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="L46" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="M46" s="1">
-        <v>46298</v>
+        <v>46289</v>
       </c>
       <c r="N46" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12136,10 +12145,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E47" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12151,19 +12160,19 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="K47" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="L47" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="M47" s="1">
-        <v>46298</v>
+        <v>46289</v>
       </c>
       <c r="N47" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12177,34 +12186,34 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E48" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="F48">
         <v>2</v>
       </c>
       <c r="G48">
-        <v>1729.85</v>
+        <v>1729.86</v>
       </c>
       <c r="H48">
-        <v>3459.7</v>
+        <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>382</v>
+        <v>548</v>
       </c>
       <c r="K48" t="s">
-        <v>382</v>
+        <v>548</v>
       </c>
       <c r="L48" t="s">
-        <v>382</v>
+        <v>548</v>
       </c>
       <c r="M48" s="1">
-        <v>46303</v>
+        <v>46314</v>
       </c>
       <c r="N48" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12218,10 +12227,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E49" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12233,19 +12242,19 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>382</v>
+        <v>548</v>
       </c>
       <c r="K49" t="s">
-        <v>382</v>
+        <v>548</v>
       </c>
       <c r="L49" t="s">
-        <v>382</v>
+        <v>548</v>
       </c>
       <c r="M49" s="1">
-        <v>46303</v>
+        <v>46314</v>
       </c>
       <c r="N49" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12259,10 +12268,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E50" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12283,10 +12292,10 @@
         <v>382</v>
       </c>
       <c r="M50" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N50" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12300,10 +12309,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E51" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12324,10 +12333,10 @@
         <v>382</v>
       </c>
       <c r="M51" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N51" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12341,10 +12350,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E52" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12365,10 +12374,10 @@
         <v>382</v>
       </c>
       <c r="M52" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N52" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12382,10 +12391,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E53" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12406,10 +12415,51 @@
         <v>382</v>
       </c>
       <c r="M53" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N53" t="s">
-        <v>547</v>
+        <v>550</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
+      <c r="A54" t="s">
+        <v>458</v>
+      </c>
+      <c r="B54" t="s">
+        <v>172</v>
+      </c>
+      <c r="C54" t="s">
+        <v>173</v>
+      </c>
+      <c r="D54" t="s">
+        <v>504</v>
+      </c>
+      <c r="E54" t="s">
+        <v>544</v>
+      </c>
+      <c r="F54">
+        <v>4</v>
+      </c>
+      <c r="G54">
+        <v>968.8099999999999</v>
+      </c>
+      <c r="H54">
+        <v>3875.24</v>
+      </c>
+      <c r="I54" t="s">
+        <v>548</v>
+      </c>
+      <c r="K54" t="s">
+        <v>548</v>
+      </c>
+      <c r="L54" t="s">
+        <v>548</v>
+      </c>
+      <c r="M54" s="1">
+        <v>46314</v>
+      </c>
+      <c r="N54" t="s">
+        <v>550</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/07/2026 20:53)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2412" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="553">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1665,6 +1665,12 @@
   </si>
   <si>
     <t>Validada</t>
+  </si>
+  <si>
+    <t>EMPENHADO</t>
+  </si>
+  <si>
+    <t>IMEDIATO</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10204,19 +10210,19 @@
         <v>545</v>
       </c>
       <c r="J2" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K2" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L2" t="s">
-        <v>546</v>
-      </c>
-      <c r="M2" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M2" t="s">
+        <v>550</v>
       </c>
       <c r="N2" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -10248,19 +10254,19 @@
         <v>545</v>
       </c>
       <c r="J3" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K3" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L3" t="s">
-        <v>546</v>
-      </c>
-      <c r="M3" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M3" t="s">
+        <v>550</v>
       </c>
       <c r="N3" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -10292,19 +10298,19 @@
         <v>545</v>
       </c>
       <c r="J4" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K4" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L4" t="s">
-        <v>546</v>
-      </c>
-      <c r="M4" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M4" t="s">
+        <v>550</v>
       </c>
       <c r="N4" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -10348,7 +10354,7 @@
         <v>46234</v>
       </c>
       <c r="N5" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -10380,19 +10386,19 @@
         <v>545</v>
       </c>
       <c r="J6" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K6" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L6" t="s">
-        <v>546</v>
-      </c>
-      <c r="M6" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M6" t="s">
+        <v>550</v>
       </c>
       <c r="N6" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -10424,19 +10430,19 @@
         <v>545</v>
       </c>
       <c r="J7" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K7" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L7" t="s">
-        <v>546</v>
-      </c>
-      <c r="M7" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M7" t="s">
+        <v>550</v>
       </c>
       <c r="N7" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -10480,7 +10486,7 @@
         <v>46299</v>
       </c>
       <c r="N8" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10512,19 +10518,19 @@
         <v>545</v>
       </c>
       <c r="J9" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K9" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L9" t="s">
-        <v>546</v>
-      </c>
-      <c r="M9" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M9" t="s">
+        <v>550</v>
       </c>
       <c r="N9" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -10568,7 +10574,7 @@
         <v>46299</v>
       </c>
       <c r="N10" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10612,7 +10618,7 @@
         <v>46299</v>
       </c>
       <c r="N11" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10685,19 +10691,19 @@
         <v>380</v>
       </c>
       <c r="J13" t="s">
-        <v>546</v>
+        <v>380</v>
       </c>
       <c r="K13" t="s">
-        <v>546</v>
+        <v>380</v>
       </c>
       <c r="L13" t="s">
-        <v>546</v>
-      </c>
-      <c r="M13" s="1">
-        <v>46234</v>
+        <v>380</v>
+      </c>
+      <c r="M13" t="s">
+        <v>551</v>
       </c>
       <c r="N13" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -10729,19 +10735,19 @@
         <v>545</v>
       </c>
       <c r="J14" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K14" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L14" t="s">
-        <v>546</v>
-      </c>
-      <c r="M14" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M14" t="s">
+        <v>550</v>
       </c>
       <c r="N14" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -10785,7 +10791,7 @@
         <v>46314</v>
       </c>
       <c r="N15" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10829,7 +10835,7 @@
         <v>46299</v>
       </c>
       <c r="N16" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10873,7 +10879,7 @@
         <v>46314</v>
       </c>
       <c r="N17" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10917,7 +10923,7 @@
         <v>46299</v>
       </c>
       <c r="N18" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10961,7 +10967,7 @@
         <v>46299</v>
       </c>
       <c r="N19" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11005,7 +11011,7 @@
         <v>46299</v>
       </c>
       <c r="N20" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11049,7 +11055,7 @@
         <v>46299</v>
       </c>
       <c r="N21" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11081,19 +11087,19 @@
         <v>545</v>
       </c>
       <c r="J22" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K22" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L22" t="s">
-        <v>546</v>
-      </c>
-      <c r="M22" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M22" t="s">
+        <v>550</v>
       </c>
       <c r="N22" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="23" spans="1:14">
@@ -11125,19 +11131,19 @@
         <v>545</v>
       </c>
       <c r="J23" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K23" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L23" t="s">
-        <v>546</v>
-      </c>
-      <c r="M23" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M23" t="s">
+        <v>550</v>
       </c>
       <c r="N23" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -11169,19 +11175,19 @@
         <v>545</v>
       </c>
       <c r="J24" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K24" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L24" t="s">
-        <v>546</v>
-      </c>
-      <c r="M24" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M24" t="s">
+        <v>550</v>
       </c>
       <c r="N24" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -11225,7 +11231,7 @@
         <v>46314</v>
       </c>
       <c r="N25" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11257,19 +11263,19 @@
         <v>545</v>
       </c>
       <c r="J26" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="K26" t="s">
-        <v>546</v>
+        <v>387</v>
       </c>
       <c r="L26" t="s">
-        <v>546</v>
-      </c>
-      <c r="M26" s="1">
-        <v>46234</v>
+        <v>387</v>
+      </c>
+      <c r="M26" t="s">
+        <v>550</v>
       </c>
       <c r="N26" t="s">
-        <v>550</v>
+        <v>395</v>
       </c>
     </row>
     <row r="27" spans="1:14">
@@ -11313,7 +11319,7 @@
         <v>46299</v>
       </c>
       <c r="N27" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11357,7 +11363,7 @@
         <v>46299</v>
       </c>
       <c r="N28" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11401,7 +11407,7 @@
         <v>46299</v>
       </c>
       <c r="N29" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11445,7 +11451,7 @@
         <v>46299</v>
       </c>
       <c r="N30" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11489,7 +11495,7 @@
         <v>46314</v>
       </c>
       <c r="N31" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11533,7 +11539,7 @@
         <v>46314</v>
       </c>
       <c r="N32" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11577,7 +11583,7 @@
         <v>46314</v>
       </c>
       <c r="N33" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11621,7 +11627,7 @@
         <v>46299</v>
       </c>
       <c r="N34" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11665,7 +11671,7 @@
         <v>46314</v>
       </c>
       <c r="N35" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11697,19 +11703,19 @@
         <v>547</v>
       </c>
       <c r="J36" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K36" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L36" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="M36" s="1">
-        <v>46314</v>
+        <v>46299</v>
       </c>
       <c r="N36" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11741,19 +11747,19 @@
         <v>547</v>
       </c>
       <c r="J37" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K37" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L37" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="M37" s="1">
-        <v>46314</v>
+        <v>46299</v>
       </c>
       <c r="N37" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11785,19 +11791,19 @@
         <v>547</v>
       </c>
       <c r="J38" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K38" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L38" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="M38" s="1">
-        <v>46314</v>
+        <v>46299</v>
       </c>
       <c r="N38" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11841,7 +11847,7 @@
         <v>46314</v>
       </c>
       <c r="N39" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11873,19 +11879,19 @@
         <v>547</v>
       </c>
       <c r="J40" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="K40" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L40" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="M40" s="1">
-        <v>46314</v>
+        <v>46299</v>
       </c>
       <c r="N40" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11916,17 +11922,20 @@
       <c r="I41" t="s">
         <v>382</v>
       </c>
+      <c r="J41" t="s">
+        <v>549</v>
+      </c>
       <c r="K41" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="L41" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="M41" s="1">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="N41" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11957,17 +11966,20 @@
       <c r="I42" t="s">
         <v>547</v>
       </c>
+      <c r="J42" t="s">
+        <v>549</v>
+      </c>
       <c r="K42" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="L42" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="M42" s="1">
-        <v>46289</v>
+        <v>46299</v>
       </c>
       <c r="N42" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -11998,17 +12010,20 @@
       <c r="I43" t="s">
         <v>548</v>
       </c>
+      <c r="J43" t="s">
+        <v>549</v>
+      </c>
       <c r="K43" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L43" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="M43" s="1">
-        <v>46314</v>
+        <v>46299</v>
       </c>
       <c r="N43" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12039,17 +12054,20 @@
       <c r="I44" t="s">
         <v>382</v>
       </c>
+      <c r="J44" t="s">
+        <v>549</v>
+      </c>
       <c r="K44" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="L44" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="M44" s="1">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="N44" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12080,17 +12098,20 @@
       <c r="I45" t="s">
         <v>382</v>
       </c>
+      <c r="J45" t="s">
+        <v>549</v>
+      </c>
       <c r="K45" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="L45" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="M45" s="1">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="N45" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12121,17 +12142,20 @@
       <c r="I46" t="s">
         <v>547</v>
       </c>
+      <c r="J46" t="s">
+        <v>549</v>
+      </c>
       <c r="K46" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="L46" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="M46" s="1">
-        <v>46289</v>
+        <v>46299</v>
       </c>
       <c r="N46" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12162,17 +12186,20 @@
       <c r="I47" t="s">
         <v>547</v>
       </c>
+      <c r="J47" t="s">
+        <v>549</v>
+      </c>
       <c r="K47" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="L47" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="M47" s="1">
-        <v>46289</v>
+        <v>46299</v>
       </c>
       <c r="N47" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12203,6 +12230,9 @@
       <c r="I48" t="s">
         <v>548</v>
       </c>
+      <c r="J48" t="s">
+        <v>548</v>
+      </c>
       <c r="K48" t="s">
         <v>548</v>
       </c>
@@ -12213,7 +12243,7 @@
         <v>46314</v>
       </c>
       <c r="N48" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12244,6 +12274,9 @@
       <c r="I49" t="s">
         <v>548</v>
       </c>
+      <c r="J49" t="s">
+        <v>548</v>
+      </c>
       <c r="K49" t="s">
         <v>548</v>
       </c>
@@ -12254,7 +12287,7 @@
         <v>46314</v>
       </c>
       <c r="N49" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12285,17 +12318,20 @@
       <c r="I50" t="s">
         <v>382</v>
       </c>
+      <c r="J50" t="s">
+        <v>549</v>
+      </c>
       <c r="K50" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="L50" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="M50" s="1">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="N50" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12326,17 +12362,20 @@
       <c r="I51" t="s">
         <v>382</v>
       </c>
+      <c r="J51" t="s">
+        <v>549</v>
+      </c>
       <c r="K51" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="L51" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="M51" s="1">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="N51" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12367,17 +12406,20 @@
       <c r="I52" t="s">
         <v>382</v>
       </c>
+      <c r="J52" t="s">
+        <v>549</v>
+      </c>
       <c r="K52" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="L52" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="M52" s="1">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="N52" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12408,17 +12450,20 @@
       <c r="I53" t="s">
         <v>382</v>
       </c>
+      <c r="J53" t="s">
+        <v>549</v>
+      </c>
       <c r="K53" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="L53" t="s">
-        <v>382</v>
+        <v>549</v>
       </c>
       <c r="M53" s="1">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="N53" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12449,6 +12494,9 @@
       <c r="I54" t="s">
         <v>548</v>
       </c>
+      <c r="J54" t="s">
+        <v>548</v>
+      </c>
       <c r="K54" t="s">
         <v>548</v>
       </c>
@@ -12459,7 +12507,7 @@
         <v>46314</v>
       </c>
       <c r="N54" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (22/07/2026 12:03)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1683,8 +1683,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1700,7 +1708,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1708,12 +1716,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2013,55 +2039,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2105,7 +2131,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2149,7 +2175,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2193,7 +2219,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2319,7 +2345,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2363,7 +2389,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2407,7 +2433,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2454,7 +2480,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2577,7 +2603,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2621,7 +2647,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2665,7 +2691,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2756,7 +2782,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2800,7 +2826,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2926,7 +2952,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2970,7 +2996,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3055,7 +3081,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3102,7 +3128,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3149,7 +3175,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3193,7 +3219,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3237,7 +3263,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3322,7 +3348,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3407,7 +3433,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3454,7 +3480,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3498,7 +3524,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3542,7 +3568,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3627,7 +3653,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3671,7 +3697,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3715,7 +3741,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3800,7 +3826,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3844,7 +3870,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3888,7 +3914,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4099,7 +4125,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4143,7 +4169,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4187,7 +4213,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4278,7 +4304,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4322,7 +4348,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4404,7 +4430,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4448,7 +4474,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4627,7 +4653,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4671,7 +4697,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4715,7 +4741,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4759,7 +4785,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4850,7 +4876,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4894,7 +4920,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -4941,7 +4967,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -4985,7 +5011,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5032,7 +5058,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5120,7 +5146,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5164,7 +5190,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5208,7 +5234,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5252,7 +5278,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5425,7 +5451,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5469,7 +5495,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5513,7 +5539,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5780,7 +5806,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5824,7 +5850,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5868,7 +5894,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5912,7 +5938,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6390,7 +6416,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6434,7 +6460,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6478,7 +6504,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6604,7 +6630,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6648,7 +6674,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6695,7 +6721,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6739,7 +6765,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6865,7 +6891,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6909,7 +6935,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -6994,7 +7020,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7038,7 +7064,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7082,7 +7108,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7387,7 +7413,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7554,7 +7580,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7598,7 +7624,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7642,7 +7668,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7903,7 +7929,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7947,7 +7973,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8032,7 +8058,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8158,7 +8184,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8202,7 +8228,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8287,7 +8313,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8331,7 +8357,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8375,7 +8401,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8680,7 +8706,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8847,7 +8873,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8891,7 +8917,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8935,7 +8961,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9064,7 +9090,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9108,7 +9134,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9152,7 +9178,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10029,7 +10055,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10114,7 +10140,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10129,55 +10155,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10350,8 +10376,8 @@
       <c r="L5" t="s">
         <v>546</v>
       </c>
-      <c r="M5" s="1">
-        <v>46234</v>
+      <c r="M5" s="2">
+        <v>46235</v>
       </c>
       <c r="N5" t="s">
         <v>552</v>
@@ -10482,8 +10508,8 @@
       <c r="L8" t="s">
         <v>549</v>
       </c>
-      <c r="M8" s="1">
-        <v>46299</v>
+      <c r="M8" s="2">
+        <v>46300</v>
       </c>
       <c r="N8" t="s">
         <v>552</v>
@@ -10570,8 +10596,8 @@
       <c r="L10" t="s">
         <v>549</v>
       </c>
-      <c r="M10" s="1">
-        <v>46299</v>
+      <c r="M10" s="2">
+        <v>46300</v>
       </c>
       <c r="N10" t="s">
         <v>552</v>
@@ -10614,8 +10640,8 @@
       <c r="L11" t="s">
         <v>549</v>
       </c>
-      <c r="M11" s="1">
-        <v>46299</v>
+      <c r="M11" s="2">
+        <v>46300</v>
       </c>
       <c r="N11" t="s">
         <v>552</v>
@@ -10787,8 +10813,8 @@
       <c r="L15" t="s">
         <v>548</v>
       </c>
-      <c r="M15" s="1">
-        <v>46314</v>
+      <c r="M15" s="2">
+        <v>46315</v>
       </c>
       <c r="N15" t="s">
         <v>552</v>
@@ -10831,8 +10857,8 @@
       <c r="L16" t="s">
         <v>549</v>
       </c>
-      <c r="M16" s="1">
-        <v>46299</v>
+      <c r="M16" s="2">
+        <v>46300</v>
       </c>
       <c r="N16" t="s">
         <v>552</v>
@@ -10875,8 +10901,8 @@
       <c r="L17" t="s">
         <v>548</v>
       </c>
-      <c r="M17" s="1">
-        <v>46314</v>
+      <c r="M17" s="2">
+        <v>46315</v>
       </c>
       <c r="N17" t="s">
         <v>552</v>
@@ -10919,8 +10945,8 @@
       <c r="L18" t="s">
         <v>549</v>
       </c>
-      <c r="M18" s="1">
-        <v>46299</v>
+      <c r="M18" s="2">
+        <v>46300</v>
       </c>
       <c r="N18" t="s">
         <v>552</v>
@@ -10963,8 +10989,8 @@
       <c r="L19" t="s">
         <v>549</v>
       </c>
-      <c r="M19" s="1">
-        <v>46299</v>
+      <c r="M19" s="2">
+        <v>46300</v>
       </c>
       <c r="N19" t="s">
         <v>552</v>
@@ -11007,8 +11033,8 @@
       <c r="L20" t="s">
         <v>549</v>
       </c>
-      <c r="M20" s="1">
-        <v>46299</v>
+      <c r="M20" s="2">
+        <v>46300</v>
       </c>
       <c r="N20" t="s">
         <v>552</v>
@@ -11051,8 +11077,8 @@
       <c r="L21" t="s">
         <v>549</v>
       </c>
-      <c r="M21" s="1">
-        <v>46299</v>
+      <c r="M21" s="2">
+        <v>46300</v>
       </c>
       <c r="N21" t="s">
         <v>552</v>
@@ -11227,8 +11253,8 @@
       <c r="L25" t="s">
         <v>548</v>
       </c>
-      <c r="M25" s="1">
-        <v>46314</v>
+      <c r="M25" s="2">
+        <v>46315</v>
       </c>
       <c r="N25" t="s">
         <v>552</v>
@@ -11315,8 +11341,8 @@
       <c r="L27" t="s">
         <v>549</v>
       </c>
-      <c r="M27" s="1">
-        <v>46299</v>
+      <c r="M27" s="2">
+        <v>46300</v>
       </c>
       <c r="N27" t="s">
         <v>552</v>
@@ -11359,8 +11385,8 @@
       <c r="L28" t="s">
         <v>549</v>
       </c>
-      <c r="M28" s="1">
-        <v>46299</v>
+      <c r="M28" s="2">
+        <v>46300</v>
       </c>
       <c r="N28" t="s">
         <v>552</v>
@@ -11403,8 +11429,8 @@
       <c r="L29" t="s">
         <v>549</v>
       </c>
-      <c r="M29" s="1">
-        <v>46299</v>
+      <c r="M29" s="2">
+        <v>46300</v>
       </c>
       <c r="N29" t="s">
         <v>552</v>
@@ -11447,8 +11473,8 @@
       <c r="L30" t="s">
         <v>549</v>
       </c>
-      <c r="M30" s="1">
-        <v>46299</v>
+      <c r="M30" s="2">
+        <v>46300</v>
       </c>
       <c r="N30" t="s">
         <v>552</v>
@@ -11491,8 +11517,8 @@
       <c r="L31" t="s">
         <v>548</v>
       </c>
-      <c r="M31" s="1">
-        <v>46314</v>
+      <c r="M31" s="2">
+        <v>46315</v>
       </c>
       <c r="N31" t="s">
         <v>552</v>
@@ -11535,8 +11561,8 @@
       <c r="L32" t="s">
         <v>548</v>
       </c>
-      <c r="M32" s="1">
-        <v>46314</v>
+      <c r="M32" s="2">
+        <v>46315</v>
       </c>
       <c r="N32" t="s">
         <v>552</v>
@@ -11579,8 +11605,8 @@
       <c r="L33" t="s">
         <v>548</v>
       </c>
-      <c r="M33" s="1">
-        <v>46314</v>
+      <c r="M33" s="2">
+        <v>46315</v>
       </c>
       <c r="N33" t="s">
         <v>552</v>
@@ -11623,8 +11649,8 @@
       <c r="L34" t="s">
         <v>549</v>
       </c>
-      <c r="M34" s="1">
-        <v>46299</v>
+      <c r="M34" s="2">
+        <v>46300</v>
       </c>
       <c r="N34" t="s">
         <v>552</v>
@@ -11667,8 +11693,8 @@
       <c r="L35" t="s">
         <v>548</v>
       </c>
-      <c r="M35" s="1">
-        <v>46314</v>
+      <c r="M35" s="2">
+        <v>46315</v>
       </c>
       <c r="N35" t="s">
         <v>552</v>
@@ -11711,8 +11737,8 @@
       <c r="L36" t="s">
         <v>549</v>
       </c>
-      <c r="M36" s="1">
-        <v>46299</v>
+      <c r="M36" s="2">
+        <v>46300</v>
       </c>
       <c r="N36" t="s">
         <v>552</v>
@@ -11755,8 +11781,8 @@
       <c r="L37" t="s">
         <v>549</v>
       </c>
-      <c r="M37" s="1">
-        <v>46299</v>
+      <c r="M37" s="2">
+        <v>46300</v>
       </c>
       <c r="N37" t="s">
         <v>552</v>
@@ -11799,8 +11825,8 @@
       <c r="L38" t="s">
         <v>549</v>
       </c>
-      <c r="M38" s="1">
-        <v>46299</v>
+      <c r="M38" s="2">
+        <v>46300</v>
       </c>
       <c r="N38" t="s">
         <v>552</v>
@@ -11843,8 +11869,8 @@
       <c r="L39" t="s">
         <v>548</v>
       </c>
-      <c r="M39" s="1">
-        <v>46314</v>
+      <c r="M39" s="2">
+        <v>46315</v>
       </c>
       <c r="N39" t="s">
         <v>552</v>
@@ -11887,8 +11913,8 @@
       <c r="L40" t="s">
         <v>549</v>
       </c>
-      <c r="M40" s="1">
-        <v>46299</v>
+      <c r="M40" s="2">
+        <v>46300</v>
       </c>
       <c r="N40" t="s">
         <v>552</v>
@@ -11931,8 +11957,8 @@
       <c r="L41" t="s">
         <v>549</v>
       </c>
-      <c r="M41" s="1">
-        <v>46299</v>
+      <c r="M41" s="2">
+        <v>46300</v>
       </c>
       <c r="N41" t="s">
         <v>552</v>
@@ -11975,8 +12001,8 @@
       <c r="L42" t="s">
         <v>549</v>
       </c>
-      <c r="M42" s="1">
-        <v>46299</v>
+      <c r="M42" s="2">
+        <v>46300</v>
       </c>
       <c r="N42" t="s">
         <v>552</v>
@@ -12019,8 +12045,8 @@
       <c r="L43" t="s">
         <v>549</v>
       </c>
-      <c r="M43" s="1">
-        <v>46299</v>
+      <c r="M43" s="2">
+        <v>46300</v>
       </c>
       <c r="N43" t="s">
         <v>552</v>
@@ -12063,8 +12089,8 @@
       <c r="L44" t="s">
         <v>549</v>
       </c>
-      <c r="M44" s="1">
-        <v>46299</v>
+      <c r="M44" s="2">
+        <v>46300</v>
       </c>
       <c r="N44" t="s">
         <v>552</v>
@@ -12107,8 +12133,8 @@
       <c r="L45" t="s">
         <v>549</v>
       </c>
-      <c r="M45" s="1">
-        <v>46299</v>
+      <c r="M45" s="2">
+        <v>46300</v>
       </c>
       <c r="N45" t="s">
         <v>552</v>
@@ -12151,8 +12177,8 @@
       <c r="L46" t="s">
         <v>549</v>
       </c>
-      <c r="M46" s="1">
-        <v>46299</v>
+      <c r="M46" s="2">
+        <v>46300</v>
       </c>
       <c r="N46" t="s">
         <v>552</v>
@@ -12195,8 +12221,8 @@
       <c r="L47" t="s">
         <v>549</v>
       </c>
-      <c r="M47" s="1">
-        <v>46299</v>
+      <c r="M47" s="2">
+        <v>46300</v>
       </c>
       <c r="N47" t="s">
         <v>552</v>
@@ -12239,8 +12265,8 @@
       <c r="L48" t="s">
         <v>548</v>
       </c>
-      <c r="M48" s="1">
-        <v>46314</v>
+      <c r="M48" s="2">
+        <v>46315</v>
       </c>
       <c r="N48" t="s">
         <v>552</v>
@@ -12283,8 +12309,8 @@
       <c r="L49" t="s">
         <v>548</v>
       </c>
-      <c r="M49" s="1">
-        <v>46314</v>
+      <c r="M49" s="2">
+        <v>46315</v>
       </c>
       <c r="N49" t="s">
         <v>552</v>
@@ -12327,8 +12353,8 @@
       <c r="L50" t="s">
         <v>549</v>
       </c>
-      <c r="M50" s="1">
-        <v>46299</v>
+      <c r="M50" s="2">
+        <v>46300</v>
       </c>
       <c r="N50" t="s">
         <v>552</v>
@@ -12371,8 +12397,8 @@
       <c r="L51" t="s">
         <v>549</v>
       </c>
-      <c r="M51" s="1">
-        <v>46299</v>
+      <c r="M51" s="2">
+        <v>46300</v>
       </c>
       <c r="N51" t="s">
         <v>552</v>
@@ -12415,8 +12441,8 @@
       <c r="L52" t="s">
         <v>549</v>
       </c>
-      <c r="M52" s="1">
-        <v>46299</v>
+      <c r="M52" s="2">
+        <v>46300</v>
       </c>
       <c r="N52" t="s">
         <v>552</v>
@@ -12459,8 +12485,8 @@
       <c r="L53" t="s">
         <v>549</v>
       </c>
-      <c r="M53" s="1">
-        <v>46299</v>
+      <c r="M53" s="2">
+        <v>46300</v>
       </c>
       <c r="N53" t="s">
         <v>552</v>
@@ -12503,8 +12529,8 @@
       <c r="L54" t="s">
         <v>548</v>
       </c>
-      <c r="M54" s="1">
-        <v>46314</v>
+      <c r="M54" s="2">
+        <v>46315</v>
       </c>
       <c r="N54" t="s">
         <v>552</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (22/07/2026 16:10)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1683,16 +1683,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1708,7 +1700,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1716,30 +1708,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2039,55 +2013,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2131,7 +2105,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2175,7 +2149,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2219,7 +2193,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2345,7 +2319,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2389,7 +2363,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2433,7 +2407,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2480,7 +2454,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2603,7 +2577,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2647,7 +2621,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2691,7 +2665,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2782,7 +2756,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2826,7 +2800,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2952,7 +2926,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2996,7 +2970,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3081,7 +3055,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3128,7 +3102,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3175,7 +3149,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3219,7 +3193,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3263,7 +3237,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3348,7 +3322,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3433,7 +3407,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3480,7 +3454,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3524,7 +3498,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3568,7 +3542,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3653,7 +3627,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3697,7 +3671,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3741,7 +3715,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3826,7 +3800,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3870,7 +3844,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3914,7 +3888,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4125,7 +4099,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4169,7 +4143,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4213,7 +4187,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4304,7 +4278,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4348,7 +4322,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4430,7 +4404,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4474,7 +4448,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4653,7 +4627,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4697,7 +4671,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4741,7 +4715,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4785,7 +4759,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4876,7 +4850,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4920,7 +4894,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -4967,7 +4941,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5011,7 +4985,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5058,7 +5032,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5146,7 +5120,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5190,7 +5164,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5234,7 +5208,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5278,7 +5252,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5451,7 +5425,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5495,7 +5469,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5539,7 +5513,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5806,7 +5780,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5850,7 +5824,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5894,7 +5868,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5938,7 +5912,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6390,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6460,7 +6434,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6504,7 +6478,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6630,7 +6604,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6674,7 +6648,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6721,7 +6695,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6765,7 +6739,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6891,7 +6865,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -6935,7 +6909,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7020,7 +6994,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7064,7 +7038,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7108,7 +7082,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7413,7 +7387,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7580,7 +7554,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7624,7 +7598,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7668,7 +7642,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -7929,7 +7903,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7973,7 +7947,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8058,7 +8032,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8184,7 +8158,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8228,7 +8202,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8313,7 +8287,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8357,7 +8331,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8401,7 +8375,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8706,7 +8680,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8873,7 +8847,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8917,7 +8891,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8961,7 +8935,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9090,7 +9064,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9134,7 +9108,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9178,7 +9152,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10055,7 +10029,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10140,7 +10114,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10155,55 +10129,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10376,7 +10350,7 @@
       <c r="L5" t="s">
         <v>546</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="1">
         <v>46235</v>
       </c>
       <c r="N5" t="s">
@@ -10508,7 +10482,7 @@
       <c r="L8" t="s">
         <v>549</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46300</v>
       </c>
       <c r="N8" t="s">
@@ -10596,7 +10570,7 @@
       <c r="L10" t="s">
         <v>549</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46300</v>
       </c>
       <c r="N10" t="s">
@@ -10640,7 +10614,7 @@
       <c r="L11" t="s">
         <v>549</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46300</v>
       </c>
       <c r="N11" t="s">
@@ -10813,7 +10787,7 @@
       <c r="L15" t="s">
         <v>548</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46315</v>
       </c>
       <c r="N15" t="s">
@@ -10857,7 +10831,7 @@
       <c r="L16" t="s">
         <v>549</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46300</v>
       </c>
       <c r="N16" t="s">
@@ -10901,7 +10875,7 @@
       <c r="L17" t="s">
         <v>548</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46315</v>
       </c>
       <c r="N17" t="s">
@@ -10945,7 +10919,7 @@
       <c r="L18" t="s">
         <v>549</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46300</v>
       </c>
       <c r="N18" t="s">
@@ -10989,7 +10963,7 @@
       <c r="L19" t="s">
         <v>549</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46300</v>
       </c>
       <c r="N19" t="s">
@@ -11033,7 +11007,7 @@
       <c r="L20" t="s">
         <v>549</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46300</v>
       </c>
       <c r="N20" t="s">
@@ -11077,7 +11051,7 @@
       <c r="L21" t="s">
         <v>549</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46300</v>
       </c>
       <c r="N21" t="s">
@@ -11253,7 +11227,7 @@
       <c r="L25" t="s">
         <v>548</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46315</v>
       </c>
       <c r="N25" t="s">
@@ -11341,7 +11315,7 @@
       <c r="L27" t="s">
         <v>549</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46300</v>
       </c>
       <c r="N27" t="s">
@@ -11385,7 +11359,7 @@
       <c r="L28" t="s">
         <v>549</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46300</v>
       </c>
       <c r="N28" t="s">
@@ -11429,7 +11403,7 @@
       <c r="L29" t="s">
         <v>549</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46300</v>
       </c>
       <c r="N29" t="s">
@@ -11473,7 +11447,7 @@
       <c r="L30" t="s">
         <v>549</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46300</v>
       </c>
       <c r="N30" t="s">
@@ -11517,7 +11491,7 @@
       <c r="L31" t="s">
         <v>548</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46315</v>
       </c>
       <c r="N31" t="s">
@@ -11561,7 +11535,7 @@
       <c r="L32" t="s">
         <v>548</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46315</v>
       </c>
       <c r="N32" t="s">
@@ -11605,7 +11579,7 @@
       <c r="L33" t="s">
         <v>548</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46315</v>
       </c>
       <c r="N33" t="s">
@@ -11649,7 +11623,7 @@
       <c r="L34" t="s">
         <v>549</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46300</v>
       </c>
       <c r="N34" t="s">
@@ -11693,7 +11667,7 @@
       <c r="L35" t="s">
         <v>548</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46315</v>
       </c>
       <c r="N35" t="s">
@@ -11737,7 +11711,7 @@
       <c r="L36" t="s">
         <v>549</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46300</v>
       </c>
       <c r="N36" t="s">
@@ -11781,7 +11755,7 @@
       <c r="L37" t="s">
         <v>549</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46300</v>
       </c>
       <c r="N37" t="s">
@@ -11825,7 +11799,7 @@
       <c r="L38" t="s">
         <v>549</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46300</v>
       </c>
       <c r="N38" t="s">
@@ -11869,7 +11843,7 @@
       <c r="L39" t="s">
         <v>548</v>
       </c>
-      <c r="M39" s="2">
+      <c r="M39" s="1">
         <v>46315</v>
       </c>
       <c r="N39" t="s">
@@ -11913,7 +11887,7 @@
       <c r="L40" t="s">
         <v>549</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46300</v>
       </c>
       <c r="N40" t="s">
@@ -11957,7 +11931,7 @@
       <c r="L41" t="s">
         <v>549</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46300</v>
       </c>
       <c r="N41" t="s">
@@ -12001,7 +11975,7 @@
       <c r="L42" t="s">
         <v>549</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46300</v>
       </c>
       <c r="N42" t="s">
@@ -12045,7 +12019,7 @@
       <c r="L43" t="s">
         <v>549</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46300</v>
       </c>
       <c r="N43" t="s">
@@ -12089,7 +12063,7 @@
       <c r="L44" t="s">
         <v>549</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46300</v>
       </c>
       <c r="N44" t="s">
@@ -12133,7 +12107,7 @@
       <c r="L45" t="s">
         <v>549</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46300</v>
       </c>
       <c r="N45" t="s">
@@ -12177,7 +12151,7 @@
       <c r="L46" t="s">
         <v>549</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46300</v>
       </c>
       <c r="N46" t="s">
@@ -12221,7 +12195,7 @@
       <c r="L47" t="s">
         <v>549</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46300</v>
       </c>
       <c r="N47" t="s">
@@ -12265,7 +12239,7 @@
       <c r="L48" t="s">
         <v>548</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46315</v>
       </c>
       <c r="N48" t="s">
@@ -12309,7 +12283,7 @@
       <c r="L49" t="s">
         <v>548</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46315</v>
       </c>
       <c r="N49" t="s">
@@ -12353,7 +12327,7 @@
       <c r="L50" t="s">
         <v>549</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46300</v>
       </c>
       <c r="N50" t="s">
@@ -12397,7 +12371,7 @@
       <c r="L51" t="s">
         <v>549</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46300</v>
       </c>
       <c r="N51" t="s">
@@ -12441,7 +12415,7 @@
       <c r="L52" t="s">
         <v>549</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46300</v>
       </c>
       <c r="N52" t="s">
@@ -12485,7 +12459,7 @@
       <c r="L53" t="s">
         <v>549</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46300</v>
       </c>
       <c r="N53" t="s">
@@ -12529,7 +12503,7 @@
       <c r="L54" t="s">
         <v>548</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46315</v>
       </c>
       <c r="N54" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (23/07/2026 06:40)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10351,7 +10351,7 @@
         <v>546</v>
       </c>
       <c r="M5" s="1">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="N5" t="s">
         <v>552</v>
@@ -10483,7 +10483,7 @@
         <v>549</v>
       </c>
       <c r="M8" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N8" t="s">
         <v>552</v>
@@ -10571,7 +10571,7 @@
         <v>549</v>
       </c>
       <c r="M10" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N10" t="s">
         <v>552</v>
@@ -10615,7 +10615,7 @@
         <v>549</v>
       </c>
       <c r="M11" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N11" t="s">
         <v>552</v>
@@ -10788,7 +10788,7 @@
         <v>548</v>
       </c>
       <c r="M15" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N15" t="s">
         <v>552</v>
@@ -10832,7 +10832,7 @@
         <v>549</v>
       </c>
       <c r="M16" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N16" t="s">
         <v>552</v>
@@ -10876,7 +10876,7 @@
         <v>548</v>
       </c>
       <c r="M17" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N17" t="s">
         <v>552</v>
@@ -10920,7 +10920,7 @@
         <v>549</v>
       </c>
       <c r="M18" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N18" t="s">
         <v>552</v>
@@ -10964,7 +10964,7 @@
         <v>549</v>
       </c>
       <c r="M19" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N19" t="s">
         <v>552</v>
@@ -11008,7 +11008,7 @@
         <v>549</v>
       </c>
       <c r="M20" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N20" t="s">
         <v>552</v>
@@ -11052,7 +11052,7 @@
         <v>549</v>
       </c>
       <c r="M21" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N21" t="s">
         <v>552</v>
@@ -11228,7 +11228,7 @@
         <v>548</v>
       </c>
       <c r="M25" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N25" t="s">
         <v>552</v>
@@ -11316,7 +11316,7 @@
         <v>549</v>
       </c>
       <c r="M27" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N27" t="s">
         <v>552</v>
@@ -11360,7 +11360,7 @@
         <v>549</v>
       </c>
       <c r="M28" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N28" t="s">
         <v>552</v>
@@ -11404,7 +11404,7 @@
         <v>549</v>
       </c>
       <c r="M29" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N29" t="s">
         <v>552</v>
@@ -11448,7 +11448,7 @@
         <v>549</v>
       </c>
       <c r="M30" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N30" t="s">
         <v>552</v>
@@ -11492,7 +11492,7 @@
         <v>548</v>
       </c>
       <c r="M31" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N31" t="s">
         <v>552</v>
@@ -11536,7 +11536,7 @@
         <v>548</v>
       </c>
       <c r="M32" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N32" t="s">
         <v>552</v>
@@ -11580,7 +11580,7 @@
         <v>548</v>
       </c>
       <c r="M33" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N33" t="s">
         <v>552</v>
@@ -11624,7 +11624,7 @@
         <v>549</v>
       </c>
       <c r="M34" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N34" t="s">
         <v>552</v>
@@ -11668,7 +11668,7 @@
         <v>548</v>
       </c>
       <c r="M35" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N35" t="s">
         <v>552</v>
@@ -11712,7 +11712,7 @@
         <v>549</v>
       </c>
       <c r="M36" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N36" t="s">
         <v>552</v>
@@ -11756,7 +11756,7 @@
         <v>549</v>
       </c>
       <c r="M37" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N37" t="s">
         <v>552</v>
@@ -11800,7 +11800,7 @@
         <v>549</v>
       </c>
       <c r="M38" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N38" t="s">
         <v>552</v>
@@ -11844,7 +11844,7 @@
         <v>548</v>
       </c>
       <c r="M39" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N39" t="s">
         <v>552</v>
@@ -11888,7 +11888,7 @@
         <v>549</v>
       </c>
       <c r="M40" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N40" t="s">
         <v>552</v>
@@ -11932,7 +11932,7 @@
         <v>549</v>
       </c>
       <c r="M41" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N41" t="s">
         <v>552</v>
@@ -11976,7 +11976,7 @@
         <v>549</v>
       </c>
       <c r="M42" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N42" t="s">
         <v>552</v>
@@ -12020,7 +12020,7 @@
         <v>549</v>
       </c>
       <c r="M43" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N43" t="s">
         <v>552</v>
@@ -12064,7 +12064,7 @@
         <v>549</v>
       </c>
       <c r="M44" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N44" t="s">
         <v>552</v>
@@ -12108,7 +12108,7 @@
         <v>549</v>
       </c>
       <c r="M45" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N45" t="s">
         <v>552</v>
@@ -12152,7 +12152,7 @@
         <v>549</v>
       </c>
       <c r="M46" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N46" t="s">
         <v>552</v>
@@ -12196,7 +12196,7 @@
         <v>549</v>
       </c>
       <c r="M47" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N47" t="s">
         <v>552</v>
@@ -12240,7 +12240,7 @@
         <v>548</v>
       </c>
       <c r="M48" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N48" t="s">
         <v>552</v>
@@ -12284,7 +12284,7 @@
         <v>548</v>
       </c>
       <c r="M49" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N49" t="s">
         <v>552</v>
@@ -12328,7 +12328,7 @@
         <v>549</v>
       </c>
       <c r="M50" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N50" t="s">
         <v>552</v>
@@ -12372,7 +12372,7 @@
         <v>549</v>
       </c>
       <c r="M51" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N51" t="s">
         <v>552</v>
@@ -12416,7 +12416,7 @@
         <v>549</v>
       </c>
       <c r="M52" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N52" t="s">
         <v>552</v>
@@ -12460,7 +12460,7 @@
         <v>549</v>
       </c>
       <c r="M53" s="1">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N53" t="s">
         <v>552</v>
@@ -12504,7 +12504,7 @@
         <v>548</v>
       </c>
       <c r="M54" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N54" t="s">
         <v>552</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (23/07/2026 11:42)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1683,8 +1683,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1700,7 +1708,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1708,12 +1716,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2013,55 +2039,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2105,7 +2131,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2149,7 +2175,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2193,7 +2219,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2319,7 +2345,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2363,7 +2389,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2407,7 +2433,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2454,7 +2480,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2577,7 +2603,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2621,7 +2647,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2665,7 +2691,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2709,7 +2735,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2756,7 +2782,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2800,7 +2826,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2926,7 +2952,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2970,7 +2996,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3055,7 +3081,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3102,7 +3128,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3149,7 +3175,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3193,7 +3219,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3237,7 +3263,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3322,7 +3348,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3407,7 +3433,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3454,7 +3480,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3498,7 +3524,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3542,7 +3568,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3627,7 +3653,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3671,7 +3697,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3715,7 +3741,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3800,7 +3826,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3844,7 +3870,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3888,7 +3914,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3932,7 +3958,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4099,7 +4125,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4143,7 +4169,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4187,7 +4213,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4231,7 +4257,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4278,7 +4304,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4322,7 +4348,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4404,7 +4430,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4448,7 +4474,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4536,7 +4562,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4580,7 +4606,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4627,7 +4653,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4671,7 +4697,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4715,7 +4741,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4759,7 +4785,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4803,7 +4829,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4850,7 +4876,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4894,7 +4920,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -4941,7 +4967,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -4985,7 +5011,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5032,7 +5058,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5120,7 +5146,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5164,7 +5190,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5208,7 +5234,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5252,7 +5278,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5296,7 +5322,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5340,7 +5366,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5425,7 +5451,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5469,7 +5495,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5513,7 +5539,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5557,7 +5583,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5601,7 +5627,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5645,7 +5671,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5689,7 +5715,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5733,7 +5759,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5780,7 +5806,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5824,7 +5850,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5868,7 +5894,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5912,7 +5938,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5956,7 +5982,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6000,7 +6026,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6044,7 +6070,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6088,7 +6114,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6132,7 +6158,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6220,7 +6246,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6264,7 +6290,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6390,7 +6416,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6434,7 +6460,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6478,7 +6504,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6522,7 +6548,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6604,7 +6630,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6648,7 +6674,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6695,7 +6721,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6739,7 +6765,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6865,7 +6891,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6909,7 +6935,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -6994,7 +7020,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7038,7 +7064,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7082,7 +7108,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7126,7 +7152,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7170,7 +7196,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7214,7 +7240,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7258,7 +7284,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7302,7 +7328,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7387,7 +7413,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7554,7 +7580,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7598,7 +7624,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7642,7 +7668,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7686,7 +7712,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7730,7 +7756,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7774,7 +7800,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7818,7 +7844,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7903,7 +7929,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7947,7 +7973,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8032,7 +8058,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8158,7 +8184,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8202,7 +8228,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8287,7 +8313,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8331,7 +8357,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8375,7 +8401,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8419,7 +8445,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8463,7 +8489,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8507,7 +8533,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8551,7 +8577,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8595,7 +8621,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8680,7 +8706,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8847,7 +8873,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8891,7 +8917,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8935,7 +8961,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8979,7 +9005,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9064,7 +9090,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9108,7 +9134,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9152,7 +9178,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9196,7 +9222,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9240,7 +9266,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9284,7 +9310,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9328,7 +9354,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9372,7 +9398,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9416,7 +9442,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9460,7 +9486,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9504,7 +9530,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9548,7 +9574,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9592,7 +9618,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9636,7 +9662,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9680,7 +9706,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9724,7 +9750,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9768,7 +9794,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9812,7 +9838,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9856,7 +9882,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9900,7 +9926,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9944,7 +9970,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10029,7 +10055,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10114,7 +10140,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10129,55 +10155,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10350,7 +10376,7 @@
       <c r="L5" t="s">
         <v>546</v>
       </c>
-      <c r="M5" s="1">
+      <c r="M5" s="2">
         <v>46236</v>
       </c>
       <c r="N5" t="s">
@@ -10482,7 +10508,7 @@
       <c r="L8" t="s">
         <v>549</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46301</v>
       </c>
       <c r="N8" t="s">
@@ -10570,7 +10596,7 @@
       <c r="L10" t="s">
         <v>549</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46301</v>
       </c>
       <c r="N10" t="s">
@@ -10614,7 +10640,7 @@
       <c r="L11" t="s">
         <v>549</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46301</v>
       </c>
       <c r="N11" t="s">
@@ -10787,7 +10813,7 @@
       <c r="L15" t="s">
         <v>548</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46316</v>
       </c>
       <c r="N15" t="s">
@@ -10831,7 +10857,7 @@
       <c r="L16" t="s">
         <v>549</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46301</v>
       </c>
       <c r="N16" t="s">
@@ -10875,7 +10901,7 @@
       <c r="L17" t="s">
         <v>548</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46316</v>
       </c>
       <c r="N17" t="s">
@@ -10919,7 +10945,7 @@
       <c r="L18" t="s">
         <v>549</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46301</v>
       </c>
       <c r="N18" t="s">
@@ -10963,7 +10989,7 @@
       <c r="L19" t="s">
         <v>549</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46301</v>
       </c>
       <c r="N19" t="s">
@@ -11007,7 +11033,7 @@
       <c r="L20" t="s">
         <v>549</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46301</v>
       </c>
       <c r="N20" t="s">
@@ -11051,7 +11077,7 @@
       <c r="L21" t="s">
         <v>549</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46301</v>
       </c>
       <c r="N21" t="s">
@@ -11227,7 +11253,7 @@
       <c r="L25" t="s">
         <v>548</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46316</v>
       </c>
       <c r="N25" t="s">
@@ -11315,7 +11341,7 @@
       <c r="L27" t="s">
         <v>549</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46301</v>
       </c>
       <c r="N27" t="s">
@@ -11359,7 +11385,7 @@
       <c r="L28" t="s">
         <v>549</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46301</v>
       </c>
       <c r="N28" t="s">
@@ -11403,7 +11429,7 @@
       <c r="L29" t="s">
         <v>549</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46301</v>
       </c>
       <c r="N29" t="s">
@@ -11447,7 +11473,7 @@
       <c r="L30" t="s">
         <v>549</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46301</v>
       </c>
       <c r="N30" t="s">
@@ -11491,7 +11517,7 @@
       <c r="L31" t="s">
         <v>548</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46316</v>
       </c>
       <c r="N31" t="s">
@@ -11535,7 +11561,7 @@
       <c r="L32" t="s">
         <v>548</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46316</v>
       </c>
       <c r="N32" t="s">
@@ -11579,7 +11605,7 @@
       <c r="L33" t="s">
         <v>548</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46316</v>
       </c>
       <c r="N33" t="s">
@@ -11623,7 +11649,7 @@
       <c r="L34" t="s">
         <v>549</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46301</v>
       </c>
       <c r="N34" t="s">
@@ -11667,7 +11693,7 @@
       <c r="L35" t="s">
         <v>548</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46316</v>
       </c>
       <c r="N35" t="s">
@@ -11711,7 +11737,7 @@
       <c r="L36" t="s">
         <v>549</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46301</v>
       </c>
       <c r="N36" t="s">
@@ -11755,7 +11781,7 @@
       <c r="L37" t="s">
         <v>549</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46301</v>
       </c>
       <c r="N37" t="s">
@@ -11799,7 +11825,7 @@
       <c r="L38" t="s">
         <v>549</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46301</v>
       </c>
       <c r="N38" t="s">
@@ -11843,7 +11869,7 @@
       <c r="L39" t="s">
         <v>548</v>
       </c>
-      <c r="M39" s="1">
+      <c r="M39" s="2">
         <v>46316</v>
       </c>
       <c r="N39" t="s">
@@ -11887,7 +11913,7 @@
       <c r="L40" t="s">
         <v>549</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46301</v>
       </c>
       <c r="N40" t="s">
@@ -11931,7 +11957,7 @@
       <c r="L41" t="s">
         <v>549</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46301</v>
       </c>
       <c r="N41" t="s">
@@ -11975,7 +12001,7 @@
       <c r="L42" t="s">
         <v>549</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46301</v>
       </c>
       <c r="N42" t="s">
@@ -12019,7 +12045,7 @@
       <c r="L43" t="s">
         <v>549</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46301</v>
       </c>
       <c r="N43" t="s">
@@ -12063,7 +12089,7 @@
       <c r="L44" t="s">
         <v>549</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46301</v>
       </c>
       <c r="N44" t="s">
@@ -12107,7 +12133,7 @@
       <c r="L45" t="s">
         <v>549</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46301</v>
       </c>
       <c r="N45" t="s">
@@ -12151,7 +12177,7 @@
       <c r="L46" t="s">
         <v>549</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46301</v>
       </c>
       <c r="N46" t="s">
@@ -12195,7 +12221,7 @@
       <c r="L47" t="s">
         <v>549</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46301</v>
       </c>
       <c r="N47" t="s">
@@ -12239,7 +12265,7 @@
       <c r="L48" t="s">
         <v>548</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46316</v>
       </c>
       <c r="N48" t="s">
@@ -12283,7 +12309,7 @@
       <c r="L49" t="s">
         <v>548</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46316</v>
       </c>
       <c r="N49" t="s">
@@ -12327,7 +12353,7 @@
       <c r="L50" t="s">
         <v>549</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46301</v>
       </c>
       <c r="N50" t="s">
@@ -12371,7 +12397,7 @@
       <c r="L51" t="s">
         <v>549</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46301</v>
       </c>
       <c r="N51" t="s">
@@ -12415,7 +12441,7 @@
       <c r="L52" t="s">
         <v>549</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46301</v>
       </c>
       <c r="N52" t="s">
@@ -12459,7 +12485,7 @@
       <c r="L53" t="s">
         <v>549</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46301</v>
       </c>
       <c r="N53" t="s">
@@ -12503,7 +12529,7 @@
       <c r="L54" t="s">
         <v>548</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46316</v>
       </c>
       <c r="N54" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (23/07/2026 16:18)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1683,16 +1683,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1708,7 +1700,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1716,30 +1708,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2039,55 +2013,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2131,7 +2105,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2175,7 +2149,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2219,7 +2193,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2345,7 +2319,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2389,7 +2363,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2433,7 +2407,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2480,7 +2454,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2603,7 +2577,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2647,7 +2621,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2691,7 +2665,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2735,7 +2709,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2782,7 +2756,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2826,7 +2800,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2952,7 +2926,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2996,7 +2970,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3081,7 +3055,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3128,7 +3102,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3175,7 +3149,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3219,7 +3193,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3263,7 +3237,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3348,7 +3322,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3433,7 +3407,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3480,7 +3454,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3524,7 +3498,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3568,7 +3542,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3653,7 +3627,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3697,7 +3671,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3741,7 +3715,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3826,7 +3800,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3870,7 +3844,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3914,7 +3888,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3958,7 +3932,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4125,7 +4099,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4169,7 +4143,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4213,7 +4187,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4257,7 +4231,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4304,7 +4278,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4348,7 +4322,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4430,7 +4404,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4474,7 +4448,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4562,7 +4536,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4606,7 +4580,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4653,7 +4627,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4697,7 +4671,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4741,7 +4715,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4785,7 +4759,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4829,7 +4803,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4876,7 +4850,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4920,7 +4894,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -4967,7 +4941,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5011,7 +4985,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5058,7 +5032,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5146,7 +5120,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5190,7 +5164,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5234,7 +5208,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5278,7 +5252,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5322,7 +5296,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5366,7 +5340,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5451,7 +5425,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5495,7 +5469,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5539,7 +5513,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5583,7 +5557,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5627,7 +5601,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5671,7 +5645,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5715,7 +5689,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5759,7 +5733,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5806,7 +5780,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5850,7 +5824,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5894,7 +5868,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5938,7 +5912,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5982,7 +5956,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6026,7 +6000,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6070,7 +6044,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6114,7 +6088,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6158,7 +6132,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6246,7 +6220,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6290,7 +6264,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6416,7 +6390,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6460,7 +6434,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6504,7 +6478,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6548,7 +6522,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6630,7 +6604,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6674,7 +6648,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6721,7 +6695,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6765,7 +6739,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6891,7 +6865,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -6935,7 +6909,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7020,7 +6994,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7064,7 +7038,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7108,7 +7082,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7152,7 +7126,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7196,7 +7170,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7240,7 +7214,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7284,7 +7258,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7328,7 +7302,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7413,7 +7387,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7580,7 +7554,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7624,7 +7598,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7668,7 +7642,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7712,7 +7686,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7756,7 +7730,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7800,7 +7774,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7844,7 +7818,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -7929,7 +7903,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7973,7 +7947,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8058,7 +8032,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8184,7 +8158,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8228,7 +8202,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8313,7 +8287,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8357,7 +8331,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8401,7 +8375,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8445,7 +8419,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8489,7 +8463,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8533,7 +8507,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8577,7 +8551,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8621,7 +8595,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8706,7 +8680,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8873,7 +8847,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8917,7 +8891,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -8961,7 +8935,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9005,7 +8979,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9090,7 +9064,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9134,7 +9108,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9178,7 +9152,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9222,7 +9196,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9266,7 +9240,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9310,7 +9284,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9354,7 +9328,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9398,7 +9372,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9442,7 +9416,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9486,7 +9460,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9530,7 +9504,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9574,7 +9548,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9618,7 +9592,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9662,7 +9636,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9706,7 +9680,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9750,7 +9724,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9794,7 +9768,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9838,7 +9812,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9882,7 +9856,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -9926,7 +9900,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9970,7 +9944,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10055,7 +10029,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10140,7 +10114,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10155,55 +10129,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10376,7 +10350,7 @@
       <c r="L5" t="s">
         <v>546</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="1">
         <v>46236</v>
       </c>
       <c r="N5" t="s">
@@ -10508,7 +10482,7 @@
       <c r="L8" t="s">
         <v>549</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46301</v>
       </c>
       <c r="N8" t="s">
@@ -10596,7 +10570,7 @@
       <c r="L10" t="s">
         <v>549</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46301</v>
       </c>
       <c r="N10" t="s">
@@ -10640,7 +10614,7 @@
       <c r="L11" t="s">
         <v>549</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46301</v>
       </c>
       <c r="N11" t="s">
@@ -10813,7 +10787,7 @@
       <c r="L15" t="s">
         <v>548</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46316</v>
       </c>
       <c r="N15" t="s">
@@ -10857,7 +10831,7 @@
       <c r="L16" t="s">
         <v>549</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46301</v>
       </c>
       <c r="N16" t="s">
@@ -10901,7 +10875,7 @@
       <c r="L17" t="s">
         <v>548</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46316</v>
       </c>
       <c r="N17" t="s">
@@ -10945,7 +10919,7 @@
       <c r="L18" t="s">
         <v>549</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46301</v>
       </c>
       <c r="N18" t="s">
@@ -10989,7 +10963,7 @@
       <c r="L19" t="s">
         <v>549</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46301</v>
       </c>
       <c r="N19" t="s">
@@ -11033,7 +11007,7 @@
       <c r="L20" t="s">
         <v>549</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46301</v>
       </c>
       <c r="N20" t="s">
@@ -11077,7 +11051,7 @@
       <c r="L21" t="s">
         <v>549</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46301</v>
       </c>
       <c r="N21" t="s">
@@ -11253,7 +11227,7 @@
       <c r="L25" t="s">
         <v>548</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46316</v>
       </c>
       <c r="N25" t="s">
@@ -11341,7 +11315,7 @@
       <c r="L27" t="s">
         <v>549</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46301</v>
       </c>
       <c r="N27" t="s">
@@ -11385,7 +11359,7 @@
       <c r="L28" t="s">
         <v>549</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46301</v>
       </c>
       <c r="N28" t="s">
@@ -11429,7 +11403,7 @@
       <c r="L29" t="s">
         <v>549</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46301</v>
       </c>
       <c r="N29" t="s">
@@ -11473,7 +11447,7 @@
       <c r="L30" t="s">
         <v>549</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46301</v>
       </c>
       <c r="N30" t="s">
@@ -11517,7 +11491,7 @@
       <c r="L31" t="s">
         <v>548</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46316</v>
       </c>
       <c r="N31" t="s">
@@ -11561,7 +11535,7 @@
       <c r="L32" t="s">
         <v>548</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46316</v>
       </c>
       <c r="N32" t="s">
@@ -11605,7 +11579,7 @@
       <c r="L33" t="s">
         <v>548</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46316</v>
       </c>
       <c r="N33" t="s">
@@ -11649,7 +11623,7 @@
       <c r="L34" t="s">
         <v>549</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46301</v>
       </c>
       <c r="N34" t="s">
@@ -11693,7 +11667,7 @@
       <c r="L35" t="s">
         <v>548</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46316</v>
       </c>
       <c r="N35" t="s">
@@ -11737,7 +11711,7 @@
       <c r="L36" t="s">
         <v>549</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46301</v>
       </c>
       <c r="N36" t="s">
@@ -11781,7 +11755,7 @@
       <c r="L37" t="s">
         <v>549</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46301</v>
       </c>
       <c r="N37" t="s">
@@ -11825,7 +11799,7 @@
       <c r="L38" t="s">
         <v>549</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46301</v>
       </c>
       <c r="N38" t="s">
@@ -11869,7 +11843,7 @@
       <c r="L39" t="s">
         <v>548</v>
       </c>
-      <c r="M39" s="2">
+      <c r="M39" s="1">
         <v>46316</v>
       </c>
       <c r="N39" t="s">
@@ -11913,7 +11887,7 @@
       <c r="L40" t="s">
         <v>549</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46301</v>
       </c>
       <c r="N40" t="s">
@@ -11957,7 +11931,7 @@
       <c r="L41" t="s">
         <v>549</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46301</v>
       </c>
       <c r="N41" t="s">
@@ -12001,7 +11975,7 @@
       <c r="L42" t="s">
         <v>549</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46301</v>
       </c>
       <c r="N42" t="s">
@@ -12045,7 +12019,7 @@
       <c r="L43" t="s">
         <v>549</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46301</v>
       </c>
       <c r="N43" t="s">
@@ -12089,7 +12063,7 @@
       <c r="L44" t="s">
         <v>549</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46301</v>
       </c>
       <c r="N44" t="s">
@@ -12133,7 +12107,7 @@
       <c r="L45" t="s">
         <v>549</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46301</v>
       </c>
       <c r="N45" t="s">
@@ -12177,7 +12151,7 @@
       <c r="L46" t="s">
         <v>549</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46301</v>
       </c>
       <c r="N46" t="s">
@@ -12221,7 +12195,7 @@
       <c r="L47" t="s">
         <v>549</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46301</v>
       </c>
       <c r="N47" t="s">
@@ -12265,7 +12239,7 @@
       <c r="L48" t="s">
         <v>548</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46316</v>
       </c>
       <c r="N48" t="s">
@@ -12309,7 +12283,7 @@
       <c r="L49" t="s">
         <v>548</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46316</v>
       </c>
       <c r="N49" t="s">
@@ -12353,7 +12327,7 @@
       <c r="L50" t="s">
         <v>549</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46301</v>
       </c>
       <c r="N50" t="s">
@@ -12397,7 +12371,7 @@
       <c r="L51" t="s">
         <v>549</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46301</v>
       </c>
       <c r="N51" t="s">
@@ -12441,7 +12415,7 @@
       <c r="L52" t="s">
         <v>549</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46301</v>
       </c>
       <c r="N52" t="s">
@@ -12485,7 +12459,7 @@
       <c r="L53" t="s">
         <v>549</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46301</v>
       </c>
       <c r="N53" t="s">
@@ -12529,7 +12503,7 @@
       <c r="L54" t="s">
         <v>548</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46316</v>
       </c>
       <c r="N54" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (24/07/2026 17:53)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10351,7 +10351,7 @@
         <v>546</v>
       </c>
       <c r="M5" s="1">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="N5" t="s">
         <v>552</v>
@@ -10483,7 +10483,7 @@
         <v>549</v>
       </c>
       <c r="M8" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N8" t="s">
         <v>552</v>
@@ -10571,7 +10571,7 @@
         <v>549</v>
       </c>
       <c r="M10" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N10" t="s">
         <v>552</v>
@@ -10615,7 +10615,7 @@
         <v>549</v>
       </c>
       <c r="M11" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N11" t="s">
         <v>552</v>
@@ -10788,7 +10788,7 @@
         <v>548</v>
       </c>
       <c r="M15" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N15" t="s">
         <v>552</v>
@@ -10832,7 +10832,7 @@
         <v>549</v>
       </c>
       <c r="M16" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N16" t="s">
         <v>552</v>
@@ -10876,7 +10876,7 @@
         <v>548</v>
       </c>
       <c r="M17" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N17" t="s">
         <v>552</v>
@@ -10920,7 +10920,7 @@
         <v>549</v>
       </c>
       <c r="M18" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N18" t="s">
         <v>552</v>
@@ -10964,7 +10964,7 @@
         <v>549</v>
       </c>
       <c r="M19" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N19" t="s">
         <v>552</v>
@@ -11008,7 +11008,7 @@
         <v>549</v>
       </c>
       <c r="M20" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N20" t="s">
         <v>552</v>
@@ -11052,7 +11052,7 @@
         <v>549</v>
       </c>
       <c r="M21" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N21" t="s">
         <v>552</v>
@@ -11228,7 +11228,7 @@
         <v>548</v>
       </c>
       <c r="M25" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N25" t="s">
         <v>552</v>
@@ -11316,7 +11316,7 @@
         <v>549</v>
       </c>
       <c r="M27" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N27" t="s">
         <v>552</v>
@@ -11360,7 +11360,7 @@
         <v>549</v>
       </c>
       <c r="M28" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N28" t="s">
         <v>552</v>
@@ -11404,7 +11404,7 @@
         <v>549</v>
       </c>
       <c r="M29" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N29" t="s">
         <v>552</v>
@@ -11448,7 +11448,7 @@
         <v>549</v>
       </c>
       <c r="M30" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N30" t="s">
         <v>552</v>
@@ -11492,7 +11492,7 @@
         <v>548</v>
       </c>
       <c r="M31" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N31" t="s">
         <v>552</v>
@@ -11536,7 +11536,7 @@
         <v>548</v>
       </c>
       <c r="M32" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N32" t="s">
         <v>552</v>
@@ -11580,7 +11580,7 @@
         <v>548</v>
       </c>
       <c r="M33" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N33" t="s">
         <v>552</v>
@@ -11624,7 +11624,7 @@
         <v>549</v>
       </c>
       <c r="M34" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N34" t="s">
         <v>552</v>
@@ -11668,7 +11668,7 @@
         <v>548</v>
       </c>
       <c r="M35" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N35" t="s">
         <v>552</v>
@@ -11712,7 +11712,7 @@
         <v>549</v>
       </c>
       <c r="M36" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N36" t="s">
         <v>552</v>
@@ -11756,7 +11756,7 @@
         <v>549</v>
       </c>
       <c r="M37" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N37" t="s">
         <v>552</v>
@@ -11800,7 +11800,7 @@
         <v>549</v>
       </c>
       <c r="M38" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N38" t="s">
         <v>552</v>
@@ -11844,7 +11844,7 @@
         <v>548</v>
       </c>
       <c r="M39" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N39" t="s">
         <v>552</v>
@@ -11888,7 +11888,7 @@
         <v>549</v>
       </c>
       <c r="M40" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N40" t="s">
         <v>552</v>
@@ -11932,7 +11932,7 @@
         <v>549</v>
       </c>
       <c r="M41" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N41" t="s">
         <v>552</v>
@@ -11976,7 +11976,7 @@
         <v>549</v>
       </c>
       <c r="M42" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N42" t="s">
         <v>552</v>
@@ -12020,7 +12020,7 @@
         <v>549</v>
       </c>
       <c r="M43" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N43" t="s">
         <v>552</v>
@@ -12064,7 +12064,7 @@
         <v>549</v>
       </c>
       <c r="M44" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N44" t="s">
         <v>552</v>
@@ -12108,7 +12108,7 @@
         <v>549</v>
       </c>
       <c r="M45" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N45" t="s">
         <v>552</v>
@@ -12152,7 +12152,7 @@
         <v>549</v>
       </c>
       <c r="M46" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N46" t="s">
         <v>552</v>
@@ -12196,7 +12196,7 @@
         <v>549</v>
       </c>
       <c r="M47" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N47" t="s">
         <v>552</v>
@@ -12240,7 +12240,7 @@
         <v>548</v>
       </c>
       <c r="M48" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N48" t="s">
         <v>552</v>
@@ -12284,7 +12284,7 @@
         <v>548</v>
       </c>
       <c r="M49" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N49" t="s">
         <v>552</v>
@@ -12328,7 +12328,7 @@
         <v>549</v>
       </c>
       <c r="M50" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N50" t="s">
         <v>552</v>
@@ -12372,7 +12372,7 @@
         <v>549</v>
       </c>
       <c r="M51" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N51" t="s">
         <v>552</v>
@@ -12416,7 +12416,7 @@
         <v>549</v>
       </c>
       <c r="M52" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N52" t="s">
         <v>552</v>
@@ -12460,7 +12460,7 @@
         <v>549</v>
       </c>
       <c r="M53" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="N53" t="s">
         <v>552</v>
@@ -12504,7 +12504,7 @@
         <v>548</v>
       </c>
       <c r="M54" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="N54" t="s">
         <v>552</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (25/07/2026 03:08)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10351,7 +10351,7 @@
         <v>546</v>
       </c>
       <c r="M5" s="1">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="N5" t="s">
         <v>552</v>
@@ -10483,7 +10483,7 @@
         <v>549</v>
       </c>
       <c r="M8" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N8" t="s">
         <v>552</v>
@@ -10571,7 +10571,7 @@
         <v>549</v>
       </c>
       <c r="M10" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N10" t="s">
         <v>552</v>
@@ -10615,7 +10615,7 @@
         <v>549</v>
       </c>
       <c r="M11" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N11" t="s">
         <v>552</v>
@@ -10788,7 +10788,7 @@
         <v>548</v>
       </c>
       <c r="M15" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N15" t="s">
         <v>552</v>
@@ -10832,7 +10832,7 @@
         <v>549</v>
       </c>
       <c r="M16" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N16" t="s">
         <v>552</v>
@@ -10876,7 +10876,7 @@
         <v>548</v>
       </c>
       <c r="M17" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N17" t="s">
         <v>552</v>
@@ -10920,7 +10920,7 @@
         <v>549</v>
       </c>
       <c r="M18" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N18" t="s">
         <v>552</v>
@@ -10964,7 +10964,7 @@
         <v>549</v>
       </c>
       <c r="M19" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N19" t="s">
         <v>552</v>
@@ -11008,7 +11008,7 @@
         <v>549</v>
       </c>
       <c r="M20" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N20" t="s">
         <v>552</v>
@@ -11052,7 +11052,7 @@
         <v>549</v>
       </c>
       <c r="M21" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N21" t="s">
         <v>552</v>
@@ -11228,7 +11228,7 @@
         <v>548</v>
       </c>
       <c r="M25" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N25" t="s">
         <v>552</v>
@@ -11316,7 +11316,7 @@
         <v>549</v>
       </c>
       <c r="M27" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N27" t="s">
         <v>552</v>
@@ -11360,7 +11360,7 @@
         <v>549</v>
       </c>
       <c r="M28" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N28" t="s">
         <v>552</v>
@@ -11404,7 +11404,7 @@
         <v>549</v>
       </c>
       <c r="M29" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N29" t="s">
         <v>552</v>
@@ -11448,7 +11448,7 @@
         <v>549</v>
       </c>
       <c r="M30" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N30" t="s">
         <v>552</v>
@@ -11492,7 +11492,7 @@
         <v>548</v>
       </c>
       <c r="M31" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N31" t="s">
         <v>552</v>
@@ -11536,7 +11536,7 @@
         <v>548</v>
       </c>
       <c r="M32" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N32" t="s">
         <v>552</v>
@@ -11580,7 +11580,7 @@
         <v>548</v>
       </c>
       <c r="M33" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N33" t="s">
         <v>552</v>
@@ -11624,7 +11624,7 @@
         <v>549</v>
       </c>
       <c r="M34" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N34" t="s">
         <v>552</v>
@@ -11668,7 +11668,7 @@
         <v>548</v>
       </c>
       <c r="M35" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N35" t="s">
         <v>552</v>
@@ -11712,7 +11712,7 @@
         <v>549</v>
       </c>
       <c r="M36" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N36" t="s">
         <v>552</v>
@@ -11756,7 +11756,7 @@
         <v>549</v>
       </c>
       <c r="M37" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N37" t="s">
         <v>552</v>
@@ -11800,7 +11800,7 @@
         <v>549</v>
       </c>
       <c r="M38" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N38" t="s">
         <v>552</v>
@@ -11844,7 +11844,7 @@
         <v>548</v>
       </c>
       <c r="M39" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N39" t="s">
         <v>552</v>
@@ -11888,7 +11888,7 @@
         <v>549</v>
       </c>
       <c r="M40" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N40" t="s">
         <v>552</v>
@@ -11932,7 +11932,7 @@
         <v>549</v>
       </c>
       <c r="M41" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N41" t="s">
         <v>552</v>
@@ -11976,7 +11976,7 @@
         <v>549</v>
       </c>
       <c r="M42" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N42" t="s">
         <v>552</v>
@@ -12020,7 +12020,7 @@
         <v>549</v>
       </c>
       <c r="M43" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N43" t="s">
         <v>552</v>
@@ -12064,7 +12064,7 @@
         <v>549</v>
       </c>
       <c r="M44" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N44" t="s">
         <v>552</v>
@@ -12108,7 +12108,7 @@
         <v>549</v>
       </c>
       <c r="M45" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N45" t="s">
         <v>552</v>
@@ -12152,7 +12152,7 @@
         <v>549</v>
       </c>
       <c r="M46" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N46" t="s">
         <v>552</v>
@@ -12196,7 +12196,7 @@
         <v>549</v>
       </c>
       <c r="M47" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N47" t="s">
         <v>552</v>
@@ -12240,7 +12240,7 @@
         <v>548</v>
       </c>
       <c r="M48" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N48" t="s">
         <v>552</v>
@@ -12284,7 +12284,7 @@
         <v>548</v>
       </c>
       <c r="M49" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N49" t="s">
         <v>552</v>
@@ -12328,7 +12328,7 @@
         <v>549</v>
       </c>
       <c r="M50" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N50" t="s">
         <v>552</v>
@@ -12372,7 +12372,7 @@
         <v>549</v>
       </c>
       <c r="M51" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N51" t="s">
         <v>552</v>
@@ -12416,7 +12416,7 @@
         <v>549</v>
       </c>
       <c r="M52" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N52" t="s">
         <v>552</v>
@@ -12460,7 +12460,7 @@
         <v>549</v>
       </c>
       <c r="M53" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N53" t="s">
         <v>552</v>
@@ -12504,7 +12504,7 @@
         <v>548</v>
       </c>
       <c r="M54" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N54" t="s">
         <v>552</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (27/07/2026 14:23)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10351,7 +10351,7 @@
         <v>546</v>
       </c>
       <c r="M5" s="1">
-        <v>46238</v>
+        <v>46240</v>
       </c>
       <c r="N5" t="s">
         <v>552</v>
@@ -10483,7 +10483,7 @@
         <v>549</v>
       </c>
       <c r="M8" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N8" t="s">
         <v>552</v>
@@ -10571,7 +10571,7 @@
         <v>549</v>
       </c>
       <c r="M10" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N10" t="s">
         <v>552</v>
@@ -10615,7 +10615,7 @@
         <v>549</v>
       </c>
       <c r="M11" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N11" t="s">
         <v>552</v>
@@ -10788,7 +10788,7 @@
         <v>548</v>
       </c>
       <c r="M15" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N15" t="s">
         <v>552</v>
@@ -10832,7 +10832,7 @@
         <v>549</v>
       </c>
       <c r="M16" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N16" t="s">
         <v>552</v>
@@ -10876,7 +10876,7 @@
         <v>548</v>
       </c>
       <c r="M17" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N17" t="s">
         <v>552</v>
@@ -10920,7 +10920,7 @@
         <v>549</v>
       </c>
       <c r="M18" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N18" t="s">
         <v>552</v>
@@ -10964,7 +10964,7 @@
         <v>549</v>
       </c>
       <c r="M19" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N19" t="s">
         <v>552</v>
@@ -11008,7 +11008,7 @@
         <v>549</v>
       </c>
       <c r="M20" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N20" t="s">
         <v>552</v>
@@ -11052,7 +11052,7 @@
         <v>549</v>
       </c>
       <c r="M21" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N21" t="s">
         <v>552</v>
@@ -11228,7 +11228,7 @@
         <v>548</v>
       </c>
       <c r="M25" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N25" t="s">
         <v>552</v>
@@ -11316,7 +11316,7 @@
         <v>549</v>
       </c>
       <c r="M27" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N27" t="s">
         <v>552</v>
@@ -11360,7 +11360,7 @@
         <v>549</v>
       </c>
       <c r="M28" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N28" t="s">
         <v>552</v>
@@ -11404,7 +11404,7 @@
         <v>549</v>
       </c>
       <c r="M29" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N29" t="s">
         <v>552</v>
@@ -11448,7 +11448,7 @@
         <v>549</v>
       </c>
       <c r="M30" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N30" t="s">
         <v>552</v>
@@ -11492,7 +11492,7 @@
         <v>548</v>
       </c>
       <c r="M31" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N31" t="s">
         <v>552</v>
@@ -11536,7 +11536,7 @@
         <v>548</v>
       </c>
       <c r="M32" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N32" t="s">
         <v>552</v>
@@ -11580,7 +11580,7 @@
         <v>548</v>
       </c>
       <c r="M33" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N33" t="s">
         <v>552</v>
@@ -11624,7 +11624,7 @@
         <v>549</v>
       </c>
       <c r="M34" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N34" t="s">
         <v>552</v>
@@ -11668,7 +11668,7 @@
         <v>548</v>
       </c>
       <c r="M35" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N35" t="s">
         <v>552</v>
@@ -11712,7 +11712,7 @@
         <v>549</v>
       </c>
       <c r="M36" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N36" t="s">
         <v>552</v>
@@ -11756,7 +11756,7 @@
         <v>549</v>
       </c>
       <c r="M37" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N37" t="s">
         <v>552</v>
@@ -11800,7 +11800,7 @@
         <v>549</v>
       </c>
       <c r="M38" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N38" t="s">
         <v>552</v>
@@ -11844,7 +11844,7 @@
         <v>548</v>
       </c>
       <c r="M39" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N39" t="s">
         <v>552</v>
@@ -11888,7 +11888,7 @@
         <v>549</v>
       </c>
       <c r="M40" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N40" t="s">
         <v>552</v>
@@ -11932,7 +11932,7 @@
         <v>549</v>
       </c>
       <c r="M41" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N41" t="s">
         <v>552</v>
@@ -11976,7 +11976,7 @@
         <v>549</v>
       </c>
       <c r="M42" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N42" t="s">
         <v>552</v>
@@ -12020,7 +12020,7 @@
         <v>549</v>
       </c>
       <c r="M43" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N43" t="s">
         <v>552</v>
@@ -12064,7 +12064,7 @@
         <v>549</v>
       </c>
       <c r="M44" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N44" t="s">
         <v>552</v>
@@ -12108,7 +12108,7 @@
         <v>549</v>
       </c>
       <c r="M45" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N45" t="s">
         <v>552</v>
@@ -12152,7 +12152,7 @@
         <v>549</v>
       </c>
       <c r="M46" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N46" t="s">
         <v>552</v>
@@ -12196,7 +12196,7 @@
         <v>549</v>
       </c>
       <c r="M47" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N47" t="s">
         <v>552</v>
@@ -12240,7 +12240,7 @@
         <v>548</v>
       </c>
       <c r="M48" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N48" t="s">
         <v>552</v>
@@ -12284,7 +12284,7 @@
         <v>548</v>
       </c>
       <c r="M49" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N49" t="s">
         <v>552</v>
@@ -12328,7 +12328,7 @@
         <v>549</v>
       </c>
       <c r="M50" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N50" t="s">
         <v>552</v>
@@ -12372,7 +12372,7 @@
         <v>549</v>
       </c>
       <c r="M51" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N51" t="s">
         <v>552</v>
@@ -12416,7 +12416,7 @@
         <v>549</v>
       </c>
       <c r="M52" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N52" t="s">
         <v>552</v>
@@ -12460,7 +12460,7 @@
         <v>549</v>
       </c>
       <c r="M53" s="1">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="N53" t="s">
         <v>552</v>
@@ -12504,7 +12504,7 @@
         <v>548</v>
       </c>
       <c r="M54" s="1">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="N54" t="s">
         <v>552</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (28/07/2026 05:08)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10351,7 +10351,7 @@
         <v>546</v>
       </c>
       <c r="M5" s="1">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="N5" t="s">
         <v>552</v>
@@ -10483,7 +10483,7 @@
         <v>549</v>
       </c>
       <c r="M8" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N8" t="s">
         <v>552</v>
@@ -10571,7 +10571,7 @@
         <v>549</v>
       </c>
       <c r="M10" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N10" t="s">
         <v>552</v>
@@ -10615,7 +10615,7 @@
         <v>549</v>
       </c>
       <c r="M11" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N11" t="s">
         <v>552</v>
@@ -10788,7 +10788,7 @@
         <v>548</v>
       </c>
       <c r="M15" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N15" t="s">
         <v>552</v>
@@ -10832,7 +10832,7 @@
         <v>549</v>
       </c>
       <c r="M16" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N16" t="s">
         <v>552</v>
@@ -10876,7 +10876,7 @@
         <v>548</v>
       </c>
       <c r="M17" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N17" t="s">
         <v>552</v>
@@ -10920,7 +10920,7 @@
         <v>549</v>
       </c>
       <c r="M18" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N18" t="s">
         <v>552</v>
@@ -10964,7 +10964,7 @@
         <v>549</v>
       </c>
       <c r="M19" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N19" t="s">
         <v>552</v>
@@ -11008,7 +11008,7 @@
         <v>549</v>
       </c>
       <c r="M20" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N20" t="s">
         <v>552</v>
@@ -11052,7 +11052,7 @@
         <v>549</v>
       </c>
       <c r="M21" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N21" t="s">
         <v>552</v>
@@ -11228,7 +11228,7 @@
         <v>548</v>
       </c>
       <c r="M25" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N25" t="s">
         <v>552</v>
@@ -11316,7 +11316,7 @@
         <v>549</v>
       </c>
       <c r="M27" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N27" t="s">
         <v>552</v>
@@ -11360,7 +11360,7 @@
         <v>549</v>
       </c>
       <c r="M28" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N28" t="s">
         <v>552</v>
@@ -11404,7 +11404,7 @@
         <v>549</v>
       </c>
       <c r="M29" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N29" t="s">
         <v>552</v>
@@ -11448,7 +11448,7 @@
         <v>549</v>
       </c>
       <c r="M30" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N30" t="s">
         <v>552</v>
@@ -11492,7 +11492,7 @@
         <v>548</v>
       </c>
       <c r="M31" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N31" t="s">
         <v>552</v>
@@ -11536,7 +11536,7 @@
         <v>548</v>
       </c>
       <c r="M32" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N32" t="s">
         <v>552</v>
@@ -11580,7 +11580,7 @@
         <v>548</v>
       </c>
       <c r="M33" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N33" t="s">
         <v>552</v>
@@ -11624,7 +11624,7 @@
         <v>549</v>
       </c>
       <c r="M34" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N34" t="s">
         <v>552</v>
@@ -11668,7 +11668,7 @@
         <v>548</v>
       </c>
       <c r="M35" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N35" t="s">
         <v>552</v>
@@ -11712,7 +11712,7 @@
         <v>549</v>
       </c>
       <c r="M36" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N36" t="s">
         <v>552</v>
@@ -11756,7 +11756,7 @@
         <v>549</v>
       </c>
       <c r="M37" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N37" t="s">
         <v>552</v>
@@ -11800,7 +11800,7 @@
         <v>549</v>
       </c>
       <c r="M38" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N38" t="s">
         <v>552</v>
@@ -11844,7 +11844,7 @@
         <v>548</v>
       </c>
       <c r="M39" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N39" t="s">
         <v>552</v>
@@ -11888,7 +11888,7 @@
         <v>549</v>
       </c>
       <c r="M40" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N40" t="s">
         <v>552</v>
@@ -11932,7 +11932,7 @@
         <v>549</v>
       </c>
       <c r="M41" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N41" t="s">
         <v>552</v>
@@ -11976,7 +11976,7 @@
         <v>549</v>
       </c>
       <c r="M42" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N42" t="s">
         <v>552</v>
@@ -12020,7 +12020,7 @@
         <v>549</v>
       </c>
       <c r="M43" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N43" t="s">
         <v>552</v>
@@ -12064,7 +12064,7 @@
         <v>549</v>
       </c>
       <c r="M44" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N44" t="s">
         <v>552</v>
@@ -12108,7 +12108,7 @@
         <v>549</v>
       </c>
       <c r="M45" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N45" t="s">
         <v>552</v>
@@ -12152,7 +12152,7 @@
         <v>549</v>
       </c>
       <c r="M46" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N46" t="s">
         <v>552</v>
@@ -12196,7 +12196,7 @@
         <v>549</v>
       </c>
       <c r="M47" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N47" t="s">
         <v>552</v>
@@ -12240,7 +12240,7 @@
         <v>548</v>
       </c>
       <c r="M48" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N48" t="s">
         <v>552</v>
@@ -12284,7 +12284,7 @@
         <v>548</v>
       </c>
       <c r="M49" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N49" t="s">
         <v>552</v>
@@ -12328,7 +12328,7 @@
         <v>549</v>
       </c>
       <c r="M50" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N50" t="s">
         <v>552</v>
@@ -12372,7 +12372,7 @@
         <v>549</v>
       </c>
       <c r="M51" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N51" t="s">
         <v>552</v>
@@ -12416,7 +12416,7 @@
         <v>549</v>
       </c>
       <c r="M52" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N52" t="s">
         <v>552</v>
@@ -12460,7 +12460,7 @@
         <v>549</v>
       </c>
       <c r="M53" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N53" t="s">
         <v>552</v>
@@ -12504,7 +12504,7 @@
         <v>548</v>
       </c>
       <c r="M54" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N54" t="s">
         <v>552</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (29/07/2026 13:13)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10351,7 +10351,7 @@
         <v>546</v>
       </c>
       <c r="M5" s="1">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="N5" t="s">
         <v>552</v>
@@ -10483,7 +10483,7 @@
         <v>549</v>
       </c>
       <c r="M8" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N8" t="s">
         <v>552</v>
@@ -10571,7 +10571,7 @@
         <v>549</v>
       </c>
       <c r="M10" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N10" t="s">
         <v>552</v>
@@ -10615,7 +10615,7 @@
         <v>549</v>
       </c>
       <c r="M11" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N11" t="s">
         <v>552</v>
@@ -10788,7 +10788,7 @@
         <v>548</v>
       </c>
       <c r="M15" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N15" t="s">
         <v>552</v>
@@ -10832,7 +10832,7 @@
         <v>549</v>
       </c>
       <c r="M16" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N16" t="s">
         <v>552</v>
@@ -10876,7 +10876,7 @@
         <v>548</v>
       </c>
       <c r="M17" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N17" t="s">
         <v>552</v>
@@ -10920,7 +10920,7 @@
         <v>549</v>
       </c>
       <c r="M18" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N18" t="s">
         <v>552</v>
@@ -10964,7 +10964,7 @@
         <v>549</v>
       </c>
       <c r="M19" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N19" t="s">
         <v>552</v>
@@ -11008,7 +11008,7 @@
         <v>549</v>
       </c>
       <c r="M20" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N20" t="s">
         <v>552</v>
@@ -11052,7 +11052,7 @@
         <v>549</v>
       </c>
       <c r="M21" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N21" t="s">
         <v>552</v>
@@ -11228,7 +11228,7 @@
         <v>548</v>
       </c>
       <c r="M25" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N25" t="s">
         <v>552</v>
@@ -11316,7 +11316,7 @@
         <v>549</v>
       </c>
       <c r="M27" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N27" t="s">
         <v>552</v>
@@ -11360,7 +11360,7 @@
         <v>549</v>
       </c>
       <c r="M28" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N28" t="s">
         <v>552</v>
@@ -11404,7 +11404,7 @@
         <v>549</v>
       </c>
       <c r="M29" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N29" t="s">
         <v>552</v>
@@ -11448,7 +11448,7 @@
         <v>549</v>
       </c>
       <c r="M30" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N30" t="s">
         <v>552</v>
@@ -11492,7 +11492,7 @@
         <v>548</v>
       </c>
       <c r="M31" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N31" t="s">
         <v>552</v>
@@ -11536,7 +11536,7 @@
         <v>548</v>
       </c>
       <c r="M32" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N32" t="s">
         <v>552</v>
@@ -11580,7 +11580,7 @@
         <v>548</v>
       </c>
       <c r="M33" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N33" t="s">
         <v>552</v>
@@ -11624,7 +11624,7 @@
         <v>549</v>
       </c>
       <c r="M34" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N34" t="s">
         <v>552</v>
@@ -11668,7 +11668,7 @@
         <v>548</v>
       </c>
       <c r="M35" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N35" t="s">
         <v>552</v>
@@ -11712,7 +11712,7 @@
         <v>549</v>
       </c>
       <c r="M36" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N36" t="s">
         <v>552</v>
@@ -11756,7 +11756,7 @@
         <v>549</v>
       </c>
       <c r="M37" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N37" t="s">
         <v>552</v>
@@ -11800,7 +11800,7 @@
         <v>549</v>
       </c>
       <c r="M38" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N38" t="s">
         <v>552</v>
@@ -11844,7 +11844,7 @@
         <v>548</v>
       </c>
       <c r="M39" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N39" t="s">
         <v>552</v>
@@ -11888,7 +11888,7 @@
         <v>549</v>
       </c>
       <c r="M40" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N40" t="s">
         <v>552</v>
@@ -11932,7 +11932,7 @@
         <v>549</v>
       </c>
       <c r="M41" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N41" t="s">
         <v>552</v>
@@ -11976,7 +11976,7 @@
         <v>549</v>
       </c>
       <c r="M42" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N42" t="s">
         <v>552</v>
@@ -12020,7 +12020,7 @@
         <v>549</v>
       </c>
       <c r="M43" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N43" t="s">
         <v>552</v>
@@ -12064,7 +12064,7 @@
         <v>549</v>
       </c>
       <c r="M44" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N44" t="s">
         <v>552</v>
@@ -12108,7 +12108,7 @@
         <v>549</v>
       </c>
       <c r="M45" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N45" t="s">
         <v>552</v>
@@ -12152,7 +12152,7 @@
         <v>549</v>
       </c>
       <c r="M46" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N46" t="s">
         <v>552</v>
@@ -12196,7 +12196,7 @@
         <v>549</v>
       </c>
       <c r="M47" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N47" t="s">
         <v>552</v>
@@ -12240,7 +12240,7 @@
         <v>548</v>
       </c>
       <c r="M48" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N48" t="s">
         <v>552</v>
@@ -12284,7 +12284,7 @@
         <v>548</v>
       </c>
       <c r="M49" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N49" t="s">
         <v>552</v>
@@ -12328,7 +12328,7 @@
         <v>549</v>
       </c>
       <c r="M50" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N50" t="s">
         <v>552</v>
@@ -12372,7 +12372,7 @@
         <v>549</v>
       </c>
       <c r="M51" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N51" t="s">
         <v>552</v>
@@ -12416,7 +12416,7 @@
         <v>549</v>
       </c>
       <c r="M52" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N52" t="s">
         <v>552</v>
@@ -12460,7 +12460,7 @@
         <v>549</v>
       </c>
       <c r="M53" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N53" t="s">
         <v>552</v>
@@ -12504,7 +12504,7 @@
         <v>548</v>
       </c>
       <c r="M54" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N54" t="s">
         <v>552</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (30/07/2026 13:20)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2492" uniqueCount="570">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1394,6 +1394,24 @@
     <t>LST202001U8</t>
   </si>
   <si>
+    <t>LST203002U8</t>
+  </si>
+  <si>
+    <t>LST203005U8</t>
+  </si>
+  <si>
+    <t>LST205005U8</t>
+  </si>
+  <si>
+    <t>LST208014U8</t>
+  </si>
+  <si>
+    <t>LST209004U8</t>
+  </si>
+  <si>
+    <t>LST209005U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1532,6 +1550,21 @@
     <t>2611137-7</t>
   </si>
   <si>
+    <t>SK208-157A0</t>
+  </si>
+  <si>
+    <t>2662018-5</t>
+  </si>
+  <si>
+    <t>5950028-10</t>
+  </si>
+  <si>
+    <t>1214134-1</t>
+  </si>
+  <si>
+    <t>2643057-1</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1652,6 +1685,21 @@
     <t>CAP MAIN LAND</t>
   </si>
   <si>
+    <t>AIR COND SYSTEM INST KIT</t>
+  </si>
+  <si>
+    <t>TUBE ASSY-LONG</t>
+  </si>
+  <si>
+    <t>Vant, Breather</t>
+  </si>
+  <si>
+    <t>BELLCRANK ASSY</t>
+  </si>
+  <si>
+    <t>BOOT N G STEER</t>
+  </si>
+  <si>
     <t>Empenho Solicitado</t>
   </si>
   <si>
@@ -1661,10 +1709,13 @@
     <t>Selecionada em Plano</t>
   </si>
   <si>
+    <t>Validada</t>
+  </si>
+  <si>
     <t>Análise do Pedido</t>
   </si>
   <si>
-    <t>Validada</t>
+    <t>Em Discrepância</t>
   </si>
   <si>
     <t>EMPENHADO</t>
@@ -10125,7 +10176,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q54"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10207,7 +10258,7 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J2" t="s">
         <v>387</v>
@@ -10219,7 +10270,7 @@
         <v>387</v>
       </c>
       <c r="M2" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N2" t="s">
         <v>395</v>
@@ -10251,7 +10302,7 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J3" t="s">
         <v>387</v>
@@ -10263,7 +10314,7 @@
         <v>387</v>
       </c>
       <c r="M3" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N3" t="s">
         <v>395</v>
@@ -10280,7 +10331,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10295,7 +10346,7 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J4" t="s">
         <v>387</v>
@@ -10307,7 +10358,7 @@
         <v>387</v>
       </c>
       <c r="M4" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N4" t="s">
         <v>395</v>
@@ -10324,10 +10375,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="E5" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10339,22 +10390,22 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>546</v>
+        <v>562</v>
       </c>
       <c r="J5" t="s">
-        <v>546</v>
+        <v>562</v>
       </c>
       <c r="K5" t="s">
-        <v>546</v>
+        <v>562</v>
       </c>
       <c r="L5" t="s">
-        <v>546</v>
+        <v>562</v>
       </c>
       <c r="M5" s="1">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="N5" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -10383,7 +10434,7 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J6" t="s">
         <v>387</v>
@@ -10395,7 +10446,7 @@
         <v>387</v>
       </c>
       <c r="M6" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N6" t="s">
         <v>395</v>
@@ -10427,7 +10478,7 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J7" t="s">
         <v>387</v>
@@ -10439,7 +10490,7 @@
         <v>387</v>
       </c>
       <c r="M7" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N7" t="s">
         <v>395</v>
@@ -10471,22 +10522,22 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J8" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K8" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L8" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M8" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N8" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10500,7 +10551,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10515,7 +10566,7 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J9" t="s">
         <v>387</v>
@@ -10527,7 +10578,7 @@
         <v>387</v>
       </c>
       <c r="M9" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N9" t="s">
         <v>395</v>
@@ -10544,10 +10595,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="E10" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10562,19 +10613,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K10" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L10" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M10" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N10" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10588,7 +10639,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10606,19 +10657,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K11" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L11" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M11" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N11" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10632,10 +10683,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="E12" t="s">
-        <v>507</v>
+        <v>518</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -10700,7 +10751,7 @@
         <v>380</v>
       </c>
       <c r="M13" t="s">
-        <v>551</v>
+        <v>568</v>
       </c>
       <c r="N13" t="s">
         <v>395</v>
@@ -10717,10 +10768,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="E14" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -10732,7 +10783,7 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J14" t="s">
         <v>387</v>
@@ -10744,7 +10795,7 @@
         <v>387</v>
       </c>
       <c r="M14" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N14" t="s">
         <v>395</v>
@@ -10761,10 +10812,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="E15" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -10776,22 +10827,22 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J15" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K15" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L15" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N15" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10805,10 +10856,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="E16" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -10823,19 +10874,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K16" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L16" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M16" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N16" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10849,10 +10900,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="E17" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -10864,22 +10915,22 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J17" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K17" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L17" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N17" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10893,10 +10944,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="E18" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -10911,19 +10962,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K18" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L18" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M18" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N18" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10937,10 +10988,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="E19" t="s">
-        <v>513</v>
+        <v>524</v>
       </c>
       <c r="F19">
         <v>4</v>
@@ -10955,19 +11006,19 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K19" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L19" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M19" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N19" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -10981,10 +11032,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="E20" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -10999,19 +11050,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K20" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L20" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M20" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N20" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11025,10 +11076,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="E21" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11043,19 +11094,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K21" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L21" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M21" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N21" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11069,10 +11120,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="E22" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11084,7 +11135,7 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J22" t="s">
         <v>387</v>
@@ -11096,7 +11147,7 @@
         <v>387</v>
       </c>
       <c r="M22" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N22" t="s">
         <v>395</v>
@@ -11113,10 +11164,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="E23" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11128,7 +11179,7 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J23" t="s">
         <v>387</v>
@@ -11140,7 +11191,7 @@
         <v>387</v>
       </c>
       <c r="M23" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N23" t="s">
         <v>395</v>
@@ -11157,7 +11208,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11172,7 +11223,7 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J24" t="s">
         <v>387</v>
@@ -11184,7 +11235,7 @@
         <v>387</v>
       </c>
       <c r="M24" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N24" t="s">
         <v>395</v>
@@ -11201,10 +11252,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="E25" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11216,22 +11267,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="J25" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K25" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L25" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M25" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N25" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11245,10 +11296,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="E26" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11260,7 +11311,7 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="J26" t="s">
         <v>387</v>
@@ -11272,7 +11323,7 @@
         <v>387</v>
       </c>
       <c r="M26" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="N26" t="s">
         <v>395</v>
@@ -11289,10 +11340,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="E27" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11304,22 +11355,22 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J27" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K27" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L27" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M27" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N27" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11333,10 +11384,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="E28" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11351,19 +11402,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K28" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L28" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M28" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N28" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11377,10 +11428,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="E29" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11392,22 +11443,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J29" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K29" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L29" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M29" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N29" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11421,10 +11472,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="E30" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11439,19 +11490,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K30" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L30" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M30" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N30" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11465,10 +11516,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="E31" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11480,22 +11531,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>548</v>
+        <v>566</v>
       </c>
       <c r="J31" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K31" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L31" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M31" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N31" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11509,10 +11560,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="E32" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11524,22 +11575,22 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J32" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K32" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L32" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N32" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11553,10 +11604,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="E33" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11568,22 +11619,22 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J33" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K33" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L33" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N33" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11597,10 +11648,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="E34" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11612,22 +11663,22 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J34" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K34" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L34" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M34" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N34" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11641,10 +11692,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="E35" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11656,22 +11707,22 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J35" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K35" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L35" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N35" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11685,10 +11736,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="E36" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -11700,22 +11751,22 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J36" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K36" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L36" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M36" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N36" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11729,10 +11780,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="E37" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -11744,22 +11795,22 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J37" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K37" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L37" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M37" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N37" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11773,10 +11824,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="E38" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -11788,22 +11839,22 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J38" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K38" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L38" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M38" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N38" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11817,10 +11868,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="E39" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -11832,22 +11883,22 @@
         <v>312.36</v>
       </c>
       <c r="I39" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="J39" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K39" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L39" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N39" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11861,10 +11912,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="E40" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -11876,22 +11927,22 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J40" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K40" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L40" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M40" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N40" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11905,10 +11956,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="E41" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -11923,19 +11974,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K41" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L41" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M41" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N41" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11964,22 +12015,22 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J42" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K42" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L42" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M42" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N42" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -11993,10 +12044,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E43" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -12008,22 +12059,22 @@
         <v>5000</v>
       </c>
       <c r="I43" t="s">
-        <v>548</v>
+        <v>566</v>
       </c>
       <c r="J43" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K43" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L43" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M43" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N43" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12037,7 +12088,7 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
@@ -12055,19 +12106,19 @@
         <v>382</v>
       </c>
       <c r="J44" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K44" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L44" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M44" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N44" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12081,10 +12132,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="E45" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12099,19 +12150,19 @@
         <v>382</v>
       </c>
       <c r="J45" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K45" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L45" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M45" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N45" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12125,10 +12176,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="E46" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12140,22 +12191,22 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J46" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K46" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L46" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M46" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N46" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12169,10 +12220,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="E47" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12184,22 +12235,22 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="J47" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K47" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L47" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M47" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N47" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12213,10 +12264,10 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="E48" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -12228,22 +12279,22 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>548</v>
+        <v>566</v>
       </c>
       <c r="J48" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K48" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L48" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M48" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N48" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12257,10 +12308,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="E49" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12272,22 +12323,22 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="J49" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K49" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L49" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M49" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N49" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12301,10 +12352,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="E50" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12316,22 +12367,22 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>382</v>
+        <v>565</v>
       </c>
       <c r="J50" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K50" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L50" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M50" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N50" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12345,10 +12396,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="E51" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12363,19 +12414,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K51" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L51" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M51" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N51" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12389,10 +12440,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E52" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12407,19 +12458,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K52" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L52" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M52" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N52" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12433,10 +12484,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="E53" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12451,19 +12502,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="K53" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="L53" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
       <c r="M53" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N53" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12477,10 +12528,10 @@
         <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="E54" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
       <c r="F54">
         <v>4</v>
@@ -12492,22 +12543,268 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>548</v>
+        <v>566</v>
       </c>
       <c r="J54" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="K54" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="L54" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="M54" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N54" t="s">
-        <v>552</v>
+        <v>569</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14">
+      <c r="A55" t="s">
+        <v>459</v>
+      </c>
+      <c r="B55" t="s">
+        <v>172</v>
+      </c>
+      <c r="C55" t="s">
+        <v>173</v>
+      </c>
+      <c r="D55" t="s">
+        <v>511</v>
+      </c>
+      <c r="E55" t="s">
+        <v>556</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55">
+        <v>78000</v>
+      </c>
+      <c r="H55">
+        <v>78000</v>
+      </c>
+      <c r="I55" t="s">
+        <v>382</v>
+      </c>
+      <c r="K55" t="s">
+        <v>382</v>
+      </c>
+      <c r="L55" t="s">
+        <v>382</v>
+      </c>
+      <c r="M55" s="1">
+        <v>46313</v>
+      </c>
+      <c r="N55" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
+      <c r="A56" t="s">
+        <v>460</v>
+      </c>
+      <c r="B56" t="s">
+        <v>172</v>
+      </c>
+      <c r="C56" t="s">
+        <v>173</v>
+      </c>
+      <c r="D56" t="s">
+        <v>512</v>
+      </c>
+      <c r="E56" t="s">
+        <v>557</v>
+      </c>
+      <c r="F56">
+        <v>1</v>
+      </c>
+      <c r="G56">
+        <v>3576.55</v>
+      </c>
+      <c r="H56">
+        <v>3576.55</v>
+      </c>
+      <c r="I56" t="s">
+        <v>565</v>
+      </c>
+      <c r="K56" t="s">
+        <v>565</v>
+      </c>
+      <c r="L56" t="s">
+        <v>565</v>
+      </c>
+      <c r="M56" s="1">
+        <v>46323</v>
+      </c>
+      <c r="N56" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14">
+      <c r="A57" t="s">
+        <v>461</v>
+      </c>
+      <c r="B57" t="s">
+        <v>172</v>
+      </c>
+      <c r="C57" t="s">
+        <v>173</v>
+      </c>
+      <c r="D57" t="s">
+        <v>513</v>
+      </c>
+      <c r="E57" t="s">
+        <v>558</v>
+      </c>
+      <c r="F57">
+        <v>1</v>
+      </c>
+      <c r="G57">
+        <v>908.11</v>
+      </c>
+      <c r="H57">
+        <v>908.11</v>
+      </c>
+      <c r="I57" t="s">
+        <v>565</v>
+      </c>
+      <c r="K57" t="s">
+        <v>565</v>
+      </c>
+      <c r="L57" t="s">
+        <v>565</v>
+      </c>
+      <c r="M57" s="1">
+        <v>46323</v>
+      </c>
+      <c r="N57" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
+      <c r="A58" t="s">
+        <v>462</v>
+      </c>
+      <c r="B58" t="s">
+        <v>172</v>
+      </c>
+      <c r="C58" t="s">
+        <v>173</v>
+      </c>
+      <c r="D58" t="s">
+        <v>514</v>
+      </c>
+      <c r="E58" t="s">
+        <v>559</v>
+      </c>
+      <c r="F58">
+        <v>4</v>
+      </c>
+      <c r="G58">
+        <v>375.2</v>
+      </c>
+      <c r="H58">
+        <v>1500.8</v>
+      </c>
+      <c r="I58" t="s">
+        <v>565</v>
+      </c>
+      <c r="K58" t="s">
+        <v>565</v>
+      </c>
+      <c r="L58" t="s">
+        <v>565</v>
+      </c>
+      <c r="M58" s="1">
+        <v>46323</v>
+      </c>
+      <c r="N58" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14">
+      <c r="A59" t="s">
+        <v>463</v>
+      </c>
+      <c r="B59" t="s">
+        <v>172</v>
+      </c>
+      <c r="C59" t="s">
+        <v>173</v>
+      </c>
+      <c r="D59" t="s">
+        <v>229</v>
+      </c>
+      <c r="E59" t="s">
+        <v>331</v>
+      </c>
+      <c r="F59">
+        <v>2</v>
+      </c>
+      <c r="G59">
+        <v>435</v>
+      </c>
+      <c r="H59">
+        <v>870</v>
+      </c>
+      <c r="I59" t="s">
+        <v>565</v>
+      </c>
+      <c r="K59" t="s">
+        <v>565</v>
+      </c>
+      <c r="L59" t="s">
+        <v>565</v>
+      </c>
+      <c r="M59" s="1">
+        <v>46323</v>
+      </c>
+      <c r="N59" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
+      <c r="A60" t="s">
+        <v>464</v>
+      </c>
+      <c r="B60" t="s">
+        <v>172</v>
+      </c>
+      <c r="C60" t="s">
+        <v>173</v>
+      </c>
+      <c r="D60" t="s">
+        <v>515</v>
+      </c>
+      <c r="E60" t="s">
+        <v>560</v>
+      </c>
+      <c r="F60">
+        <v>3</v>
+      </c>
+      <c r="G60">
+        <v>459.84</v>
+      </c>
+      <c r="H60">
+        <v>1379.52</v>
+      </c>
+      <c r="I60" t="s">
+        <v>565</v>
+      </c>
+      <c r="K60" t="s">
+        <v>565</v>
+      </c>
+      <c r="L60" t="s">
+        <v>565</v>
+      </c>
+      <c r="M60" s="1">
+        <v>46323</v>
+      </c>
+      <c r="N60" t="s">
+        <v>569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (31/07/2026 05:12)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10402,7 +10402,7 @@
         <v>562</v>
       </c>
       <c r="M5" s="1">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="N5" t="s">
         <v>569</v>
@@ -10534,7 +10534,7 @@
         <v>564</v>
       </c>
       <c r="M8" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N8" t="s">
         <v>569</v>
@@ -10622,7 +10622,7 @@
         <v>564</v>
       </c>
       <c r="M10" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N10" t="s">
         <v>569</v>
@@ -10666,7 +10666,7 @@
         <v>564</v>
       </c>
       <c r="M11" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N11" t="s">
         <v>569</v>
@@ -10839,7 +10839,7 @@
         <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N15" t="s">
         <v>569</v>
@@ -10883,7 +10883,7 @@
         <v>564</v>
       </c>
       <c r="M16" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N16" t="s">
         <v>569</v>
@@ -10927,7 +10927,7 @@
         <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N17" t="s">
         <v>569</v>
@@ -10971,7 +10971,7 @@
         <v>564</v>
       </c>
       <c r="M18" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N18" t="s">
         <v>569</v>
@@ -11015,7 +11015,7 @@
         <v>564</v>
       </c>
       <c r="M19" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N19" t="s">
         <v>569</v>
@@ -11059,7 +11059,7 @@
         <v>564</v>
       </c>
       <c r="M20" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N20" t="s">
         <v>569</v>
@@ -11103,7 +11103,7 @@
         <v>564</v>
       </c>
       <c r="M21" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N21" t="s">
         <v>569</v>
@@ -11279,7 +11279,7 @@
         <v>565</v>
       </c>
       <c r="M25" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N25" t="s">
         <v>569</v>
@@ -11367,7 +11367,7 @@
         <v>564</v>
       </c>
       <c r="M27" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N27" t="s">
         <v>569</v>
@@ -11411,7 +11411,7 @@
         <v>564</v>
       </c>
       <c r="M28" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N28" t="s">
         <v>569</v>
@@ -11455,7 +11455,7 @@
         <v>564</v>
       </c>
       <c r="M29" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N29" t="s">
         <v>569</v>
@@ -11499,7 +11499,7 @@
         <v>564</v>
       </c>
       <c r="M30" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N30" t="s">
         <v>569</v>
@@ -11543,7 +11543,7 @@
         <v>565</v>
       </c>
       <c r="M31" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N31" t="s">
         <v>569</v>
@@ -11587,7 +11587,7 @@
         <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N32" t="s">
         <v>569</v>
@@ -11631,7 +11631,7 @@
         <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N33" t="s">
         <v>569</v>
@@ -11675,7 +11675,7 @@
         <v>564</v>
       </c>
       <c r="M34" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N34" t="s">
         <v>569</v>
@@ -11719,7 +11719,7 @@
         <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N35" t="s">
         <v>569</v>
@@ -11763,7 +11763,7 @@
         <v>564</v>
       </c>
       <c r="M36" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N36" t="s">
         <v>569</v>
@@ -11807,7 +11807,7 @@
         <v>564</v>
       </c>
       <c r="M37" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N37" t="s">
         <v>569</v>
@@ -11851,7 +11851,7 @@
         <v>564</v>
       </c>
       <c r="M38" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N38" t="s">
         <v>569</v>
@@ -11895,7 +11895,7 @@
         <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N39" t="s">
         <v>569</v>
@@ -11939,7 +11939,7 @@
         <v>564</v>
       </c>
       <c r="M40" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N40" t="s">
         <v>569</v>
@@ -11983,7 +11983,7 @@
         <v>564</v>
       </c>
       <c r="M41" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N41" t="s">
         <v>569</v>
@@ -12027,7 +12027,7 @@
         <v>564</v>
       </c>
       <c r="M42" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N42" t="s">
         <v>569</v>
@@ -12071,7 +12071,7 @@
         <v>564</v>
       </c>
       <c r="M43" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N43" t="s">
         <v>569</v>
@@ -12115,7 +12115,7 @@
         <v>564</v>
       </c>
       <c r="M44" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N44" t="s">
         <v>569</v>
@@ -12159,7 +12159,7 @@
         <v>564</v>
       </c>
       <c r="M45" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N45" t="s">
         <v>569</v>
@@ -12203,7 +12203,7 @@
         <v>564</v>
       </c>
       <c r="M46" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N46" t="s">
         <v>569</v>
@@ -12247,7 +12247,7 @@
         <v>564</v>
       </c>
       <c r="M47" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N47" t="s">
         <v>569</v>
@@ -12291,7 +12291,7 @@
         <v>565</v>
       </c>
       <c r="M48" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N48" t="s">
         <v>569</v>
@@ -12335,7 +12335,7 @@
         <v>565</v>
       </c>
       <c r="M49" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N49" t="s">
         <v>569</v>
@@ -12379,7 +12379,7 @@
         <v>564</v>
       </c>
       <c r="M50" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N50" t="s">
         <v>569</v>
@@ -12423,7 +12423,7 @@
         <v>564</v>
       </c>
       <c r="M51" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N51" t="s">
         <v>569</v>
@@ -12467,7 +12467,7 @@
         <v>564</v>
       </c>
       <c r="M52" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N52" t="s">
         <v>569</v>
@@ -12511,7 +12511,7 @@
         <v>564</v>
       </c>
       <c r="M53" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="N53" t="s">
         <v>569</v>
@@ -12555,7 +12555,7 @@
         <v>565</v>
       </c>
       <c r="M54" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N54" t="s">
         <v>569</v>
@@ -12596,7 +12596,7 @@
         <v>382</v>
       </c>
       <c r="M55" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N55" t="s">
         <v>569</v>
@@ -12637,7 +12637,7 @@
         <v>565</v>
       </c>
       <c r="M56" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N56" t="s">
         <v>569</v>
@@ -12678,7 +12678,7 @@
         <v>565</v>
       </c>
       <c r="M57" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N57" t="s">
         <v>569</v>
@@ -12719,7 +12719,7 @@
         <v>565</v>
       </c>
       <c r="M58" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N58" t="s">
         <v>569</v>
@@ -12760,7 +12760,7 @@
         <v>565</v>
       </c>
       <c r="M59" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N59" t="s">
         <v>569</v>
@@ -12801,7 +12801,7 @@
         <v>565</v>
       </c>
       <c r="M60" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="N60" t="s">
         <v>569</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (03/08/2026 14:31)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10402,7 +10402,7 @@
         <v>562</v>
       </c>
       <c r="M5" s="1">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="N5" t="s">
         <v>569</v>
@@ -10534,7 +10534,7 @@
         <v>564</v>
       </c>
       <c r="M8" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N8" t="s">
         <v>569</v>
@@ -10622,7 +10622,7 @@
         <v>564</v>
       </c>
       <c r="M10" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N10" t="s">
         <v>569</v>
@@ -10666,7 +10666,7 @@
         <v>564</v>
       </c>
       <c r="M11" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N11" t="s">
         <v>569</v>
@@ -10839,7 +10839,7 @@
         <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N15" t="s">
         <v>569</v>
@@ -10883,7 +10883,7 @@
         <v>564</v>
       </c>
       <c r="M16" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N16" t="s">
         <v>569</v>
@@ -10927,7 +10927,7 @@
         <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N17" t="s">
         <v>569</v>
@@ -10971,7 +10971,7 @@
         <v>564</v>
       </c>
       <c r="M18" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N18" t="s">
         <v>569</v>
@@ -11015,7 +11015,7 @@
         <v>564</v>
       </c>
       <c r="M19" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N19" t="s">
         <v>569</v>
@@ -11059,7 +11059,7 @@
         <v>564</v>
       </c>
       <c r="M20" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N20" t="s">
         <v>569</v>
@@ -11103,7 +11103,7 @@
         <v>564</v>
       </c>
       <c r="M21" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N21" t="s">
         <v>569</v>
@@ -11279,7 +11279,7 @@
         <v>565</v>
       </c>
       <c r="M25" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N25" t="s">
         <v>569</v>
@@ -11367,7 +11367,7 @@
         <v>564</v>
       </c>
       <c r="M27" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N27" t="s">
         <v>569</v>
@@ -11411,7 +11411,7 @@
         <v>564</v>
       </c>
       <c r="M28" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N28" t="s">
         <v>569</v>
@@ -11455,7 +11455,7 @@
         <v>564</v>
       </c>
       <c r="M29" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N29" t="s">
         <v>569</v>
@@ -11499,7 +11499,7 @@
         <v>564</v>
       </c>
       <c r="M30" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N30" t="s">
         <v>569</v>
@@ -11543,7 +11543,7 @@
         <v>565</v>
       </c>
       <c r="M31" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N31" t="s">
         <v>569</v>
@@ -11587,7 +11587,7 @@
         <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N32" t="s">
         <v>569</v>
@@ -11631,7 +11631,7 @@
         <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N33" t="s">
         <v>569</v>
@@ -11675,7 +11675,7 @@
         <v>564</v>
       </c>
       <c r="M34" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N34" t="s">
         <v>569</v>
@@ -11719,7 +11719,7 @@
         <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N35" t="s">
         <v>569</v>
@@ -11763,7 +11763,7 @@
         <v>564</v>
       </c>
       <c r="M36" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N36" t="s">
         <v>569</v>
@@ -11807,7 +11807,7 @@
         <v>564</v>
       </c>
       <c r="M37" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N37" t="s">
         <v>569</v>
@@ -11851,7 +11851,7 @@
         <v>564</v>
       </c>
       <c r="M38" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N38" t="s">
         <v>569</v>
@@ -11895,7 +11895,7 @@
         <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N39" t="s">
         <v>569</v>
@@ -11939,7 +11939,7 @@
         <v>564</v>
       </c>
       <c r="M40" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N40" t="s">
         <v>569</v>
@@ -11983,7 +11983,7 @@
         <v>564</v>
       </c>
       <c r="M41" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N41" t="s">
         <v>569</v>
@@ -12027,7 +12027,7 @@
         <v>564</v>
       </c>
       <c r="M42" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N42" t="s">
         <v>569</v>
@@ -12071,7 +12071,7 @@
         <v>564</v>
       </c>
       <c r="M43" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N43" t="s">
         <v>569</v>
@@ -12115,7 +12115,7 @@
         <v>564</v>
       </c>
       <c r="M44" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N44" t="s">
         <v>569</v>
@@ -12159,7 +12159,7 @@
         <v>564</v>
       </c>
       <c r="M45" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N45" t="s">
         <v>569</v>
@@ -12203,7 +12203,7 @@
         <v>564</v>
       </c>
       <c r="M46" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N46" t="s">
         <v>569</v>
@@ -12247,7 +12247,7 @@
         <v>564</v>
       </c>
       <c r="M47" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N47" t="s">
         <v>569</v>
@@ -12291,7 +12291,7 @@
         <v>565</v>
       </c>
       <c r="M48" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N48" t="s">
         <v>569</v>
@@ -12335,7 +12335,7 @@
         <v>565</v>
       </c>
       <c r="M49" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N49" t="s">
         <v>569</v>
@@ -12379,7 +12379,7 @@
         <v>564</v>
       </c>
       <c r="M50" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N50" t="s">
         <v>569</v>
@@ -12423,7 +12423,7 @@
         <v>564</v>
       </c>
       <c r="M51" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N51" t="s">
         <v>569</v>
@@ -12467,7 +12467,7 @@
         <v>564</v>
       </c>
       <c r="M52" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N52" t="s">
         <v>569</v>
@@ -12511,7 +12511,7 @@
         <v>564</v>
       </c>
       <c r="M53" s="1">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="N53" t="s">
         <v>569</v>
@@ -12555,7 +12555,7 @@
         <v>565</v>
       </c>
       <c r="M54" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N54" t="s">
         <v>569</v>
@@ -12596,7 +12596,7 @@
         <v>382</v>
       </c>
       <c r="M55" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N55" t="s">
         <v>569</v>
@@ -12637,7 +12637,7 @@
         <v>565</v>
       </c>
       <c r="M56" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N56" t="s">
         <v>569</v>
@@ -12678,7 +12678,7 @@
         <v>565</v>
       </c>
       <c r="M57" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N57" t="s">
         <v>569</v>
@@ -12719,7 +12719,7 @@
         <v>565</v>
       </c>
       <c r="M58" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N58" t="s">
         <v>569</v>
@@ -12760,7 +12760,7 @@
         <v>565</v>
       </c>
       <c r="M59" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N59" t="s">
         <v>569</v>
@@ -12801,7 +12801,7 @@
         <v>565</v>
       </c>
       <c r="M60" s="1">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="N60" t="s">
         <v>569</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (04/08/2026 05:12)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10402,7 +10402,7 @@
         <v>562</v>
       </c>
       <c r="M5" s="1">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="N5" t="s">
         <v>569</v>
@@ -10534,7 +10534,7 @@
         <v>564</v>
       </c>
       <c r="M8" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N8" t="s">
         <v>569</v>
@@ -10622,7 +10622,7 @@
         <v>564</v>
       </c>
       <c r="M10" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N10" t="s">
         <v>569</v>
@@ -10666,7 +10666,7 @@
         <v>564</v>
       </c>
       <c r="M11" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N11" t="s">
         <v>569</v>
@@ -10839,7 +10839,7 @@
         <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N15" t="s">
         <v>569</v>
@@ -10883,7 +10883,7 @@
         <v>564</v>
       </c>
       <c r="M16" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N16" t="s">
         <v>569</v>
@@ -10927,7 +10927,7 @@
         <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N17" t="s">
         <v>569</v>
@@ -10971,7 +10971,7 @@
         <v>564</v>
       </c>
       <c r="M18" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N18" t="s">
         <v>569</v>
@@ -11015,7 +11015,7 @@
         <v>564</v>
       </c>
       <c r="M19" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N19" t="s">
         <v>569</v>
@@ -11059,7 +11059,7 @@
         <v>564</v>
       </c>
       <c r="M20" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N20" t="s">
         <v>569</v>
@@ -11103,7 +11103,7 @@
         <v>564</v>
       </c>
       <c r="M21" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N21" t="s">
         <v>569</v>
@@ -11279,7 +11279,7 @@
         <v>565</v>
       </c>
       <c r="M25" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N25" t="s">
         <v>569</v>
@@ -11367,7 +11367,7 @@
         <v>564</v>
       </c>
       <c r="M27" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N27" t="s">
         <v>569</v>
@@ -11411,7 +11411,7 @@
         <v>564</v>
       </c>
       <c r="M28" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N28" t="s">
         <v>569</v>
@@ -11455,7 +11455,7 @@
         <v>564</v>
       </c>
       <c r="M29" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N29" t="s">
         <v>569</v>
@@ -11499,7 +11499,7 @@
         <v>564</v>
       </c>
       <c r="M30" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N30" t="s">
         <v>569</v>
@@ -11543,7 +11543,7 @@
         <v>565</v>
       </c>
       <c r="M31" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N31" t="s">
         <v>569</v>
@@ -11587,7 +11587,7 @@
         <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N32" t="s">
         <v>569</v>
@@ -11631,7 +11631,7 @@
         <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N33" t="s">
         <v>569</v>
@@ -11675,7 +11675,7 @@
         <v>564</v>
       </c>
       <c r="M34" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N34" t="s">
         <v>569</v>
@@ -11719,7 +11719,7 @@
         <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N35" t="s">
         <v>569</v>
@@ -11763,7 +11763,7 @@
         <v>564</v>
       </c>
       <c r="M36" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N36" t="s">
         <v>569</v>
@@ -11807,7 +11807,7 @@
         <v>564</v>
       </c>
       <c r="M37" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N37" t="s">
         <v>569</v>
@@ -11851,7 +11851,7 @@
         <v>564</v>
       </c>
       <c r="M38" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N38" t="s">
         <v>569</v>
@@ -11895,7 +11895,7 @@
         <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N39" t="s">
         <v>569</v>
@@ -11939,7 +11939,7 @@
         <v>564</v>
       </c>
       <c r="M40" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N40" t="s">
         <v>569</v>
@@ -11983,7 +11983,7 @@
         <v>564</v>
       </c>
       <c r="M41" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N41" t="s">
         <v>569</v>
@@ -12027,7 +12027,7 @@
         <v>564</v>
       </c>
       <c r="M42" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N42" t="s">
         <v>569</v>
@@ -12071,7 +12071,7 @@
         <v>564</v>
       </c>
       <c r="M43" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N43" t="s">
         <v>569</v>
@@ -12115,7 +12115,7 @@
         <v>564</v>
       </c>
       <c r="M44" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N44" t="s">
         <v>569</v>
@@ -12159,7 +12159,7 @@
         <v>564</v>
       </c>
       <c r="M45" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N45" t="s">
         <v>569</v>
@@ -12203,7 +12203,7 @@
         <v>564</v>
       </c>
       <c r="M46" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N46" t="s">
         <v>569</v>
@@ -12247,7 +12247,7 @@
         <v>564</v>
       </c>
       <c r="M47" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N47" t="s">
         <v>569</v>
@@ -12291,7 +12291,7 @@
         <v>565</v>
       </c>
       <c r="M48" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N48" t="s">
         <v>569</v>
@@ -12335,7 +12335,7 @@
         <v>565</v>
       </c>
       <c r="M49" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N49" t="s">
         <v>569</v>
@@ -12379,7 +12379,7 @@
         <v>564</v>
       </c>
       <c r="M50" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N50" t="s">
         <v>569</v>
@@ -12423,7 +12423,7 @@
         <v>564</v>
       </c>
       <c r="M51" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N51" t="s">
         <v>569</v>
@@ -12467,7 +12467,7 @@
         <v>564</v>
       </c>
       <c r="M52" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N52" t="s">
         <v>569</v>
@@ -12511,7 +12511,7 @@
         <v>564</v>
       </c>
       <c r="M53" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N53" t="s">
         <v>569</v>
@@ -12555,7 +12555,7 @@
         <v>565</v>
       </c>
       <c r="M54" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N54" t="s">
         <v>569</v>
@@ -12596,7 +12596,7 @@
         <v>382</v>
       </c>
       <c r="M55" s="1">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="N55" t="s">
         <v>569</v>
@@ -12637,7 +12637,7 @@
         <v>565</v>
       </c>
       <c r="M56" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N56" t="s">
         <v>569</v>
@@ -12678,7 +12678,7 @@
         <v>565</v>
       </c>
       <c r="M57" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N57" t="s">
         <v>569</v>
@@ -12719,7 +12719,7 @@
         <v>565</v>
       </c>
       <c r="M58" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N58" t="s">
         <v>569</v>
@@ -12760,7 +12760,7 @@
         <v>565</v>
       </c>
       <c r="M59" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N59" t="s">
         <v>569</v>
@@ -12801,7 +12801,7 @@
         <v>565</v>
       </c>
       <c r="M60" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N60" t="s">
         <v>569</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (05/08/2026 05:11)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10402,7 +10402,7 @@
         <v>562</v>
       </c>
       <c r="M5" s="1">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="N5" t="s">
         <v>569</v>
@@ -10534,7 +10534,7 @@
         <v>564</v>
       </c>
       <c r="M8" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N8" t="s">
         <v>569</v>
@@ -10622,7 +10622,7 @@
         <v>564</v>
       </c>
       <c r="M10" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N10" t="s">
         <v>569</v>
@@ -10666,7 +10666,7 @@
         <v>564</v>
       </c>
       <c r="M11" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N11" t="s">
         <v>569</v>
@@ -10839,7 +10839,7 @@
         <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N15" t="s">
         <v>569</v>
@@ -10883,7 +10883,7 @@
         <v>564</v>
       </c>
       <c r="M16" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N16" t="s">
         <v>569</v>
@@ -10927,7 +10927,7 @@
         <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N17" t="s">
         <v>569</v>
@@ -10971,7 +10971,7 @@
         <v>564</v>
       </c>
       <c r="M18" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N18" t="s">
         <v>569</v>
@@ -11015,7 +11015,7 @@
         <v>564</v>
       </c>
       <c r="M19" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N19" t="s">
         <v>569</v>
@@ -11059,7 +11059,7 @@
         <v>564</v>
       </c>
       <c r="M20" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N20" t="s">
         <v>569</v>
@@ -11103,7 +11103,7 @@
         <v>564</v>
       </c>
       <c r="M21" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N21" t="s">
         <v>569</v>
@@ -11279,7 +11279,7 @@
         <v>565</v>
       </c>
       <c r="M25" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N25" t="s">
         <v>569</v>
@@ -11367,7 +11367,7 @@
         <v>564</v>
       </c>
       <c r="M27" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N27" t="s">
         <v>569</v>
@@ -11411,7 +11411,7 @@
         <v>564</v>
       </c>
       <c r="M28" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N28" t="s">
         <v>569</v>
@@ -11455,7 +11455,7 @@
         <v>564</v>
       </c>
       <c r="M29" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N29" t="s">
         <v>569</v>
@@ -11499,7 +11499,7 @@
         <v>564</v>
       </c>
       <c r="M30" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N30" t="s">
         <v>569</v>
@@ -11543,7 +11543,7 @@
         <v>565</v>
       </c>
       <c r="M31" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N31" t="s">
         <v>569</v>
@@ -11587,7 +11587,7 @@
         <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N32" t="s">
         <v>569</v>
@@ -11631,7 +11631,7 @@
         <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N33" t="s">
         <v>569</v>
@@ -11675,7 +11675,7 @@
         <v>564</v>
       </c>
       <c r="M34" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N34" t="s">
         <v>569</v>
@@ -11719,7 +11719,7 @@
         <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N35" t="s">
         <v>569</v>
@@ -11763,7 +11763,7 @@
         <v>564</v>
       </c>
       <c r="M36" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N36" t="s">
         <v>569</v>
@@ -11807,7 +11807,7 @@
         <v>564</v>
       </c>
       <c r="M37" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N37" t="s">
         <v>569</v>
@@ -11851,7 +11851,7 @@
         <v>564</v>
       </c>
       <c r="M38" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N38" t="s">
         <v>569</v>
@@ -11895,7 +11895,7 @@
         <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N39" t="s">
         <v>569</v>
@@ -11939,7 +11939,7 @@
         <v>564</v>
       </c>
       <c r="M40" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N40" t="s">
         <v>569</v>
@@ -11983,7 +11983,7 @@
         <v>564</v>
       </c>
       <c r="M41" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N41" t="s">
         <v>569</v>
@@ -12027,7 +12027,7 @@
         <v>564</v>
       </c>
       <c r="M42" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N42" t="s">
         <v>569</v>
@@ -12071,7 +12071,7 @@
         <v>564</v>
       </c>
       <c r="M43" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N43" t="s">
         <v>569</v>
@@ -12115,7 +12115,7 @@
         <v>564</v>
       </c>
       <c r="M44" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N44" t="s">
         <v>569</v>
@@ -12159,7 +12159,7 @@
         <v>564</v>
       </c>
       <c r="M45" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N45" t="s">
         <v>569</v>
@@ -12203,7 +12203,7 @@
         <v>564</v>
       </c>
       <c r="M46" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N46" t="s">
         <v>569</v>
@@ -12247,7 +12247,7 @@
         <v>564</v>
       </c>
       <c r="M47" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N47" t="s">
         <v>569</v>
@@ -12291,7 +12291,7 @@
         <v>565</v>
       </c>
       <c r="M48" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N48" t="s">
         <v>569</v>
@@ -12335,7 +12335,7 @@
         <v>565</v>
       </c>
       <c r="M49" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N49" t="s">
         <v>569</v>
@@ -12379,7 +12379,7 @@
         <v>564</v>
       </c>
       <c r="M50" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N50" t="s">
         <v>569</v>
@@ -12423,7 +12423,7 @@
         <v>564</v>
       </c>
       <c r="M51" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N51" t="s">
         <v>569</v>
@@ -12467,7 +12467,7 @@
         <v>564</v>
       </c>
       <c r="M52" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N52" t="s">
         <v>569</v>
@@ -12511,7 +12511,7 @@
         <v>564</v>
       </c>
       <c r="M53" s="1">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="N53" t="s">
         <v>569</v>
@@ -12555,7 +12555,7 @@
         <v>565</v>
       </c>
       <c r="M54" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N54" t="s">
         <v>569</v>
@@ -12596,7 +12596,7 @@
         <v>382</v>
       </c>
       <c r="M55" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N55" t="s">
         <v>569</v>
@@ -12637,7 +12637,7 @@
         <v>565</v>
       </c>
       <c r="M56" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N56" t="s">
         <v>569</v>
@@ -12678,7 +12678,7 @@
         <v>565</v>
       </c>
       <c r="M57" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N57" t="s">
         <v>569</v>
@@ -12719,7 +12719,7 @@
         <v>565</v>
       </c>
       <c r="M58" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N58" t="s">
         <v>569</v>
@@ -12760,7 +12760,7 @@
         <v>565</v>
       </c>
       <c r="M59" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N59" t="s">
         <v>569</v>
@@ -12801,7 +12801,7 @@
         <v>565</v>
       </c>
       <c r="M60" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N60" t="s">
         <v>569</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (05/08/2026 15:42)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2492" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="572">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1412,6 +1412,9 @@
     <t>LST209005U8</t>
   </si>
   <si>
+    <t>LST216004U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1565,6 +1568,9 @@
     <t>2643057-1</t>
   </si>
   <si>
+    <t>S3100-527</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1691,7 +1697,7 @@
     <t>TUBE ASSY-LONG</t>
   </si>
   <si>
-    <t>Vant, Breather</t>
+    <t>VANT,BREATHER</t>
   </si>
   <si>
     <t>BELLCRANK ASSY</t>
@@ -1700,28 +1706,28 @@
     <t>BOOT N G STEER</t>
   </si>
   <si>
+    <t>NAV STROBE LIGHT ASSEMBLYRIGHT</t>
+  </si>
+  <si>
     <t>Empenho Solicitado</t>
   </si>
   <si>
     <t>Mapa Gerado</t>
   </si>
   <si>
-    <t>Selecionada em Plano</t>
+    <t>Selecionada para Cotação</t>
   </si>
   <si>
     <t>Validada</t>
   </si>
   <si>
+    <t>Em Discrepância</t>
+  </si>
+  <si>
     <t>Análise do Pedido</t>
   </si>
   <si>
-    <t>Em Discrepância</t>
-  </si>
-  <si>
-    <t>EMPENHADO</t>
-  </si>
-  <si>
-    <t>IMEDIATO</t>
+    <t>Selecionada para cotação</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10176,7 +10182,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q60"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10258,7 +10264,7 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J2" t="s">
         <v>387</v>
@@ -10268,9 +10274,6 @@
       </c>
       <c r="L2" t="s">
         <v>387</v>
-      </c>
-      <c r="M2" t="s">
-        <v>567</v>
       </c>
       <c r="N2" t="s">
         <v>395</v>
@@ -10302,7 +10305,7 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J3" t="s">
         <v>387</v>
@@ -10312,9 +10315,6 @@
       </c>
       <c r="L3" t="s">
         <v>387</v>
-      </c>
-      <c r="M3" t="s">
-        <v>567</v>
       </c>
       <c r="N3" t="s">
         <v>395</v>
@@ -10331,7 +10331,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10346,7 +10346,7 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J4" t="s">
         <v>387</v>
@@ -10356,9 +10356,6 @@
       </c>
       <c r="L4" t="s">
         <v>387</v>
-      </c>
-      <c r="M4" t="s">
-        <v>567</v>
       </c>
       <c r="N4" t="s">
         <v>395</v>
@@ -10375,10 +10372,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E5" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10390,22 +10387,22 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="J5" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="K5" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="L5" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="M5" s="1">
         <v>46249</v>
       </c>
       <c r="N5" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -10434,7 +10431,7 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J6" t="s">
         <v>387</v>
@@ -10444,9 +10441,6 @@
       </c>
       <c r="L6" t="s">
         <v>387</v>
-      </c>
-      <c r="M6" t="s">
-        <v>567</v>
       </c>
       <c r="N6" t="s">
         <v>395</v>
@@ -10478,7 +10472,7 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J7" t="s">
         <v>387</v>
@@ -10488,9 +10482,6 @@
       </c>
       <c r="L7" t="s">
         <v>387</v>
-      </c>
-      <c r="M7" t="s">
-        <v>567</v>
       </c>
       <c r="N7" t="s">
         <v>395</v>
@@ -10522,22 +10513,22 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J8" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K8" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L8" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M8" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N8" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10551,7 +10542,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10566,7 +10557,7 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J9" t="s">
         <v>387</v>
@@ -10576,9 +10567,6 @@
       </c>
       <c r="L9" t="s">
         <v>387</v>
-      </c>
-      <c r="M9" t="s">
-        <v>567</v>
       </c>
       <c r="N9" t="s">
         <v>395</v>
@@ -10595,10 +10583,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E10" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10613,19 +10601,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K10" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L10" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M10" s="1">
         <v>46314</v>
       </c>
       <c r="N10" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10639,7 +10627,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10657,19 +10645,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K11" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L11" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M11" s="1">
         <v>46314</v>
       </c>
       <c r="N11" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10683,10 +10671,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E12" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -10739,19 +10727,16 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>380</v>
+        <v>564</v>
       </c>
       <c r="J13" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="K13" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="L13" t="s">
-        <v>380</v>
-      </c>
-      <c r="M13" t="s">
-        <v>568</v>
+        <v>387</v>
       </c>
       <c r="N13" t="s">
         <v>395</v>
@@ -10768,10 +10753,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E14" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -10783,7 +10768,7 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J14" t="s">
         <v>387</v>
@@ -10793,9 +10778,6 @@
       </c>
       <c r="L14" t="s">
         <v>387</v>
-      </c>
-      <c r="M14" t="s">
-        <v>567</v>
       </c>
       <c r="N14" t="s">
         <v>395</v>
@@ -10812,10 +10794,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E15" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -10827,22 +10809,22 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J15" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="K15" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="L15" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="M15" s="1">
-        <v>46329</v>
+        <v>46284</v>
       </c>
       <c r="N15" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10856,10 +10838,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E16" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -10874,19 +10856,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K16" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L16" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M16" s="1">
         <v>46314</v>
       </c>
       <c r="N16" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10900,10 +10882,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E17" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -10915,22 +10897,22 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J17" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="K17" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="L17" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="M17" s="1">
-        <v>46329</v>
+        <v>46284</v>
       </c>
       <c r="N17" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10944,10 +10926,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E18" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -10962,19 +10944,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K18" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L18" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M18" s="1">
         <v>46314</v>
       </c>
       <c r="N18" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10988,10 +10970,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E19" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="F19">
         <v>4</v>
@@ -11006,19 +10988,19 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K19" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L19" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M19" s="1">
         <v>46314</v>
       </c>
       <c r="N19" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11032,10 +11014,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E20" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -11050,19 +11032,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K20" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L20" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M20" s="1">
         <v>46314</v>
       </c>
       <c r="N20" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11076,10 +11058,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E21" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11094,19 +11076,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K21" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L21" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M21" s="1">
         <v>46314</v>
       </c>
       <c r="N21" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11120,10 +11102,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E22" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11135,7 +11117,7 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J22" t="s">
         <v>387</v>
@@ -11145,9 +11127,6 @@
       </c>
       <c r="L22" t="s">
         <v>387</v>
-      </c>
-      <c r="M22" t="s">
-        <v>567</v>
       </c>
       <c r="N22" t="s">
         <v>395</v>
@@ -11164,10 +11143,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E23" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11179,7 +11158,7 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J23" t="s">
         <v>387</v>
@@ -11189,9 +11168,6 @@
       </c>
       <c r="L23" t="s">
         <v>387</v>
-      </c>
-      <c r="M23" t="s">
-        <v>567</v>
       </c>
       <c r="N23" t="s">
         <v>395</v>
@@ -11208,7 +11184,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11223,7 +11199,7 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J24" t="s">
         <v>387</v>
@@ -11233,9 +11209,6 @@
       </c>
       <c r="L24" t="s">
         <v>387</v>
-      </c>
-      <c r="M24" t="s">
-        <v>567</v>
       </c>
       <c r="N24" t="s">
         <v>395</v>
@@ -11252,10 +11225,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E25" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11267,22 +11240,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="J25" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="K25" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="L25" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="M25" s="1">
-        <v>46329</v>
+        <v>46314</v>
       </c>
       <c r="N25" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11296,10 +11269,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E26" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11311,7 +11284,7 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="J26" t="s">
         <v>387</v>
@@ -11321,9 +11294,6 @@
       </c>
       <c r="L26" t="s">
         <v>387</v>
-      </c>
-      <c r="M26" t="s">
-        <v>567</v>
       </c>
       <c r="N26" t="s">
         <v>395</v>
@@ -11340,10 +11310,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E27" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11355,22 +11325,22 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J27" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K27" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L27" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M27" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N27" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11384,10 +11354,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E28" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11402,19 +11372,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K28" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L28" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M28" s="1">
         <v>46314</v>
       </c>
       <c r="N28" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11428,10 +11398,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E29" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11443,22 +11413,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J29" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K29" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L29" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M29" s="1">
         <v>46314</v>
       </c>
       <c r="N29" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11472,10 +11442,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E30" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11490,19 +11460,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K30" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L30" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M30" s="1">
         <v>46314</v>
       </c>
       <c r="N30" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11516,10 +11486,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E31" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11531,22 +11501,19 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J31" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K31" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L31" t="s">
-        <v>565</v>
-      </c>
-      <c r="M31" s="1">
-        <v>46329</v>
+        <v>568</v>
       </c>
       <c r="N31" t="s">
-        <v>569</v>
+        <v>395</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11560,10 +11527,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E32" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11575,22 +11542,22 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J32" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="K32" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="L32" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="M32" s="1">
-        <v>46329</v>
+        <v>46284</v>
       </c>
       <c r="N32" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11604,10 +11571,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E33" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11619,22 +11586,22 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J33" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="K33" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="L33" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="M33" s="1">
-        <v>46329</v>
+        <v>46284</v>
       </c>
       <c r="N33" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11648,10 +11615,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E34" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11663,22 +11630,22 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J34" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K34" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L34" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M34" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N34" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11692,10 +11659,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E35" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11707,22 +11674,22 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J35" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="K35" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="L35" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="M35" s="1">
-        <v>46329</v>
+        <v>46284</v>
       </c>
       <c r="N35" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11736,10 +11703,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E36" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -11751,22 +11718,22 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J36" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K36" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L36" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M36" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N36" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11780,10 +11747,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E37" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -11795,22 +11762,22 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J37" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K37" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L37" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M37" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N37" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11824,10 +11791,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E38" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -11839,22 +11806,22 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J38" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K38" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L38" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M38" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N38" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11868,10 +11835,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E39" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -11883,22 +11850,22 @@
         <v>312.36</v>
       </c>
       <c r="I39" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J39" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="K39" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="L39" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="M39" s="1">
-        <v>46329</v>
+        <v>46284</v>
       </c>
       <c r="N39" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11912,10 +11879,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E40" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -11927,22 +11894,22 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J40" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K40" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L40" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M40" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N40" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11956,10 +11923,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E41" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -11974,19 +11941,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K41" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L41" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M41" s="1">
         <v>46314</v>
       </c>
       <c r="N41" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12015,22 +11982,22 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J42" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K42" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L42" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M42" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N42" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -12044,10 +12011,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E43" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -12059,22 +12026,19 @@
         <v>5000</v>
       </c>
       <c r="I43" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J43" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="K43" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="L43" t="s">
-        <v>564</v>
-      </c>
-      <c r="M43" s="1">
-        <v>46314</v>
+        <v>568</v>
       </c>
       <c r="N43" t="s">
-        <v>569</v>
+        <v>395</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12088,7 +12052,7 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
@@ -12106,19 +12070,19 @@
         <v>382</v>
       </c>
       <c r="J44" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K44" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L44" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M44" s="1">
         <v>46314</v>
       </c>
       <c r="N44" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12132,10 +12096,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E45" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12150,19 +12114,19 @@
         <v>382</v>
       </c>
       <c r="J45" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K45" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L45" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M45" s="1">
         <v>46314</v>
       </c>
       <c r="N45" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12176,10 +12140,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E46" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12191,22 +12155,22 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J46" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K46" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L46" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M46" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N46" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12220,10 +12184,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="E47" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12235,22 +12199,22 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="J47" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="K47" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="L47" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M47" s="1">
-        <v>46314</v>
+        <v>46284</v>
       </c>
       <c r="N47" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12264,10 +12228,10 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E48" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -12279,22 +12243,19 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J48" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K48" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L48" t="s">
-        <v>565</v>
-      </c>
-      <c r="M48" s="1">
-        <v>46329</v>
+        <v>568</v>
       </c>
       <c r="N48" t="s">
-        <v>569</v>
+        <v>395</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12308,10 +12269,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E49" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12323,22 +12284,22 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="J49" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="K49" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="L49" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="M49" s="1">
-        <v>46329</v>
+        <v>46314</v>
       </c>
       <c r="N49" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12352,10 +12313,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E50" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12367,22 +12328,22 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="J50" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K50" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L50" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M50" s="1">
         <v>46314</v>
       </c>
       <c r="N50" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12396,10 +12357,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E51" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12414,19 +12375,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K51" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L51" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M51" s="1">
         <v>46314</v>
       </c>
       <c r="N51" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12440,10 +12401,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E52" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12458,19 +12419,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K52" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L52" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M52" s="1">
         <v>46314</v>
       </c>
       <c r="N52" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12484,10 +12445,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E53" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12502,19 +12463,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="K53" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="L53" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M53" s="1">
         <v>46314</v>
       </c>
       <c r="N53" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12528,10 +12489,10 @@
         <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E54" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="F54">
         <v>4</v>
@@ -12543,22 +12504,22 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J54" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="K54" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="L54" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="M54" s="1">
         <v>46329</v>
       </c>
       <c r="N54" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12572,10 +12533,10 @@
         <v>173</v>
       </c>
       <c r="D55" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E55" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="F55">
         <v>1</v>
@@ -12589,17 +12550,20 @@
       <c r="I55" t="s">
         <v>382</v>
       </c>
+      <c r="J55" t="s">
+        <v>567</v>
+      </c>
       <c r="K55" t="s">
-        <v>382</v>
+        <v>567</v>
       </c>
       <c r="L55" t="s">
-        <v>382</v>
+        <v>567</v>
       </c>
       <c r="M55" s="1">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="N55" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12613,10 +12577,10 @@
         <v>173</v>
       </c>
       <c r="D56" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E56" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -12628,19 +12592,22 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
-        <v>565</v>
+        <v>569</v>
+      </c>
+      <c r="J56" t="s">
+        <v>569</v>
       </c>
       <c r="K56" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="L56" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="M56" s="1">
         <v>46329</v>
       </c>
       <c r="N56" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12654,10 +12621,10 @@
         <v>173</v>
       </c>
       <c r="D57" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E57" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -12669,19 +12636,22 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
-        <v>565</v>
+        <v>569</v>
+      </c>
+      <c r="J57" t="s">
+        <v>569</v>
       </c>
       <c r="K57" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="L57" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="M57" s="1">
         <v>46329</v>
       </c>
       <c r="N57" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12695,10 +12665,10 @@
         <v>173</v>
       </c>
       <c r="D58" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E58" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="F58">
         <v>4</v>
@@ -12710,19 +12680,22 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
-        <v>565</v>
+        <v>569</v>
+      </c>
+      <c r="J58" t="s">
+        <v>569</v>
       </c>
       <c r="K58" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="L58" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="M58" s="1">
         <v>46329</v>
       </c>
       <c r="N58" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -12751,19 +12724,22 @@
         <v>870</v>
       </c>
       <c r="I59" t="s">
-        <v>565</v>
+        <v>569</v>
+      </c>
+      <c r="J59" t="s">
+        <v>567</v>
       </c>
       <c r="K59" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="L59" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46329</v>
+        <v>46314</v>
       </c>
       <c r="N59" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -12777,10 +12753,10 @@
         <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E60" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -12792,19 +12768,66 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
-        <v>565</v>
+        <v>569</v>
+      </c>
+      <c r="J60" t="s">
+        <v>569</v>
       </c>
       <c r="K60" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="L60" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="M60" s="1">
         <v>46329</v>
       </c>
       <c r="N60" t="s">
-        <v>569</v>
+        <v>571</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14">
+      <c r="A61" t="s">
+        <v>465</v>
+      </c>
+      <c r="B61" t="s">
+        <v>172</v>
+      </c>
+      <c r="C61" t="s">
+        <v>173</v>
+      </c>
+      <c r="D61" t="s">
+        <v>517</v>
+      </c>
+      <c r="E61" t="s">
+        <v>563</v>
+      </c>
+      <c r="F61">
+        <v>5</v>
+      </c>
+      <c r="G61">
+        <v>1129.01</v>
+      </c>
+      <c r="H61">
+        <v>5645.05</v>
+      </c>
+      <c r="I61" t="s">
+        <v>382</v>
+      </c>
+      <c r="J61" t="s">
+        <v>567</v>
+      </c>
+      <c r="K61" t="s">
+        <v>567</v>
+      </c>
+      <c r="L61" t="s">
+        <v>567</v>
+      </c>
+      <c r="M61" s="1">
+        <v>46314</v>
+      </c>
+      <c r="N61" t="s">
+        <v>571</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (06/08/2026 10:02)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10399,7 +10399,7 @@
         <v>565</v>
       </c>
       <c r="M5" s="1">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="N5" t="s">
         <v>571</v>
@@ -10525,7 +10525,7 @@
         <v>570</v>
       </c>
       <c r="M8" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N8" t="s">
         <v>571</v>
@@ -10610,7 +10610,7 @@
         <v>567</v>
       </c>
       <c r="M10" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N10" t="s">
         <v>571</v>
@@ -10654,7 +10654,7 @@
         <v>567</v>
       </c>
       <c r="M11" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N11" t="s">
         <v>571</v>
@@ -10821,7 +10821,7 @@
         <v>570</v>
       </c>
       <c r="M15" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N15" t="s">
         <v>571</v>
@@ -10865,7 +10865,7 @@
         <v>567</v>
       </c>
       <c r="M16" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N16" t="s">
         <v>571</v>
@@ -10909,7 +10909,7 @@
         <v>570</v>
       </c>
       <c r="M17" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N17" t="s">
         <v>571</v>
@@ -10953,7 +10953,7 @@
         <v>567</v>
       </c>
       <c r="M18" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N18" t="s">
         <v>571</v>
@@ -10997,7 +10997,7 @@
         <v>567</v>
       </c>
       <c r="M19" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N19" t="s">
         <v>571</v>
@@ -11041,7 +11041,7 @@
         <v>567</v>
       </c>
       <c r="M20" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N20" t="s">
         <v>571</v>
@@ -11085,7 +11085,7 @@
         <v>567</v>
       </c>
       <c r="M21" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N21" t="s">
         <v>571</v>
@@ -11252,7 +11252,7 @@
         <v>567</v>
       </c>
       <c r="M25" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N25" t="s">
         <v>571</v>
@@ -11337,7 +11337,7 @@
         <v>570</v>
       </c>
       <c r="M27" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N27" t="s">
         <v>571</v>
@@ -11381,7 +11381,7 @@
         <v>567</v>
       </c>
       <c r="M28" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N28" t="s">
         <v>571</v>
@@ -11425,7 +11425,7 @@
         <v>567</v>
       </c>
       <c r="M29" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N29" t="s">
         <v>571</v>
@@ -11469,7 +11469,7 @@
         <v>567</v>
       </c>
       <c r="M30" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N30" t="s">
         <v>571</v>
@@ -11554,7 +11554,7 @@
         <v>570</v>
       </c>
       <c r="M32" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N32" t="s">
         <v>571</v>
@@ -11598,7 +11598,7 @@
         <v>570</v>
       </c>
       <c r="M33" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N33" t="s">
         <v>571</v>
@@ -11642,7 +11642,7 @@
         <v>570</v>
       </c>
       <c r="M34" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N34" t="s">
         <v>571</v>
@@ -11686,7 +11686,7 @@
         <v>570</v>
       </c>
       <c r="M35" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N35" t="s">
         <v>571</v>
@@ -11730,7 +11730,7 @@
         <v>570</v>
       </c>
       <c r="M36" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N36" t="s">
         <v>571</v>
@@ -11774,7 +11774,7 @@
         <v>570</v>
       </c>
       <c r="M37" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N37" t="s">
         <v>571</v>
@@ -11818,7 +11818,7 @@
         <v>570</v>
       </c>
       <c r="M38" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N38" t="s">
         <v>571</v>
@@ -11862,7 +11862,7 @@
         <v>570</v>
       </c>
       <c r="M39" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N39" t="s">
         <v>571</v>
@@ -11906,7 +11906,7 @@
         <v>570</v>
       </c>
       <c r="M40" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N40" t="s">
         <v>571</v>
@@ -11950,7 +11950,7 @@
         <v>567</v>
       </c>
       <c r="M41" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N41" t="s">
         <v>571</v>
@@ -11994,7 +11994,7 @@
         <v>570</v>
       </c>
       <c r="M42" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N42" t="s">
         <v>571</v>
@@ -12079,7 +12079,7 @@
         <v>567</v>
       </c>
       <c r="M44" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N44" t="s">
         <v>571</v>
@@ -12123,7 +12123,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N45" t="s">
         <v>571</v>
@@ -12167,7 +12167,7 @@
         <v>570</v>
       </c>
       <c r="M46" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N46" t="s">
         <v>571</v>
@@ -12211,7 +12211,7 @@
         <v>570</v>
       </c>
       <c r="M47" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N47" t="s">
         <v>571</v>
@@ -12296,7 +12296,7 @@
         <v>567</v>
       </c>
       <c r="M49" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N49" t="s">
         <v>571</v>
@@ -12340,7 +12340,7 @@
         <v>567</v>
       </c>
       <c r="M50" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N50" t="s">
         <v>571</v>
@@ -12384,7 +12384,7 @@
         <v>567</v>
       </c>
       <c r="M51" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N51" t="s">
         <v>571</v>
@@ -12428,7 +12428,7 @@
         <v>567</v>
       </c>
       <c r="M52" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N52" t="s">
         <v>571</v>
@@ -12472,7 +12472,7 @@
         <v>567</v>
       </c>
       <c r="M53" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N53" t="s">
         <v>571</v>
@@ -12516,7 +12516,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N54" t="s">
         <v>571</v>
@@ -12560,7 +12560,7 @@
         <v>567</v>
       </c>
       <c r="M55" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N55" t="s">
         <v>571</v>
@@ -12604,7 +12604,7 @@
         <v>569</v>
       </c>
       <c r="M56" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N56" t="s">
         <v>571</v>
@@ -12648,7 +12648,7 @@
         <v>569</v>
       </c>
       <c r="M57" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N57" t="s">
         <v>571</v>
@@ -12692,7 +12692,7 @@
         <v>569</v>
       </c>
       <c r="M58" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N58" t="s">
         <v>571</v>
@@ -12736,7 +12736,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N59" t="s">
         <v>571</v>
@@ -12780,7 +12780,7 @@
         <v>569</v>
       </c>
       <c r="M60" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N60" t="s">
         <v>571</v>
@@ -12824,7 +12824,7 @@
         <v>567</v>
       </c>
       <c r="M61" s="1">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="N61" t="s">
         <v>571</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (07/08/2026 08:52)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10399,7 +10399,7 @@
         <v>565</v>
       </c>
       <c r="M5" s="1">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="N5" t="s">
         <v>571</v>
@@ -10525,7 +10525,7 @@
         <v>570</v>
       </c>
       <c r="M8" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N8" t="s">
         <v>571</v>
@@ -10610,7 +10610,7 @@
         <v>567</v>
       </c>
       <c r="M10" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N10" t="s">
         <v>571</v>
@@ -10654,7 +10654,7 @@
         <v>567</v>
       </c>
       <c r="M11" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N11" t="s">
         <v>571</v>
@@ -10821,7 +10821,7 @@
         <v>570</v>
       </c>
       <c r="M15" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N15" t="s">
         <v>571</v>
@@ -10865,7 +10865,7 @@
         <v>567</v>
       </c>
       <c r="M16" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N16" t="s">
         <v>571</v>
@@ -10909,7 +10909,7 @@
         <v>570</v>
       </c>
       <c r="M17" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N17" t="s">
         <v>571</v>
@@ -10953,7 +10953,7 @@
         <v>567</v>
       </c>
       <c r="M18" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N18" t="s">
         <v>571</v>
@@ -10997,7 +10997,7 @@
         <v>567</v>
       </c>
       <c r="M19" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N19" t="s">
         <v>571</v>
@@ -11041,7 +11041,7 @@
         <v>567</v>
       </c>
       <c r="M20" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N20" t="s">
         <v>571</v>
@@ -11085,7 +11085,7 @@
         <v>567</v>
       </c>
       <c r="M21" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N21" t="s">
         <v>571</v>
@@ -11252,7 +11252,7 @@
         <v>567</v>
       </c>
       <c r="M25" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N25" t="s">
         <v>571</v>
@@ -11337,7 +11337,7 @@
         <v>570</v>
       </c>
       <c r="M27" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N27" t="s">
         <v>571</v>
@@ -11381,7 +11381,7 @@
         <v>567</v>
       </c>
       <c r="M28" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N28" t="s">
         <v>571</v>
@@ -11425,7 +11425,7 @@
         <v>567</v>
       </c>
       <c r="M29" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N29" t="s">
         <v>571</v>
@@ -11469,7 +11469,7 @@
         <v>567</v>
       </c>
       <c r="M30" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N30" t="s">
         <v>571</v>
@@ -11554,7 +11554,7 @@
         <v>570</v>
       </c>
       <c r="M32" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N32" t="s">
         <v>571</v>
@@ -11598,7 +11598,7 @@
         <v>570</v>
       </c>
       <c r="M33" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N33" t="s">
         <v>571</v>
@@ -11642,7 +11642,7 @@
         <v>570</v>
       </c>
       <c r="M34" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N34" t="s">
         <v>571</v>
@@ -11686,7 +11686,7 @@
         <v>570</v>
       </c>
       <c r="M35" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N35" t="s">
         <v>571</v>
@@ -11730,7 +11730,7 @@
         <v>570</v>
       </c>
       <c r="M36" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N36" t="s">
         <v>571</v>
@@ -11774,7 +11774,7 @@
         <v>570</v>
       </c>
       <c r="M37" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N37" t="s">
         <v>571</v>
@@ -11818,7 +11818,7 @@
         <v>570</v>
       </c>
       <c r="M38" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N38" t="s">
         <v>571</v>
@@ -11862,7 +11862,7 @@
         <v>570</v>
       </c>
       <c r="M39" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N39" t="s">
         <v>571</v>
@@ -11906,7 +11906,7 @@
         <v>570</v>
       </c>
       <c r="M40" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N40" t="s">
         <v>571</v>
@@ -11950,7 +11950,7 @@
         <v>567</v>
       </c>
       <c r="M41" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N41" t="s">
         <v>571</v>
@@ -11994,7 +11994,7 @@
         <v>570</v>
       </c>
       <c r="M42" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N42" t="s">
         <v>571</v>
@@ -12079,7 +12079,7 @@
         <v>567</v>
       </c>
       <c r="M44" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N44" t="s">
         <v>571</v>
@@ -12123,7 +12123,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N45" t="s">
         <v>571</v>
@@ -12167,7 +12167,7 @@
         <v>570</v>
       </c>
       <c r="M46" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N46" t="s">
         <v>571</v>
@@ -12211,7 +12211,7 @@
         <v>570</v>
       </c>
       <c r="M47" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N47" t="s">
         <v>571</v>
@@ -12296,7 +12296,7 @@
         <v>567</v>
       </c>
       <c r="M49" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N49" t="s">
         <v>571</v>
@@ -12340,7 +12340,7 @@
         <v>567</v>
       </c>
       <c r="M50" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N50" t="s">
         <v>571</v>
@@ -12384,7 +12384,7 @@
         <v>567</v>
       </c>
       <c r="M51" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N51" t="s">
         <v>571</v>
@@ -12428,7 +12428,7 @@
         <v>567</v>
       </c>
       <c r="M52" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N52" t="s">
         <v>571</v>
@@ -12472,7 +12472,7 @@
         <v>567</v>
       </c>
       <c r="M53" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N53" t="s">
         <v>571</v>
@@ -12516,7 +12516,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="N54" t="s">
         <v>571</v>
@@ -12560,7 +12560,7 @@
         <v>567</v>
       </c>
       <c r="M55" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N55" t="s">
         <v>571</v>
@@ -12604,7 +12604,7 @@
         <v>569</v>
       </c>
       <c r="M56" s="1">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="N56" t="s">
         <v>571</v>
@@ -12648,7 +12648,7 @@
         <v>569</v>
       </c>
       <c r="M57" s="1">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="N57" t="s">
         <v>571</v>
@@ -12692,7 +12692,7 @@
         <v>569</v>
       </c>
       <c r="M58" s="1">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="N58" t="s">
         <v>571</v>
@@ -12736,7 +12736,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N59" t="s">
         <v>571</v>
@@ -12780,7 +12780,7 @@
         <v>569</v>
       </c>
       <c r="M60" s="1">
-        <v>46330</v>
+        <v>46331</v>
       </c>
       <c r="N60" t="s">
         <v>571</v>
@@ -12824,7 +12824,7 @@
         <v>567</v>
       </c>
       <c r="M61" s="1">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="N61" t="s">
         <v>571</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (07/08/2026 11:17)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="573">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1712,19 +1712,22 @@
     <t>Empenho Solicitado</t>
   </si>
   <si>
+    <t>Aguardando Intenção de Recurso</t>
+  </si>
+  <si>
+    <t>Em Cotação</t>
+  </si>
+  <si>
+    <t>Validada</t>
+  </si>
+  <si>
+    <t>Em Discrepância</t>
+  </si>
+  <si>
+    <t>Análise do Pedido</t>
+  </si>
+  <si>
     <t>Mapa Gerado</t>
-  </si>
-  <si>
-    <t>Selecionada para Cotação</t>
-  </si>
-  <si>
-    <t>Validada</t>
-  </si>
-  <si>
-    <t>Em Discrepância</t>
-  </si>
-  <si>
-    <t>Análise do Pedido</t>
   </si>
   <si>
     <t>Selecionada para cotação</t>
@@ -10390,19 +10393,19 @@
         <v>565</v>
       </c>
       <c r="J5" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="K5" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="L5" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="M5" s="1">
         <v>46251</v>
       </c>
       <c r="N5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -10516,19 +10519,19 @@
         <v>566</v>
       </c>
       <c r="J8" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K8" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L8" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M8" s="1">
         <v>46286</v>
       </c>
       <c r="N8" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10613,7 +10616,7 @@
         <v>46316</v>
       </c>
       <c r="N10" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10657,7 +10660,7 @@
         <v>46316</v>
       </c>
       <c r="N11" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10812,19 +10815,19 @@
         <v>566</v>
       </c>
       <c r="J15" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K15" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L15" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M15" s="1">
         <v>46286</v>
       </c>
       <c r="N15" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10868,7 +10871,7 @@
         <v>46316</v>
       </c>
       <c r="N16" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10900,19 +10903,19 @@
         <v>566</v>
       </c>
       <c r="J17" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K17" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L17" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M17" s="1">
         <v>46286</v>
       </c>
       <c r="N17" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10956,7 +10959,7 @@
         <v>46316</v>
       </c>
       <c r="N18" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -11000,7 +11003,7 @@
         <v>46316</v>
       </c>
       <c r="N19" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11044,7 +11047,7 @@
         <v>46316</v>
       </c>
       <c r="N20" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11088,7 +11091,7 @@
         <v>46316</v>
       </c>
       <c r="N21" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11255,7 +11258,7 @@
         <v>46316</v>
       </c>
       <c r="N25" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11328,19 +11331,19 @@
         <v>566</v>
       </c>
       <c r="J27" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K27" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L27" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M27" s="1">
         <v>46286</v>
       </c>
       <c r="N27" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11384,7 +11387,7 @@
         <v>46316</v>
       </c>
       <c r="N28" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11428,7 +11431,7 @@
         <v>46316</v>
       </c>
       <c r="N29" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11472,7 +11475,7 @@
         <v>46316</v>
       </c>
       <c r="N30" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11501,7 +11504,7 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="J31" t="s">
         <v>568</v>
@@ -11545,19 +11548,19 @@
         <v>566</v>
       </c>
       <c r="J32" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K32" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L32" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M32" s="1">
         <v>46286</v>
       </c>
       <c r="N32" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11589,19 +11592,19 @@
         <v>566</v>
       </c>
       <c r="J33" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K33" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L33" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M33" s="1">
         <v>46286</v>
       </c>
       <c r="N33" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11633,19 +11636,19 @@
         <v>566</v>
       </c>
       <c r="J34" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K34" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L34" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M34" s="1">
         <v>46286</v>
       </c>
       <c r="N34" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11677,19 +11680,19 @@
         <v>566</v>
       </c>
       <c r="J35" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K35" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L35" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M35" s="1">
         <v>46286</v>
       </c>
       <c r="N35" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11721,19 +11724,19 @@
         <v>566</v>
       </c>
       <c r="J36" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K36" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L36" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M36" s="1">
         <v>46286</v>
       </c>
       <c r="N36" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11765,19 +11768,19 @@
         <v>566</v>
       </c>
       <c r="J37" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K37" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L37" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M37" s="1">
         <v>46286</v>
       </c>
       <c r="N37" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11809,19 +11812,19 @@
         <v>566</v>
       </c>
       <c r="J38" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K38" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L38" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M38" s="1">
         <v>46286</v>
       </c>
       <c r="N38" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11853,19 +11856,19 @@
         <v>566</v>
       </c>
       <c r="J39" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K39" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L39" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M39" s="1">
         <v>46286</v>
       </c>
       <c r="N39" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11897,19 +11900,19 @@
         <v>566</v>
       </c>
       <c r="J40" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K40" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L40" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M40" s="1">
         <v>46286</v>
       </c>
       <c r="N40" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11953,7 +11956,7 @@
         <v>46316</v>
       </c>
       <c r="N41" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11985,19 +11988,19 @@
         <v>566</v>
       </c>
       <c r="J42" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K42" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L42" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M42" s="1">
         <v>46286</v>
       </c>
       <c r="N42" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -12082,7 +12085,7 @@
         <v>46316</v>
       </c>
       <c r="N44" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12126,7 +12129,7 @@
         <v>46316</v>
       </c>
       <c r="N45" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12158,19 +12161,19 @@
         <v>566</v>
       </c>
       <c r="J46" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K46" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L46" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M46" s="1">
         <v>46286</v>
       </c>
       <c r="N46" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12202,19 +12205,19 @@
         <v>566</v>
       </c>
       <c r="J47" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K47" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L47" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M47" s="1">
         <v>46286</v>
       </c>
       <c r="N47" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12299,7 +12302,7 @@
         <v>46316</v>
       </c>
       <c r="N49" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12343,7 +12346,7 @@
         <v>46316</v>
       </c>
       <c r="N50" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12387,7 +12390,7 @@
         <v>46316</v>
       </c>
       <c r="N51" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12431,7 +12434,7 @@
         <v>46316</v>
       </c>
       <c r="N52" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12475,7 +12478,7 @@
         <v>46316</v>
       </c>
       <c r="N53" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12519,7 +12522,7 @@
         <v>46331</v>
       </c>
       <c r="N54" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12563,7 +12566,7 @@
         <v>46316</v>
       </c>
       <c r="N55" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12607,7 +12610,7 @@
         <v>46331</v>
       </c>
       <c r="N56" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12636,7 +12639,7 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="J57" t="s">
         <v>569</v>
@@ -12651,7 +12654,7 @@
         <v>46331</v>
       </c>
       <c r="N57" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12695,7 +12698,7 @@
         <v>46331</v>
       </c>
       <c r="N58" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -12739,7 +12742,7 @@
         <v>46316</v>
       </c>
       <c r="N59" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -12783,7 +12786,7 @@
         <v>46331</v>
       </c>
       <c r="N60" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -12827,7 +12830,7 @@
         <v>46316</v>
       </c>
       <c r="N61" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (10/08/2026 08:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10402,7 +10402,7 @@
         <v>570</v>
       </c>
       <c r="M5" s="1">
-        <v>46251</v>
+        <v>46254</v>
       </c>
       <c r="N5" t="s">
         <v>572</v>
@@ -10528,7 +10528,7 @@
         <v>571</v>
       </c>
       <c r="M8" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10613,7 +10613,7 @@
         <v>567</v>
       </c>
       <c r="M10" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10657,7 +10657,7 @@
         <v>567</v>
       </c>
       <c r="M11" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10824,7 +10824,7 @@
         <v>571</v>
       </c>
       <c r="M15" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10868,7 +10868,7 @@
         <v>567</v>
       </c>
       <c r="M16" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10912,7 +10912,7 @@
         <v>571</v>
       </c>
       <c r="M17" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10956,7 +10956,7 @@
         <v>567</v>
       </c>
       <c r="M18" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -11000,7 +11000,7 @@
         <v>567</v>
       </c>
       <c r="M19" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11044,7 +11044,7 @@
         <v>567</v>
       </c>
       <c r="M20" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11088,7 +11088,7 @@
         <v>567</v>
       </c>
       <c r="M21" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11255,7 +11255,7 @@
         <v>567</v>
       </c>
       <c r="M25" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11340,7 +11340,7 @@
         <v>571</v>
       </c>
       <c r="M27" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11384,7 +11384,7 @@
         <v>567</v>
       </c>
       <c r="M28" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11428,7 +11428,7 @@
         <v>567</v>
       </c>
       <c r="M29" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11472,7 +11472,7 @@
         <v>567</v>
       </c>
       <c r="M30" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>571</v>
       </c>
       <c r="M32" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>571</v>
       </c>
       <c r="M33" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>571</v>
       </c>
       <c r="M34" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>571</v>
       </c>
       <c r="M35" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>571</v>
       </c>
       <c r="M36" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>571</v>
       </c>
       <c r="M37" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>571</v>
       </c>
       <c r="M38" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>571</v>
       </c>
       <c r="M39" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>571</v>
       </c>
       <c r="M40" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>567</v>
       </c>
       <c r="M41" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>571</v>
       </c>
       <c r="M42" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12082,7 +12082,7 @@
         <v>567</v>
       </c>
       <c r="M44" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12126,7 +12126,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12170,7 +12170,7 @@
         <v>571</v>
       </c>
       <c r="M46" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12214,7 +12214,7 @@
         <v>571</v>
       </c>
       <c r="M47" s="1">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12299,7 +12299,7 @@
         <v>567</v>
       </c>
       <c r="M49" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12343,7 +12343,7 @@
         <v>567</v>
       </c>
       <c r="M50" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12387,7 +12387,7 @@
         <v>567</v>
       </c>
       <c r="M51" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12431,7 +12431,7 @@
         <v>567</v>
       </c>
       <c r="M52" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12475,7 +12475,7 @@
         <v>567</v>
       </c>
       <c r="M53" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12519,7 +12519,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46331</v>
+        <v>46334</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12563,7 +12563,7 @@
         <v>567</v>
       </c>
       <c r="M55" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12607,7 +12607,7 @@
         <v>569</v>
       </c>
       <c r="M56" s="1">
-        <v>46331</v>
+        <v>46334</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12651,7 +12651,7 @@
         <v>569</v>
       </c>
       <c r="M57" s="1">
-        <v>46331</v>
+        <v>46334</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12695,7 +12695,7 @@
         <v>569</v>
       </c>
       <c r="M58" s="1">
-        <v>46331</v>
+        <v>46334</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12739,7 +12739,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12783,7 +12783,7 @@
         <v>569</v>
       </c>
       <c r="M60" s="1">
-        <v>46331</v>
+        <v>46334</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12827,7 +12827,7 @@
         <v>567</v>
       </c>
       <c r="M61" s="1">
-        <v>46316</v>
+        <v>46319</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (11/08/2026 08:52)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10402,7 +10402,7 @@
         <v>570</v>
       </c>
       <c r="M5" s="1">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N5" t="s">
         <v>572</v>
@@ -10528,7 +10528,7 @@
         <v>571</v>
       </c>
       <c r="M8" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10613,7 +10613,7 @@
         <v>567</v>
       </c>
       <c r="M10" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10657,7 +10657,7 @@
         <v>567</v>
       </c>
       <c r="M11" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10824,7 +10824,7 @@
         <v>571</v>
       </c>
       <c r="M15" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10868,7 +10868,7 @@
         <v>567</v>
       </c>
       <c r="M16" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10912,7 +10912,7 @@
         <v>571</v>
       </c>
       <c r="M17" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10956,7 +10956,7 @@
         <v>567</v>
       </c>
       <c r="M18" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -11000,7 +11000,7 @@
         <v>567</v>
       </c>
       <c r="M19" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11044,7 +11044,7 @@
         <v>567</v>
       </c>
       <c r="M20" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11088,7 +11088,7 @@
         <v>567</v>
       </c>
       <c r="M21" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11255,7 +11255,7 @@
         <v>567</v>
       </c>
       <c r="M25" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11340,7 +11340,7 @@
         <v>571</v>
       </c>
       <c r="M27" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11384,7 +11384,7 @@
         <v>567</v>
       </c>
       <c r="M28" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11428,7 +11428,7 @@
         <v>567</v>
       </c>
       <c r="M29" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11472,7 +11472,7 @@
         <v>567</v>
       </c>
       <c r="M30" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>571</v>
       </c>
       <c r="M32" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>571</v>
       </c>
       <c r="M33" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>571</v>
       </c>
       <c r="M34" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>571</v>
       </c>
       <c r="M35" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>571</v>
       </c>
       <c r="M36" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>571</v>
       </c>
       <c r="M37" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>571</v>
       </c>
       <c r="M38" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>571</v>
       </c>
       <c r="M39" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>571</v>
       </c>
       <c r="M40" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>567</v>
       </c>
       <c r="M41" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>571</v>
       </c>
       <c r="M42" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12082,7 +12082,7 @@
         <v>567</v>
       </c>
       <c r="M44" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12126,7 +12126,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12170,7 +12170,7 @@
         <v>571</v>
       </c>
       <c r="M46" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12214,7 +12214,7 @@
         <v>571</v>
       </c>
       <c r="M47" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12299,7 +12299,7 @@
         <v>567</v>
       </c>
       <c r="M49" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12343,7 +12343,7 @@
         <v>567</v>
       </c>
       <c r="M50" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12387,7 +12387,7 @@
         <v>567</v>
       </c>
       <c r="M51" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12431,7 +12431,7 @@
         <v>567</v>
       </c>
       <c r="M52" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12475,7 +12475,7 @@
         <v>567</v>
       </c>
       <c r="M53" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12519,7 +12519,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12563,7 +12563,7 @@
         <v>567</v>
       </c>
       <c r="M55" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12607,7 +12607,7 @@
         <v>569</v>
       </c>
       <c r="M56" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12651,7 +12651,7 @@
         <v>569</v>
       </c>
       <c r="M57" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12695,7 +12695,7 @@
         <v>569</v>
       </c>
       <c r="M58" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12739,7 +12739,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12783,7 +12783,7 @@
         <v>569</v>
       </c>
       <c r="M60" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12827,7 +12827,7 @@
         <v>567</v>
       </c>
       <c r="M61" s="1">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (12/08/2026 08:55)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10402,7 +10402,7 @@
         <v>570</v>
       </c>
       <c r="M5" s="1">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="N5" t="s">
         <v>572</v>
@@ -10528,7 +10528,7 @@
         <v>571</v>
       </c>
       <c r="M8" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10613,7 +10613,7 @@
         <v>567</v>
       </c>
       <c r="M10" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10657,7 +10657,7 @@
         <v>567</v>
       </c>
       <c r="M11" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10824,7 +10824,7 @@
         <v>571</v>
       </c>
       <c r="M15" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10868,7 +10868,7 @@
         <v>567</v>
       </c>
       <c r="M16" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10912,7 +10912,7 @@
         <v>571</v>
       </c>
       <c r="M17" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10956,7 +10956,7 @@
         <v>567</v>
       </c>
       <c r="M18" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -11000,7 +11000,7 @@
         <v>567</v>
       </c>
       <c r="M19" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11044,7 +11044,7 @@
         <v>567</v>
       </c>
       <c r="M20" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11088,7 +11088,7 @@
         <v>567</v>
       </c>
       <c r="M21" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11255,7 +11255,7 @@
         <v>567</v>
       </c>
       <c r="M25" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11340,7 +11340,7 @@
         <v>571</v>
       </c>
       <c r="M27" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11384,7 +11384,7 @@
         <v>567</v>
       </c>
       <c r="M28" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11428,7 +11428,7 @@
         <v>567</v>
       </c>
       <c r="M29" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11472,7 +11472,7 @@
         <v>567</v>
       </c>
       <c r="M30" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>571</v>
       </c>
       <c r="M32" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>571</v>
       </c>
       <c r="M33" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>571</v>
       </c>
       <c r="M34" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>571</v>
       </c>
       <c r="M35" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>571</v>
       </c>
       <c r="M36" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>571</v>
       </c>
       <c r="M37" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>571</v>
       </c>
       <c r="M38" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>571</v>
       </c>
       <c r="M39" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>571</v>
       </c>
       <c r="M40" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>567</v>
       </c>
       <c r="M41" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>571</v>
       </c>
       <c r="M42" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12082,7 +12082,7 @@
         <v>567</v>
       </c>
       <c r="M44" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12126,7 +12126,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12170,7 +12170,7 @@
         <v>571</v>
       </c>
       <c r="M46" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12214,7 +12214,7 @@
         <v>571</v>
       </c>
       <c r="M47" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12299,7 +12299,7 @@
         <v>567</v>
       </c>
       <c r="M49" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12343,7 +12343,7 @@
         <v>567</v>
       </c>
       <c r="M50" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12387,7 +12387,7 @@
         <v>567</v>
       </c>
       <c r="M51" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12431,7 +12431,7 @@
         <v>567</v>
       </c>
       <c r="M52" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12475,7 +12475,7 @@
         <v>567</v>
       </c>
       <c r="M53" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12519,7 +12519,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12563,7 +12563,7 @@
         <v>567</v>
       </c>
       <c r="M55" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12607,7 +12607,7 @@
         <v>569</v>
       </c>
       <c r="M56" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12651,7 +12651,7 @@
         <v>569</v>
       </c>
       <c r="M57" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12695,7 +12695,7 @@
         <v>569</v>
       </c>
       <c r="M58" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12739,7 +12739,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12783,7 +12783,7 @@
         <v>569</v>
       </c>
       <c r="M60" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12827,7 +12827,7 @@
         <v>567</v>
       </c>
       <c r="M61" s="1">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (12/08/2026 15:02)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1712,25 +1712,25 @@
     <t>Empenho Solicitado</t>
   </si>
   <si>
-    <t>Aguardando Intenção de Recurso</t>
-  </si>
-  <si>
     <t>Em Cotação</t>
   </si>
   <si>
+    <t>Selecionada em Plano</t>
+  </si>
+  <si>
+    <t>Análise do Pedido</t>
+  </si>
+  <si>
+    <t>Mapa Gerado</t>
+  </si>
+  <si>
+    <t>Selecionada para cotação</t>
+  </si>
+  <si>
     <t>Validada</t>
   </si>
   <si>
     <t>Em Discrepância</t>
-  </si>
-  <si>
-    <t>Análise do Pedido</t>
-  </si>
-  <si>
-    <t>Mapa Gerado</t>
-  </si>
-  <si>
-    <t>Selecionada para cotação</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10390,16 +10390,16 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>565</v>
+        <v>380</v>
       </c>
       <c r="J5" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K5" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L5" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M5" s="1">
         <v>46256</v>
@@ -10516,16 +10516,16 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J8" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K8" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L8" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M8" s="1">
         <v>46291</v>
@@ -10604,13 +10604,13 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K10" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L10" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M10" s="1">
         <v>46321</v>
@@ -10648,13 +10648,13 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K11" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L11" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M11" s="1">
         <v>46321</v>
@@ -10812,16 +10812,16 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J15" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K15" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L15" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M15" s="1">
         <v>46291</v>
@@ -10859,13 +10859,13 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K16" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L16" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M16" s="1">
         <v>46321</v>
@@ -10900,16 +10900,16 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J17" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K17" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L17" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M17" s="1">
         <v>46291</v>
@@ -10947,13 +10947,13 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K18" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L18" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M18" s="1">
         <v>46321</v>
@@ -10991,13 +10991,13 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K19" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L19" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M19" s="1">
         <v>46321</v>
@@ -11035,13 +11035,13 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K20" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L20" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M20" s="1">
         <v>46321</v>
@@ -11079,13 +11079,13 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K21" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L21" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M21" s="1">
         <v>46321</v>
@@ -11243,16 +11243,16 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J25" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K25" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L25" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M25" s="1">
         <v>46321</v>
@@ -11328,16 +11328,16 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J27" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K27" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L27" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M27" s="1">
         <v>46291</v>
@@ -11375,13 +11375,13 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K28" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L28" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M28" s="1">
         <v>46321</v>
@@ -11416,16 +11416,16 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J29" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K29" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L29" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M29" s="1">
         <v>46321</v>
@@ -11463,13 +11463,13 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K30" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L30" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M30" s="1">
         <v>46321</v>
@@ -11504,16 +11504,16 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J31" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K31" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L31" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="N31" t="s">
         <v>395</v>
@@ -11545,16 +11545,16 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J32" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K32" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L32" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M32" s="1">
         <v>46291</v>
@@ -11589,16 +11589,16 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J33" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K33" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L33" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M33" s="1">
         <v>46291</v>
@@ -11633,16 +11633,16 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J34" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K34" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L34" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M34" s="1">
         <v>46291</v>
@@ -11677,16 +11677,16 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J35" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K35" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L35" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M35" s="1">
         <v>46291</v>
@@ -11721,16 +11721,16 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J36" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K36" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L36" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M36" s="1">
         <v>46291</v>
@@ -11765,16 +11765,16 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J37" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K37" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L37" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M37" s="1">
         <v>46291</v>
@@ -11809,16 +11809,16 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J38" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K38" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L38" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M38" s="1">
         <v>46291</v>
@@ -11853,16 +11853,16 @@
         <v>312.36</v>
       </c>
       <c r="I39" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J39" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K39" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L39" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M39" s="1">
         <v>46291</v>
@@ -11897,16 +11897,16 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J40" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K40" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L40" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M40" s="1">
         <v>46291</v>
@@ -11944,13 +11944,13 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K41" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L41" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M41" s="1">
         <v>46321</v>
@@ -11985,16 +11985,16 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J42" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K42" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L42" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M42" s="1">
         <v>46291</v>
@@ -12029,16 +12029,16 @@
         <v>5000</v>
       </c>
       <c r="I43" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="J43" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K43" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L43" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="N43" t="s">
         <v>395</v>
@@ -12073,13 +12073,13 @@
         <v>382</v>
       </c>
       <c r="J44" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K44" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L44" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M44" s="1">
         <v>46321</v>
@@ -12114,16 +12114,16 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>382</v>
+        <v>567</v>
       </c>
       <c r="J45" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K45" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L45" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M45" s="1">
         <v>46321</v>
@@ -12158,16 +12158,16 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J46" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K46" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L46" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M46" s="1">
         <v>46291</v>
@@ -12202,16 +12202,16 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J47" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K47" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L47" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M47" s="1">
         <v>46291</v>
@@ -12246,16 +12246,16 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="J48" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K48" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L48" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="N48" t="s">
         <v>395</v>
@@ -12287,16 +12287,16 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J49" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K49" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L49" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M49" s="1">
         <v>46321</v>
@@ -12331,16 +12331,16 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J50" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K50" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L50" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M50" s="1">
         <v>46321</v>
@@ -12378,13 +12378,13 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K51" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L51" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M51" s="1">
         <v>46321</v>
@@ -12422,13 +12422,13 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K52" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L52" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M52" s="1">
         <v>46321</v>
@@ -12466,13 +12466,13 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K53" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L53" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M53" s="1">
         <v>46321</v>
@@ -12507,16 +12507,16 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="J54" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="K54" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="L54" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="M54" s="1">
         <v>46336</v>
@@ -12554,13 +12554,13 @@
         <v>382</v>
       </c>
       <c r="J55" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K55" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L55" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M55" s="1">
         <v>46321</v>
@@ -12595,16 +12595,16 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="J56" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="K56" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="L56" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="M56" s="1">
         <v>46336</v>
@@ -12639,16 +12639,16 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
+        <v>566</v>
+      </c>
+      <c r="J57" t="s">
         <v>567</v>
       </c>
-      <c r="J57" t="s">
-        <v>569</v>
-      </c>
       <c r="K57" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="L57" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="M57" s="1">
         <v>46336</v>
@@ -12683,16 +12683,16 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="J58" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="K58" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="L58" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="M58" s="1">
         <v>46336</v>
@@ -12721,22 +12721,22 @@
         <v>2</v>
       </c>
       <c r="G59">
-        <v>435</v>
+        <v>434.99</v>
       </c>
       <c r="H59">
-        <v>870</v>
+        <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="J59" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K59" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L59" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M59" s="1">
         <v>46321</v>
@@ -12771,16 +12771,16 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="J60" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="K60" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="L60" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="M60" s="1">
         <v>46336</v>
@@ -12815,16 +12815,16 @@
         <v>5645.05</v>
       </c>
       <c r="I61" t="s">
-        <v>382</v>
+        <v>566</v>
       </c>
       <c r="J61" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K61" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L61" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M61" s="1">
         <v>46321</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (12/08/2026 17:04)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="570">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1721,16 +1721,7 @@
     <t>Análise do Pedido</t>
   </si>
   <si>
-    <t>Mapa Gerado</t>
-  </si>
-  <si>
-    <t>Selecionada para cotação</t>
-  </si>
-  <si>
     <t>Validada</t>
-  </si>
-  <si>
-    <t>Em Discrepância</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10393,19 +10384,16 @@
         <v>380</v>
       </c>
       <c r="J5" t="s">
-        <v>568</v>
+        <v>380</v>
       </c>
       <c r="K5" t="s">
-        <v>568</v>
+        <v>380</v>
       </c>
       <c r="L5" t="s">
-        <v>568</v>
-      </c>
-      <c r="M5" s="1">
-        <v>46256</v>
+        <v>380</v>
       </c>
       <c r="N5" t="s">
-        <v>572</v>
+        <v>395</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -10519,19 +10507,19 @@
         <v>565</v>
       </c>
       <c r="J8" t="s">
+        <v>565</v>
+      </c>
+      <c r="K8" t="s">
+        <v>565</v>
+      </c>
+      <c r="L8" t="s">
+        <v>565</v>
+      </c>
+      <c r="M8" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N8" t="s">
         <v>569</v>
-      </c>
-      <c r="K8" t="s">
-        <v>569</v>
-      </c>
-      <c r="L8" t="s">
-        <v>569</v>
-      </c>
-      <c r="M8" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N8" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10604,19 +10592,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K10" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L10" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M10" s="1">
         <v>46321</v>
       </c>
       <c r="N10" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10648,19 +10636,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K11" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L11" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M11" s="1">
         <v>46321</v>
       </c>
       <c r="N11" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10815,19 +10803,19 @@
         <v>565</v>
       </c>
       <c r="J15" t="s">
+        <v>565</v>
+      </c>
+      <c r="K15" t="s">
+        <v>565</v>
+      </c>
+      <c r="L15" t="s">
+        <v>565</v>
+      </c>
+      <c r="M15" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N15" t="s">
         <v>569</v>
-      </c>
-      <c r="K15" t="s">
-        <v>569</v>
-      </c>
-      <c r="L15" t="s">
-        <v>569</v>
-      </c>
-      <c r="M15" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N15" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10859,19 +10847,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K16" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L16" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M16" s="1">
         <v>46321</v>
       </c>
       <c r="N16" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10903,19 +10891,19 @@
         <v>565</v>
       </c>
       <c r="J17" t="s">
+        <v>565</v>
+      </c>
+      <c r="K17" t="s">
+        <v>565</v>
+      </c>
+      <c r="L17" t="s">
+        <v>565</v>
+      </c>
+      <c r="M17" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N17" t="s">
         <v>569</v>
-      </c>
-      <c r="K17" t="s">
-        <v>569</v>
-      </c>
-      <c r="L17" t="s">
-        <v>569</v>
-      </c>
-      <c r="M17" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N17" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10947,19 +10935,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K18" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L18" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M18" s="1">
         <v>46321</v>
       </c>
       <c r="N18" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10991,19 +10979,19 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K19" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L19" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M19" s="1">
         <v>46321</v>
       </c>
       <c r="N19" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11035,19 +11023,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K20" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L20" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M20" s="1">
         <v>46321</v>
       </c>
       <c r="N20" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11079,19 +11067,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K21" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L21" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M21" s="1">
         <v>46321</v>
       </c>
       <c r="N21" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11246,19 +11234,19 @@
         <v>566</v>
       </c>
       <c r="J25" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K25" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L25" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M25" s="1">
         <v>46321</v>
       </c>
       <c r="N25" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11331,19 +11319,19 @@
         <v>565</v>
       </c>
       <c r="J27" t="s">
+        <v>565</v>
+      </c>
+      <c r="K27" t="s">
+        <v>565</v>
+      </c>
+      <c r="L27" t="s">
+        <v>565</v>
+      </c>
+      <c r="M27" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N27" t="s">
         <v>569</v>
-      </c>
-      <c r="K27" t="s">
-        <v>569</v>
-      </c>
-      <c r="L27" t="s">
-        <v>569</v>
-      </c>
-      <c r="M27" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N27" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11375,19 +11363,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K28" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L28" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M28" s="1">
         <v>46321</v>
       </c>
       <c r="N28" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11419,19 +11407,19 @@
         <v>566</v>
       </c>
       <c r="J29" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K29" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L29" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M29" s="1">
         <v>46321</v>
       </c>
       <c r="N29" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11463,19 +11451,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K30" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L30" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M30" s="1">
         <v>46321</v>
       </c>
       <c r="N30" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11507,16 +11495,19 @@
         <v>566</v>
       </c>
       <c r="J31" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="K31" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="L31" t="s">
-        <v>571</v>
+        <v>568</v>
+      </c>
+      <c r="M31" s="1">
+        <v>46321</v>
       </c>
       <c r="N31" t="s">
-        <v>395</v>
+        <v>569</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11548,19 +11539,19 @@
         <v>565</v>
       </c>
       <c r="J32" t="s">
+        <v>565</v>
+      </c>
+      <c r="K32" t="s">
+        <v>565</v>
+      </c>
+      <c r="L32" t="s">
+        <v>565</v>
+      </c>
+      <c r="M32" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N32" t="s">
         <v>569</v>
-      </c>
-      <c r="K32" t="s">
-        <v>569</v>
-      </c>
-      <c r="L32" t="s">
-        <v>569</v>
-      </c>
-      <c r="M32" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N32" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11592,19 +11583,19 @@
         <v>565</v>
       </c>
       <c r="J33" t="s">
+        <v>565</v>
+      </c>
+      <c r="K33" t="s">
+        <v>565</v>
+      </c>
+      <c r="L33" t="s">
+        <v>565</v>
+      </c>
+      <c r="M33" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N33" t="s">
         <v>569</v>
-      </c>
-      <c r="K33" t="s">
-        <v>569</v>
-      </c>
-      <c r="L33" t="s">
-        <v>569</v>
-      </c>
-      <c r="M33" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N33" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11636,19 +11627,19 @@
         <v>565</v>
       </c>
       <c r="J34" t="s">
+        <v>565</v>
+      </c>
+      <c r="K34" t="s">
+        <v>565</v>
+      </c>
+      <c r="L34" t="s">
+        <v>565</v>
+      </c>
+      <c r="M34" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N34" t="s">
         <v>569</v>
-      </c>
-      <c r="K34" t="s">
-        <v>569</v>
-      </c>
-      <c r="L34" t="s">
-        <v>569</v>
-      </c>
-      <c r="M34" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N34" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11680,19 +11671,19 @@
         <v>565</v>
       </c>
       <c r="J35" t="s">
+        <v>565</v>
+      </c>
+      <c r="K35" t="s">
+        <v>565</v>
+      </c>
+      <c r="L35" t="s">
+        <v>565</v>
+      </c>
+      <c r="M35" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N35" t="s">
         <v>569</v>
-      </c>
-      <c r="K35" t="s">
-        <v>569</v>
-      </c>
-      <c r="L35" t="s">
-        <v>569</v>
-      </c>
-      <c r="M35" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N35" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11724,19 +11715,19 @@
         <v>565</v>
       </c>
       <c r="J36" t="s">
+        <v>565</v>
+      </c>
+      <c r="K36" t="s">
+        <v>565</v>
+      </c>
+      <c r="L36" t="s">
+        <v>565</v>
+      </c>
+      <c r="M36" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N36" t="s">
         <v>569</v>
-      </c>
-      <c r="K36" t="s">
-        <v>569</v>
-      </c>
-      <c r="L36" t="s">
-        <v>569</v>
-      </c>
-      <c r="M36" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N36" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11768,19 +11759,19 @@
         <v>565</v>
       </c>
       <c r="J37" t="s">
+        <v>565</v>
+      </c>
+      <c r="K37" t="s">
+        <v>565</v>
+      </c>
+      <c r="L37" t="s">
+        <v>565</v>
+      </c>
+      <c r="M37" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N37" t="s">
         <v>569</v>
-      </c>
-      <c r="K37" t="s">
-        <v>569</v>
-      </c>
-      <c r="L37" t="s">
-        <v>569</v>
-      </c>
-      <c r="M37" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N37" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11812,19 +11803,19 @@
         <v>565</v>
       </c>
       <c r="J38" t="s">
+        <v>565</v>
+      </c>
+      <c r="K38" t="s">
+        <v>565</v>
+      </c>
+      <c r="L38" t="s">
+        <v>565</v>
+      </c>
+      <c r="M38" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N38" t="s">
         <v>569</v>
-      </c>
-      <c r="K38" t="s">
-        <v>569</v>
-      </c>
-      <c r="L38" t="s">
-        <v>569</v>
-      </c>
-      <c r="M38" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N38" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11856,19 +11847,19 @@
         <v>565</v>
       </c>
       <c r="J39" t="s">
+        <v>565</v>
+      </c>
+      <c r="K39" t="s">
+        <v>565</v>
+      </c>
+      <c r="L39" t="s">
+        <v>565</v>
+      </c>
+      <c r="M39" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N39" t="s">
         <v>569</v>
-      </c>
-      <c r="K39" t="s">
-        <v>569</v>
-      </c>
-      <c r="L39" t="s">
-        <v>569</v>
-      </c>
-      <c r="M39" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N39" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11900,19 +11891,19 @@
         <v>565</v>
       </c>
       <c r="J40" t="s">
+        <v>565</v>
+      </c>
+      <c r="K40" t="s">
+        <v>565</v>
+      </c>
+      <c r="L40" t="s">
+        <v>565</v>
+      </c>
+      <c r="M40" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N40" t="s">
         <v>569</v>
-      </c>
-      <c r="K40" t="s">
-        <v>569</v>
-      </c>
-      <c r="L40" t="s">
-        <v>569</v>
-      </c>
-      <c r="M40" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N40" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11944,19 +11935,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K41" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L41" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M41" s="1">
         <v>46321</v>
       </c>
       <c r="N41" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11988,19 +11979,19 @@
         <v>565</v>
       </c>
       <c r="J42" t="s">
+        <v>565</v>
+      </c>
+      <c r="K42" t="s">
+        <v>565</v>
+      </c>
+      <c r="L42" t="s">
+        <v>565</v>
+      </c>
+      <c r="M42" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N42" t="s">
         <v>569</v>
-      </c>
-      <c r="K42" t="s">
-        <v>569</v>
-      </c>
-      <c r="L42" t="s">
-        <v>569</v>
-      </c>
-      <c r="M42" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N42" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -12032,16 +12023,19 @@
         <v>567</v>
       </c>
       <c r="J43" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="K43" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="L43" t="s">
-        <v>571</v>
+        <v>567</v>
+      </c>
+      <c r="M43" s="1">
+        <v>46336</v>
       </c>
       <c r="N43" t="s">
-        <v>395</v>
+        <v>569</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12073,19 +12067,19 @@
         <v>382</v>
       </c>
       <c r="J44" t="s">
-        <v>570</v>
+        <v>392</v>
       </c>
       <c r="K44" t="s">
-        <v>570</v>
+        <v>392</v>
       </c>
       <c r="L44" t="s">
-        <v>570</v>
+        <v>392</v>
       </c>
       <c r="M44" s="1">
-        <v>46321</v>
+        <v>46326</v>
       </c>
       <c r="N44" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12117,19 +12111,19 @@
         <v>567</v>
       </c>
       <c r="J45" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="K45" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="L45" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46321</v>
+        <v>46336</v>
       </c>
       <c r="N45" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12161,19 +12155,19 @@
         <v>565</v>
       </c>
       <c r="J46" t="s">
+        <v>565</v>
+      </c>
+      <c r="K46" t="s">
+        <v>565</v>
+      </c>
+      <c r="L46" t="s">
+        <v>565</v>
+      </c>
+      <c r="M46" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N46" t="s">
         <v>569</v>
-      </c>
-      <c r="K46" t="s">
-        <v>569</v>
-      </c>
-      <c r="L46" t="s">
-        <v>569</v>
-      </c>
-      <c r="M46" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N46" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12205,19 +12199,19 @@
         <v>565</v>
       </c>
       <c r="J47" t="s">
+        <v>565</v>
+      </c>
+      <c r="K47" t="s">
+        <v>565</v>
+      </c>
+      <c r="L47" t="s">
+        <v>565</v>
+      </c>
+      <c r="M47" s="1">
+        <v>46276</v>
+      </c>
+      <c r="N47" t="s">
         <v>569</v>
-      </c>
-      <c r="K47" t="s">
-        <v>569</v>
-      </c>
-      <c r="L47" t="s">
-        <v>569</v>
-      </c>
-      <c r="M47" s="1">
-        <v>46291</v>
-      </c>
-      <c r="N47" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12249,16 +12243,19 @@
         <v>567</v>
       </c>
       <c r="J48" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="K48" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="L48" t="s">
-        <v>571</v>
+        <v>567</v>
+      </c>
+      <c r="M48" s="1">
+        <v>46336</v>
       </c>
       <c r="N48" t="s">
-        <v>395</v>
+        <v>569</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12290,19 +12287,19 @@
         <v>566</v>
       </c>
       <c r="J49" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K49" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L49" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M49" s="1">
         <v>46321</v>
       </c>
       <c r="N49" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12334,19 +12331,19 @@
         <v>566</v>
       </c>
       <c r="J50" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K50" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L50" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M50" s="1">
         <v>46321</v>
       </c>
       <c r="N50" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12378,19 +12375,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K51" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L51" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M51" s="1">
         <v>46321</v>
       </c>
       <c r="N51" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12422,19 +12419,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K52" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L52" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M52" s="1">
         <v>46321</v>
       </c>
       <c r="N52" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12466,19 +12463,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K53" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L53" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M53" s="1">
         <v>46321</v>
       </c>
       <c r="N53" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12522,7 +12519,7 @@
         <v>46336</v>
       </c>
       <c r="N54" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12554,19 +12551,19 @@
         <v>382</v>
       </c>
       <c r="J55" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K55" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L55" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M55" s="1">
         <v>46321</v>
       </c>
       <c r="N55" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12598,19 +12595,19 @@
         <v>566</v>
       </c>
       <c r="J56" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K56" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="L56" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="M56" s="1">
-        <v>46336</v>
+        <v>46321</v>
       </c>
       <c r="N56" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12642,19 +12639,19 @@
         <v>566</v>
       </c>
       <c r="J57" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K57" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="L57" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="M57" s="1">
-        <v>46336</v>
+        <v>46321</v>
       </c>
       <c r="N57" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12686,19 +12683,19 @@
         <v>566</v>
       </c>
       <c r="J58" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K58" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="L58" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="M58" s="1">
-        <v>46336</v>
+        <v>46321</v>
       </c>
       <c r="N58" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -12730,19 +12727,19 @@
         <v>567</v>
       </c>
       <c r="J59" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="K59" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="L59" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46321</v>
+        <v>46336</v>
       </c>
       <c r="N59" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -12774,19 +12771,19 @@
         <v>566</v>
       </c>
       <c r="J60" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="K60" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="L60" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="M60" s="1">
-        <v>46336</v>
+        <v>46321</v>
       </c>
       <c r="N60" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -12818,19 +12815,19 @@
         <v>566</v>
       </c>
       <c r="J61" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="K61" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="L61" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M61" s="1">
         <v>46321</v>
       </c>
       <c r="N61" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (13/08/2026 08:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10516,7 +10516,7 @@
         <v>565</v>
       </c>
       <c r="M8" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N8" t="s">
         <v>569</v>
@@ -10601,7 +10601,7 @@
         <v>568</v>
       </c>
       <c r="M10" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N10" t="s">
         <v>569</v>
@@ -10645,7 +10645,7 @@
         <v>568</v>
       </c>
       <c r="M11" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N11" t="s">
         <v>569</v>
@@ -10812,7 +10812,7 @@
         <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N15" t="s">
         <v>569</v>
@@ -10856,7 +10856,7 @@
         <v>568</v>
       </c>
       <c r="M16" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N16" t="s">
         <v>569</v>
@@ -10900,7 +10900,7 @@
         <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N17" t="s">
         <v>569</v>
@@ -10944,7 +10944,7 @@
         <v>568</v>
       </c>
       <c r="M18" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N18" t="s">
         <v>569</v>
@@ -10988,7 +10988,7 @@
         <v>568</v>
       </c>
       <c r="M19" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N19" t="s">
         <v>569</v>
@@ -11032,7 +11032,7 @@
         <v>568</v>
       </c>
       <c r="M20" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N20" t="s">
         <v>569</v>
@@ -11076,7 +11076,7 @@
         <v>568</v>
       </c>
       <c r="M21" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N21" t="s">
         <v>569</v>
@@ -11243,7 +11243,7 @@
         <v>568</v>
       </c>
       <c r="M25" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N25" t="s">
         <v>569</v>
@@ -11328,7 +11328,7 @@
         <v>565</v>
       </c>
       <c r="M27" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N27" t="s">
         <v>569</v>
@@ -11372,7 +11372,7 @@
         <v>568</v>
       </c>
       <c r="M28" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N28" t="s">
         <v>569</v>
@@ -11416,7 +11416,7 @@
         <v>568</v>
       </c>
       <c r="M29" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N29" t="s">
         <v>569</v>
@@ -11460,7 +11460,7 @@
         <v>568</v>
       </c>
       <c r="M30" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N30" t="s">
         <v>569</v>
@@ -11504,7 +11504,7 @@
         <v>568</v>
       </c>
       <c r="M31" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N31" t="s">
         <v>569</v>
@@ -11548,7 +11548,7 @@
         <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N32" t="s">
         <v>569</v>
@@ -11592,7 +11592,7 @@
         <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N33" t="s">
         <v>569</v>
@@ -11636,7 +11636,7 @@
         <v>565</v>
       </c>
       <c r="M34" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N34" t="s">
         <v>569</v>
@@ -11680,7 +11680,7 @@
         <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N35" t="s">
         <v>569</v>
@@ -11724,7 +11724,7 @@
         <v>565</v>
       </c>
       <c r="M36" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N36" t="s">
         <v>569</v>
@@ -11768,7 +11768,7 @@
         <v>565</v>
       </c>
       <c r="M37" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N37" t="s">
         <v>569</v>
@@ -11812,7 +11812,7 @@
         <v>565</v>
       </c>
       <c r="M38" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N38" t="s">
         <v>569</v>
@@ -11856,7 +11856,7 @@
         <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N39" t="s">
         <v>569</v>
@@ -11900,7 +11900,7 @@
         <v>565</v>
       </c>
       <c r="M40" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N40" t="s">
         <v>569</v>
@@ -11944,7 +11944,7 @@
         <v>568</v>
       </c>
       <c r="M41" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N41" t="s">
         <v>569</v>
@@ -11988,7 +11988,7 @@
         <v>565</v>
       </c>
       <c r="M42" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N42" t="s">
         <v>569</v>
@@ -12032,7 +12032,7 @@
         <v>567</v>
       </c>
       <c r="M43" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N43" t="s">
         <v>569</v>
@@ -12076,7 +12076,7 @@
         <v>392</v>
       </c>
       <c r="M44" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N44" t="s">
         <v>569</v>
@@ -12120,7 +12120,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N45" t="s">
         <v>569</v>
@@ -12164,7 +12164,7 @@
         <v>565</v>
       </c>
       <c r="M46" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N46" t="s">
         <v>569</v>
@@ -12208,7 +12208,7 @@
         <v>565</v>
       </c>
       <c r="M47" s="1">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="N47" t="s">
         <v>569</v>
@@ -12252,7 +12252,7 @@
         <v>567</v>
       </c>
       <c r="M48" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N48" t="s">
         <v>569</v>
@@ -12296,7 +12296,7 @@
         <v>568</v>
       </c>
       <c r="M49" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N49" t="s">
         <v>569</v>
@@ -12340,7 +12340,7 @@
         <v>568</v>
       </c>
       <c r="M50" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N50" t="s">
         <v>569</v>
@@ -12384,7 +12384,7 @@
         <v>568</v>
       </c>
       <c r="M51" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N51" t="s">
         <v>569</v>
@@ -12428,7 +12428,7 @@
         <v>568</v>
       </c>
       <c r="M52" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N52" t="s">
         <v>569</v>
@@ -12472,7 +12472,7 @@
         <v>568</v>
       </c>
       <c r="M53" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N53" t="s">
         <v>569</v>
@@ -12516,7 +12516,7 @@
         <v>567</v>
       </c>
       <c r="M54" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N54" t="s">
         <v>569</v>
@@ -12560,7 +12560,7 @@
         <v>568</v>
       </c>
       <c r="M55" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N55" t="s">
         <v>569</v>
@@ -12604,7 +12604,7 @@
         <v>568</v>
       </c>
       <c r="M56" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N56" t="s">
         <v>569</v>
@@ -12648,7 +12648,7 @@
         <v>568</v>
       </c>
       <c r="M57" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N57" t="s">
         <v>569</v>
@@ -12692,7 +12692,7 @@
         <v>568</v>
       </c>
       <c r="M58" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N58" t="s">
         <v>569</v>
@@ -12736,7 +12736,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N59" t="s">
         <v>569</v>
@@ -12780,7 +12780,7 @@
         <v>568</v>
       </c>
       <c r="M60" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N60" t="s">
         <v>569</v>
@@ -12824,7 +12824,7 @@
         <v>568</v>
       </c>
       <c r="M61" s="1">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="N61" t="s">
         <v>569</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (14/08/2026 08:53)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10516,7 +10516,7 @@
         <v>565</v>
       </c>
       <c r="M8" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N8" t="s">
         <v>569</v>
@@ -10601,7 +10601,7 @@
         <v>568</v>
       </c>
       <c r="M10" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N10" t="s">
         <v>569</v>
@@ -10645,7 +10645,7 @@
         <v>568</v>
       </c>
       <c r="M11" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N11" t="s">
         <v>569</v>
@@ -10812,7 +10812,7 @@
         <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N15" t="s">
         <v>569</v>
@@ -10856,7 +10856,7 @@
         <v>568</v>
       </c>
       <c r="M16" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N16" t="s">
         <v>569</v>
@@ -10900,7 +10900,7 @@
         <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N17" t="s">
         <v>569</v>
@@ -10944,7 +10944,7 @@
         <v>568</v>
       </c>
       <c r="M18" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N18" t="s">
         <v>569</v>
@@ -10988,7 +10988,7 @@
         <v>568</v>
       </c>
       <c r="M19" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N19" t="s">
         <v>569</v>
@@ -11032,7 +11032,7 @@
         <v>568</v>
       </c>
       <c r="M20" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N20" t="s">
         <v>569</v>
@@ -11076,7 +11076,7 @@
         <v>568</v>
       </c>
       <c r="M21" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N21" t="s">
         <v>569</v>
@@ -11243,7 +11243,7 @@
         <v>568</v>
       </c>
       <c r="M25" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N25" t="s">
         <v>569</v>
@@ -11328,7 +11328,7 @@
         <v>565</v>
       </c>
       <c r="M27" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N27" t="s">
         <v>569</v>
@@ -11372,7 +11372,7 @@
         <v>568</v>
       </c>
       <c r="M28" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N28" t="s">
         <v>569</v>
@@ -11416,7 +11416,7 @@
         <v>568</v>
       </c>
       <c r="M29" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N29" t="s">
         <v>569</v>
@@ -11460,7 +11460,7 @@
         <v>568</v>
       </c>
       <c r="M30" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N30" t="s">
         <v>569</v>
@@ -11504,7 +11504,7 @@
         <v>568</v>
       </c>
       <c r="M31" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N31" t="s">
         <v>569</v>
@@ -11548,7 +11548,7 @@
         <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N32" t="s">
         <v>569</v>
@@ -11592,7 +11592,7 @@
         <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N33" t="s">
         <v>569</v>
@@ -11636,7 +11636,7 @@
         <v>565</v>
       </c>
       <c r="M34" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N34" t="s">
         <v>569</v>
@@ -11680,7 +11680,7 @@
         <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N35" t="s">
         <v>569</v>
@@ -11724,7 +11724,7 @@
         <v>565</v>
       </c>
       <c r="M36" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N36" t="s">
         <v>569</v>
@@ -11768,7 +11768,7 @@
         <v>565</v>
       </c>
       <c r="M37" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N37" t="s">
         <v>569</v>
@@ -11812,7 +11812,7 @@
         <v>565</v>
       </c>
       <c r="M38" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N38" t="s">
         <v>569</v>
@@ -11856,7 +11856,7 @@
         <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N39" t="s">
         <v>569</v>
@@ -11900,7 +11900,7 @@
         <v>565</v>
       </c>
       <c r="M40" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N40" t="s">
         <v>569</v>
@@ -11944,7 +11944,7 @@
         <v>568</v>
       </c>
       <c r="M41" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N41" t="s">
         <v>569</v>
@@ -11988,7 +11988,7 @@
         <v>565</v>
       </c>
       <c r="M42" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N42" t="s">
         <v>569</v>
@@ -12032,7 +12032,7 @@
         <v>567</v>
       </c>
       <c r="M43" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N43" t="s">
         <v>569</v>
@@ -12076,7 +12076,7 @@
         <v>392</v>
       </c>
       <c r="M44" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N44" t="s">
         <v>569</v>
@@ -12120,7 +12120,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N45" t="s">
         <v>569</v>
@@ -12164,7 +12164,7 @@
         <v>565</v>
       </c>
       <c r="M46" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N46" t="s">
         <v>569</v>
@@ -12208,7 +12208,7 @@
         <v>565</v>
       </c>
       <c r="M47" s="1">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="N47" t="s">
         <v>569</v>
@@ -12252,7 +12252,7 @@
         <v>567</v>
       </c>
       <c r="M48" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N48" t="s">
         <v>569</v>
@@ -12296,7 +12296,7 @@
         <v>568</v>
       </c>
       <c r="M49" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N49" t="s">
         <v>569</v>
@@ -12340,7 +12340,7 @@
         <v>568</v>
       </c>
       <c r="M50" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N50" t="s">
         <v>569</v>
@@ -12384,7 +12384,7 @@
         <v>568</v>
       </c>
       <c r="M51" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N51" t="s">
         <v>569</v>
@@ -12428,7 +12428,7 @@
         <v>568</v>
       </c>
       <c r="M52" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N52" t="s">
         <v>569</v>
@@ -12472,7 +12472,7 @@
         <v>568</v>
       </c>
       <c r="M53" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N53" t="s">
         <v>569</v>
@@ -12516,7 +12516,7 @@
         <v>567</v>
       </c>
       <c r="M54" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N54" t="s">
         <v>569</v>
@@ -12560,7 +12560,7 @@
         <v>568</v>
       </c>
       <c r="M55" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N55" t="s">
         <v>569</v>
@@ -12604,7 +12604,7 @@
         <v>568</v>
       </c>
       <c r="M56" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N56" t="s">
         <v>569</v>
@@ -12648,7 +12648,7 @@
         <v>568</v>
       </c>
       <c r="M57" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N57" t="s">
         <v>569</v>
@@ -12692,7 +12692,7 @@
         <v>568</v>
       </c>
       <c r="M58" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N58" t="s">
         <v>569</v>
@@ -12736,7 +12736,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N59" t="s">
         <v>569</v>
@@ -12780,7 +12780,7 @@
         <v>568</v>
       </c>
       <c r="M60" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N60" t="s">
         <v>569</v>
@@ -12824,7 +12824,7 @@
         <v>568</v>
       </c>
       <c r="M61" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="N61" t="s">
         <v>569</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (17/08/2026 08:35)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10516,7 +10516,7 @@
         <v>565</v>
       </c>
       <c r="M8" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N8" t="s">
         <v>569</v>
@@ -10601,7 +10601,7 @@
         <v>568</v>
       </c>
       <c r="M10" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N10" t="s">
         <v>569</v>
@@ -10645,7 +10645,7 @@
         <v>568</v>
       </c>
       <c r="M11" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N11" t="s">
         <v>569</v>
@@ -10812,7 +10812,7 @@
         <v>565</v>
       </c>
       <c r="M15" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N15" t="s">
         <v>569</v>
@@ -10856,7 +10856,7 @@
         <v>568</v>
       </c>
       <c r="M16" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N16" t="s">
         <v>569</v>
@@ -10900,7 +10900,7 @@
         <v>565</v>
       </c>
       <c r="M17" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N17" t="s">
         <v>569</v>
@@ -10944,7 +10944,7 @@
         <v>568</v>
       </c>
       <c r="M18" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N18" t="s">
         <v>569</v>
@@ -10988,7 +10988,7 @@
         <v>568</v>
       </c>
       <c r="M19" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N19" t="s">
         <v>569</v>
@@ -11032,7 +11032,7 @@
         <v>568</v>
       </c>
       <c r="M20" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N20" t="s">
         <v>569</v>
@@ -11076,7 +11076,7 @@
         <v>568</v>
       </c>
       <c r="M21" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N21" t="s">
         <v>569</v>
@@ -11243,7 +11243,7 @@
         <v>568</v>
       </c>
       <c r="M25" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N25" t="s">
         <v>569</v>
@@ -11328,7 +11328,7 @@
         <v>565</v>
       </c>
       <c r="M27" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N27" t="s">
         <v>569</v>
@@ -11372,7 +11372,7 @@
         <v>568</v>
       </c>
       <c r="M28" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N28" t="s">
         <v>569</v>
@@ -11416,7 +11416,7 @@
         <v>568</v>
       </c>
       <c r="M29" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N29" t="s">
         <v>569</v>
@@ -11460,7 +11460,7 @@
         <v>568</v>
       </c>
       <c r="M30" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N30" t="s">
         <v>569</v>
@@ -11504,7 +11504,7 @@
         <v>568</v>
       </c>
       <c r="M31" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N31" t="s">
         <v>569</v>
@@ -11548,7 +11548,7 @@
         <v>565</v>
       </c>
       <c r="M32" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N32" t="s">
         <v>569</v>
@@ -11592,7 +11592,7 @@
         <v>565</v>
       </c>
       <c r="M33" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N33" t="s">
         <v>569</v>
@@ -11636,7 +11636,7 @@
         <v>565</v>
       </c>
       <c r="M34" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N34" t="s">
         <v>569</v>
@@ -11680,7 +11680,7 @@
         <v>565</v>
       </c>
       <c r="M35" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N35" t="s">
         <v>569</v>
@@ -11724,7 +11724,7 @@
         <v>565</v>
       </c>
       <c r="M36" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N36" t="s">
         <v>569</v>
@@ -11768,7 +11768,7 @@
         <v>565</v>
       </c>
       <c r="M37" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N37" t="s">
         <v>569</v>
@@ -11812,7 +11812,7 @@
         <v>565</v>
       </c>
       <c r="M38" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N38" t="s">
         <v>569</v>
@@ -11856,7 +11856,7 @@
         <v>565</v>
       </c>
       <c r="M39" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N39" t="s">
         <v>569</v>
@@ -11900,7 +11900,7 @@
         <v>565</v>
       </c>
       <c r="M40" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N40" t="s">
         <v>569</v>
@@ -11944,7 +11944,7 @@
         <v>568</v>
       </c>
       <c r="M41" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N41" t="s">
         <v>569</v>
@@ -11988,7 +11988,7 @@
         <v>565</v>
       </c>
       <c r="M42" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N42" t="s">
         <v>569</v>
@@ -12032,7 +12032,7 @@
         <v>567</v>
       </c>
       <c r="M43" s="1">
-        <v>46338</v>
+        <v>46341</v>
       </c>
       <c r="N43" t="s">
         <v>569</v>
@@ -12076,7 +12076,7 @@
         <v>392</v>
       </c>
       <c r="M44" s="1">
-        <v>46328</v>
+        <v>46331</v>
       </c>
       <c r="N44" t="s">
         <v>569</v>
@@ -12120,7 +12120,7 @@
         <v>567</v>
       </c>
       <c r="M45" s="1">
-        <v>46338</v>
+        <v>46341</v>
       </c>
       <c r="N45" t="s">
         <v>569</v>
@@ -12164,7 +12164,7 @@
         <v>565</v>
       </c>
       <c r="M46" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N46" t="s">
         <v>569</v>
@@ -12208,7 +12208,7 @@
         <v>565</v>
       </c>
       <c r="M47" s="1">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="N47" t="s">
         <v>569</v>
@@ -12252,7 +12252,7 @@
         <v>567</v>
       </c>
       <c r="M48" s="1">
-        <v>46338</v>
+        <v>46341</v>
       </c>
       <c r="N48" t="s">
         <v>569</v>
@@ -12296,7 +12296,7 @@
         <v>568</v>
       </c>
       <c r="M49" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N49" t="s">
         <v>569</v>
@@ -12340,7 +12340,7 @@
         <v>568</v>
       </c>
       <c r="M50" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N50" t="s">
         <v>569</v>
@@ -12384,7 +12384,7 @@
         <v>568</v>
       </c>
       <c r="M51" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N51" t="s">
         <v>569</v>
@@ -12428,7 +12428,7 @@
         <v>568</v>
       </c>
       <c r="M52" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N52" t="s">
         <v>569</v>
@@ -12472,7 +12472,7 @@
         <v>568</v>
       </c>
       <c r="M53" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N53" t="s">
         <v>569</v>
@@ -12516,7 +12516,7 @@
         <v>567</v>
       </c>
       <c r="M54" s="1">
-        <v>46338</v>
+        <v>46341</v>
       </c>
       <c r="N54" t="s">
         <v>569</v>
@@ -12560,7 +12560,7 @@
         <v>568</v>
       </c>
       <c r="M55" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N55" t="s">
         <v>569</v>
@@ -12604,7 +12604,7 @@
         <v>568</v>
       </c>
       <c r="M56" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N56" t="s">
         <v>569</v>
@@ -12648,7 +12648,7 @@
         <v>568</v>
       </c>
       <c r="M57" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N57" t="s">
         <v>569</v>
@@ -12692,7 +12692,7 @@
         <v>568</v>
       </c>
       <c r="M58" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N58" t="s">
         <v>569</v>
@@ -12736,7 +12736,7 @@
         <v>567</v>
       </c>
       <c r="M59" s="1">
-        <v>46338</v>
+        <v>46341</v>
       </c>
       <c r="N59" t="s">
         <v>569</v>
@@ -12780,7 +12780,7 @@
         <v>568</v>
       </c>
       <c r="M60" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N60" t="s">
         <v>569</v>
@@ -12824,7 +12824,7 @@
         <v>568</v>
       </c>
       <c r="M61" s="1">
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="N61" t="s">
         <v>569</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (17/08/2026 14:36)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2505" uniqueCount="573">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1415,6 +1415,9 @@
     <t>LST216004U8</t>
   </si>
   <si>
+    <t>LST225001U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1571,6 +1574,9 @@
     <t>S3100-527</t>
   </si>
   <si>
+    <t>71014</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1707,6 +1713,9 @@
   </si>
   <si>
     <t>NAV STROBE LIGHT ASSEMBLYRIGHT</t>
+  </si>
+  <si>
+    <t>CAP - Confirmation of the requested PN and condition of the material is required..</t>
   </si>
   <si>
     <t>Empenho Solicitado</t>
@@ -10176,7 +10185,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q61"/>
+  <dimension ref="A1:Q62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10258,7 +10267,7 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J2" t="s">
         <v>387</v>
@@ -10299,7 +10308,7 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J3" t="s">
         <v>387</v>
@@ -10325,7 +10334,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10340,7 +10349,7 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J4" t="s">
         <v>387</v>
@@ -10366,10 +10375,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E5" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10422,7 +10431,7 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J6" t="s">
         <v>387</v>
@@ -10463,7 +10472,7 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J7" t="s">
         <v>387</v>
@@ -10504,22 +10513,22 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J8" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K8" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L8" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M8" s="1">
         <v>46281</v>
       </c>
       <c r="N8" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10533,7 +10542,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10548,7 +10557,7 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J9" t="s">
         <v>387</v>
@@ -10574,10 +10583,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E10" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10592,19 +10601,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K10" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L10" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M10" s="1">
         <v>46326</v>
       </c>
       <c r="N10" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10618,7 +10627,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10636,19 +10645,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K11" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L11" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M11" s="1">
         <v>46326</v>
       </c>
       <c r="N11" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10662,10 +10671,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E12" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -10718,7 +10727,7 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J13" t="s">
         <v>387</v>
@@ -10744,10 +10753,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E14" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -10759,7 +10768,7 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J14" t="s">
         <v>387</v>
@@ -10785,10 +10794,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E15" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -10800,22 +10809,22 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J15" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K15" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L15" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M15" s="1">
         <v>46281</v>
       </c>
       <c r="N15" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10829,10 +10838,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E16" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -10847,19 +10856,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K16" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L16" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M16" s="1">
         <v>46326</v>
       </c>
       <c r="N16" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10873,10 +10882,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E17" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -10888,22 +10897,22 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J17" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K17" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L17" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M17" s="1">
         <v>46281</v>
       </c>
       <c r="N17" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10917,10 +10926,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E18" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -10935,19 +10944,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K18" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L18" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M18" s="1">
         <v>46326</v>
       </c>
       <c r="N18" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10961,10 +10970,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E19" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="F19">
         <v>4</v>
@@ -10979,19 +10988,19 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K19" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L19" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M19" s="1">
         <v>46326</v>
       </c>
       <c r="N19" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11005,10 +11014,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E20" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -11023,19 +11032,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K20" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L20" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M20" s="1">
         <v>46326</v>
       </c>
       <c r="N20" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11049,10 +11058,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E21" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11067,19 +11076,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K21" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L21" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M21" s="1">
         <v>46326</v>
       </c>
       <c r="N21" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11093,10 +11102,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E22" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11108,7 +11117,7 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J22" t="s">
         <v>387</v>
@@ -11134,10 +11143,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E23" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11149,7 +11158,7 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J23" t="s">
         <v>387</v>
@@ -11175,7 +11184,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11190,7 +11199,7 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J24" t="s">
         <v>387</v>
@@ -11216,10 +11225,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E25" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11231,22 +11240,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J25" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K25" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L25" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M25" s="1">
         <v>46326</v>
       </c>
       <c r="N25" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11260,10 +11269,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E26" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11275,7 +11284,7 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="J26" t="s">
         <v>387</v>
@@ -11301,10 +11310,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E27" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11316,22 +11325,22 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J27" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K27" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L27" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M27" s="1">
         <v>46281</v>
       </c>
       <c r="N27" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11345,10 +11354,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E28" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11363,19 +11372,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K28" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L28" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M28" s="1">
         <v>46326</v>
       </c>
       <c r="N28" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11389,10 +11398,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E29" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11404,22 +11413,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J29" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K29" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L29" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M29" s="1">
         <v>46326</v>
       </c>
       <c r="N29" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11433,10 +11442,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E30" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11451,19 +11460,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K30" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L30" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M30" s="1">
         <v>46326</v>
       </c>
       <c r="N30" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11477,10 +11486,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E31" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11492,22 +11501,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J31" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K31" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L31" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M31" s="1">
         <v>46326</v>
       </c>
       <c r="N31" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11521,10 +11530,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E32" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11536,22 +11545,22 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J32" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K32" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L32" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M32" s="1">
         <v>46281</v>
       </c>
       <c r="N32" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11565,10 +11574,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E33" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11580,22 +11589,22 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J33" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K33" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L33" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M33" s="1">
         <v>46281</v>
       </c>
       <c r="N33" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11609,10 +11618,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E34" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11624,22 +11633,22 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J34" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K34" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L34" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M34" s="1">
         <v>46281</v>
       </c>
       <c r="N34" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11653,10 +11662,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E35" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11668,22 +11677,22 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J35" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K35" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L35" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M35" s="1">
         <v>46281</v>
       </c>
       <c r="N35" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11697,10 +11706,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E36" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -11712,22 +11721,22 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J36" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K36" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L36" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M36" s="1">
         <v>46281</v>
       </c>
       <c r="N36" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11741,10 +11750,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E37" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -11756,22 +11765,22 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J37" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K37" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L37" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M37" s="1">
         <v>46281</v>
       </c>
       <c r="N37" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11785,10 +11794,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E38" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -11800,22 +11809,22 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J38" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K38" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L38" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M38" s="1">
         <v>46281</v>
       </c>
       <c r="N38" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11829,10 +11838,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E39" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -11844,22 +11853,22 @@
         <v>312.36</v>
       </c>
       <c r="I39" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J39" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K39" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L39" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M39" s="1">
         <v>46281</v>
       </c>
       <c r="N39" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11873,10 +11882,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E40" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -11888,22 +11897,22 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J40" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K40" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L40" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M40" s="1">
         <v>46281</v>
       </c>
       <c r="N40" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11917,10 +11926,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E41" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -11935,19 +11944,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K41" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L41" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M41" s="1">
         <v>46326</v>
       </c>
       <c r="N41" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11976,22 +11985,22 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J42" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K42" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L42" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M42" s="1">
         <v>46281</v>
       </c>
       <c r="N42" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -12005,10 +12014,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E43" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -12020,22 +12029,22 @@
         <v>5000</v>
       </c>
       <c r="I43" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="J43" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K43" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L43" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M43" s="1">
         <v>46341</v>
       </c>
       <c r="N43" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12049,22 +12058,22 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
       </c>
       <c r="F44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G44">
-        <v>163.13</v>
+        <v>176.26</v>
       </c>
       <c r="H44">
-        <v>163.13</v>
+        <v>352.52</v>
       </c>
       <c r="I44" t="s">
-        <v>382</v>
+        <v>570</v>
       </c>
       <c r="J44" t="s">
         <v>392</v>
@@ -12079,7 +12088,7 @@
         <v>46331</v>
       </c>
       <c r="N44" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12093,10 +12102,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E45" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12108,22 +12117,22 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="J45" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K45" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L45" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M45" s="1">
         <v>46341</v>
       </c>
       <c r="N45" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12137,10 +12146,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="E46" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12152,22 +12161,22 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J46" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K46" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L46" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M46" s="1">
         <v>46281</v>
       </c>
       <c r="N46" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12181,10 +12190,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E47" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12196,22 +12205,22 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="J47" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="K47" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="L47" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="M47" s="1">
         <v>46281</v>
       </c>
       <c r="N47" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12225,10 +12234,10 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E48" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -12240,22 +12249,22 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="J48" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K48" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L48" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M48" s="1">
         <v>46341</v>
       </c>
       <c r="N48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12269,10 +12278,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E49" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12284,22 +12293,22 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J49" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K49" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L49" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M49" s="1">
         <v>46326</v>
       </c>
       <c r="N49" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12313,10 +12322,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E50" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12328,22 +12337,22 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J50" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K50" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L50" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M50" s="1">
         <v>46326</v>
       </c>
       <c r="N50" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12357,10 +12366,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E51" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12375,19 +12384,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K51" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L51" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M51" s="1">
         <v>46326</v>
       </c>
       <c r="N51" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12401,10 +12410,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E52" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12419,19 +12428,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K52" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L52" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M52" s="1">
         <v>46326</v>
       </c>
       <c r="N52" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12445,10 +12454,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E53" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12463,19 +12472,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K53" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L53" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M53" s="1">
         <v>46326</v>
       </c>
       <c r="N53" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12489,10 +12498,10 @@
         <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E54" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F54">
         <v>4</v>
@@ -12504,22 +12513,22 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="J54" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K54" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L54" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M54" s="1">
         <v>46341</v>
       </c>
       <c r="N54" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12533,10 +12542,10 @@
         <v>173</v>
       </c>
       <c r="D55" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E55" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="F55">
         <v>1</v>
@@ -12551,19 +12560,19 @@
         <v>382</v>
       </c>
       <c r="J55" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K55" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L55" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M55" s="1">
         <v>46326</v>
       </c>
       <c r="N55" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12577,10 +12586,10 @@
         <v>173</v>
       </c>
       <c r="D56" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E56" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -12592,22 +12601,22 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J56" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K56" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L56" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M56" s="1">
         <v>46326</v>
       </c>
       <c r="N56" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12621,10 +12630,10 @@
         <v>173</v>
       </c>
       <c r="D57" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E57" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -12636,22 +12645,22 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J57" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K57" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L57" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M57" s="1">
         <v>46326</v>
       </c>
       <c r="N57" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12665,10 +12674,10 @@
         <v>173</v>
       </c>
       <c r="D58" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E58" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="F58">
         <v>4</v>
@@ -12680,22 +12689,22 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J58" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K58" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L58" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M58" s="1">
         <v>46326</v>
       </c>
       <c r="N58" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -12724,22 +12733,22 @@
         <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="J59" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="K59" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="L59" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="M59" s="1">
         <v>46341</v>
       </c>
       <c r="N59" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -12753,10 +12762,10 @@
         <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E60" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -12768,22 +12777,22 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J60" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K60" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L60" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M60" s="1">
         <v>46326</v>
       </c>
       <c r="N60" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -12797,10 +12806,10 @@
         <v>173</v>
       </c>
       <c r="D61" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E61" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="F61">
         <v>5</v>
@@ -12812,22 +12821,63 @@
         <v>5645.05</v>
       </c>
       <c r="I61" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="J61" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K61" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="L61" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="M61" s="1">
         <v>46326</v>
       </c>
       <c r="N61" t="s">
-        <v>569</v>
+        <v>572</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
+      <c r="A62" t="s">
+        <v>466</v>
+      </c>
+      <c r="B62" t="s">
+        <v>172</v>
+      </c>
+      <c r="C62" t="s">
+        <v>173</v>
+      </c>
+      <c r="D62" t="s">
+        <v>519</v>
+      </c>
+      <c r="E62" t="s">
+        <v>566</v>
+      </c>
+      <c r="F62">
+        <v>21</v>
+      </c>
+      <c r="G62">
+        <v>9.76</v>
+      </c>
+      <c r="H62">
+        <v>204.96</v>
+      </c>
+      <c r="I62" t="s">
+        <v>570</v>
+      </c>
+      <c r="K62" t="s">
+        <v>570</v>
+      </c>
+      <c r="L62" t="s">
+        <v>570</v>
+      </c>
+      <c r="M62" s="1">
+        <v>46341</v>
+      </c>
+      <c r="N62" t="s">
+        <v>572</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (17/08/2026 16:36)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2505" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="573">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1715,7 +1715,7 @@
     <t>NAV STROBE LIGHT ASSEMBLYRIGHT</t>
   </si>
   <si>
-    <t>CAP - Confirmation of the requested PN and condition of the material is required..</t>
+    <t>CAP</t>
   </si>
   <si>
     <t>Empenho Solicitado</t>
@@ -12076,16 +12076,16 @@
         <v>570</v>
       </c>
       <c r="J44" t="s">
-        <v>392</v>
+        <v>570</v>
       </c>
       <c r="K44" t="s">
-        <v>392</v>
+        <v>570</v>
       </c>
       <c r="L44" t="s">
-        <v>392</v>
+        <v>570</v>
       </c>
       <c r="M44" s="1">
-        <v>46331</v>
+        <v>46341</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12252,16 +12252,16 @@
         <v>571</v>
       </c>
       <c r="J48" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K48" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L48" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M48" s="1">
-        <v>46341</v>
+        <v>46326</v>
       </c>
       <c r="N48" t="s">
         <v>572</v>
@@ -12516,16 +12516,16 @@
         <v>571</v>
       </c>
       <c r="J54" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K54" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L54" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M54" s="1">
-        <v>46341</v>
+        <v>46326</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12865,6 +12865,9 @@
         <v>204.96</v>
       </c>
       <c r="I62" t="s">
+        <v>570</v>
+      </c>
+      <c r="J62" t="s">
         <v>570</v>
       </c>
       <c r="K62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (18/08/2026 08:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10525,7 +10525,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10610,7 +10610,7 @@
         <v>571</v>
       </c>
       <c r="M10" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10654,7 +10654,7 @@
         <v>571</v>
       </c>
       <c r="M11" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10821,7 +10821,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10865,7 +10865,7 @@
         <v>571</v>
       </c>
       <c r="M16" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10909,7 +10909,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10953,7 +10953,7 @@
         <v>571</v>
       </c>
       <c r="M18" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -10997,7 +10997,7 @@
         <v>571</v>
       </c>
       <c r="M19" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11041,7 +11041,7 @@
         <v>571</v>
       </c>
       <c r="M20" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11085,7 +11085,7 @@
         <v>571</v>
       </c>
       <c r="M21" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11252,7 +11252,7 @@
         <v>571</v>
       </c>
       <c r="M25" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11337,7 +11337,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11381,7 +11381,7 @@
         <v>571</v>
       </c>
       <c r="M28" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11425,7 +11425,7 @@
         <v>571</v>
       </c>
       <c r="M29" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11469,7 +11469,7 @@
         <v>571</v>
       </c>
       <c r="M30" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11513,7 +11513,7 @@
         <v>571</v>
       </c>
       <c r="M31" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N31" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>571</v>
       </c>
       <c r="M41" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12041,7 +12041,7 @@
         <v>570</v>
       </c>
       <c r="M43" s="1">
-        <v>46341</v>
+        <v>46342</v>
       </c>
       <c r="N43" t="s">
         <v>572</v>
@@ -12085,7 +12085,7 @@
         <v>570</v>
       </c>
       <c r="M44" s="1">
-        <v>46341</v>
+        <v>46342</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12129,7 +12129,7 @@
         <v>570</v>
       </c>
       <c r="M45" s="1">
-        <v>46341</v>
+        <v>46342</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12173,7 +12173,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12217,7 +12217,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12261,7 +12261,7 @@
         <v>571</v>
       </c>
       <c r="M48" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N48" t="s">
         <v>572</v>
@@ -12305,7 +12305,7 @@
         <v>571</v>
       </c>
       <c r="M49" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12349,7 +12349,7 @@
         <v>571</v>
       </c>
       <c r="M50" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12393,7 +12393,7 @@
         <v>571</v>
       </c>
       <c r="M51" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12437,7 +12437,7 @@
         <v>571</v>
       </c>
       <c r="M52" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12481,7 +12481,7 @@
         <v>571</v>
       </c>
       <c r="M53" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12525,7 +12525,7 @@
         <v>571</v>
       </c>
       <c r="M54" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12569,7 +12569,7 @@
         <v>571</v>
       </c>
       <c r="M55" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12613,7 +12613,7 @@
         <v>571</v>
       </c>
       <c r="M56" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12657,7 +12657,7 @@
         <v>571</v>
       </c>
       <c r="M57" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12701,7 +12701,7 @@
         <v>571</v>
       </c>
       <c r="M58" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12745,7 +12745,7 @@
         <v>570</v>
       </c>
       <c r="M59" s="1">
-        <v>46341</v>
+        <v>46342</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12789,7 +12789,7 @@
         <v>571</v>
       </c>
       <c r="M60" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12833,7 +12833,7 @@
         <v>571</v>
       </c>
       <c r="M61" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>
@@ -12877,7 +12877,7 @@
         <v>570</v>
       </c>
       <c r="M62" s="1">
-        <v>46341</v>
+        <v>46342</v>
       </c>
       <c r="N62" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (18/08/2026 12:32)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,8 +1743,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1760,7 +1768,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1768,12 +1776,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2073,55 +2099,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2165,7 +2191,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2209,7 +2235,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2253,7 +2279,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2379,7 +2405,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2423,7 +2449,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2467,7 +2493,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2514,7 +2540,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2637,7 +2663,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2681,7 +2707,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2725,7 +2751,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2769,7 +2795,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2816,7 +2842,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2860,7 +2886,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2986,7 +3012,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3030,7 +3056,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3115,7 +3141,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3162,7 +3188,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3209,7 +3235,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3253,7 +3279,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3297,7 +3323,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3382,7 +3408,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3467,7 +3493,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3514,7 +3540,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3558,7 +3584,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3602,7 +3628,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3687,7 +3713,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3731,7 +3757,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3775,7 +3801,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3860,7 +3886,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3904,7 +3930,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3948,7 +3974,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3992,7 +4018,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4159,7 +4185,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4203,7 +4229,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4247,7 +4273,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4291,7 +4317,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4338,7 +4364,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4382,7 +4408,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4596,7 +4622,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4640,7 +4666,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4687,7 +4713,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4731,7 +4757,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4775,7 +4801,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4819,7 +4845,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4910,7 +4936,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4954,7 +4980,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5001,7 +5027,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5045,7 +5071,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5092,7 +5118,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5180,7 +5206,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5224,7 +5250,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5268,7 +5294,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5312,7 +5338,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5356,7 +5382,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5400,7 +5426,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5485,7 +5511,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5529,7 +5555,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5573,7 +5599,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5617,7 +5643,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5661,7 +5687,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5705,7 +5731,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5749,7 +5775,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5793,7 +5819,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5840,7 +5866,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5884,7 +5910,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5928,7 +5954,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5972,7 +5998,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6016,7 +6042,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6060,7 +6086,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6104,7 +6130,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6148,7 +6174,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6192,7 +6218,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6280,7 +6306,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6324,7 +6350,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6450,7 +6476,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6494,7 +6520,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6538,7 +6564,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6582,7 +6608,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6664,7 +6690,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6708,7 +6734,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6755,7 +6781,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6799,7 +6825,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6925,7 +6951,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6969,7 +6995,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7054,7 +7080,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7098,7 +7124,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7142,7 +7168,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7186,7 +7212,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7230,7 +7256,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7274,7 +7300,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7318,7 +7344,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7362,7 +7388,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7447,7 +7473,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7614,7 +7640,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7658,7 +7684,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7702,7 +7728,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7746,7 +7772,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7790,7 +7816,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7834,7 +7860,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7878,7 +7904,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7963,7 +7989,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8007,7 +8033,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8092,7 +8118,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8218,7 +8244,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8262,7 +8288,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8347,7 +8373,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8391,7 +8417,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8435,7 +8461,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8479,7 +8505,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8523,7 +8549,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8567,7 +8593,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8611,7 +8637,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8655,7 +8681,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8740,7 +8766,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8907,7 +8933,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8951,7 +8977,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8995,7 +9021,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9039,7 +9065,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9124,7 +9150,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9168,7 +9194,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9212,7 +9238,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9256,7 +9282,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9300,7 +9326,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9344,7 +9370,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9388,7 +9414,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9432,7 +9458,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9476,7 +9502,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9520,7 +9546,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9564,7 +9590,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9608,7 +9634,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9652,7 +9678,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9696,7 +9722,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9740,7 +9766,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9784,7 +9810,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9828,7 +9854,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9872,7 +9898,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9916,7 +9942,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9960,7 +9986,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10004,7 +10030,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10089,7 +10115,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10174,7 +10200,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10189,55 +10215,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10524,7 +10550,7 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46282</v>
       </c>
       <c r="N8" t="s">
@@ -10609,7 +10635,7 @@
       <c r="L10" t="s">
         <v>571</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46327</v>
       </c>
       <c r="N10" t="s">
@@ -10653,7 +10679,7 @@
       <c r="L11" t="s">
         <v>571</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46327</v>
       </c>
       <c r="N11" t="s">
@@ -10820,7 +10846,7 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46282</v>
       </c>
       <c r="N15" t="s">
@@ -10864,7 +10890,7 @@
       <c r="L16" t="s">
         <v>571</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46327</v>
       </c>
       <c r="N16" t="s">
@@ -10908,7 +10934,7 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46282</v>
       </c>
       <c r="N17" t="s">
@@ -10952,7 +10978,7 @@
       <c r="L18" t="s">
         <v>571</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46327</v>
       </c>
       <c r="N18" t="s">
@@ -10996,7 +11022,7 @@
       <c r="L19" t="s">
         <v>571</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46327</v>
       </c>
       <c r="N19" t="s">
@@ -11040,7 +11066,7 @@
       <c r="L20" t="s">
         <v>571</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46327</v>
       </c>
       <c r="N20" t="s">
@@ -11084,7 +11110,7 @@
       <c r="L21" t="s">
         <v>571</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46327</v>
       </c>
       <c r="N21" t="s">
@@ -11251,7 +11277,7 @@
       <c r="L25" t="s">
         <v>571</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46327</v>
       </c>
       <c r="N25" t="s">
@@ -11336,7 +11362,7 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46282</v>
       </c>
       <c r="N27" t="s">
@@ -11380,7 +11406,7 @@
       <c r="L28" t="s">
         <v>571</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46327</v>
       </c>
       <c r="N28" t="s">
@@ -11424,7 +11450,7 @@
       <c r="L29" t="s">
         <v>571</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46327</v>
       </c>
       <c r="N29" t="s">
@@ -11468,7 +11494,7 @@
       <c r="L30" t="s">
         <v>571</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46327</v>
       </c>
       <c r="N30" t="s">
@@ -11512,7 +11538,7 @@
       <c r="L31" t="s">
         <v>571</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46327</v>
       </c>
       <c r="N31" t="s">
@@ -11556,7 +11582,7 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46282</v>
       </c>
       <c r="N32" t="s">
@@ -11600,7 +11626,7 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46282</v>
       </c>
       <c r="N33" t="s">
@@ -11644,7 +11670,7 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46282</v>
       </c>
       <c r="N34" t="s">
@@ -11688,7 +11714,7 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46282</v>
       </c>
       <c r="N35" t="s">
@@ -11732,7 +11758,7 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46282</v>
       </c>
       <c r="N36" t="s">
@@ -11776,7 +11802,7 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46282</v>
       </c>
       <c r="N37" t="s">
@@ -11820,7 +11846,7 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46282</v>
       </c>
       <c r="N38" t="s">
@@ -11864,7 +11890,7 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="1">
+      <c r="M39" s="2">
         <v>46282</v>
       </c>
       <c r="N39" t="s">
@@ -11908,7 +11934,7 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46282</v>
       </c>
       <c r="N40" t="s">
@@ -11952,7 +11978,7 @@
       <c r="L41" t="s">
         <v>571</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46327</v>
       </c>
       <c r="N41" t="s">
@@ -11996,7 +12022,7 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46282</v>
       </c>
       <c r="N42" t="s">
@@ -12040,7 +12066,7 @@
       <c r="L43" t="s">
         <v>570</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46342</v>
       </c>
       <c r="N43" t="s">
@@ -12084,7 +12110,7 @@
       <c r="L44" t="s">
         <v>570</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46342</v>
       </c>
       <c r="N44" t="s">
@@ -12128,7 +12154,7 @@
       <c r="L45" t="s">
         <v>570</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46342</v>
       </c>
       <c r="N45" t="s">
@@ -12172,7 +12198,7 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46282</v>
       </c>
       <c r="N46" t="s">
@@ -12216,7 +12242,7 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46282</v>
       </c>
       <c r="N47" t="s">
@@ -12260,7 +12286,7 @@
       <c r="L48" t="s">
         <v>571</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46327</v>
       </c>
       <c r="N48" t="s">
@@ -12304,7 +12330,7 @@
       <c r="L49" t="s">
         <v>571</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46327</v>
       </c>
       <c r="N49" t="s">
@@ -12348,7 +12374,7 @@
       <c r="L50" t="s">
         <v>571</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46327</v>
       </c>
       <c r="N50" t="s">
@@ -12392,7 +12418,7 @@
       <c r="L51" t="s">
         <v>571</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46327</v>
       </c>
       <c r="N51" t="s">
@@ -12436,7 +12462,7 @@
       <c r="L52" t="s">
         <v>571</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46327</v>
       </c>
       <c r="N52" t="s">
@@ -12480,7 +12506,7 @@
       <c r="L53" t="s">
         <v>571</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46327</v>
       </c>
       <c r="N53" t="s">
@@ -12524,7 +12550,7 @@
       <c r="L54" t="s">
         <v>571</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46327</v>
       </c>
       <c r="N54" t="s">
@@ -12568,7 +12594,7 @@
       <c r="L55" t="s">
         <v>571</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46327</v>
       </c>
       <c r="N55" t="s">
@@ -12612,7 +12638,7 @@
       <c r="L56" t="s">
         <v>571</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46327</v>
       </c>
       <c r="N56" t="s">
@@ -12656,7 +12682,7 @@
       <c r="L57" t="s">
         <v>571</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46327</v>
       </c>
       <c r="N57" t="s">
@@ -12700,7 +12726,7 @@
       <c r="L58" t="s">
         <v>571</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46327</v>
       </c>
       <c r="N58" t="s">
@@ -12744,7 +12770,7 @@
       <c r="L59" t="s">
         <v>570</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46342</v>
       </c>
       <c r="N59" t="s">
@@ -12788,7 +12814,7 @@
       <c r="L60" t="s">
         <v>571</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46327</v>
       </c>
       <c r="N60" t="s">
@@ -12832,7 +12858,7 @@
       <c r="L61" t="s">
         <v>571</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46327</v>
       </c>
       <c r="N61" t="s">
@@ -12876,7 +12902,7 @@
       <c r="L62" t="s">
         <v>570</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46342</v>
       </c>
       <c r="N62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (18/08/2026 12:40)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,16 +1743,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1768,7 +1760,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1776,30 +1768,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2099,55 +2073,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2191,7 +2165,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2235,7 +2209,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2279,7 +2253,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2405,7 +2379,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2449,7 +2423,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2493,7 +2467,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2540,7 +2514,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2663,7 +2637,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2707,7 +2681,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2751,7 +2725,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2795,7 +2769,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2842,7 +2816,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2886,7 +2860,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3012,7 +2986,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3056,7 +3030,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3141,7 +3115,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3188,7 +3162,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3235,7 +3209,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3279,7 +3253,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3323,7 +3297,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3408,7 +3382,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3493,7 +3467,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3540,7 +3514,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3584,7 +3558,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3628,7 +3602,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3713,7 +3687,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3757,7 +3731,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3801,7 +3775,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3886,7 +3860,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3930,7 +3904,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3974,7 +3948,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4018,7 +3992,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4185,7 +4159,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4229,7 +4203,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4273,7 +4247,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4317,7 +4291,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4364,7 +4338,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4408,7 +4382,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4622,7 +4596,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4666,7 +4640,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4713,7 +4687,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4757,7 +4731,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4801,7 +4775,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4845,7 +4819,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4889,7 +4863,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4936,7 +4910,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4980,7 +4954,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5027,7 +5001,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5071,7 +5045,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5118,7 +5092,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5206,7 +5180,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5250,7 +5224,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5294,7 +5268,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5338,7 +5312,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5382,7 +5356,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5426,7 +5400,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5511,7 +5485,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5555,7 +5529,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5599,7 +5573,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5643,7 +5617,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5687,7 +5661,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5731,7 +5705,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5775,7 +5749,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5819,7 +5793,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5866,7 +5840,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5910,7 +5884,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5954,7 +5928,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5998,7 +5972,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6042,7 +6016,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6086,7 +6060,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6130,7 +6104,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6174,7 +6148,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6218,7 +6192,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6306,7 +6280,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6350,7 +6324,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6476,7 +6450,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6520,7 +6494,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6564,7 +6538,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6608,7 +6582,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6690,7 +6664,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6734,7 +6708,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6781,7 +6755,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6825,7 +6799,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6951,7 +6925,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -6995,7 +6969,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7080,7 +7054,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7124,7 +7098,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7168,7 +7142,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7212,7 +7186,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7256,7 +7230,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7300,7 +7274,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7344,7 +7318,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7388,7 +7362,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7473,7 +7447,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7640,7 +7614,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7684,7 +7658,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7728,7 +7702,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7772,7 +7746,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7816,7 +7790,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7860,7 +7834,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7904,7 +7878,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -7989,7 +7963,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8033,7 +8007,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8118,7 +8092,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8244,7 +8218,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8288,7 +8262,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8373,7 +8347,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8417,7 +8391,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8461,7 +8435,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8505,7 +8479,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8549,7 +8523,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8593,7 +8567,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8637,7 +8611,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8681,7 +8655,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8766,7 +8740,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8933,7 +8907,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8977,7 +8951,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9021,7 +8995,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9065,7 +9039,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9150,7 +9124,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9194,7 +9168,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9238,7 +9212,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9282,7 +9256,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9326,7 +9300,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9370,7 +9344,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9414,7 +9388,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9458,7 +9432,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9502,7 +9476,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9546,7 +9520,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9590,7 +9564,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9634,7 +9608,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9678,7 +9652,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9722,7 +9696,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9766,7 +9740,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9810,7 +9784,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9854,7 +9828,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9898,7 +9872,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9942,7 +9916,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -9986,7 +9960,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10030,7 +10004,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10115,7 +10089,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10200,7 +10174,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10215,55 +10189,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10550,7 +10524,7 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46282</v>
       </c>
       <c r="N8" t="s">
@@ -10635,7 +10609,7 @@
       <c r="L10" t="s">
         <v>571</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46327</v>
       </c>
       <c r="N10" t="s">
@@ -10679,7 +10653,7 @@
       <c r="L11" t="s">
         <v>571</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46327</v>
       </c>
       <c r="N11" t="s">
@@ -10846,7 +10820,7 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46282</v>
       </c>
       <c r="N15" t="s">
@@ -10890,7 +10864,7 @@
       <c r="L16" t="s">
         <v>571</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46327</v>
       </c>
       <c r="N16" t="s">
@@ -10934,7 +10908,7 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46282</v>
       </c>
       <c r="N17" t="s">
@@ -10978,7 +10952,7 @@
       <c r="L18" t="s">
         <v>571</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46327</v>
       </c>
       <c r="N18" t="s">
@@ -11022,7 +10996,7 @@
       <c r="L19" t="s">
         <v>571</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46327</v>
       </c>
       <c r="N19" t="s">
@@ -11066,7 +11040,7 @@
       <c r="L20" t="s">
         <v>571</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46327</v>
       </c>
       <c r="N20" t="s">
@@ -11110,7 +11084,7 @@
       <c r="L21" t="s">
         <v>571</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46327</v>
       </c>
       <c r="N21" t="s">
@@ -11277,7 +11251,7 @@
       <c r="L25" t="s">
         <v>571</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46327</v>
       </c>
       <c r="N25" t="s">
@@ -11362,7 +11336,7 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46282</v>
       </c>
       <c r="N27" t="s">
@@ -11406,7 +11380,7 @@
       <c r="L28" t="s">
         <v>571</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46327</v>
       </c>
       <c r="N28" t="s">
@@ -11450,7 +11424,7 @@
       <c r="L29" t="s">
         <v>571</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46327</v>
       </c>
       <c r="N29" t="s">
@@ -11494,7 +11468,7 @@
       <c r="L30" t="s">
         <v>571</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46327</v>
       </c>
       <c r="N30" t="s">
@@ -11538,7 +11512,7 @@
       <c r="L31" t="s">
         <v>571</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46327</v>
       </c>
       <c r="N31" t="s">
@@ -11582,7 +11556,7 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46282</v>
       </c>
       <c r="N32" t="s">
@@ -11626,7 +11600,7 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46282</v>
       </c>
       <c r="N33" t="s">
@@ -11670,7 +11644,7 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46282</v>
       </c>
       <c r="N34" t="s">
@@ -11714,7 +11688,7 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46282</v>
       </c>
       <c r="N35" t="s">
@@ -11758,7 +11732,7 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46282</v>
       </c>
       <c r="N36" t="s">
@@ -11802,7 +11776,7 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46282</v>
       </c>
       <c r="N37" t="s">
@@ -11846,7 +11820,7 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46282</v>
       </c>
       <c r="N38" t="s">
@@ -11890,7 +11864,7 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="2">
+      <c r="M39" s="1">
         <v>46282</v>
       </c>
       <c r="N39" t="s">
@@ -11934,7 +11908,7 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46282</v>
       </c>
       <c r="N40" t="s">
@@ -11978,7 +11952,7 @@
       <c r="L41" t="s">
         <v>571</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46327</v>
       </c>
       <c r="N41" t="s">
@@ -12022,7 +11996,7 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46282</v>
       </c>
       <c r="N42" t="s">
@@ -12066,7 +12040,7 @@
       <c r="L43" t="s">
         <v>570</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46342</v>
       </c>
       <c r="N43" t="s">
@@ -12110,7 +12084,7 @@
       <c r="L44" t="s">
         <v>570</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46342</v>
       </c>
       <c r="N44" t="s">
@@ -12154,7 +12128,7 @@
       <c r="L45" t="s">
         <v>570</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46342</v>
       </c>
       <c r="N45" t="s">
@@ -12198,7 +12172,7 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46282</v>
       </c>
       <c r="N46" t="s">
@@ -12242,7 +12216,7 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46282</v>
       </c>
       <c r="N47" t="s">
@@ -12286,7 +12260,7 @@
       <c r="L48" t="s">
         <v>571</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46327</v>
       </c>
       <c r="N48" t="s">
@@ -12330,7 +12304,7 @@
       <c r="L49" t="s">
         <v>571</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46327</v>
       </c>
       <c r="N49" t="s">
@@ -12374,7 +12348,7 @@
       <c r="L50" t="s">
         <v>571</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46327</v>
       </c>
       <c r="N50" t="s">
@@ -12418,7 +12392,7 @@
       <c r="L51" t="s">
         <v>571</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46327</v>
       </c>
       <c r="N51" t="s">
@@ -12462,7 +12436,7 @@
       <c r="L52" t="s">
         <v>571</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46327</v>
       </c>
       <c r="N52" t="s">
@@ -12506,7 +12480,7 @@
       <c r="L53" t="s">
         <v>571</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46327</v>
       </c>
       <c r="N53" t="s">
@@ -12550,7 +12524,7 @@
       <c r="L54" t="s">
         <v>571</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46327</v>
       </c>
       <c r="N54" t="s">
@@ -12594,7 +12568,7 @@
       <c r="L55" t="s">
         <v>571</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46327</v>
       </c>
       <c r="N55" t="s">
@@ -12638,7 +12612,7 @@
       <c r="L56" t="s">
         <v>571</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46327</v>
       </c>
       <c r="N56" t="s">
@@ -12682,7 +12656,7 @@
       <c r="L57" t="s">
         <v>571</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46327</v>
       </c>
       <c r="N57" t="s">
@@ -12726,7 +12700,7 @@
       <c r="L58" t="s">
         <v>571</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46327</v>
       </c>
       <c r="N58" t="s">
@@ -12770,7 +12744,7 @@
       <c r="L59" t="s">
         <v>570</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46342</v>
       </c>
       <c r="N59" t="s">
@@ -12814,7 +12788,7 @@
       <c r="L60" t="s">
         <v>571</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46327</v>
       </c>
       <c r="N60" t="s">
@@ -12858,7 +12832,7 @@
       <c r="L61" t="s">
         <v>571</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46327</v>
       </c>
       <c r="N61" t="s">
@@ -12902,7 +12876,7 @@
       <c r="L62" t="s">
         <v>570</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46342</v>
       </c>
       <c r="N62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (19/08/2026 08:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10525,7 +10525,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10610,7 +10610,7 @@
         <v>571</v>
       </c>
       <c r="M10" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10654,7 +10654,7 @@
         <v>571</v>
       </c>
       <c r="M11" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10821,7 +10821,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10865,7 +10865,7 @@
         <v>571</v>
       </c>
       <c r="M16" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10909,7 +10909,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10953,7 +10953,7 @@
         <v>571</v>
       </c>
       <c r="M18" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -10997,7 +10997,7 @@
         <v>571</v>
       </c>
       <c r="M19" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11041,7 +11041,7 @@
         <v>571</v>
       </c>
       <c r="M20" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11085,7 +11085,7 @@
         <v>571</v>
       </c>
       <c r="M21" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11252,7 +11252,7 @@
         <v>571</v>
       </c>
       <c r="M25" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11337,7 +11337,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11381,7 +11381,7 @@
         <v>571</v>
       </c>
       <c r="M28" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11425,7 +11425,7 @@
         <v>571</v>
       </c>
       <c r="M29" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11469,7 +11469,7 @@
         <v>571</v>
       </c>
       <c r="M30" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11513,7 +11513,7 @@
         <v>571</v>
       </c>
       <c r="M31" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N31" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>571</v>
       </c>
       <c r="M41" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12041,7 +12041,7 @@
         <v>570</v>
       </c>
       <c r="M43" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N43" t="s">
         <v>572</v>
@@ -12085,7 +12085,7 @@
         <v>570</v>
       </c>
       <c r="M44" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12129,7 +12129,7 @@
         <v>570</v>
       </c>
       <c r="M45" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12173,7 +12173,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12217,7 +12217,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12261,7 +12261,7 @@
         <v>571</v>
       </c>
       <c r="M48" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N48" t="s">
         <v>572</v>
@@ -12305,7 +12305,7 @@
         <v>571</v>
       </c>
       <c r="M49" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12349,7 +12349,7 @@
         <v>571</v>
       </c>
       <c r="M50" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12393,7 +12393,7 @@
         <v>571</v>
       </c>
       <c r="M51" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12437,7 +12437,7 @@
         <v>571</v>
       </c>
       <c r="M52" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12481,7 +12481,7 @@
         <v>571</v>
       </c>
       <c r="M53" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12525,7 +12525,7 @@
         <v>571</v>
       </c>
       <c r="M54" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12569,7 +12569,7 @@
         <v>571</v>
       </c>
       <c r="M55" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12613,7 +12613,7 @@
         <v>571</v>
       </c>
       <c r="M56" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12657,7 +12657,7 @@
         <v>571</v>
       </c>
       <c r="M57" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12701,7 +12701,7 @@
         <v>571</v>
       </c>
       <c r="M58" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12745,7 +12745,7 @@
         <v>570</v>
       </c>
       <c r="M59" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12789,7 +12789,7 @@
         <v>571</v>
       </c>
       <c r="M60" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12833,7 +12833,7 @@
         <v>571</v>
       </c>
       <c r="M61" s="1">
-        <v>46327</v>
+        <v>46328</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>
@@ -12877,7 +12877,7 @@
         <v>570</v>
       </c>
       <c r="M62" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N62" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (19/08/2026 13:07)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,8 +1743,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1760,7 +1768,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1768,12 +1776,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2073,55 +2099,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2165,7 +2191,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2209,7 +2235,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2253,7 +2279,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2379,7 +2405,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2423,7 +2449,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2467,7 +2493,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2514,7 +2540,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2637,7 +2663,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2681,7 +2707,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2725,7 +2751,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2769,7 +2795,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2816,7 +2842,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2860,7 +2886,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2986,7 +3012,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3030,7 +3056,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3115,7 +3141,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3162,7 +3188,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3209,7 +3235,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3253,7 +3279,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3297,7 +3323,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3382,7 +3408,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3467,7 +3493,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3514,7 +3540,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3558,7 +3584,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3602,7 +3628,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3687,7 +3713,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3731,7 +3757,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3775,7 +3801,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3860,7 +3886,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3904,7 +3930,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3948,7 +3974,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3992,7 +4018,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4159,7 +4185,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4203,7 +4229,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4247,7 +4273,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4291,7 +4317,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4338,7 +4364,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4382,7 +4408,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4596,7 +4622,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4640,7 +4666,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4687,7 +4713,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4731,7 +4757,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4775,7 +4801,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4819,7 +4845,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4910,7 +4936,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4954,7 +4980,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5001,7 +5027,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5045,7 +5071,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5092,7 +5118,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5180,7 +5206,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5224,7 +5250,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5268,7 +5294,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5312,7 +5338,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5356,7 +5382,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5400,7 +5426,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5485,7 +5511,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5529,7 +5555,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5573,7 +5599,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5617,7 +5643,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5661,7 +5687,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5705,7 +5731,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5749,7 +5775,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5793,7 +5819,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5840,7 +5866,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5884,7 +5910,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5928,7 +5954,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5972,7 +5998,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6016,7 +6042,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6060,7 +6086,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6104,7 +6130,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6148,7 +6174,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6192,7 +6218,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6280,7 +6306,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6324,7 +6350,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6450,7 +6476,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6494,7 +6520,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6538,7 +6564,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6582,7 +6608,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6664,7 +6690,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6708,7 +6734,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6755,7 +6781,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6799,7 +6825,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6925,7 +6951,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6969,7 +6995,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7054,7 +7080,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7098,7 +7124,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7142,7 +7168,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7186,7 +7212,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7230,7 +7256,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7274,7 +7300,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7318,7 +7344,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7362,7 +7388,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7447,7 +7473,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7614,7 +7640,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7658,7 +7684,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7702,7 +7728,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7746,7 +7772,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7790,7 +7816,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7834,7 +7860,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7878,7 +7904,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7963,7 +7989,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8007,7 +8033,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8092,7 +8118,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8218,7 +8244,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8262,7 +8288,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8347,7 +8373,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8391,7 +8417,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8435,7 +8461,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8479,7 +8505,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8523,7 +8549,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8567,7 +8593,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8611,7 +8637,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8655,7 +8681,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8740,7 +8766,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8907,7 +8933,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8951,7 +8977,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8995,7 +9021,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9039,7 +9065,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9124,7 +9150,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9168,7 +9194,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9212,7 +9238,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9256,7 +9282,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9300,7 +9326,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9344,7 +9370,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9388,7 +9414,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9432,7 +9458,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9476,7 +9502,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9520,7 +9546,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9564,7 +9590,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9608,7 +9634,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9652,7 +9678,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9696,7 +9722,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9740,7 +9766,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9784,7 +9810,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9828,7 +9854,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9872,7 +9898,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9916,7 +9942,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9960,7 +9986,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10004,7 +10030,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10089,7 +10115,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10174,7 +10200,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10189,55 +10215,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10524,7 +10550,7 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46283</v>
       </c>
       <c r="N8" t="s">
@@ -10609,7 +10635,7 @@
       <c r="L10" t="s">
         <v>571</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46328</v>
       </c>
       <c r="N10" t="s">
@@ -10653,7 +10679,7 @@
       <c r="L11" t="s">
         <v>571</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46328</v>
       </c>
       <c r="N11" t="s">
@@ -10820,7 +10846,7 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46283</v>
       </c>
       <c r="N15" t="s">
@@ -10864,7 +10890,7 @@
       <c r="L16" t="s">
         <v>571</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46328</v>
       </c>
       <c r="N16" t="s">
@@ -10908,7 +10934,7 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46283</v>
       </c>
       <c r="N17" t="s">
@@ -10952,7 +10978,7 @@
       <c r="L18" t="s">
         <v>571</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46328</v>
       </c>
       <c r="N18" t="s">
@@ -10996,7 +11022,7 @@
       <c r="L19" t="s">
         <v>571</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46328</v>
       </c>
       <c r="N19" t="s">
@@ -11040,7 +11066,7 @@
       <c r="L20" t="s">
         <v>571</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46328</v>
       </c>
       <c r="N20" t="s">
@@ -11084,7 +11110,7 @@
       <c r="L21" t="s">
         <v>571</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46328</v>
       </c>
       <c r="N21" t="s">
@@ -11251,7 +11277,7 @@
       <c r="L25" t="s">
         <v>571</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46328</v>
       </c>
       <c r="N25" t="s">
@@ -11336,7 +11362,7 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46283</v>
       </c>
       <c r="N27" t="s">
@@ -11380,7 +11406,7 @@
       <c r="L28" t="s">
         <v>571</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46328</v>
       </c>
       <c r="N28" t="s">
@@ -11424,7 +11450,7 @@
       <c r="L29" t="s">
         <v>571</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46328</v>
       </c>
       <c r="N29" t="s">
@@ -11468,7 +11494,7 @@
       <c r="L30" t="s">
         <v>571</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46328</v>
       </c>
       <c r="N30" t="s">
@@ -11512,7 +11538,7 @@
       <c r="L31" t="s">
         <v>571</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46328</v>
       </c>
       <c r="N31" t="s">
@@ -11556,7 +11582,7 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46283</v>
       </c>
       <c r="N32" t="s">
@@ -11600,7 +11626,7 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46283</v>
       </c>
       <c r="N33" t="s">
@@ -11644,7 +11670,7 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46283</v>
       </c>
       <c r="N34" t="s">
@@ -11688,7 +11714,7 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46283</v>
       </c>
       <c r="N35" t="s">
@@ -11732,7 +11758,7 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46283</v>
       </c>
       <c r="N36" t="s">
@@ -11776,7 +11802,7 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46283</v>
       </c>
       <c r="N37" t="s">
@@ -11820,7 +11846,7 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46283</v>
       </c>
       <c r="N38" t="s">
@@ -11864,7 +11890,7 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="1">
+      <c r="M39" s="2">
         <v>46283</v>
       </c>
       <c r="N39" t="s">
@@ -11908,7 +11934,7 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46283</v>
       </c>
       <c r="N40" t="s">
@@ -11952,7 +11978,7 @@
       <c r="L41" t="s">
         <v>571</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46328</v>
       </c>
       <c r="N41" t="s">
@@ -11996,7 +12022,7 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46283</v>
       </c>
       <c r="N42" t="s">
@@ -12040,7 +12066,7 @@
       <c r="L43" t="s">
         <v>570</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46343</v>
       </c>
       <c r="N43" t="s">
@@ -12084,7 +12110,7 @@
       <c r="L44" t="s">
         <v>570</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46343</v>
       </c>
       <c r="N44" t="s">
@@ -12128,7 +12154,7 @@
       <c r="L45" t="s">
         <v>570</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46343</v>
       </c>
       <c r="N45" t="s">
@@ -12172,7 +12198,7 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46283</v>
       </c>
       <c r="N46" t="s">
@@ -12216,7 +12242,7 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46283</v>
       </c>
       <c r="N47" t="s">
@@ -12260,7 +12286,7 @@
       <c r="L48" t="s">
         <v>571</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46328</v>
       </c>
       <c r="N48" t="s">
@@ -12304,7 +12330,7 @@
       <c r="L49" t="s">
         <v>571</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46328</v>
       </c>
       <c r="N49" t="s">
@@ -12348,7 +12374,7 @@
       <c r="L50" t="s">
         <v>571</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46328</v>
       </c>
       <c r="N50" t="s">
@@ -12392,7 +12418,7 @@
       <c r="L51" t="s">
         <v>571</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46328</v>
       </c>
       <c r="N51" t="s">
@@ -12436,7 +12462,7 @@
       <c r="L52" t="s">
         <v>571</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46328</v>
       </c>
       <c r="N52" t="s">
@@ -12480,7 +12506,7 @@
       <c r="L53" t="s">
         <v>571</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46328</v>
       </c>
       <c r="N53" t="s">
@@ -12524,7 +12550,7 @@
       <c r="L54" t="s">
         <v>571</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46328</v>
       </c>
       <c r="N54" t="s">
@@ -12568,7 +12594,7 @@
       <c r="L55" t="s">
         <v>571</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46328</v>
       </c>
       <c r="N55" t="s">
@@ -12612,7 +12638,7 @@
       <c r="L56" t="s">
         <v>571</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46328</v>
       </c>
       <c r="N56" t="s">
@@ -12656,7 +12682,7 @@
       <c r="L57" t="s">
         <v>571</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46328</v>
       </c>
       <c r="N57" t="s">
@@ -12700,7 +12726,7 @@
       <c r="L58" t="s">
         <v>571</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46328</v>
       </c>
       <c r="N58" t="s">
@@ -12744,7 +12770,7 @@
       <c r="L59" t="s">
         <v>570</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46343</v>
       </c>
       <c r="N59" t="s">
@@ -12788,7 +12814,7 @@
       <c r="L60" t="s">
         <v>571</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46328</v>
       </c>
       <c r="N60" t="s">
@@ -12832,7 +12858,7 @@
       <c r="L61" t="s">
         <v>571</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46328</v>
       </c>
       <c r="N61" t="s">
@@ -12876,7 +12902,7 @@
       <c r="L62" t="s">
         <v>570</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46343</v>
       </c>
       <c r="N62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (19/08/2026 14:35)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,16 +1743,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1768,7 +1760,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1776,30 +1768,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2099,55 +2073,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2191,7 +2165,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2235,7 +2209,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2279,7 +2253,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2405,7 +2379,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2449,7 +2423,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2493,7 +2467,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2540,7 +2514,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2663,7 +2637,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2707,7 +2681,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2751,7 +2725,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2795,7 +2769,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2842,7 +2816,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2886,7 +2860,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3012,7 +2986,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3056,7 +3030,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3141,7 +3115,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3188,7 +3162,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3235,7 +3209,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3279,7 +3253,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3323,7 +3297,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3408,7 +3382,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3493,7 +3467,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3540,7 +3514,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3584,7 +3558,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3628,7 +3602,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3713,7 +3687,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3757,7 +3731,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3801,7 +3775,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3886,7 +3860,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3930,7 +3904,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3974,7 +3948,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4018,7 +3992,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4185,7 +4159,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4229,7 +4203,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4273,7 +4247,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4317,7 +4291,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4364,7 +4338,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4408,7 +4382,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4622,7 +4596,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4666,7 +4640,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4713,7 +4687,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4757,7 +4731,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4801,7 +4775,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4845,7 +4819,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4889,7 +4863,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4936,7 +4910,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4980,7 +4954,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5027,7 +5001,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5071,7 +5045,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5118,7 +5092,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5206,7 +5180,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5250,7 +5224,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5294,7 +5268,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5338,7 +5312,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5382,7 +5356,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5426,7 +5400,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5511,7 +5485,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5555,7 +5529,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5599,7 +5573,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5643,7 +5617,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5687,7 +5661,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5731,7 +5705,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5775,7 +5749,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5819,7 +5793,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5866,7 +5840,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5910,7 +5884,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5954,7 +5928,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5998,7 +5972,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6042,7 +6016,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6086,7 +6060,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6130,7 +6104,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6174,7 +6148,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6218,7 +6192,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6306,7 +6280,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6350,7 +6324,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6476,7 +6450,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6520,7 +6494,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6564,7 +6538,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6608,7 +6582,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6690,7 +6664,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6734,7 +6708,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6781,7 +6755,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6825,7 +6799,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6951,7 +6925,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -6995,7 +6969,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7080,7 +7054,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7124,7 +7098,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7168,7 +7142,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7212,7 +7186,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7256,7 +7230,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7300,7 +7274,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7344,7 +7318,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7388,7 +7362,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7473,7 +7447,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7640,7 +7614,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7684,7 +7658,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7728,7 +7702,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7772,7 +7746,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7816,7 +7790,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7860,7 +7834,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7904,7 +7878,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -7989,7 +7963,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8033,7 +8007,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8118,7 +8092,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8244,7 +8218,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8288,7 +8262,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8373,7 +8347,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8417,7 +8391,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8461,7 +8435,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8505,7 +8479,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8549,7 +8523,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8593,7 +8567,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8637,7 +8611,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8681,7 +8655,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8766,7 +8740,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8933,7 +8907,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8977,7 +8951,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9021,7 +8995,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9065,7 +9039,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9150,7 +9124,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9194,7 +9168,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9238,7 +9212,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9282,7 +9256,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9326,7 +9300,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9370,7 +9344,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9414,7 +9388,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9458,7 +9432,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9502,7 +9476,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9546,7 +9520,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9590,7 +9564,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9634,7 +9608,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9678,7 +9652,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9722,7 +9696,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9766,7 +9740,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9810,7 +9784,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9854,7 +9828,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9898,7 +9872,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9942,7 +9916,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -9986,7 +9960,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10030,7 +10004,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10115,7 +10089,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10200,7 +10174,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10215,55 +10189,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10550,7 +10524,7 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46283</v>
       </c>
       <c r="N8" t="s">
@@ -10635,7 +10609,7 @@
       <c r="L10" t="s">
         <v>571</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46328</v>
       </c>
       <c r="N10" t="s">
@@ -10679,7 +10653,7 @@
       <c r="L11" t="s">
         <v>571</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46328</v>
       </c>
       <c r="N11" t="s">
@@ -10846,7 +10820,7 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46283</v>
       </c>
       <c r="N15" t="s">
@@ -10890,7 +10864,7 @@
       <c r="L16" t="s">
         <v>571</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46328</v>
       </c>
       <c r="N16" t="s">
@@ -10934,7 +10908,7 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46283</v>
       </c>
       <c r="N17" t="s">
@@ -10978,7 +10952,7 @@
       <c r="L18" t="s">
         <v>571</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46328</v>
       </c>
       <c r="N18" t="s">
@@ -11022,7 +10996,7 @@
       <c r="L19" t="s">
         <v>571</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46328</v>
       </c>
       <c r="N19" t="s">
@@ -11066,7 +11040,7 @@
       <c r="L20" t="s">
         <v>571</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46328</v>
       </c>
       <c r="N20" t="s">
@@ -11110,7 +11084,7 @@
       <c r="L21" t="s">
         <v>571</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46328</v>
       </c>
       <c r="N21" t="s">
@@ -11277,7 +11251,7 @@
       <c r="L25" t="s">
         <v>571</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46328</v>
       </c>
       <c r="N25" t="s">
@@ -11362,7 +11336,7 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46283</v>
       </c>
       <c r="N27" t="s">
@@ -11406,7 +11380,7 @@
       <c r="L28" t="s">
         <v>571</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46328</v>
       </c>
       <c r="N28" t="s">
@@ -11450,7 +11424,7 @@
       <c r="L29" t="s">
         <v>571</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46328</v>
       </c>
       <c r="N29" t="s">
@@ -11494,7 +11468,7 @@
       <c r="L30" t="s">
         <v>571</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46328</v>
       </c>
       <c r="N30" t="s">
@@ -11538,7 +11512,7 @@
       <c r="L31" t="s">
         <v>571</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46328</v>
       </c>
       <c r="N31" t="s">
@@ -11582,7 +11556,7 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46283</v>
       </c>
       <c r="N32" t="s">
@@ -11626,7 +11600,7 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46283</v>
       </c>
       <c r="N33" t="s">
@@ -11670,7 +11644,7 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46283</v>
       </c>
       <c r="N34" t="s">
@@ -11714,7 +11688,7 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46283</v>
       </c>
       <c r="N35" t="s">
@@ -11758,7 +11732,7 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46283</v>
       </c>
       <c r="N36" t="s">
@@ -11802,7 +11776,7 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46283</v>
       </c>
       <c r="N37" t="s">
@@ -11846,7 +11820,7 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46283</v>
       </c>
       <c r="N38" t="s">
@@ -11890,7 +11864,7 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="2">
+      <c r="M39" s="1">
         <v>46283</v>
       </c>
       <c r="N39" t="s">
@@ -11934,7 +11908,7 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46283</v>
       </c>
       <c r="N40" t="s">
@@ -11978,7 +11952,7 @@
       <c r="L41" t="s">
         <v>571</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46328</v>
       </c>
       <c r="N41" t="s">
@@ -12022,7 +11996,7 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46283</v>
       </c>
       <c r="N42" t="s">
@@ -12066,7 +12040,7 @@
       <c r="L43" t="s">
         <v>570</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46343</v>
       </c>
       <c r="N43" t="s">
@@ -12110,7 +12084,7 @@
       <c r="L44" t="s">
         <v>570</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46343</v>
       </c>
       <c r="N44" t="s">
@@ -12154,7 +12128,7 @@
       <c r="L45" t="s">
         <v>570</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46343</v>
       </c>
       <c r="N45" t="s">
@@ -12198,7 +12172,7 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46283</v>
       </c>
       <c r="N46" t="s">
@@ -12242,7 +12216,7 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46283</v>
       </c>
       <c r="N47" t="s">
@@ -12286,7 +12260,7 @@
       <c r="L48" t="s">
         <v>571</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46328</v>
       </c>
       <c r="N48" t="s">
@@ -12330,7 +12304,7 @@
       <c r="L49" t="s">
         <v>571</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46328</v>
       </c>
       <c r="N49" t="s">
@@ -12374,7 +12348,7 @@
       <c r="L50" t="s">
         <v>571</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46328</v>
       </c>
       <c r="N50" t="s">
@@ -12418,7 +12392,7 @@
       <c r="L51" t="s">
         <v>571</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46328</v>
       </c>
       <c r="N51" t="s">
@@ -12462,7 +12436,7 @@
       <c r="L52" t="s">
         <v>571</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46328</v>
       </c>
       <c r="N52" t="s">
@@ -12506,7 +12480,7 @@
       <c r="L53" t="s">
         <v>571</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46328</v>
       </c>
       <c r="N53" t="s">
@@ -12550,7 +12524,7 @@
       <c r="L54" t="s">
         <v>571</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46328</v>
       </c>
       <c r="N54" t="s">
@@ -12594,7 +12568,7 @@
       <c r="L55" t="s">
         <v>571</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46328</v>
       </c>
       <c r="N55" t="s">
@@ -12638,7 +12612,7 @@
       <c r="L56" t="s">
         <v>571</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46328</v>
       </c>
       <c r="N56" t="s">
@@ -12682,7 +12656,7 @@
       <c r="L57" t="s">
         <v>571</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46328</v>
       </c>
       <c r="N57" t="s">
@@ -12726,7 +12700,7 @@
       <c r="L58" t="s">
         <v>571</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46328</v>
       </c>
       <c r="N58" t="s">
@@ -12770,7 +12744,7 @@
       <c r="L59" t="s">
         <v>570</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46343</v>
       </c>
       <c r="N59" t="s">
@@ -12814,7 +12788,7 @@
       <c r="L60" t="s">
         <v>571</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46328</v>
       </c>
       <c r="N60" t="s">
@@ -12858,7 +12832,7 @@
       <c r="L61" t="s">
         <v>571</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46328</v>
       </c>
       <c r="N61" t="s">
@@ -12902,7 +12876,7 @@
       <c r="L62" t="s">
         <v>570</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46343</v>
       </c>
       <c r="N62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (20/08/2026 08:36)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10525,7 +10525,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10610,7 +10610,7 @@
         <v>571</v>
       </c>
       <c r="M10" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10654,7 +10654,7 @@
         <v>571</v>
       </c>
       <c r="M11" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10821,7 +10821,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10865,7 +10865,7 @@
         <v>571</v>
       </c>
       <c r="M16" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10909,7 +10909,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10953,7 +10953,7 @@
         <v>571</v>
       </c>
       <c r="M18" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -10997,7 +10997,7 @@
         <v>571</v>
       </c>
       <c r="M19" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11041,7 +11041,7 @@
         <v>571</v>
       </c>
       <c r="M20" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11085,7 +11085,7 @@
         <v>571</v>
       </c>
       <c r="M21" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11252,7 +11252,7 @@
         <v>571</v>
       </c>
       <c r="M25" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11337,7 +11337,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11381,7 +11381,7 @@
         <v>571</v>
       </c>
       <c r="M28" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11425,7 +11425,7 @@
         <v>571</v>
       </c>
       <c r="M29" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11469,7 +11469,7 @@
         <v>571</v>
       </c>
       <c r="M30" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11513,7 +11513,7 @@
         <v>571</v>
       </c>
       <c r="M31" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N31" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>571</v>
       </c>
       <c r="M41" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12041,7 +12041,7 @@
         <v>570</v>
       </c>
       <c r="M43" s="1">
-        <v>46343</v>
+        <v>46344</v>
       </c>
       <c r="N43" t="s">
         <v>572</v>
@@ -12085,7 +12085,7 @@
         <v>570</v>
       </c>
       <c r="M44" s="1">
-        <v>46343</v>
+        <v>46344</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12129,7 +12129,7 @@
         <v>570</v>
       </c>
       <c r="M45" s="1">
-        <v>46343</v>
+        <v>46344</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12173,7 +12173,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12217,7 +12217,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12261,7 +12261,7 @@
         <v>571</v>
       </c>
       <c r="M48" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N48" t="s">
         <v>572</v>
@@ -12305,7 +12305,7 @@
         <v>571</v>
       </c>
       <c r="M49" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12349,7 +12349,7 @@
         <v>571</v>
       </c>
       <c r="M50" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12393,7 +12393,7 @@
         <v>571</v>
       </c>
       <c r="M51" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12437,7 +12437,7 @@
         <v>571</v>
       </c>
       <c r="M52" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12481,7 +12481,7 @@
         <v>571</v>
       </c>
       <c r="M53" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12525,7 +12525,7 @@
         <v>571</v>
       </c>
       <c r="M54" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12569,7 +12569,7 @@
         <v>571</v>
       </c>
       <c r="M55" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12613,7 +12613,7 @@
         <v>571</v>
       </c>
       <c r="M56" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12657,7 +12657,7 @@
         <v>571</v>
       </c>
       <c r="M57" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12701,7 +12701,7 @@
         <v>571</v>
       </c>
       <c r="M58" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12745,7 +12745,7 @@
         <v>570</v>
       </c>
       <c r="M59" s="1">
-        <v>46343</v>
+        <v>46344</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12789,7 +12789,7 @@
         <v>571</v>
       </c>
       <c r="M60" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12833,7 +12833,7 @@
         <v>571</v>
       </c>
       <c r="M61" s="1">
-        <v>46328</v>
+        <v>46329</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>
@@ -12877,7 +12877,7 @@
         <v>570</v>
       </c>
       <c r="M62" s="1">
-        <v>46343</v>
+        <v>46344</v>
       </c>
       <c r="N62" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (20/08/2026 16:39)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1724,13 +1724,13 @@
     <t>Em Cotação</t>
   </si>
   <si>
+    <t>Validada</t>
+  </si>
+  <si>
     <t>Selecionada em Plano</t>
   </si>
   <si>
     <t>Análise do Pedido</t>
-  </si>
-  <si>
-    <t>Validada</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10601,13 +10601,13 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K10" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L10" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M10" s="1">
         <v>46329</v>
@@ -10645,13 +10645,13 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K11" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L11" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M11" s="1">
         <v>46329</v>
@@ -10856,13 +10856,13 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K16" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L16" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M16" s="1">
         <v>46329</v>
@@ -10944,13 +10944,13 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K18" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L18" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M18" s="1">
         <v>46329</v>
@@ -10988,13 +10988,13 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K19" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L19" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M19" s="1">
         <v>46329</v>
@@ -11032,13 +11032,13 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K20" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L20" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M20" s="1">
         <v>46329</v>
@@ -11076,13 +11076,13 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K21" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L21" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M21" s="1">
         <v>46329</v>
@@ -11243,13 +11243,13 @@
         <v>569</v>
       </c>
       <c r="J25" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K25" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L25" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M25" s="1">
         <v>46329</v>
@@ -11372,13 +11372,13 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K28" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L28" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M28" s="1">
         <v>46329</v>
@@ -11413,16 +11413,16 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
+        <v>570</v>
+      </c>
+      <c r="J29" t="s">
         <v>569</v>
       </c>
-      <c r="J29" t="s">
-        <v>571</v>
-      </c>
       <c r="K29" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L29" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M29" s="1">
         <v>46329</v>
@@ -11460,13 +11460,13 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K30" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L30" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M30" s="1">
         <v>46329</v>
@@ -11501,16 +11501,16 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
+        <v>570</v>
+      </c>
+      <c r="J31" t="s">
         <v>569</v>
       </c>
-      <c r="J31" t="s">
-        <v>571</v>
-      </c>
       <c r="K31" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L31" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M31" s="1">
         <v>46329</v>
@@ -11944,13 +11944,13 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K41" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L41" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M41" s="1">
         <v>46329</v>
@@ -12029,16 +12029,16 @@
         <v>5000</v>
       </c>
       <c r="I43" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="J43" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K43" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L43" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M43" s="1">
         <v>46344</v>
@@ -12073,16 +12073,16 @@
         <v>352.52</v>
       </c>
       <c r="I44" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="J44" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K44" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L44" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M44" s="1">
         <v>46344</v>
@@ -12117,19 +12117,19 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="J45" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="K45" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="L45" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="M45" s="1">
-        <v>46344</v>
+        <v>46329</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12249,16 +12249,16 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="J48" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K48" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L48" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M48" s="1">
         <v>46329</v>
@@ -12293,16 +12293,16 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
+        <v>570</v>
+      </c>
+      <c r="J49" t="s">
         <v>569</v>
       </c>
-      <c r="J49" t="s">
-        <v>571</v>
-      </c>
       <c r="K49" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L49" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M49" s="1">
         <v>46329</v>
@@ -12337,16 +12337,16 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
+        <v>570</v>
+      </c>
+      <c r="J50" t="s">
         <v>569</v>
       </c>
-      <c r="J50" t="s">
-        <v>571</v>
-      </c>
       <c r="K50" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L50" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M50" s="1">
         <v>46329</v>
@@ -12384,13 +12384,13 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K51" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L51" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M51" s="1">
         <v>46329</v>
@@ -12428,13 +12428,13 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K52" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L52" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M52" s="1">
         <v>46329</v>
@@ -12472,13 +12472,13 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K53" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L53" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M53" s="1">
         <v>46329</v>
@@ -12513,16 +12513,16 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="J54" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K54" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L54" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M54" s="1">
         <v>46329</v>
@@ -12560,13 +12560,13 @@
         <v>382</v>
       </c>
       <c r="J55" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="K55" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L55" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M55" s="1">
         <v>46329</v>
@@ -12601,16 +12601,16 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
+        <v>570</v>
+      </c>
+      <c r="J56" t="s">
         <v>569</v>
       </c>
-      <c r="J56" t="s">
-        <v>571</v>
-      </c>
       <c r="K56" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L56" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M56" s="1">
         <v>46329</v>
@@ -12645,16 +12645,16 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
+        <v>570</v>
+      </c>
+      <c r="J57" t="s">
         <v>569</v>
       </c>
-      <c r="J57" t="s">
-        <v>571</v>
-      </c>
       <c r="K57" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L57" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M57" s="1">
         <v>46329</v>
@@ -12689,16 +12689,16 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
+        <v>570</v>
+      </c>
+      <c r="J58" t="s">
         <v>569</v>
       </c>
-      <c r="J58" t="s">
-        <v>571</v>
-      </c>
       <c r="K58" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L58" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M58" s="1">
         <v>46329</v>
@@ -12733,19 +12733,19 @@
         <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="J59" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="K59" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="L59" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="M59" s="1">
-        <v>46344</v>
+        <v>46329</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12777,16 +12777,16 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
+        <v>570</v>
+      </c>
+      <c r="J60" t="s">
         <v>569</v>
       </c>
-      <c r="J60" t="s">
-        <v>571</v>
-      </c>
       <c r="K60" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L60" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M60" s="1">
         <v>46329</v>
@@ -12821,16 +12821,16 @@
         <v>5645.05</v>
       </c>
       <c r="I61" t="s">
+        <v>570</v>
+      </c>
+      <c r="J61" t="s">
         <v>569</v>
       </c>
-      <c r="J61" t="s">
-        <v>571</v>
-      </c>
       <c r="K61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="L61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M61" s="1">
         <v>46329</v>
@@ -12865,16 +12865,16 @@
         <v>204.96</v>
       </c>
       <c r="I62" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="J62" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K62" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L62" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="M62" s="1">
         <v>46344</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/08/2026 08:34)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10525,7 +10525,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10610,7 +10610,7 @@
         <v>569</v>
       </c>
       <c r="M10" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10654,7 +10654,7 @@
         <v>569</v>
       </c>
       <c r="M11" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10821,7 +10821,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10865,7 +10865,7 @@
         <v>569</v>
       </c>
       <c r="M16" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10909,7 +10909,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10953,7 +10953,7 @@
         <v>569</v>
       </c>
       <c r="M18" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -10997,7 +10997,7 @@
         <v>569</v>
       </c>
       <c r="M19" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11041,7 +11041,7 @@
         <v>569</v>
       </c>
       <c r="M20" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11085,7 +11085,7 @@
         <v>569</v>
       </c>
       <c r="M21" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11252,7 +11252,7 @@
         <v>569</v>
       </c>
       <c r="M25" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11337,7 +11337,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11381,7 +11381,7 @@
         <v>569</v>
       </c>
       <c r="M28" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11425,7 +11425,7 @@
         <v>569</v>
       </c>
       <c r="M29" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11469,7 +11469,7 @@
         <v>569</v>
       </c>
       <c r="M30" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11513,7 +11513,7 @@
         <v>569</v>
       </c>
       <c r="M31" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N31" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>569</v>
       </c>
       <c r="M41" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12041,7 +12041,7 @@
         <v>571</v>
       </c>
       <c r="M43" s="1">
-        <v>46344</v>
+        <v>46345</v>
       </c>
       <c r="N43" t="s">
         <v>572</v>
@@ -12085,7 +12085,7 @@
         <v>571</v>
       </c>
       <c r="M44" s="1">
-        <v>46344</v>
+        <v>46345</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12129,7 +12129,7 @@
         <v>569</v>
       </c>
       <c r="M45" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12173,7 +12173,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12217,7 +12217,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12261,7 +12261,7 @@
         <v>569</v>
       </c>
       <c r="M48" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N48" t="s">
         <v>572</v>
@@ -12305,7 +12305,7 @@
         <v>569</v>
       </c>
       <c r="M49" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12349,7 +12349,7 @@
         <v>569</v>
       </c>
       <c r="M50" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12393,7 +12393,7 @@
         <v>569</v>
       </c>
       <c r="M51" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12437,7 +12437,7 @@
         <v>569</v>
       </c>
       <c r="M52" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12481,7 +12481,7 @@
         <v>569</v>
       </c>
       <c r="M53" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12525,7 +12525,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12569,7 +12569,7 @@
         <v>569</v>
       </c>
       <c r="M55" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12613,7 +12613,7 @@
         <v>569</v>
       </c>
       <c r="M56" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12657,7 +12657,7 @@
         <v>569</v>
       </c>
       <c r="M57" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12701,7 +12701,7 @@
         <v>569</v>
       </c>
       <c r="M58" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12745,7 +12745,7 @@
         <v>569</v>
       </c>
       <c r="M59" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12789,7 +12789,7 @@
         <v>569</v>
       </c>
       <c r="M60" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12833,7 +12833,7 @@
         <v>569</v>
       </c>
       <c r="M61" s="1">
-        <v>46329</v>
+        <v>46330</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>
@@ -12877,7 +12877,7 @@
         <v>571</v>
       </c>
       <c r="M62" s="1">
-        <v>46344</v>
+        <v>46345</v>
       </c>
       <c r="N62" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/08/2026 09:07)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,8 +1743,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1760,7 +1768,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1768,12 +1776,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2073,55 +2099,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2165,7 +2191,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2209,7 +2235,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2253,7 +2279,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2379,7 +2405,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2423,7 +2449,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2467,7 +2493,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2514,7 +2540,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2637,7 +2663,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2681,7 +2707,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2725,7 +2751,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2769,7 +2795,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2816,7 +2842,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2860,7 +2886,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2986,7 +3012,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3030,7 +3056,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3115,7 +3141,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3162,7 +3188,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3209,7 +3235,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3253,7 +3279,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3297,7 +3323,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3382,7 +3408,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3467,7 +3493,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3514,7 +3540,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3558,7 +3584,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3602,7 +3628,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3687,7 +3713,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3731,7 +3757,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3775,7 +3801,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3860,7 +3886,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3904,7 +3930,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3948,7 +3974,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3992,7 +4018,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4159,7 +4185,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4203,7 +4229,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4247,7 +4273,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4291,7 +4317,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4338,7 +4364,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4382,7 +4408,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4596,7 +4622,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4640,7 +4666,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4687,7 +4713,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4731,7 +4757,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4775,7 +4801,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4819,7 +4845,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4910,7 +4936,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4954,7 +4980,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5001,7 +5027,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5045,7 +5071,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5092,7 +5118,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5180,7 +5206,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5224,7 +5250,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5268,7 +5294,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5312,7 +5338,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5356,7 +5382,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5400,7 +5426,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5485,7 +5511,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5529,7 +5555,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5573,7 +5599,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5617,7 +5643,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5661,7 +5687,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5705,7 +5731,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5749,7 +5775,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5793,7 +5819,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5840,7 +5866,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5884,7 +5910,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5928,7 +5954,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5972,7 +5998,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6016,7 +6042,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6060,7 +6086,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6104,7 +6130,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6148,7 +6174,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6192,7 +6218,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6280,7 +6306,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6324,7 +6350,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6450,7 +6476,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6494,7 +6520,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6538,7 +6564,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6582,7 +6608,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6664,7 +6690,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6708,7 +6734,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6755,7 +6781,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6799,7 +6825,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6925,7 +6951,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6969,7 +6995,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7054,7 +7080,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7098,7 +7124,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7142,7 +7168,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7186,7 +7212,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7230,7 +7256,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7274,7 +7300,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7318,7 +7344,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7362,7 +7388,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7447,7 +7473,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7614,7 +7640,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7658,7 +7684,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7702,7 +7728,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7746,7 +7772,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7790,7 +7816,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7834,7 +7860,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7878,7 +7904,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7963,7 +7989,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8007,7 +8033,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8092,7 +8118,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8218,7 +8244,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8262,7 +8288,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8347,7 +8373,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8391,7 +8417,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8435,7 +8461,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8479,7 +8505,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8523,7 +8549,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8567,7 +8593,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8611,7 +8637,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8655,7 +8681,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8740,7 +8766,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8907,7 +8933,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8951,7 +8977,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8995,7 +9021,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9039,7 +9065,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9124,7 +9150,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9168,7 +9194,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9212,7 +9238,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9256,7 +9282,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9300,7 +9326,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9344,7 +9370,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9388,7 +9414,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9432,7 +9458,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9476,7 +9502,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9520,7 +9546,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9564,7 +9590,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9608,7 +9634,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9652,7 +9678,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9696,7 +9722,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9740,7 +9766,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9784,7 +9810,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9828,7 +9854,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9872,7 +9898,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9916,7 +9942,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9960,7 +9986,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10004,7 +10030,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10089,7 +10115,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10174,7 +10200,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10189,55 +10215,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10524,7 +10550,7 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46285</v>
       </c>
       <c r="N8" t="s">
@@ -10609,7 +10635,7 @@
       <c r="L10" t="s">
         <v>569</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46330</v>
       </c>
       <c r="N10" t="s">
@@ -10653,7 +10679,7 @@
       <c r="L11" t="s">
         <v>569</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46330</v>
       </c>
       <c r="N11" t="s">
@@ -10820,7 +10846,7 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46285</v>
       </c>
       <c r="N15" t="s">
@@ -10864,7 +10890,7 @@
       <c r="L16" t="s">
         <v>569</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46330</v>
       </c>
       <c r="N16" t="s">
@@ -10908,7 +10934,7 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46285</v>
       </c>
       <c r="N17" t="s">
@@ -10952,7 +10978,7 @@
       <c r="L18" t="s">
         <v>569</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46330</v>
       </c>
       <c r="N18" t="s">
@@ -10996,7 +11022,7 @@
       <c r="L19" t="s">
         <v>569</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46330</v>
       </c>
       <c r="N19" t="s">
@@ -11040,7 +11066,7 @@
       <c r="L20" t="s">
         <v>569</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46330</v>
       </c>
       <c r="N20" t="s">
@@ -11084,7 +11110,7 @@
       <c r="L21" t="s">
         <v>569</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46330</v>
       </c>
       <c r="N21" t="s">
@@ -11251,7 +11277,7 @@
       <c r="L25" t="s">
         <v>569</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46330</v>
       </c>
       <c r="N25" t="s">
@@ -11336,7 +11362,7 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46285</v>
       </c>
       <c r="N27" t="s">
@@ -11380,7 +11406,7 @@
       <c r="L28" t="s">
         <v>569</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46330</v>
       </c>
       <c r="N28" t="s">
@@ -11424,7 +11450,7 @@
       <c r="L29" t="s">
         <v>569</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46330</v>
       </c>
       <c r="N29" t="s">
@@ -11468,7 +11494,7 @@
       <c r="L30" t="s">
         <v>569</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46330</v>
       </c>
       <c r="N30" t="s">
@@ -11512,7 +11538,7 @@
       <c r="L31" t="s">
         <v>569</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46330</v>
       </c>
       <c r="N31" t="s">
@@ -11556,7 +11582,7 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46285</v>
       </c>
       <c r="N32" t="s">
@@ -11600,7 +11626,7 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46285</v>
       </c>
       <c r="N33" t="s">
@@ -11644,7 +11670,7 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46285</v>
       </c>
       <c r="N34" t="s">
@@ -11688,7 +11714,7 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46285</v>
       </c>
       <c r="N35" t="s">
@@ -11732,7 +11758,7 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46285</v>
       </c>
       <c r="N36" t="s">
@@ -11776,7 +11802,7 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46285</v>
       </c>
       <c r="N37" t="s">
@@ -11820,7 +11846,7 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46285</v>
       </c>
       <c r="N38" t="s">
@@ -11864,7 +11890,7 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="1">
+      <c r="M39" s="2">
         <v>46285</v>
       </c>
       <c r="N39" t="s">
@@ -11908,7 +11934,7 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46285</v>
       </c>
       <c r="N40" t="s">
@@ -11952,7 +11978,7 @@
       <c r="L41" t="s">
         <v>569</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46330</v>
       </c>
       <c r="N41" t="s">
@@ -11996,7 +12022,7 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46285</v>
       </c>
       <c r="N42" t="s">
@@ -12040,7 +12066,7 @@
       <c r="L43" t="s">
         <v>571</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46345</v>
       </c>
       <c r="N43" t="s">
@@ -12084,7 +12110,7 @@
       <c r="L44" t="s">
         <v>571</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46345</v>
       </c>
       <c r="N44" t="s">
@@ -12128,7 +12154,7 @@
       <c r="L45" t="s">
         <v>569</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46330</v>
       </c>
       <c r="N45" t="s">
@@ -12172,7 +12198,7 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46285</v>
       </c>
       <c r="N46" t="s">
@@ -12216,7 +12242,7 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46285</v>
       </c>
       <c r="N47" t="s">
@@ -12260,7 +12286,7 @@
       <c r="L48" t="s">
         <v>569</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46330</v>
       </c>
       <c r="N48" t="s">
@@ -12304,7 +12330,7 @@
       <c r="L49" t="s">
         <v>569</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46330</v>
       </c>
       <c r="N49" t="s">
@@ -12348,7 +12374,7 @@
       <c r="L50" t="s">
         <v>569</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46330</v>
       </c>
       <c r="N50" t="s">
@@ -12392,7 +12418,7 @@
       <c r="L51" t="s">
         <v>569</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46330</v>
       </c>
       <c r="N51" t="s">
@@ -12436,7 +12462,7 @@
       <c r="L52" t="s">
         <v>569</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46330</v>
       </c>
       <c r="N52" t="s">
@@ -12480,7 +12506,7 @@
       <c r="L53" t="s">
         <v>569</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46330</v>
       </c>
       <c r="N53" t="s">
@@ -12524,7 +12550,7 @@
       <c r="L54" t="s">
         <v>569</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46330</v>
       </c>
       <c r="N54" t="s">
@@ -12568,7 +12594,7 @@
       <c r="L55" t="s">
         <v>569</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46330</v>
       </c>
       <c r="N55" t="s">
@@ -12612,7 +12638,7 @@
       <c r="L56" t="s">
         <v>569</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46330</v>
       </c>
       <c r="N56" t="s">
@@ -12656,7 +12682,7 @@
       <c r="L57" t="s">
         <v>569</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46330</v>
       </c>
       <c r="N57" t="s">
@@ -12700,7 +12726,7 @@
       <c r="L58" t="s">
         <v>569</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46330</v>
       </c>
       <c r="N58" t="s">
@@ -12744,7 +12770,7 @@
       <c r="L59" t="s">
         <v>569</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46330</v>
       </c>
       <c r="N59" t="s">
@@ -12788,7 +12814,7 @@
       <c r="L60" t="s">
         <v>569</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46330</v>
       </c>
       <c r="N60" t="s">
@@ -12832,7 +12858,7 @@
       <c r="L61" t="s">
         <v>569</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46330</v>
       </c>
       <c r="N61" t="s">
@@ -12876,7 +12902,7 @@
       <c r="L62" t="s">
         <v>571</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46345</v>
       </c>
       <c r="N62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (21/08/2026 10:52)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,16 +1743,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1768,7 +1760,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1776,30 +1768,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2099,55 +2073,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2191,7 +2165,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2235,7 +2209,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2279,7 +2253,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2405,7 +2379,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2449,7 +2423,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2493,7 +2467,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2540,7 +2514,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2663,7 +2637,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2707,7 +2681,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2751,7 +2725,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2795,7 +2769,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2842,7 +2816,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2886,7 +2860,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3012,7 +2986,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3056,7 +3030,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3141,7 +3115,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3188,7 +3162,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3235,7 +3209,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3279,7 +3253,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3323,7 +3297,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3408,7 +3382,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3493,7 +3467,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3540,7 +3514,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3584,7 +3558,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3628,7 +3602,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3713,7 +3687,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3757,7 +3731,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3801,7 +3775,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3886,7 +3860,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3930,7 +3904,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3974,7 +3948,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4018,7 +3992,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4185,7 +4159,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4229,7 +4203,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4273,7 +4247,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4317,7 +4291,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4364,7 +4338,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4408,7 +4382,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4622,7 +4596,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4666,7 +4640,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4713,7 +4687,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4757,7 +4731,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4801,7 +4775,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4845,7 +4819,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4889,7 +4863,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4936,7 +4910,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4980,7 +4954,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5027,7 +5001,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5071,7 +5045,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5118,7 +5092,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5206,7 +5180,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5250,7 +5224,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5294,7 +5268,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5338,7 +5312,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5382,7 +5356,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5426,7 +5400,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5511,7 +5485,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5555,7 +5529,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5599,7 +5573,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5643,7 +5617,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5687,7 +5661,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5731,7 +5705,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5775,7 +5749,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5819,7 +5793,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5866,7 +5840,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5910,7 +5884,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5954,7 +5928,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5998,7 +5972,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6042,7 +6016,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6086,7 +6060,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6130,7 +6104,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6174,7 +6148,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6218,7 +6192,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6306,7 +6280,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6350,7 +6324,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6476,7 +6450,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6520,7 +6494,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6564,7 +6538,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6608,7 +6582,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6690,7 +6664,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6734,7 +6708,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6781,7 +6755,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6825,7 +6799,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6951,7 +6925,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -6995,7 +6969,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7080,7 +7054,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7124,7 +7098,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7168,7 +7142,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7212,7 +7186,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7256,7 +7230,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7300,7 +7274,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7344,7 +7318,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7388,7 +7362,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7473,7 +7447,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7640,7 +7614,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7684,7 +7658,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7728,7 +7702,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7772,7 +7746,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7816,7 +7790,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7860,7 +7834,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7904,7 +7878,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -7989,7 +7963,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8033,7 +8007,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8118,7 +8092,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8244,7 +8218,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8288,7 +8262,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8373,7 +8347,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8417,7 +8391,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8461,7 +8435,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8505,7 +8479,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8549,7 +8523,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8593,7 +8567,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8637,7 +8611,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8681,7 +8655,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8766,7 +8740,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8933,7 +8907,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8977,7 +8951,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9021,7 +8995,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9065,7 +9039,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9150,7 +9124,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9194,7 +9168,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9238,7 +9212,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9282,7 +9256,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9326,7 +9300,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9370,7 +9344,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9414,7 +9388,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9458,7 +9432,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9502,7 +9476,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9546,7 +9520,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9590,7 +9564,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9634,7 +9608,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9678,7 +9652,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9722,7 +9696,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9766,7 +9740,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9810,7 +9784,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9854,7 +9828,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9898,7 +9872,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9942,7 +9916,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -9986,7 +9960,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10030,7 +10004,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10115,7 +10089,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10200,7 +10174,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10215,55 +10189,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10550,7 +10524,7 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46285</v>
       </c>
       <c r="N8" t="s">
@@ -10635,7 +10609,7 @@
       <c r="L10" t="s">
         <v>569</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46330</v>
       </c>
       <c r="N10" t="s">
@@ -10679,7 +10653,7 @@
       <c r="L11" t="s">
         <v>569</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46330</v>
       </c>
       <c r="N11" t="s">
@@ -10846,7 +10820,7 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46285</v>
       </c>
       <c r="N15" t="s">
@@ -10890,7 +10864,7 @@
       <c r="L16" t="s">
         <v>569</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46330</v>
       </c>
       <c r="N16" t="s">
@@ -10934,7 +10908,7 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46285</v>
       </c>
       <c r="N17" t="s">
@@ -10978,7 +10952,7 @@
       <c r="L18" t="s">
         <v>569</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46330</v>
       </c>
       <c r="N18" t="s">
@@ -11022,7 +10996,7 @@
       <c r="L19" t="s">
         <v>569</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46330</v>
       </c>
       <c r="N19" t="s">
@@ -11066,7 +11040,7 @@
       <c r="L20" t="s">
         <v>569</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46330</v>
       </c>
       <c r="N20" t="s">
@@ -11110,7 +11084,7 @@
       <c r="L21" t="s">
         <v>569</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46330</v>
       </c>
       <c r="N21" t="s">
@@ -11277,7 +11251,7 @@
       <c r="L25" t="s">
         <v>569</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46330</v>
       </c>
       <c r="N25" t="s">
@@ -11362,7 +11336,7 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46285</v>
       </c>
       <c r="N27" t="s">
@@ -11406,7 +11380,7 @@
       <c r="L28" t="s">
         <v>569</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46330</v>
       </c>
       <c r="N28" t="s">
@@ -11450,7 +11424,7 @@
       <c r="L29" t="s">
         <v>569</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46330</v>
       </c>
       <c r="N29" t="s">
@@ -11494,7 +11468,7 @@
       <c r="L30" t="s">
         <v>569</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46330</v>
       </c>
       <c r="N30" t="s">
@@ -11538,7 +11512,7 @@
       <c r="L31" t="s">
         <v>569</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46330</v>
       </c>
       <c r="N31" t="s">
@@ -11582,7 +11556,7 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46285</v>
       </c>
       <c r="N32" t="s">
@@ -11626,7 +11600,7 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46285</v>
       </c>
       <c r="N33" t="s">
@@ -11670,7 +11644,7 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46285</v>
       </c>
       <c r="N34" t="s">
@@ -11714,7 +11688,7 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46285</v>
       </c>
       <c r="N35" t="s">
@@ -11758,7 +11732,7 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46285</v>
       </c>
       <c r="N36" t="s">
@@ -11802,7 +11776,7 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46285</v>
       </c>
       <c r="N37" t="s">
@@ -11846,7 +11820,7 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46285</v>
       </c>
       <c r="N38" t="s">
@@ -11890,7 +11864,7 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="2">
+      <c r="M39" s="1">
         <v>46285</v>
       </c>
       <c r="N39" t="s">
@@ -11934,7 +11908,7 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46285</v>
       </c>
       <c r="N40" t="s">
@@ -11978,7 +11952,7 @@
       <c r="L41" t="s">
         <v>569</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46330</v>
       </c>
       <c r="N41" t="s">
@@ -12022,7 +11996,7 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46285</v>
       </c>
       <c r="N42" t="s">
@@ -12066,7 +12040,7 @@
       <c r="L43" t="s">
         <v>571</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46345</v>
       </c>
       <c r="N43" t="s">
@@ -12110,7 +12084,7 @@
       <c r="L44" t="s">
         <v>571</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46345</v>
       </c>
       <c r="N44" t="s">
@@ -12154,7 +12128,7 @@
       <c r="L45" t="s">
         <v>569</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46330</v>
       </c>
       <c r="N45" t="s">
@@ -12198,7 +12172,7 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46285</v>
       </c>
       <c r="N46" t="s">
@@ -12242,7 +12216,7 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46285</v>
       </c>
       <c r="N47" t="s">
@@ -12286,7 +12260,7 @@
       <c r="L48" t="s">
         <v>569</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46330</v>
       </c>
       <c r="N48" t="s">
@@ -12330,7 +12304,7 @@
       <c r="L49" t="s">
         <v>569</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46330</v>
       </c>
       <c r="N49" t="s">
@@ -12374,7 +12348,7 @@
       <c r="L50" t="s">
         <v>569</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46330</v>
       </c>
       <c r="N50" t="s">
@@ -12418,7 +12392,7 @@
       <c r="L51" t="s">
         <v>569</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46330</v>
       </c>
       <c r="N51" t="s">
@@ -12462,7 +12436,7 @@
       <c r="L52" t="s">
         <v>569</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46330</v>
       </c>
       <c r="N52" t="s">
@@ -12506,7 +12480,7 @@
       <c r="L53" t="s">
         <v>569</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46330</v>
       </c>
       <c r="N53" t="s">
@@ -12550,7 +12524,7 @@
       <c r="L54" t="s">
         <v>569</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46330</v>
       </c>
       <c r="N54" t="s">
@@ -12594,7 +12568,7 @@
       <c r="L55" t="s">
         <v>569</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46330</v>
       </c>
       <c r="N55" t="s">
@@ -12638,7 +12612,7 @@
       <c r="L56" t="s">
         <v>569</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46330</v>
       </c>
       <c r="N56" t="s">
@@ -12682,7 +12656,7 @@
       <c r="L57" t="s">
         <v>569</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46330</v>
       </c>
       <c r="N57" t="s">
@@ -12726,7 +12700,7 @@
       <c r="L58" t="s">
         <v>569</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46330</v>
       </c>
       <c r="N58" t="s">
@@ -12770,7 +12744,7 @@
       <c r="L59" t="s">
         <v>569</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46330</v>
       </c>
       <c r="N59" t="s">
@@ -12814,7 +12788,7 @@
       <c r="L60" t="s">
         <v>569</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46330</v>
       </c>
       <c r="N60" t="s">
@@ -12858,7 +12832,7 @@
       <c r="L61" t="s">
         <v>569</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46330</v>
       </c>
       <c r="N61" t="s">
@@ -12902,7 +12876,7 @@
       <c r="L62" t="s">
         <v>571</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46345</v>
       </c>
       <c r="N62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (24/08/2026 08:37)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10525,7 +10525,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10610,7 +10610,7 @@
         <v>569</v>
       </c>
       <c r="M10" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10654,7 +10654,7 @@
         <v>569</v>
       </c>
       <c r="M11" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10821,7 +10821,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10865,7 +10865,7 @@
         <v>569</v>
       </c>
       <c r="M16" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10909,7 +10909,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10953,7 +10953,7 @@
         <v>569</v>
       </c>
       <c r="M18" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -10997,7 +10997,7 @@
         <v>569</v>
       </c>
       <c r="M19" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11041,7 +11041,7 @@
         <v>569</v>
       </c>
       <c r="M20" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11085,7 +11085,7 @@
         <v>569</v>
       </c>
       <c r="M21" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11252,7 +11252,7 @@
         <v>569</v>
       </c>
       <c r="M25" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11337,7 +11337,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11381,7 +11381,7 @@
         <v>569</v>
       </c>
       <c r="M28" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11425,7 +11425,7 @@
         <v>569</v>
       </c>
       <c r="M29" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11469,7 +11469,7 @@
         <v>569</v>
       </c>
       <c r="M30" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11513,7 +11513,7 @@
         <v>569</v>
       </c>
       <c r="M31" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N31" t="s">
         <v>572</v>
@@ -11557,7 +11557,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11601,7 +11601,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11645,7 +11645,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11689,7 +11689,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11733,7 +11733,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11777,7 +11777,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11821,7 +11821,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11865,7 +11865,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11909,7 +11909,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11953,7 +11953,7 @@
         <v>569</v>
       </c>
       <c r="M41" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11997,7 +11997,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12041,7 +12041,7 @@
         <v>571</v>
       </c>
       <c r="M43" s="1">
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="N43" t="s">
         <v>572</v>
@@ -12085,7 +12085,7 @@
         <v>571</v>
       </c>
       <c r="M44" s="1">
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12129,7 +12129,7 @@
         <v>569</v>
       </c>
       <c r="M45" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12173,7 +12173,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12217,7 +12217,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12261,7 +12261,7 @@
         <v>569</v>
       </c>
       <c r="M48" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N48" t="s">
         <v>572</v>
@@ -12305,7 +12305,7 @@
         <v>569</v>
       </c>
       <c r="M49" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12349,7 +12349,7 @@
         <v>569</v>
       </c>
       <c r="M50" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12393,7 +12393,7 @@
         <v>569</v>
       </c>
       <c r="M51" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12437,7 +12437,7 @@
         <v>569</v>
       </c>
       <c r="M52" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12481,7 +12481,7 @@
         <v>569</v>
       </c>
       <c r="M53" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12525,7 +12525,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12569,7 +12569,7 @@
         <v>569</v>
       </c>
       <c r="M55" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12613,7 +12613,7 @@
         <v>569</v>
       </c>
       <c r="M56" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12657,7 +12657,7 @@
         <v>569</v>
       </c>
       <c r="M57" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12701,7 +12701,7 @@
         <v>569</v>
       </c>
       <c r="M58" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12745,7 +12745,7 @@
         <v>569</v>
       </c>
       <c r="M59" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12789,7 +12789,7 @@
         <v>569</v>
       </c>
       <c r="M60" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12833,7 +12833,7 @@
         <v>569</v>
       </c>
       <c r="M61" s="1">
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>
@@ -12877,7 +12877,7 @@
         <v>571</v>
       </c>
       <c r="M62" s="1">
-        <v>46345</v>
+        <v>46348</v>
       </c>
       <c r="N62" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (25/08/2026 08:31)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,8 +1743,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1760,7 +1768,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1768,12 +1776,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2073,55 +2099,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2165,7 +2191,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2209,7 +2235,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2253,7 +2279,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2379,7 +2405,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2423,7 +2449,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2467,7 +2493,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2514,7 +2540,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2637,7 +2663,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2681,7 +2707,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2725,7 +2751,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2769,7 +2795,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2816,7 +2842,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2860,7 +2886,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2986,7 +3012,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3030,7 +3056,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3115,7 +3141,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3162,7 +3188,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3209,7 +3235,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3253,7 +3279,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3297,7 +3323,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3382,7 +3408,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3467,7 +3493,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3514,7 +3540,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3558,7 +3584,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3602,7 +3628,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3687,7 +3713,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3731,7 +3757,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3775,7 +3801,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3860,7 +3886,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3904,7 +3930,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3948,7 +3974,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3992,7 +4018,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4159,7 +4185,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4203,7 +4229,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4247,7 +4273,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4291,7 +4317,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4338,7 +4364,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4382,7 +4408,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4464,7 +4490,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4508,7 +4534,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4596,7 +4622,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4640,7 +4666,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4687,7 +4713,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4731,7 +4757,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4775,7 +4801,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4819,7 +4845,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4863,7 +4889,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4910,7 +4936,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4954,7 +4980,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5001,7 +5027,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5045,7 +5071,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5092,7 +5118,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5180,7 +5206,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5224,7 +5250,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5268,7 +5294,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5312,7 +5338,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5356,7 +5382,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5400,7 +5426,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5485,7 +5511,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5529,7 +5555,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5573,7 +5599,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5617,7 +5643,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5661,7 +5687,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5705,7 +5731,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5749,7 +5775,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5793,7 +5819,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5840,7 +5866,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5884,7 +5910,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5928,7 +5954,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5972,7 +5998,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6016,7 +6042,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6060,7 +6086,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6104,7 +6130,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6148,7 +6174,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6192,7 +6218,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6280,7 +6306,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6324,7 +6350,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6450,7 +6476,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6494,7 +6520,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6538,7 +6564,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6582,7 +6608,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6664,7 +6690,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6708,7 +6734,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6755,7 +6781,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6799,7 +6825,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6925,7 +6951,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6969,7 +6995,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7054,7 +7080,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7098,7 +7124,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7142,7 +7168,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7186,7 +7212,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7230,7 +7256,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7274,7 +7300,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7318,7 +7344,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7362,7 +7388,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7447,7 +7473,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7614,7 +7640,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7658,7 +7684,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7702,7 +7728,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7746,7 +7772,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7790,7 +7816,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7834,7 +7860,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7878,7 +7904,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7963,7 +7989,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8007,7 +8033,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8092,7 +8118,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8218,7 +8244,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8262,7 +8288,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8347,7 +8373,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8391,7 +8417,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8435,7 +8461,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8479,7 +8505,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8523,7 +8549,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8567,7 +8593,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8611,7 +8637,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8655,7 +8681,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8740,7 +8766,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8907,7 +8933,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8951,7 +8977,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -8995,7 +9021,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9039,7 +9065,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9124,7 +9150,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9168,7 +9194,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9212,7 +9238,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9256,7 +9282,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9300,7 +9326,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9344,7 +9370,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9388,7 +9414,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9432,7 +9458,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9476,7 +9502,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9520,7 +9546,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9564,7 +9590,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9608,7 +9634,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9652,7 +9678,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9696,7 +9722,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9740,7 +9766,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9784,7 +9810,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9828,7 +9854,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9872,7 +9898,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9916,7 +9942,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9960,7 +9986,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10004,7 +10030,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10089,7 +10115,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10174,7 +10200,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10189,55 +10215,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10524,8 +10550,8 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="1">
-        <v>46288</v>
+      <c r="M8" s="2">
+        <v>46289</v>
       </c>
       <c r="N8" t="s">
         <v>572</v>
@@ -10609,8 +10635,8 @@
       <c r="L10" t="s">
         <v>569</v>
       </c>
-      <c r="M10" s="1">
-        <v>46333</v>
+      <c r="M10" s="2">
+        <v>46334</v>
       </c>
       <c r="N10" t="s">
         <v>572</v>
@@ -10653,8 +10679,8 @@
       <c r="L11" t="s">
         <v>569</v>
       </c>
-      <c r="M11" s="1">
-        <v>46333</v>
+      <c r="M11" s="2">
+        <v>46334</v>
       </c>
       <c r="N11" t="s">
         <v>572</v>
@@ -10820,8 +10846,8 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="1">
-        <v>46288</v>
+      <c r="M15" s="2">
+        <v>46289</v>
       </c>
       <c r="N15" t="s">
         <v>572</v>
@@ -10864,8 +10890,8 @@
       <c r="L16" t="s">
         <v>569</v>
       </c>
-      <c r="M16" s="1">
-        <v>46333</v>
+      <c r="M16" s="2">
+        <v>46334</v>
       </c>
       <c r="N16" t="s">
         <v>572</v>
@@ -10908,8 +10934,8 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="1">
-        <v>46288</v>
+      <c r="M17" s="2">
+        <v>46289</v>
       </c>
       <c r="N17" t="s">
         <v>572</v>
@@ -10952,8 +10978,8 @@
       <c r="L18" t="s">
         <v>569</v>
       </c>
-      <c r="M18" s="1">
-        <v>46333</v>
+      <c r="M18" s="2">
+        <v>46334</v>
       </c>
       <c r="N18" t="s">
         <v>572</v>
@@ -10996,8 +11022,8 @@
       <c r="L19" t="s">
         <v>569</v>
       </c>
-      <c r="M19" s="1">
-        <v>46333</v>
+      <c r="M19" s="2">
+        <v>46334</v>
       </c>
       <c r="N19" t="s">
         <v>572</v>
@@ -11040,8 +11066,8 @@
       <c r="L20" t="s">
         <v>569</v>
       </c>
-      <c r="M20" s="1">
-        <v>46333</v>
+      <c r="M20" s="2">
+        <v>46334</v>
       </c>
       <c r="N20" t="s">
         <v>572</v>
@@ -11084,8 +11110,8 @@
       <c r="L21" t="s">
         <v>569</v>
       </c>
-      <c r="M21" s="1">
-        <v>46333</v>
+      <c r="M21" s="2">
+        <v>46334</v>
       </c>
       <c r="N21" t="s">
         <v>572</v>
@@ -11251,8 +11277,8 @@
       <c r="L25" t="s">
         <v>569</v>
       </c>
-      <c r="M25" s="1">
-        <v>46333</v>
+      <c r="M25" s="2">
+        <v>46334</v>
       </c>
       <c r="N25" t="s">
         <v>572</v>
@@ -11336,8 +11362,8 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="1">
-        <v>46288</v>
+      <c r="M27" s="2">
+        <v>46289</v>
       </c>
       <c r="N27" t="s">
         <v>572</v>
@@ -11380,8 +11406,8 @@
       <c r="L28" t="s">
         <v>569</v>
       </c>
-      <c r="M28" s="1">
-        <v>46333</v>
+      <c r="M28" s="2">
+        <v>46334</v>
       </c>
       <c r="N28" t="s">
         <v>572</v>
@@ -11424,8 +11450,8 @@
       <c r="L29" t="s">
         <v>569</v>
       </c>
-      <c r="M29" s="1">
-        <v>46333</v>
+      <c r="M29" s="2">
+        <v>46334</v>
       </c>
       <c r="N29" t="s">
         <v>572</v>
@@ -11468,8 +11494,8 @@
       <c r="L30" t="s">
         <v>569</v>
       </c>
-      <c r="M30" s="1">
-        <v>46333</v>
+      <c r="M30" s="2">
+        <v>46334</v>
       </c>
       <c r="N30" t="s">
         <v>572</v>
@@ -11512,8 +11538,8 @@
       <c r="L31" t="s">
         <v>569</v>
       </c>
-      <c r="M31" s="1">
-        <v>46333</v>
+      <c r="M31" s="2">
+        <v>46334</v>
       </c>
       <c r="N31" t="s">
         <v>572</v>
@@ -11556,8 +11582,8 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="1">
-        <v>46288</v>
+      <c r="M32" s="2">
+        <v>46289</v>
       </c>
       <c r="N32" t="s">
         <v>572</v>
@@ -11600,8 +11626,8 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="1">
-        <v>46288</v>
+      <c r="M33" s="2">
+        <v>46289</v>
       </c>
       <c r="N33" t="s">
         <v>572</v>
@@ -11644,8 +11670,8 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="1">
-        <v>46288</v>
+      <c r="M34" s="2">
+        <v>46289</v>
       </c>
       <c r="N34" t="s">
         <v>572</v>
@@ -11688,8 +11714,8 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="1">
-        <v>46288</v>
+      <c r="M35" s="2">
+        <v>46289</v>
       </c>
       <c r="N35" t="s">
         <v>572</v>
@@ -11732,8 +11758,8 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="1">
-        <v>46288</v>
+      <c r="M36" s="2">
+        <v>46289</v>
       </c>
       <c r="N36" t="s">
         <v>572</v>
@@ -11776,8 +11802,8 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="1">
-        <v>46288</v>
+      <c r="M37" s="2">
+        <v>46289</v>
       </c>
       <c r="N37" t="s">
         <v>572</v>
@@ -11820,8 +11846,8 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="1">
-        <v>46288</v>
+      <c r="M38" s="2">
+        <v>46289</v>
       </c>
       <c r="N38" t="s">
         <v>572</v>
@@ -11864,8 +11890,8 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="1">
-        <v>46288</v>
+      <c r="M39" s="2">
+        <v>46289</v>
       </c>
       <c r="N39" t="s">
         <v>572</v>
@@ -11908,8 +11934,8 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="1">
-        <v>46288</v>
+      <c r="M40" s="2">
+        <v>46289</v>
       </c>
       <c r="N40" t="s">
         <v>572</v>
@@ -11952,8 +11978,8 @@
       <c r="L41" t="s">
         <v>569</v>
       </c>
-      <c r="M41" s="1">
-        <v>46333</v>
+      <c r="M41" s="2">
+        <v>46334</v>
       </c>
       <c r="N41" t="s">
         <v>572</v>
@@ -11996,8 +12022,8 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="1">
-        <v>46288</v>
+      <c r="M42" s="2">
+        <v>46289</v>
       </c>
       <c r="N42" t="s">
         <v>572</v>
@@ -12040,8 +12066,8 @@
       <c r="L43" t="s">
         <v>571</v>
       </c>
-      <c r="M43" s="1">
-        <v>46348</v>
+      <c r="M43" s="2">
+        <v>46349</v>
       </c>
       <c r="N43" t="s">
         <v>572</v>
@@ -12084,8 +12110,8 @@
       <c r="L44" t="s">
         <v>571</v>
       </c>
-      <c r="M44" s="1">
-        <v>46348</v>
+      <c r="M44" s="2">
+        <v>46349</v>
       </c>
       <c r="N44" t="s">
         <v>572</v>
@@ -12128,8 +12154,8 @@
       <c r="L45" t="s">
         <v>569</v>
       </c>
-      <c r="M45" s="1">
-        <v>46333</v>
+      <c r="M45" s="2">
+        <v>46334</v>
       </c>
       <c r="N45" t="s">
         <v>572</v>
@@ -12172,8 +12198,8 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="1">
-        <v>46288</v>
+      <c r="M46" s="2">
+        <v>46289</v>
       </c>
       <c r="N46" t="s">
         <v>572</v>
@@ -12216,8 +12242,8 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="1">
-        <v>46288</v>
+      <c r="M47" s="2">
+        <v>46289</v>
       </c>
       <c r="N47" t="s">
         <v>572</v>
@@ -12260,8 +12286,8 @@
       <c r="L48" t="s">
         <v>569</v>
       </c>
-      <c r="M48" s="1">
-        <v>46333</v>
+      <c r="M48" s="2">
+        <v>46334</v>
       </c>
       <c r="N48" t="s">
         <v>572</v>
@@ -12304,8 +12330,8 @@
       <c r="L49" t="s">
         <v>569</v>
       </c>
-      <c r="M49" s="1">
-        <v>46333</v>
+      <c r="M49" s="2">
+        <v>46334</v>
       </c>
       <c r="N49" t="s">
         <v>572</v>
@@ -12348,8 +12374,8 @@
       <c r="L50" t="s">
         <v>569</v>
       </c>
-      <c r="M50" s="1">
-        <v>46333</v>
+      <c r="M50" s="2">
+        <v>46334</v>
       </c>
       <c r="N50" t="s">
         <v>572</v>
@@ -12392,8 +12418,8 @@
       <c r="L51" t="s">
         <v>569</v>
       </c>
-      <c r="M51" s="1">
-        <v>46333</v>
+      <c r="M51" s="2">
+        <v>46334</v>
       </c>
       <c r="N51" t="s">
         <v>572</v>
@@ -12436,8 +12462,8 @@
       <c r="L52" t="s">
         <v>569</v>
       </c>
-      <c r="M52" s="1">
-        <v>46333</v>
+      <c r="M52" s="2">
+        <v>46334</v>
       </c>
       <c r="N52" t="s">
         <v>572</v>
@@ -12480,8 +12506,8 @@
       <c r="L53" t="s">
         <v>569</v>
       </c>
-      <c r="M53" s="1">
-        <v>46333</v>
+      <c r="M53" s="2">
+        <v>46334</v>
       </c>
       <c r="N53" t="s">
         <v>572</v>
@@ -12524,8 +12550,8 @@
       <c r="L54" t="s">
         <v>569</v>
       </c>
-      <c r="M54" s="1">
-        <v>46333</v>
+      <c r="M54" s="2">
+        <v>46334</v>
       </c>
       <c r="N54" t="s">
         <v>572</v>
@@ -12568,8 +12594,8 @@
       <c r="L55" t="s">
         <v>569</v>
       </c>
-      <c r="M55" s="1">
-        <v>46333</v>
+      <c r="M55" s="2">
+        <v>46334</v>
       </c>
       <c r="N55" t="s">
         <v>572</v>
@@ -12612,8 +12638,8 @@
       <c r="L56" t="s">
         <v>569</v>
       </c>
-      <c r="M56" s="1">
-        <v>46333</v>
+      <c r="M56" s="2">
+        <v>46334</v>
       </c>
       <c r="N56" t="s">
         <v>572</v>
@@ -12656,8 +12682,8 @@
       <c r="L57" t="s">
         <v>569</v>
       </c>
-      <c r="M57" s="1">
-        <v>46333</v>
+      <c r="M57" s="2">
+        <v>46334</v>
       </c>
       <c r="N57" t="s">
         <v>572</v>
@@ -12700,8 +12726,8 @@
       <c r="L58" t="s">
         <v>569</v>
       </c>
-      <c r="M58" s="1">
-        <v>46333</v>
+      <c r="M58" s="2">
+        <v>46334</v>
       </c>
       <c r="N58" t="s">
         <v>572</v>
@@ -12744,8 +12770,8 @@
       <c r="L59" t="s">
         <v>569</v>
       </c>
-      <c r="M59" s="1">
-        <v>46333</v>
+      <c r="M59" s="2">
+        <v>46334</v>
       </c>
       <c r="N59" t="s">
         <v>572</v>
@@ -12788,8 +12814,8 @@
       <c r="L60" t="s">
         <v>569</v>
       </c>
-      <c r="M60" s="1">
-        <v>46333</v>
+      <c r="M60" s="2">
+        <v>46334</v>
       </c>
       <c r="N60" t="s">
         <v>572</v>
@@ -12832,8 +12858,8 @@
       <c r="L61" t="s">
         <v>569</v>
       </c>
-      <c r="M61" s="1">
-        <v>46333</v>
+      <c r="M61" s="2">
+        <v>46334</v>
       </c>
       <c r="N61" t="s">
         <v>572</v>
@@ -12876,8 +12902,8 @@
       <c r="L62" t="s">
         <v>571</v>
       </c>
-      <c r="M62" s="1">
-        <v>46348</v>
+      <c r="M62" s="2">
+        <v>46349</v>
       </c>
       <c r="N62" t="s">
         <v>572</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (25/08/2026 08:37)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1743,16 +1743,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1768,7 +1760,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1776,30 +1768,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2099,55 +2073,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2191,7 +2165,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2235,7 +2209,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2279,7 +2253,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2405,7 +2379,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2449,7 +2423,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2493,7 +2467,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2540,7 +2514,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2663,7 +2637,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2707,7 +2681,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2751,7 +2725,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2795,7 +2769,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2842,7 +2816,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2886,7 +2860,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3012,7 +2986,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3056,7 +3030,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3141,7 +3115,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3188,7 +3162,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3235,7 +3209,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3279,7 +3253,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3323,7 +3297,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3408,7 +3382,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3493,7 +3467,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3540,7 +3514,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3584,7 +3558,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3628,7 +3602,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3713,7 +3687,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3757,7 +3731,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3801,7 +3775,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3886,7 +3860,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3930,7 +3904,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3974,7 +3948,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4018,7 +3992,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4185,7 +4159,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4229,7 +4203,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4273,7 +4247,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4317,7 +4291,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4364,7 +4338,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4408,7 +4382,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4490,7 +4464,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4534,7 +4508,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4622,7 +4596,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4666,7 +4640,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4713,7 +4687,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4757,7 +4731,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4801,7 +4775,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4845,7 +4819,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4889,7 +4863,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4936,7 +4910,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4980,7 +4954,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5027,7 +5001,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5071,7 +5045,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5118,7 +5092,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5206,7 +5180,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5250,7 +5224,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5294,7 +5268,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5338,7 +5312,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5382,7 +5356,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5426,7 +5400,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5511,7 +5485,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5555,7 +5529,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5599,7 +5573,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5643,7 +5617,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5687,7 +5661,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5731,7 +5705,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5775,7 +5749,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5819,7 +5793,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5866,7 +5840,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5910,7 +5884,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5954,7 +5928,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5998,7 +5972,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6042,7 +6016,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6086,7 +6060,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6130,7 +6104,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6174,7 +6148,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6218,7 +6192,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6306,7 +6280,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6350,7 +6324,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6476,7 +6450,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6520,7 +6494,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6564,7 +6538,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6608,7 +6582,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6690,7 +6664,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6734,7 +6708,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6781,7 +6755,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6825,7 +6799,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6951,7 +6925,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -6995,7 +6969,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7080,7 +7054,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7124,7 +7098,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7168,7 +7142,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7212,7 +7186,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7256,7 +7230,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7300,7 +7274,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7344,7 +7318,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7388,7 +7362,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7473,7 +7447,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7640,7 +7614,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7684,7 +7658,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7728,7 +7702,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7772,7 +7746,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7816,7 +7790,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7860,7 +7834,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7904,7 +7878,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -7989,7 +7963,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8033,7 +8007,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8118,7 +8092,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8244,7 +8218,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8288,7 +8262,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8373,7 +8347,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8417,7 +8391,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8461,7 +8435,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8505,7 +8479,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8549,7 +8523,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8593,7 +8567,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8637,7 +8611,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8681,7 +8655,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8766,7 +8740,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8933,7 +8907,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -8977,7 +8951,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9021,7 +8995,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9065,7 +9039,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9150,7 +9124,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9194,7 +9168,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9238,7 +9212,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9282,7 +9256,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9326,7 +9300,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9370,7 +9344,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9414,7 +9388,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9458,7 +9432,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9502,7 +9476,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9546,7 +9520,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9590,7 +9564,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9634,7 +9608,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9678,7 +9652,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9722,7 +9696,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9766,7 +9740,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9810,7 +9784,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9854,7 +9828,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9898,7 +9872,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9942,7 +9916,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -9986,7 +9960,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10030,7 +10004,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10115,7 +10089,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10200,7 +10174,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10215,55 +10189,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10550,7 +10524,7 @@
       <c r="L8" t="s">
         <v>568</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46289</v>
       </c>
       <c r="N8" t="s">
@@ -10635,7 +10609,7 @@
       <c r="L10" t="s">
         <v>569</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46334</v>
       </c>
       <c r="N10" t="s">
@@ -10679,7 +10653,7 @@
       <c r="L11" t="s">
         <v>569</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46334</v>
       </c>
       <c r="N11" t="s">
@@ -10846,7 +10820,7 @@
       <c r="L15" t="s">
         <v>568</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46289</v>
       </c>
       <c r="N15" t="s">
@@ -10890,7 +10864,7 @@
       <c r="L16" t="s">
         <v>569</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46334</v>
       </c>
       <c r="N16" t="s">
@@ -10934,7 +10908,7 @@
       <c r="L17" t="s">
         <v>568</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46289</v>
       </c>
       <c r="N17" t="s">
@@ -10978,7 +10952,7 @@
       <c r="L18" t="s">
         <v>569</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46334</v>
       </c>
       <c r="N18" t="s">
@@ -11022,7 +10996,7 @@
       <c r="L19" t="s">
         <v>569</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46334</v>
       </c>
       <c r="N19" t="s">
@@ -11066,7 +11040,7 @@
       <c r="L20" t="s">
         <v>569</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46334</v>
       </c>
       <c r="N20" t="s">
@@ -11110,7 +11084,7 @@
       <c r="L21" t="s">
         <v>569</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46334</v>
       </c>
       <c r="N21" t="s">
@@ -11277,7 +11251,7 @@
       <c r="L25" t="s">
         <v>569</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46334</v>
       </c>
       <c r="N25" t="s">
@@ -11362,7 +11336,7 @@
       <c r="L27" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46289</v>
       </c>
       <c r="N27" t="s">
@@ -11406,7 +11380,7 @@
       <c r="L28" t="s">
         <v>569</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46334</v>
       </c>
       <c r="N28" t="s">
@@ -11450,7 +11424,7 @@
       <c r="L29" t="s">
         <v>569</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46334</v>
       </c>
       <c r="N29" t="s">
@@ -11494,7 +11468,7 @@
       <c r="L30" t="s">
         <v>569</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46334</v>
       </c>
       <c r="N30" t="s">
@@ -11538,7 +11512,7 @@
       <c r="L31" t="s">
         <v>569</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46334</v>
       </c>
       <c r="N31" t="s">
@@ -11582,7 +11556,7 @@
       <c r="L32" t="s">
         <v>568</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46289</v>
       </c>
       <c r="N32" t="s">
@@ -11626,7 +11600,7 @@
       <c r="L33" t="s">
         <v>568</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46289</v>
       </c>
       <c r="N33" t="s">
@@ -11670,7 +11644,7 @@
       <c r="L34" t="s">
         <v>568</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46289</v>
       </c>
       <c r="N34" t="s">
@@ -11714,7 +11688,7 @@
       <c r="L35" t="s">
         <v>568</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46289</v>
       </c>
       <c r="N35" t="s">
@@ -11758,7 +11732,7 @@
       <c r="L36" t="s">
         <v>568</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46289</v>
       </c>
       <c r="N36" t="s">
@@ -11802,7 +11776,7 @@
       <c r="L37" t="s">
         <v>568</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46289</v>
       </c>
       <c r="N37" t="s">
@@ -11846,7 +11820,7 @@
       <c r="L38" t="s">
         <v>568</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46289</v>
       </c>
       <c r="N38" t="s">
@@ -11890,7 +11864,7 @@
       <c r="L39" t="s">
         <v>568</v>
       </c>
-      <c r="M39" s="2">
+      <c r="M39" s="1">
         <v>46289</v>
       </c>
       <c r="N39" t="s">
@@ -11934,7 +11908,7 @@
       <c r="L40" t="s">
         <v>568</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46289</v>
       </c>
       <c r="N40" t="s">
@@ -11978,7 +11952,7 @@
       <c r="L41" t="s">
         <v>569</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46334</v>
       </c>
       <c r="N41" t="s">
@@ -12022,7 +11996,7 @@
       <c r="L42" t="s">
         <v>568</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46289</v>
       </c>
       <c r="N42" t="s">
@@ -12066,7 +12040,7 @@
       <c r="L43" t="s">
         <v>571</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46349</v>
       </c>
       <c r="N43" t="s">
@@ -12110,7 +12084,7 @@
       <c r="L44" t="s">
         <v>571</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46349</v>
       </c>
       <c r="N44" t="s">
@@ -12154,7 +12128,7 @@
       <c r="L45" t="s">
         <v>569</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46334</v>
       </c>
       <c r="N45" t="s">
@@ -12198,7 +12172,7 @@
       <c r="L46" t="s">
         <v>568</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46289</v>
       </c>
       <c r="N46" t="s">
@@ -12242,7 +12216,7 @@
       <c r="L47" t="s">
         <v>568</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46289</v>
       </c>
       <c r="N47" t="s">
@@ -12286,7 +12260,7 @@
       <c r="L48" t="s">
         <v>569</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46334</v>
       </c>
       <c r="N48" t="s">
@@ -12330,7 +12304,7 @@
       <c r="L49" t="s">
         <v>569</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46334</v>
       </c>
       <c r="N49" t="s">
@@ -12374,7 +12348,7 @@
       <c r="L50" t="s">
         <v>569</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46334</v>
       </c>
       <c r="N50" t="s">
@@ -12418,7 +12392,7 @@
       <c r="L51" t="s">
         <v>569</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46334</v>
       </c>
       <c r="N51" t="s">
@@ -12462,7 +12436,7 @@
       <c r="L52" t="s">
         <v>569</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46334</v>
       </c>
       <c r="N52" t="s">
@@ -12506,7 +12480,7 @@
       <c r="L53" t="s">
         <v>569</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46334</v>
       </c>
       <c r="N53" t="s">
@@ -12550,7 +12524,7 @@
       <c r="L54" t="s">
         <v>569</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46334</v>
       </c>
       <c r="N54" t="s">
@@ -12594,7 +12568,7 @@
       <c r="L55" t="s">
         <v>569</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46334</v>
       </c>
       <c r="N55" t="s">
@@ -12638,7 +12612,7 @@
       <c r="L56" t="s">
         <v>569</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46334</v>
       </c>
       <c r="N56" t="s">
@@ -12682,7 +12656,7 @@
       <c r="L57" t="s">
         <v>569</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46334</v>
       </c>
       <c r="N57" t="s">
@@ -12726,7 +12700,7 @@
       <c r="L58" t="s">
         <v>569</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46334</v>
       </c>
       <c r="N58" t="s">
@@ -12770,7 +12744,7 @@
       <c r="L59" t="s">
         <v>569</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46334</v>
       </c>
       <c r="N59" t="s">
@@ -12814,7 +12788,7 @@
       <c r="L60" t="s">
         <v>569</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46334</v>
       </c>
       <c r="N60" t="s">
@@ -12858,7 +12832,7 @@
       <c r="L61" t="s">
         <v>569</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46334</v>
       </c>
       <c r="N61" t="s">
@@ -12902,7 +12876,7 @@
       <c r="L62" t="s">
         <v>571</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46349</v>
       </c>
       <c r="N62" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (26/08/2026 08:38)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="574">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1727,10 +1727,13 @@
     <t>Validada</t>
   </si>
   <si>
-    <t>Selecionada em Plano</t>
+    <t>Selecionada para Cotação</t>
   </si>
   <si>
     <t>Análise do Pedido</t>
+  </si>
+  <si>
+    <t>Selecionada para cotação</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10525,10 +10528,10 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N8" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10610,10 +10613,10 @@
         <v>569</v>
       </c>
       <c r="M10" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N10" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10654,10 +10657,10 @@
         <v>569</v>
       </c>
       <c r="M11" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N11" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10821,10 +10824,10 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N15" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10865,10 +10868,10 @@
         <v>569</v>
       </c>
       <c r="M16" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N16" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10909,10 +10912,10 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N17" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10953,10 +10956,10 @@
         <v>569</v>
       </c>
       <c r="M18" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N18" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10997,10 +11000,10 @@
         <v>569</v>
       </c>
       <c r="M19" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N19" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11041,10 +11044,10 @@
         <v>569</v>
       </c>
       <c r="M20" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N20" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11085,10 +11088,10 @@
         <v>569</v>
       </c>
       <c r="M21" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N21" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11252,10 +11255,10 @@
         <v>569</v>
       </c>
       <c r="M25" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N25" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11337,10 +11340,10 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N27" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11381,10 +11384,10 @@
         <v>569</v>
       </c>
       <c r="M28" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N28" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11416,19 +11419,19 @@
         <v>570</v>
       </c>
       <c r="J29" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K29" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L29" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M29" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N29" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11469,10 +11472,10 @@
         <v>569</v>
       </c>
       <c r="M30" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N30" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11504,19 +11507,19 @@
         <v>570</v>
       </c>
       <c r="J31" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K31" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L31" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M31" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N31" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11557,10 +11560,10 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N32" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11601,10 +11604,10 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N33" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11645,10 +11648,10 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N34" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11689,10 +11692,10 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N35" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11733,10 +11736,10 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N36" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11777,10 +11780,10 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N37" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11821,10 +11824,10 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N38" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11865,10 +11868,10 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N39" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11909,10 +11912,10 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N40" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11953,10 +11956,10 @@
         <v>569</v>
       </c>
       <c r="M41" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N41" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11997,10 +12000,10 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N42" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -12041,10 +12044,10 @@
         <v>571</v>
       </c>
       <c r="M43" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N43" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12085,10 +12088,10 @@
         <v>571</v>
       </c>
       <c r="M44" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N44" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12129,10 +12132,10 @@
         <v>569</v>
       </c>
       <c r="M45" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N45" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12173,10 +12176,10 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N46" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12217,10 +12220,10 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="N47" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12261,10 +12264,10 @@
         <v>569</v>
       </c>
       <c r="M48" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N48" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12296,19 +12299,19 @@
         <v>570</v>
       </c>
       <c r="J49" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K49" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L49" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M49" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N49" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12340,19 +12343,19 @@
         <v>570</v>
       </c>
       <c r="J50" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K50" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L50" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M50" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N50" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12393,10 +12396,10 @@
         <v>569</v>
       </c>
       <c r="M51" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N51" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12437,10 +12440,10 @@
         <v>569</v>
       </c>
       <c r="M52" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N52" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12481,10 +12484,10 @@
         <v>569</v>
       </c>
       <c r="M53" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N53" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12525,10 +12528,10 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N54" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12569,10 +12572,10 @@
         <v>569</v>
       </c>
       <c r="M55" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N55" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12604,19 +12607,19 @@
         <v>570</v>
       </c>
       <c r="J56" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K56" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L56" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M56" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N56" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12648,19 +12651,19 @@
         <v>570</v>
       </c>
       <c r="J57" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K57" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L57" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M57" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N57" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12692,19 +12695,19 @@
         <v>570</v>
       </c>
       <c r="J58" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K58" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L58" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M58" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N58" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -12745,10 +12748,10 @@
         <v>569</v>
       </c>
       <c r="M59" s="1">
-        <v>46334</v>
+        <v>46335</v>
       </c>
       <c r="N59" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -12780,19 +12783,19 @@
         <v>570</v>
       </c>
       <c r="J60" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K60" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L60" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M60" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N60" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -12824,19 +12827,19 @@
         <v>570</v>
       </c>
       <c r="J61" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="K61" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L61" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="M61" s="1">
-        <v>46334</v>
+        <v>46305</v>
       </c>
       <c r="N61" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -12877,10 +12880,10 @@
         <v>571</v>
       </c>
       <c r="M62" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N62" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (27/08/2026 18:00)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10528,7 +10528,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N8" t="s">
         <v>573</v>
@@ -10613,7 +10613,7 @@
         <v>569</v>
       </c>
       <c r="M10" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N10" t="s">
         <v>573</v>
@@ -10657,7 +10657,7 @@
         <v>569</v>
       </c>
       <c r="M11" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N11" t="s">
         <v>573</v>
@@ -10824,7 +10824,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N15" t="s">
         <v>573</v>
@@ -10868,7 +10868,7 @@
         <v>569</v>
       </c>
       <c r="M16" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N16" t="s">
         <v>573</v>
@@ -10912,7 +10912,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N17" t="s">
         <v>573</v>
@@ -10956,7 +10956,7 @@
         <v>569</v>
       </c>
       <c r="M18" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N18" t="s">
         <v>573</v>
@@ -11000,7 +11000,7 @@
         <v>569</v>
       </c>
       <c r="M19" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N19" t="s">
         <v>573</v>
@@ -11044,7 +11044,7 @@
         <v>569</v>
       </c>
       <c r="M20" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N20" t="s">
         <v>573</v>
@@ -11088,7 +11088,7 @@
         <v>569</v>
       </c>
       <c r="M21" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N21" t="s">
         <v>573</v>
@@ -11255,7 +11255,7 @@
         <v>569</v>
       </c>
       <c r="M25" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N25" t="s">
         <v>573</v>
@@ -11340,7 +11340,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N27" t="s">
         <v>573</v>
@@ -11384,7 +11384,7 @@
         <v>569</v>
       </c>
       <c r="M28" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N28" t="s">
         <v>573</v>
@@ -11428,7 +11428,7 @@
         <v>572</v>
       </c>
       <c r="M29" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N29" t="s">
         <v>573</v>
@@ -11472,7 +11472,7 @@
         <v>569</v>
       </c>
       <c r="M30" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N30" t="s">
         <v>573</v>
@@ -11516,7 +11516,7 @@
         <v>572</v>
       </c>
       <c r="M31" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N31" t="s">
         <v>573</v>
@@ -11560,7 +11560,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N32" t="s">
         <v>573</v>
@@ -11604,7 +11604,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N33" t="s">
         <v>573</v>
@@ -11648,7 +11648,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N34" t="s">
         <v>573</v>
@@ -11692,7 +11692,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N35" t="s">
         <v>573</v>
@@ -11736,7 +11736,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N36" t="s">
         <v>573</v>
@@ -11780,7 +11780,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N37" t="s">
         <v>573</v>
@@ -11824,7 +11824,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N38" t="s">
         <v>573</v>
@@ -11868,7 +11868,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N39" t="s">
         <v>573</v>
@@ -11912,7 +11912,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N40" t="s">
         <v>573</v>
@@ -11956,7 +11956,7 @@
         <v>569</v>
       </c>
       <c r="M41" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N41" t="s">
         <v>573</v>
@@ -12000,7 +12000,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N42" t="s">
         <v>573</v>
@@ -12044,7 +12044,7 @@
         <v>571</v>
       </c>
       <c r="M43" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N43" t="s">
         <v>573</v>
@@ -12088,7 +12088,7 @@
         <v>571</v>
       </c>
       <c r="M44" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N44" t="s">
         <v>573</v>
@@ -12132,7 +12132,7 @@
         <v>569</v>
       </c>
       <c r="M45" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N45" t="s">
         <v>573</v>
@@ -12176,7 +12176,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N46" t="s">
         <v>573</v>
@@ -12220,7 +12220,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="N47" t="s">
         <v>573</v>
@@ -12264,7 +12264,7 @@
         <v>569</v>
       </c>
       <c r="M48" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N48" t="s">
         <v>573</v>
@@ -12308,7 +12308,7 @@
         <v>572</v>
       </c>
       <c r="M49" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N49" t="s">
         <v>573</v>
@@ -12352,7 +12352,7 @@
         <v>572</v>
       </c>
       <c r="M50" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N50" t="s">
         <v>573</v>
@@ -12396,7 +12396,7 @@
         <v>569</v>
       </c>
       <c r="M51" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N51" t="s">
         <v>573</v>
@@ -12440,7 +12440,7 @@
         <v>569</v>
       </c>
       <c r="M52" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N52" t="s">
         <v>573</v>
@@ -12484,7 +12484,7 @@
         <v>569</v>
       </c>
       <c r="M53" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N53" t="s">
         <v>573</v>
@@ -12528,7 +12528,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N54" t="s">
         <v>573</v>
@@ -12572,7 +12572,7 @@
         <v>569</v>
       </c>
       <c r="M55" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N55" t="s">
         <v>573</v>
@@ -12616,7 +12616,7 @@
         <v>572</v>
       </c>
       <c r="M56" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N56" t="s">
         <v>573</v>
@@ -12660,7 +12660,7 @@
         <v>572</v>
       </c>
       <c r="M57" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N57" t="s">
         <v>573</v>
@@ -12704,7 +12704,7 @@
         <v>572</v>
       </c>
       <c r="M58" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N58" t="s">
         <v>573</v>
@@ -12748,7 +12748,7 @@
         <v>569</v>
       </c>
       <c r="M59" s="1">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="N59" t="s">
         <v>573</v>
@@ -12792,7 +12792,7 @@
         <v>572</v>
       </c>
       <c r="M60" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N60" t="s">
         <v>573</v>
@@ -12836,7 +12836,7 @@
         <v>572</v>
       </c>
       <c r="M61" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N61" t="s">
         <v>573</v>
@@ -12880,7 +12880,7 @@
         <v>571</v>
       </c>
       <c r="M62" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N62" t="s">
         <v>573</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (28/08/2026 02:14)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10528,7 +10528,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N8" t="s">
         <v>573</v>
@@ -10613,7 +10613,7 @@
         <v>569</v>
       </c>
       <c r="M10" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N10" t="s">
         <v>573</v>
@@ -10657,7 +10657,7 @@
         <v>569</v>
       </c>
       <c r="M11" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N11" t="s">
         <v>573</v>
@@ -10824,7 +10824,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N15" t="s">
         <v>573</v>
@@ -10868,7 +10868,7 @@
         <v>569</v>
       </c>
       <c r="M16" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N16" t="s">
         <v>573</v>
@@ -10912,7 +10912,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N17" t="s">
         <v>573</v>
@@ -10956,7 +10956,7 @@
         <v>569</v>
       </c>
       <c r="M18" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N18" t="s">
         <v>573</v>
@@ -11000,7 +11000,7 @@
         <v>569</v>
       </c>
       <c r="M19" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N19" t="s">
         <v>573</v>
@@ -11044,7 +11044,7 @@
         <v>569</v>
       </c>
       <c r="M20" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N20" t="s">
         <v>573</v>
@@ -11088,7 +11088,7 @@
         <v>569</v>
       </c>
       <c r="M21" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N21" t="s">
         <v>573</v>
@@ -11255,7 +11255,7 @@
         <v>569</v>
       </c>
       <c r="M25" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N25" t="s">
         <v>573</v>
@@ -11340,7 +11340,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N27" t="s">
         <v>573</v>
@@ -11384,7 +11384,7 @@
         <v>569</v>
       </c>
       <c r="M28" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N28" t="s">
         <v>573</v>
@@ -11428,7 +11428,7 @@
         <v>572</v>
       </c>
       <c r="M29" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N29" t="s">
         <v>573</v>
@@ -11472,7 +11472,7 @@
         <v>569</v>
       </c>
       <c r="M30" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N30" t="s">
         <v>573</v>
@@ -11516,7 +11516,7 @@
         <v>572</v>
       </c>
       <c r="M31" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N31" t="s">
         <v>573</v>
@@ -11560,7 +11560,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N32" t="s">
         <v>573</v>
@@ -11604,7 +11604,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N33" t="s">
         <v>573</v>
@@ -11648,7 +11648,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N34" t="s">
         <v>573</v>
@@ -11692,7 +11692,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N35" t="s">
         <v>573</v>
@@ -11736,7 +11736,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N36" t="s">
         <v>573</v>
@@ -11780,7 +11780,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N37" t="s">
         <v>573</v>
@@ -11824,7 +11824,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N38" t="s">
         <v>573</v>
@@ -11868,7 +11868,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N39" t="s">
         <v>573</v>
@@ -11912,7 +11912,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N40" t="s">
         <v>573</v>
@@ -11956,7 +11956,7 @@
         <v>569</v>
       </c>
       <c r="M41" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N41" t="s">
         <v>573</v>
@@ -12000,7 +12000,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N42" t="s">
         <v>573</v>
@@ -12044,7 +12044,7 @@
         <v>571</v>
       </c>
       <c r="M43" s="1">
-        <v>46351</v>
+        <v>46352</v>
       </c>
       <c r="N43" t="s">
         <v>573</v>
@@ -12088,7 +12088,7 @@
         <v>571</v>
       </c>
       <c r="M44" s="1">
-        <v>46351</v>
+        <v>46352</v>
       </c>
       <c r="N44" t="s">
         <v>573</v>
@@ -12132,7 +12132,7 @@
         <v>569</v>
       </c>
       <c r="M45" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N45" t="s">
         <v>573</v>
@@ -12176,7 +12176,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N46" t="s">
         <v>573</v>
@@ -12220,7 +12220,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="N47" t="s">
         <v>573</v>
@@ -12264,7 +12264,7 @@
         <v>569</v>
       </c>
       <c r="M48" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N48" t="s">
         <v>573</v>
@@ -12308,7 +12308,7 @@
         <v>572</v>
       </c>
       <c r="M49" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N49" t="s">
         <v>573</v>
@@ -12352,7 +12352,7 @@
         <v>572</v>
       </c>
       <c r="M50" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N50" t="s">
         <v>573</v>
@@ -12396,7 +12396,7 @@
         <v>569</v>
       </c>
       <c r="M51" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N51" t="s">
         <v>573</v>
@@ -12440,7 +12440,7 @@
         <v>569</v>
       </c>
       <c r="M52" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N52" t="s">
         <v>573</v>
@@ -12484,7 +12484,7 @@
         <v>569</v>
       </c>
       <c r="M53" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N53" t="s">
         <v>573</v>
@@ -12528,7 +12528,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N54" t="s">
         <v>573</v>
@@ -12572,7 +12572,7 @@
         <v>569</v>
       </c>
       <c r="M55" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N55" t="s">
         <v>573</v>
@@ -12616,7 +12616,7 @@
         <v>572</v>
       </c>
       <c r="M56" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N56" t="s">
         <v>573</v>
@@ -12660,7 +12660,7 @@
         <v>572</v>
       </c>
       <c r="M57" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N57" t="s">
         <v>573</v>
@@ -12704,7 +12704,7 @@
         <v>572</v>
       </c>
       <c r="M58" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N58" t="s">
         <v>573</v>
@@ -12748,7 +12748,7 @@
         <v>569</v>
       </c>
       <c r="M59" s="1">
-        <v>46336</v>
+        <v>46337</v>
       </c>
       <c r="N59" t="s">
         <v>573</v>
@@ -12792,7 +12792,7 @@
         <v>572</v>
       </c>
       <c r="M60" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N60" t="s">
         <v>573</v>
@@ -12836,7 +12836,7 @@
         <v>572</v>
       </c>
       <c r="M61" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="N61" t="s">
         <v>573</v>
@@ -12880,7 +12880,7 @@
         <v>571</v>
       </c>
       <c r="M62" s="1">
-        <v>46351</v>
+        <v>46352</v>
       </c>
       <c r="N62" t="s">
         <v>573</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (29/08/2026 01:08)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10528,7 +10528,7 @@
         <v>568</v>
       </c>
       <c r="M8" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N8" t="s">
         <v>573</v>
@@ -10613,7 +10613,7 @@
         <v>569</v>
       </c>
       <c r="M10" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N10" t="s">
         <v>573</v>
@@ -10657,7 +10657,7 @@
         <v>569</v>
       </c>
       <c r="M11" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N11" t="s">
         <v>573</v>
@@ -10824,7 +10824,7 @@
         <v>568</v>
       </c>
       <c r="M15" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N15" t="s">
         <v>573</v>
@@ -10868,7 +10868,7 @@
         <v>569</v>
       </c>
       <c r="M16" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N16" t="s">
         <v>573</v>
@@ -10912,7 +10912,7 @@
         <v>568</v>
       </c>
       <c r="M17" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N17" t="s">
         <v>573</v>
@@ -10956,7 +10956,7 @@
         <v>569</v>
       </c>
       <c r="M18" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N18" t="s">
         <v>573</v>
@@ -11000,7 +11000,7 @@
         <v>569</v>
       </c>
       <c r="M19" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N19" t="s">
         <v>573</v>
@@ -11044,7 +11044,7 @@
         <v>569</v>
       </c>
       <c r="M20" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N20" t="s">
         <v>573</v>
@@ -11088,7 +11088,7 @@
         <v>569</v>
       </c>
       <c r="M21" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N21" t="s">
         <v>573</v>
@@ -11255,7 +11255,7 @@
         <v>569</v>
       </c>
       <c r="M25" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N25" t="s">
         <v>573</v>
@@ -11340,7 +11340,7 @@
         <v>568</v>
       </c>
       <c r="M27" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N27" t="s">
         <v>573</v>
@@ -11384,7 +11384,7 @@
         <v>569</v>
       </c>
       <c r="M28" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N28" t="s">
         <v>573</v>
@@ -11428,7 +11428,7 @@
         <v>572</v>
       </c>
       <c r="M29" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N29" t="s">
         <v>573</v>
@@ -11472,7 +11472,7 @@
         <v>569</v>
       </c>
       <c r="M30" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N30" t="s">
         <v>573</v>
@@ -11516,7 +11516,7 @@
         <v>572</v>
       </c>
       <c r="M31" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N31" t="s">
         <v>573</v>
@@ -11560,7 +11560,7 @@
         <v>568</v>
       </c>
       <c r="M32" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N32" t="s">
         <v>573</v>
@@ -11604,7 +11604,7 @@
         <v>568</v>
       </c>
       <c r="M33" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N33" t="s">
         <v>573</v>
@@ -11648,7 +11648,7 @@
         <v>568</v>
       </c>
       <c r="M34" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N34" t="s">
         <v>573</v>
@@ -11692,7 +11692,7 @@
         <v>568</v>
       </c>
       <c r="M35" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N35" t="s">
         <v>573</v>
@@ -11736,7 +11736,7 @@
         <v>568</v>
       </c>
       <c r="M36" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N36" t="s">
         <v>573</v>
@@ -11780,7 +11780,7 @@
         <v>568</v>
       </c>
       <c r="M37" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N37" t="s">
         <v>573</v>
@@ -11824,7 +11824,7 @@
         <v>568</v>
       </c>
       <c r="M38" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N38" t="s">
         <v>573</v>
@@ -11868,7 +11868,7 @@
         <v>568</v>
       </c>
       <c r="M39" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N39" t="s">
         <v>573</v>
@@ -11912,7 +11912,7 @@
         <v>568</v>
       </c>
       <c r="M40" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N40" t="s">
         <v>573</v>
@@ -11956,7 +11956,7 @@
         <v>569</v>
       </c>
       <c r="M41" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N41" t="s">
         <v>573</v>
@@ -12000,7 +12000,7 @@
         <v>568</v>
       </c>
       <c r="M42" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N42" t="s">
         <v>573</v>
@@ -12044,7 +12044,7 @@
         <v>571</v>
       </c>
       <c r="M43" s="1">
-        <v>46352</v>
+        <v>46353</v>
       </c>
       <c r="N43" t="s">
         <v>573</v>
@@ -12088,7 +12088,7 @@
         <v>571</v>
       </c>
       <c r="M44" s="1">
-        <v>46352</v>
+        <v>46353</v>
       </c>
       <c r="N44" t="s">
         <v>573</v>
@@ -12132,7 +12132,7 @@
         <v>569</v>
       </c>
       <c r="M45" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N45" t="s">
         <v>573</v>
@@ -12176,7 +12176,7 @@
         <v>568</v>
       </c>
       <c r="M46" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N46" t="s">
         <v>573</v>
@@ -12220,7 +12220,7 @@
         <v>568</v>
       </c>
       <c r="M47" s="1">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="N47" t="s">
         <v>573</v>
@@ -12264,7 +12264,7 @@
         <v>569</v>
       </c>
       <c r="M48" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N48" t="s">
         <v>573</v>
@@ -12308,7 +12308,7 @@
         <v>572</v>
       </c>
       <c r="M49" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N49" t="s">
         <v>573</v>
@@ -12352,7 +12352,7 @@
         <v>572</v>
       </c>
       <c r="M50" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N50" t="s">
         <v>573</v>
@@ -12396,7 +12396,7 @@
         <v>569</v>
       </c>
       <c r="M51" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N51" t="s">
         <v>573</v>
@@ -12440,7 +12440,7 @@
         <v>569</v>
       </c>
       <c r="M52" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N52" t="s">
         <v>573</v>
@@ -12484,7 +12484,7 @@
         <v>569</v>
       </c>
       <c r="M53" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N53" t="s">
         <v>573</v>
@@ -12528,7 +12528,7 @@
         <v>569</v>
       </c>
       <c r="M54" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N54" t="s">
         <v>573</v>
@@ -12572,7 +12572,7 @@
         <v>569</v>
       </c>
       <c r="M55" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N55" t="s">
         <v>573</v>
@@ -12616,7 +12616,7 @@
         <v>572</v>
       </c>
       <c r="M56" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N56" t="s">
         <v>573</v>
@@ -12660,7 +12660,7 @@
         <v>572</v>
       </c>
       <c r="M57" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N57" t="s">
         <v>573</v>
@@ -12704,7 +12704,7 @@
         <v>572</v>
       </c>
       <c r="M58" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N58" t="s">
         <v>573</v>
@@ -12748,7 +12748,7 @@
         <v>569</v>
       </c>
       <c r="M59" s="1">
-        <v>46337</v>
+        <v>46338</v>
       </c>
       <c r="N59" t="s">
         <v>573</v>
@@ -12792,7 +12792,7 @@
         <v>572</v>
       </c>
       <c r="M60" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N60" t="s">
         <v>573</v>
@@ -12836,7 +12836,7 @@
         <v>572</v>
       </c>
       <c r="M61" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="N61" t="s">
         <v>573</v>
@@ -12880,7 +12880,7 @@
         <v>571</v>
       </c>
       <c r="M62" s="1">
-        <v>46352</v>
+        <v>46353</v>
       </c>
       <c r="N62" t="s">
         <v>573</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (31/08/2026 15:00)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2546" uniqueCount="583">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1418,6 +1418,18 @@
     <t>LST225001U8</t>
   </si>
   <si>
+    <t>LST238006U8</t>
+  </si>
+  <si>
+    <t>LST239001U8</t>
+  </si>
+  <si>
+    <t>LST240003U8</t>
+  </si>
+  <si>
+    <t>LST243001U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1577,6 +1589,15 @@
     <t>71014</t>
   </si>
   <si>
+    <t>M81934/2-32C032</t>
+  </si>
+  <si>
+    <t>2601102-1</t>
+  </si>
+  <si>
+    <t>S3461-76</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1716,6 +1737,12 @@
   </si>
   <si>
     <t>CAP</t>
+  </si>
+  <si>
+    <t>HINGE-ASSY-HOISTING</t>
+  </si>
+  <si>
+    <t>BOLT MPI</t>
   </si>
   <si>
     <t>Empenho Solicitado</t>
@@ -10188,7 +10215,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q62"/>
+  <dimension ref="A1:Q66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10270,7 +10297,7 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J2" t="s">
         <v>387</v>
@@ -10311,7 +10338,7 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J3" t="s">
         <v>387</v>
@@ -10337,7 +10364,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10352,7 +10379,7 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J4" t="s">
         <v>387</v>
@@ -10378,10 +10405,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="E5" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10434,7 +10461,7 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J6" t="s">
         <v>387</v>
@@ -10475,7 +10502,7 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J7" t="s">
         <v>387</v>
@@ -10516,22 +10543,22 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J8" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K8" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L8" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M8" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N8" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10545,7 +10572,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10560,7 +10587,7 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J9" t="s">
         <v>387</v>
@@ -10586,10 +10613,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="E10" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10604,19 +10631,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K10" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L10" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M10" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N10" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10630,7 +10657,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10648,19 +10675,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K11" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L11" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M11" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N11" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10674,10 +10701,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="E12" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -10730,7 +10757,7 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J13" t="s">
         <v>387</v>
@@ -10756,10 +10783,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="E14" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -10771,7 +10798,7 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J14" t="s">
         <v>387</v>
@@ -10797,10 +10824,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="E15" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -10812,22 +10839,22 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J15" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K15" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L15" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M15" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N15" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10841,10 +10868,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="E16" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -10859,19 +10886,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K16" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L16" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M16" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N16" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10885,10 +10912,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="E17" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -10900,22 +10927,22 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J17" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K17" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L17" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M17" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N17" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10929,10 +10956,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="E18" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -10947,19 +10974,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K18" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L18" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M18" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N18" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -10973,10 +11000,10 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="E19" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
       <c r="F19">
         <v>4</v>
@@ -10991,19 +11018,19 @@
         <v>382</v>
       </c>
       <c r="J19" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K19" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L19" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M19" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N19" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11017,10 +11044,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="E20" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -11035,19 +11062,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K20" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L20" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M20" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N20" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11061,10 +11088,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="E21" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11079,19 +11106,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K21" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L21" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M21" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N21" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11105,10 +11132,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="E22" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11120,7 +11147,7 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J22" t="s">
         <v>387</v>
@@ -11146,10 +11173,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="E23" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11161,7 +11188,7 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J23" t="s">
         <v>387</v>
@@ -11187,7 +11214,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11202,7 +11229,7 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J24" t="s">
         <v>387</v>
@@ -11228,10 +11255,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="E25" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11243,22 +11270,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="J25" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K25" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L25" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M25" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N25" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11272,10 +11299,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="E26" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11287,7 +11314,7 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="J26" t="s">
         <v>387</v>
@@ -11313,10 +11340,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="E27" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11328,22 +11355,22 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J27" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K27" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L27" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M27" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N27" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11357,10 +11384,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="E28" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11375,19 +11402,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K28" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L28" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M28" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N28" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11401,10 +11428,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="E29" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11416,22 +11443,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J29" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K29" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L29" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M29" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N29" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11445,10 +11472,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="E30" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11463,19 +11490,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K30" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L30" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M30" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N30" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11489,10 +11516,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="E31" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11504,22 +11531,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J31" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K31" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L31" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M31" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N31" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11533,10 +11560,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="E32" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11548,22 +11575,22 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J32" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K32" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L32" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M32" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N32" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11577,10 +11604,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="E33" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11592,22 +11619,22 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J33" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K33" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L33" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M33" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N33" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11621,10 +11648,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="E34" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11636,22 +11663,22 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J34" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K34" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L34" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M34" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N34" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11665,10 +11692,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="E35" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11680,22 +11707,22 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J35" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K35" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L35" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M35" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N35" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11709,10 +11736,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="E36" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -11724,22 +11751,22 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J36" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K36" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L36" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M36" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N36" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11753,10 +11780,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="E37" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -11768,22 +11795,22 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J37" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K37" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L37" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M37" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N37" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11797,10 +11824,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="E38" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -11812,22 +11839,22 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J38" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K38" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L38" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M38" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N38" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11841,10 +11868,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="E39" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -11856,22 +11883,19 @@
         <v>312.36</v>
       </c>
       <c r="I39" t="s">
-        <v>568</v>
+        <v>391</v>
       </c>
       <c r="J39" t="s">
-        <v>568</v>
+        <v>391</v>
       </c>
       <c r="K39" t="s">
-        <v>568</v>
+        <v>391</v>
       </c>
       <c r="L39" t="s">
-        <v>568</v>
-      </c>
-      <c r="M39" s="1">
-        <v>46293</v>
+        <v>391</v>
       </c>
       <c r="N39" t="s">
-        <v>573</v>
+        <v>395</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -11885,10 +11909,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="E40" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -11900,22 +11924,22 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J40" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K40" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L40" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M40" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N40" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11929,10 +11953,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="E41" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -11947,19 +11971,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K41" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L41" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M41" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N41" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -11988,22 +12012,22 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J42" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K42" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L42" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M42" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N42" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -12017,37 +12041,37 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="E43" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="F43">
         <v>1</v>
       </c>
       <c r="G43">
-        <v>5000</v>
+        <v>7890.58</v>
       </c>
       <c r="H43">
-        <v>5000</v>
+        <v>7890.58</v>
       </c>
       <c r="I43" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="J43" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="K43" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="L43" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="M43" s="1">
-        <v>46353</v>
+        <v>46355</v>
       </c>
       <c r="N43" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12061,7 +12085,7 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
@@ -12076,22 +12100,22 @@
         <v>352.52</v>
       </c>
       <c r="I44" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="J44" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="K44" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="L44" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="M44" s="1">
-        <v>46353</v>
+        <v>46340</v>
       </c>
       <c r="N44" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12105,10 +12129,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="E45" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12120,22 +12144,22 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="J45" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K45" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L45" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M45" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N45" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12149,10 +12173,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="E46" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12164,22 +12188,22 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J46" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K46" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L46" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M46" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N46" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12193,10 +12217,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="E47" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12208,22 +12232,22 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="J47" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="K47" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="L47" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="M47" s="1">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="N47" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12237,10 +12261,10 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="E48" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -12252,22 +12276,22 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="J48" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K48" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L48" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M48" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N48" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12281,10 +12305,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="E49" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12296,22 +12320,22 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J49" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K49" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L49" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M49" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N49" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12325,10 +12349,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="E50" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12340,22 +12364,22 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J50" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K50" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L50" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M50" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N50" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12369,10 +12393,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="E51" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12387,19 +12411,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K51" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L51" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M51" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N51" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12413,10 +12437,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="E52" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12431,19 +12455,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K52" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L52" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M52" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N52" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12457,10 +12481,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="E53" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12475,19 +12499,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K53" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L53" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M53" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N53" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12501,10 +12525,10 @@
         <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E54" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
       <c r="F54">
         <v>4</v>
@@ -12516,22 +12540,22 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="J54" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K54" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L54" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M54" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N54" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12545,10 +12569,10 @@
         <v>173</v>
       </c>
       <c r="D55" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="E55" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="F55">
         <v>1</v>
@@ -12563,19 +12587,19 @@
         <v>382</v>
       </c>
       <c r="J55" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K55" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L55" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M55" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N55" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12589,10 +12613,10 @@
         <v>173</v>
       </c>
       <c r="D56" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="E56" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -12604,22 +12628,22 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J56" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K56" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L56" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M56" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N56" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12633,10 +12657,10 @@
         <v>173</v>
       </c>
       <c r="D57" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="E57" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -12648,22 +12672,22 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J57" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K57" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L57" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M57" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N57" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12677,10 +12701,10 @@
         <v>173</v>
       </c>
       <c r="D58" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="E58" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
       <c r="F58">
         <v>4</v>
@@ -12692,22 +12716,22 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J58" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K58" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L58" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M58" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N58" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -12736,22 +12760,22 @@
         <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="J59" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="K59" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="L59" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="M59" s="1">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="N59" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -12765,10 +12789,10 @@
         <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="E60" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -12780,22 +12804,22 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J60" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K60" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L60" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M60" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N60" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -12809,10 +12833,10 @@
         <v>173</v>
       </c>
       <c r="D61" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="E61" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
       <c r="F61">
         <v>5</v>
@@ -12824,22 +12848,22 @@
         <v>5645.05</v>
       </c>
       <c r="I61" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="J61" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="K61" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="L61" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="M61" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="N61" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -12853,10 +12877,10 @@
         <v>173</v>
       </c>
       <c r="D62" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="E62" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
       <c r="F62">
         <v>21</v>
@@ -12868,22 +12892,198 @@
         <v>204.96</v>
       </c>
       <c r="I62" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="J62" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="K62" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="L62" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="M62" s="1">
-        <v>46353</v>
+        <v>46340</v>
       </c>
       <c r="N62" t="s">
-        <v>573</v>
+        <v>582</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14">
+      <c r="A63" t="s">
+        <v>467</v>
+      </c>
+      <c r="B63" t="s">
+        <v>172</v>
+      </c>
+      <c r="C63" t="s">
+        <v>173</v>
+      </c>
+      <c r="D63" t="s">
+        <v>233</v>
+      </c>
+      <c r="E63" t="s">
+        <v>334</v>
+      </c>
+      <c r="F63">
+        <v>100</v>
+      </c>
+      <c r="G63">
+        <v>4.37</v>
+      </c>
+      <c r="H63">
+        <v>437</v>
+      </c>
+      <c r="I63" t="s">
+        <v>382</v>
+      </c>
+      <c r="J63" t="s">
+        <v>578</v>
+      </c>
+      <c r="K63" t="s">
+        <v>578</v>
+      </c>
+      <c r="L63" t="s">
+        <v>578</v>
+      </c>
+      <c r="M63" s="1">
+        <v>46340</v>
+      </c>
+      <c r="N63" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14">
+      <c r="A64" t="s">
+        <v>468</v>
+      </c>
+      <c r="B64" t="s">
+        <v>172</v>
+      </c>
+      <c r="C64" t="s">
+        <v>173</v>
+      </c>
+      <c r="D64" t="s">
+        <v>524</v>
+      </c>
+      <c r="E64" t="s">
+        <v>308</v>
+      </c>
+      <c r="F64">
+        <v>8</v>
+      </c>
+      <c r="G64">
+        <v>249.94</v>
+      </c>
+      <c r="H64">
+        <v>1999.52</v>
+      </c>
+      <c r="I64" t="s">
+        <v>580</v>
+      </c>
+      <c r="J64" t="s">
+        <v>580</v>
+      </c>
+      <c r="K64" t="s">
+        <v>580</v>
+      </c>
+      <c r="L64" t="s">
+        <v>580</v>
+      </c>
+      <c r="M64" s="1">
+        <v>46355</v>
+      </c>
+      <c r="N64" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14">
+      <c r="A65" t="s">
+        <v>469</v>
+      </c>
+      <c r="B65" t="s">
+        <v>172</v>
+      </c>
+      <c r="C65" t="s">
+        <v>173</v>
+      </c>
+      <c r="D65" t="s">
+        <v>525</v>
+      </c>
+      <c r="E65" t="s">
+        <v>574</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+      <c r="G65">
+        <v>4742.74</v>
+      </c>
+      <c r="H65">
+        <v>9485.48</v>
+      </c>
+      <c r="I65" t="s">
+        <v>382</v>
+      </c>
+      <c r="J65" t="s">
+        <v>578</v>
+      </c>
+      <c r="K65" t="s">
+        <v>578</v>
+      </c>
+      <c r="L65" t="s">
+        <v>578</v>
+      </c>
+      <c r="M65" s="1">
+        <v>46340</v>
+      </c>
+      <c r="N65" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
+      <c r="A66" t="s">
+        <v>470</v>
+      </c>
+      <c r="B66" t="s">
+        <v>172</v>
+      </c>
+      <c r="C66" t="s">
+        <v>173</v>
+      </c>
+      <c r="D66" t="s">
+        <v>526</v>
+      </c>
+      <c r="E66" t="s">
+        <v>575</v>
+      </c>
+      <c r="F66">
+        <v>2</v>
+      </c>
+      <c r="G66">
+        <v>148.96</v>
+      </c>
+      <c r="H66">
+        <v>297.92</v>
+      </c>
+      <c r="I66" t="s">
+        <v>382</v>
+      </c>
+      <c r="J66" t="s">
+        <v>578</v>
+      </c>
+      <c r="K66" t="s">
+        <v>578</v>
+      </c>
+      <c r="L66" t="s">
+        <v>578</v>
+      </c>
+      <c r="M66" s="1">
+        <v>46340</v>
+      </c>
+      <c r="N66" t="s">
+        <v>582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (01/09/2026 11:16)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,8 +1773,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1790,7 +1798,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1798,12 +1806,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2103,55 +2129,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2195,7 +2221,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2239,7 +2265,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2283,7 +2309,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2409,7 +2435,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2453,7 +2479,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2497,7 +2523,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2544,7 +2570,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2667,7 +2693,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2711,7 +2737,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2755,7 +2781,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2799,7 +2825,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2846,7 +2872,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2890,7 +2916,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3016,7 +3042,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3060,7 +3086,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3145,7 +3171,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3192,7 +3218,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3239,7 +3265,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3283,7 +3309,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3327,7 +3353,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3412,7 +3438,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3497,7 +3523,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3544,7 +3570,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3588,7 +3614,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3632,7 +3658,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3717,7 +3743,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3761,7 +3787,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3805,7 +3831,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3890,7 +3916,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3934,7 +3960,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3978,7 +4004,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4022,7 +4048,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4189,7 +4215,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4233,7 +4259,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4277,7 +4303,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4321,7 +4347,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4368,7 +4394,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4412,7 +4438,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4494,7 +4520,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4538,7 +4564,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4626,7 +4652,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4670,7 +4696,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4717,7 +4743,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4761,7 +4787,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4805,7 +4831,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4849,7 +4875,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4893,7 +4919,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4940,7 +4966,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4984,7 +5010,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5031,7 +5057,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5075,7 +5101,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5122,7 +5148,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5210,7 +5236,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5254,7 +5280,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5298,7 +5324,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5342,7 +5368,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5386,7 +5412,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5430,7 +5456,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5515,7 +5541,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5559,7 +5585,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5603,7 +5629,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5647,7 +5673,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5691,7 +5717,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5735,7 +5761,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5779,7 +5805,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5823,7 +5849,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5870,7 +5896,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5914,7 +5940,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5958,7 +5984,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6002,7 +6028,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6046,7 +6072,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6090,7 +6116,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6134,7 +6160,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6178,7 +6204,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6222,7 +6248,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6310,7 +6336,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6354,7 +6380,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6480,7 +6506,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6524,7 +6550,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6568,7 +6594,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6612,7 +6638,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6694,7 +6720,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6738,7 +6764,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6785,7 +6811,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6829,7 +6855,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6955,7 +6981,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6999,7 +7025,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7084,7 +7110,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7128,7 +7154,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7172,7 +7198,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7216,7 +7242,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7260,7 +7286,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7304,7 +7330,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7348,7 +7374,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7392,7 +7418,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7477,7 +7503,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7644,7 +7670,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7688,7 +7714,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7732,7 +7758,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7776,7 +7802,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7820,7 +7846,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7864,7 +7890,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7908,7 +7934,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7993,7 +8019,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8037,7 +8063,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8122,7 +8148,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8248,7 +8274,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8292,7 +8318,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8377,7 +8403,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8421,7 +8447,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8465,7 +8491,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8509,7 +8535,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8553,7 +8579,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8597,7 +8623,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8641,7 +8667,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8685,7 +8711,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8770,7 +8796,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8937,7 +8963,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8981,7 +9007,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9025,7 +9051,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9069,7 +9095,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9154,7 +9180,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9198,7 +9224,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9242,7 +9268,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9286,7 +9312,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9330,7 +9356,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9374,7 +9400,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9418,7 +9444,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9462,7 +9488,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9506,7 +9532,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9550,7 +9576,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9594,7 +9620,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9638,7 +9664,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9682,7 +9708,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9726,7 +9752,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9770,7 +9796,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9814,7 +9840,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9858,7 +9884,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9902,7 +9928,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9946,7 +9972,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9990,7 +10016,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10034,7 +10060,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10119,7 +10145,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10204,7 +10230,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10219,55 +10245,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10554,8 +10580,8 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="1">
-        <v>46295</v>
+      <c r="M8" s="2">
+        <v>46296</v>
       </c>
       <c r="N8" t="s">
         <v>582</v>
@@ -10639,8 +10665,8 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="1">
-        <v>46340</v>
+      <c r="M10" s="2">
+        <v>46341</v>
       </c>
       <c r="N10" t="s">
         <v>582</v>
@@ -10683,8 +10709,8 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="1">
-        <v>46340</v>
+      <c r="M11" s="2">
+        <v>46341</v>
       </c>
       <c r="N11" t="s">
         <v>582</v>
@@ -10850,8 +10876,8 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="1">
-        <v>46295</v>
+      <c r="M15" s="2">
+        <v>46296</v>
       </c>
       <c r="N15" t="s">
         <v>582</v>
@@ -10894,8 +10920,8 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="1">
-        <v>46340</v>
+      <c r="M16" s="2">
+        <v>46341</v>
       </c>
       <c r="N16" t="s">
         <v>582</v>
@@ -10938,8 +10964,8 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="1">
-        <v>46295</v>
+      <c r="M17" s="2">
+        <v>46296</v>
       </c>
       <c r="N17" t="s">
         <v>582</v>
@@ -10982,8 +11008,8 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="1">
-        <v>46340</v>
+      <c r="M18" s="2">
+        <v>46341</v>
       </c>
       <c r="N18" t="s">
         <v>582</v>
@@ -11026,8 +11052,8 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="1">
-        <v>46340</v>
+      <c r="M19" s="2">
+        <v>46341</v>
       </c>
       <c r="N19" t="s">
         <v>582</v>
@@ -11070,8 +11096,8 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="1">
-        <v>46340</v>
+      <c r="M20" s="2">
+        <v>46341</v>
       </c>
       <c r="N20" t="s">
         <v>582</v>
@@ -11114,8 +11140,8 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="1">
-        <v>46340</v>
+      <c r="M21" s="2">
+        <v>46341</v>
       </c>
       <c r="N21" t="s">
         <v>582</v>
@@ -11281,8 +11307,8 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="1">
-        <v>46340</v>
+      <c r="M25" s="2">
+        <v>46341</v>
       </c>
       <c r="N25" t="s">
         <v>582</v>
@@ -11366,8 +11392,8 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="1">
-        <v>46295</v>
+      <c r="M27" s="2">
+        <v>46296</v>
       </c>
       <c r="N27" t="s">
         <v>582</v>
@@ -11410,8 +11436,8 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="1">
-        <v>46340</v>
+      <c r="M28" s="2">
+        <v>46341</v>
       </c>
       <c r="N28" t="s">
         <v>582</v>
@@ -11454,8 +11480,8 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="1">
-        <v>46310</v>
+      <c r="M29" s="2">
+        <v>46311</v>
       </c>
       <c r="N29" t="s">
         <v>582</v>
@@ -11498,8 +11524,8 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="1">
-        <v>46340</v>
+      <c r="M30" s="2">
+        <v>46341</v>
       </c>
       <c r="N30" t="s">
         <v>582</v>
@@ -11542,8 +11568,8 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="1">
-        <v>46310</v>
+      <c r="M31" s="2">
+        <v>46311</v>
       </c>
       <c r="N31" t="s">
         <v>582</v>
@@ -11586,8 +11612,8 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="1">
-        <v>46295</v>
+      <c r="M32" s="2">
+        <v>46296</v>
       </c>
       <c r="N32" t="s">
         <v>582</v>
@@ -11630,8 +11656,8 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="1">
-        <v>46295</v>
+      <c r="M33" s="2">
+        <v>46296</v>
       </c>
       <c r="N33" t="s">
         <v>582</v>
@@ -11674,8 +11700,8 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="1">
-        <v>46295</v>
+      <c r="M34" s="2">
+        <v>46296</v>
       </c>
       <c r="N34" t="s">
         <v>582</v>
@@ -11718,8 +11744,8 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="1">
-        <v>46295</v>
+      <c r="M35" s="2">
+        <v>46296</v>
       </c>
       <c r="N35" t="s">
         <v>582</v>
@@ -11762,8 +11788,8 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="1">
-        <v>46295</v>
+      <c r="M36" s="2">
+        <v>46296</v>
       </c>
       <c r="N36" t="s">
         <v>582</v>
@@ -11806,8 +11832,8 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="1">
-        <v>46295</v>
+      <c r="M37" s="2">
+        <v>46296</v>
       </c>
       <c r="N37" t="s">
         <v>582</v>
@@ -11850,8 +11876,8 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="1">
-        <v>46295</v>
+      <c r="M38" s="2">
+        <v>46296</v>
       </c>
       <c r="N38" t="s">
         <v>582</v>
@@ -11935,8 +11961,8 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="1">
-        <v>46295</v>
+      <c r="M40" s="2">
+        <v>46296</v>
       </c>
       <c r="N40" t="s">
         <v>582</v>
@@ -11979,8 +12005,8 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="1">
-        <v>46340</v>
+      <c r="M41" s="2">
+        <v>46341</v>
       </c>
       <c r="N41" t="s">
         <v>582</v>
@@ -12023,8 +12049,8 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="1">
-        <v>46295</v>
+      <c r="M42" s="2">
+        <v>46296</v>
       </c>
       <c r="N42" t="s">
         <v>582</v>
@@ -12067,8 +12093,8 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="1">
-        <v>46355</v>
+      <c r="M43" s="2">
+        <v>46356</v>
       </c>
       <c r="N43" t="s">
         <v>582</v>
@@ -12111,8 +12137,8 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="1">
-        <v>46340</v>
+      <c r="M44" s="2">
+        <v>46341</v>
       </c>
       <c r="N44" t="s">
         <v>582</v>
@@ -12155,8 +12181,8 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="1">
-        <v>46340</v>
+      <c r="M45" s="2">
+        <v>46341</v>
       </c>
       <c r="N45" t="s">
         <v>582</v>
@@ -12199,8 +12225,8 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="1">
-        <v>46295</v>
+      <c r="M46" s="2">
+        <v>46296</v>
       </c>
       <c r="N46" t="s">
         <v>582</v>
@@ -12243,8 +12269,8 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="1">
-        <v>46295</v>
+      <c r="M47" s="2">
+        <v>46296</v>
       </c>
       <c r="N47" t="s">
         <v>582</v>
@@ -12287,8 +12313,8 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="1">
-        <v>46340</v>
+      <c r="M48" s="2">
+        <v>46341</v>
       </c>
       <c r="N48" t="s">
         <v>582</v>
@@ -12331,8 +12357,8 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="1">
-        <v>46310</v>
+      <c r="M49" s="2">
+        <v>46311</v>
       </c>
       <c r="N49" t="s">
         <v>582</v>
@@ -12375,8 +12401,8 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="1">
-        <v>46310</v>
+      <c r="M50" s="2">
+        <v>46311</v>
       </c>
       <c r="N50" t="s">
         <v>582</v>
@@ -12419,8 +12445,8 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="1">
-        <v>46340</v>
+      <c r="M51" s="2">
+        <v>46341</v>
       </c>
       <c r="N51" t="s">
         <v>582</v>
@@ -12463,8 +12489,8 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="1">
-        <v>46340</v>
+      <c r="M52" s="2">
+        <v>46341</v>
       </c>
       <c r="N52" t="s">
         <v>582</v>
@@ -12507,8 +12533,8 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="1">
-        <v>46340</v>
+      <c r="M53" s="2">
+        <v>46341</v>
       </c>
       <c r="N53" t="s">
         <v>582</v>
@@ -12551,8 +12577,8 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="1">
-        <v>46340</v>
+      <c r="M54" s="2">
+        <v>46341</v>
       </c>
       <c r="N54" t="s">
         <v>582</v>
@@ -12595,8 +12621,8 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="1">
-        <v>46340</v>
+      <c r="M55" s="2">
+        <v>46341</v>
       </c>
       <c r="N55" t="s">
         <v>582</v>
@@ -12639,8 +12665,8 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="1">
-        <v>46310</v>
+      <c r="M56" s="2">
+        <v>46311</v>
       </c>
       <c r="N56" t="s">
         <v>582</v>
@@ -12683,8 +12709,8 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="1">
-        <v>46310</v>
+      <c r="M57" s="2">
+        <v>46311</v>
       </c>
       <c r="N57" t="s">
         <v>582</v>
@@ -12727,8 +12753,8 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="1">
-        <v>46310</v>
+      <c r="M58" s="2">
+        <v>46311</v>
       </c>
       <c r="N58" t="s">
         <v>582</v>
@@ -12771,8 +12797,8 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="1">
-        <v>46340</v>
+      <c r="M59" s="2">
+        <v>46341</v>
       </c>
       <c r="N59" t="s">
         <v>582</v>
@@ -12815,8 +12841,8 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="1">
-        <v>46310</v>
+      <c r="M60" s="2">
+        <v>46311</v>
       </c>
       <c r="N60" t="s">
         <v>582</v>
@@ -12859,8 +12885,8 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="1">
-        <v>46310</v>
+      <c r="M61" s="2">
+        <v>46311</v>
       </c>
       <c r="N61" t="s">
         <v>582</v>
@@ -12903,8 +12929,8 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="1">
-        <v>46340</v>
+      <c r="M62" s="2">
+        <v>46341</v>
       </c>
       <c r="N62" t="s">
         <v>582</v>
@@ -12947,8 +12973,8 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="1">
-        <v>46340</v>
+      <c r="M63" s="2">
+        <v>46341</v>
       </c>
       <c r="N63" t="s">
         <v>582</v>
@@ -12991,8 +13017,8 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="1">
-        <v>46355</v>
+      <c r="M64" s="2">
+        <v>46356</v>
       </c>
       <c r="N64" t="s">
         <v>582</v>
@@ -13035,8 +13061,8 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="1">
-        <v>46340</v>
+      <c r="M65" s="2">
+        <v>46341</v>
       </c>
       <c r="N65" t="s">
         <v>582</v>
@@ -13079,8 +13105,8 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="1">
-        <v>46340</v>
+      <c r="M66" s="2">
+        <v>46341</v>
       </c>
       <c r="N66" t="s">
         <v>582</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (01/09/2026 12:28)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,16 +1773,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1798,7 +1790,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1806,30 +1798,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2129,55 +2103,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2221,7 +2195,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2265,7 +2239,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2309,7 +2283,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2435,7 +2409,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2479,7 +2453,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2523,7 +2497,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2570,7 +2544,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2693,7 +2667,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2737,7 +2711,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2781,7 +2755,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2825,7 +2799,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2872,7 +2846,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2916,7 +2890,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3042,7 +3016,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3086,7 +3060,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3171,7 +3145,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3218,7 +3192,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3265,7 +3239,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3309,7 +3283,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3353,7 +3327,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3438,7 +3412,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3523,7 +3497,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3570,7 +3544,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3614,7 +3588,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3658,7 +3632,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3743,7 +3717,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3787,7 +3761,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3831,7 +3805,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3916,7 +3890,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3960,7 +3934,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4004,7 +3978,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4048,7 +4022,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4215,7 +4189,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4259,7 +4233,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4303,7 +4277,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4347,7 +4321,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4394,7 +4368,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4438,7 +4412,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4520,7 +4494,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4564,7 +4538,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4696,7 +4670,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4743,7 +4717,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4787,7 +4761,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4831,7 +4805,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4875,7 +4849,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4919,7 +4893,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4966,7 +4940,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5010,7 +4984,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5057,7 +5031,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5101,7 +5075,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5148,7 +5122,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5236,7 +5210,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5280,7 +5254,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5324,7 +5298,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5368,7 +5342,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5412,7 +5386,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5456,7 +5430,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5541,7 +5515,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5585,7 +5559,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5629,7 +5603,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5673,7 +5647,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5717,7 +5691,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5761,7 +5735,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5805,7 +5779,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5849,7 +5823,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5896,7 +5870,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5940,7 +5914,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5984,7 +5958,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6028,7 +6002,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6072,7 +6046,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6116,7 +6090,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6160,7 +6134,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6204,7 +6178,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6248,7 +6222,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6336,7 +6310,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6380,7 +6354,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6506,7 +6480,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6550,7 +6524,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6594,7 +6568,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6638,7 +6612,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6720,7 +6694,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6764,7 +6738,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6811,7 +6785,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6855,7 +6829,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6981,7 +6955,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7025,7 +6999,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7110,7 +7084,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7154,7 +7128,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7198,7 +7172,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7242,7 +7216,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7286,7 +7260,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7330,7 +7304,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7374,7 +7348,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7418,7 +7392,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7503,7 +7477,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7670,7 +7644,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7714,7 +7688,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7758,7 +7732,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7802,7 +7776,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7846,7 +7820,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7890,7 +7864,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7934,7 +7908,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8019,7 +7993,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8063,7 +8037,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8148,7 +8122,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8274,7 +8248,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8318,7 +8292,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8403,7 +8377,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8447,7 +8421,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8491,7 +8465,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8535,7 +8509,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8579,7 +8553,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8623,7 +8597,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8667,7 +8641,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8711,7 +8685,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8796,7 +8770,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8963,7 +8937,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9007,7 +8981,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9051,7 +9025,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9095,7 +9069,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9180,7 +9154,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9224,7 +9198,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9268,7 +9242,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9312,7 +9286,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9356,7 +9330,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9400,7 +9374,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9444,7 +9418,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9488,7 +9462,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9532,7 +9506,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9576,7 +9550,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9620,7 +9594,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9664,7 +9638,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9708,7 +9682,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9752,7 +9726,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9796,7 +9770,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9840,7 +9814,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9884,7 +9858,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9928,7 +9902,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9972,7 +9946,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10016,7 +9990,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10060,7 +10034,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10145,7 +10119,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10230,7 +10204,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10245,55 +10219,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10580,7 +10554,7 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46296</v>
       </c>
       <c r="N8" t="s">
@@ -10665,7 +10639,7 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46341</v>
       </c>
       <c r="N10" t="s">
@@ -10709,7 +10683,7 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46341</v>
       </c>
       <c r="N11" t="s">
@@ -10876,7 +10850,7 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46296</v>
       </c>
       <c r="N15" t="s">
@@ -10920,7 +10894,7 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46341</v>
       </c>
       <c r="N16" t="s">
@@ -10964,7 +10938,7 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46296</v>
       </c>
       <c r="N17" t="s">
@@ -11008,7 +10982,7 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46341</v>
       </c>
       <c r="N18" t="s">
@@ -11052,7 +11026,7 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46341</v>
       </c>
       <c r="N19" t="s">
@@ -11096,7 +11070,7 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46341</v>
       </c>
       <c r="N20" t="s">
@@ -11140,7 +11114,7 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46341</v>
       </c>
       <c r="N21" t="s">
@@ -11307,7 +11281,7 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46341</v>
       </c>
       <c r="N25" t="s">
@@ -11392,7 +11366,7 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46296</v>
       </c>
       <c r="N27" t="s">
@@ -11436,7 +11410,7 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46341</v>
       </c>
       <c r="N28" t="s">
@@ -11480,7 +11454,7 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46311</v>
       </c>
       <c r="N29" t="s">
@@ -11524,7 +11498,7 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46341</v>
       </c>
       <c r="N30" t="s">
@@ -11568,7 +11542,7 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46311</v>
       </c>
       <c r="N31" t="s">
@@ -11612,7 +11586,7 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46296</v>
       </c>
       <c r="N32" t="s">
@@ -11656,7 +11630,7 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46296</v>
       </c>
       <c r="N33" t="s">
@@ -11700,7 +11674,7 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46296</v>
       </c>
       <c r="N34" t="s">
@@ -11744,7 +11718,7 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46296</v>
       </c>
       <c r="N35" t="s">
@@ -11788,7 +11762,7 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46296</v>
       </c>
       <c r="N36" t="s">
@@ -11832,7 +11806,7 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46296</v>
       </c>
       <c r="N37" t="s">
@@ -11876,7 +11850,7 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46296</v>
       </c>
       <c r="N38" t="s">
@@ -11961,7 +11935,7 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46296</v>
       </c>
       <c r="N40" t="s">
@@ -12005,7 +11979,7 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46341</v>
       </c>
       <c r="N41" t="s">
@@ -12049,7 +12023,7 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46296</v>
       </c>
       <c r="N42" t="s">
@@ -12093,7 +12067,7 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46356</v>
       </c>
       <c r="N43" t="s">
@@ -12137,7 +12111,7 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46341</v>
       </c>
       <c r="N44" t="s">
@@ -12181,7 +12155,7 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46341</v>
       </c>
       <c r="N45" t="s">
@@ -12225,7 +12199,7 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46296</v>
       </c>
       <c r="N46" t="s">
@@ -12269,7 +12243,7 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46296</v>
       </c>
       <c r="N47" t="s">
@@ -12313,7 +12287,7 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46341</v>
       </c>
       <c r="N48" t="s">
@@ -12357,7 +12331,7 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46311</v>
       </c>
       <c r="N49" t="s">
@@ -12401,7 +12375,7 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46311</v>
       </c>
       <c r="N50" t="s">
@@ -12445,7 +12419,7 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46341</v>
       </c>
       <c r="N51" t="s">
@@ -12489,7 +12463,7 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46341</v>
       </c>
       <c r="N52" t="s">
@@ -12533,7 +12507,7 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46341</v>
       </c>
       <c r="N53" t="s">
@@ -12577,7 +12551,7 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46341</v>
       </c>
       <c r="N54" t="s">
@@ -12621,7 +12595,7 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46341</v>
       </c>
       <c r="N55" t="s">
@@ -12665,7 +12639,7 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46311</v>
       </c>
       <c r="N56" t="s">
@@ -12709,7 +12683,7 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46311</v>
       </c>
       <c r="N57" t="s">
@@ -12753,7 +12727,7 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46311</v>
       </c>
       <c r="N58" t="s">
@@ -12797,7 +12771,7 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46341</v>
       </c>
       <c r="N59" t="s">
@@ -12841,7 +12815,7 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46311</v>
       </c>
       <c r="N60" t="s">
@@ -12885,7 +12859,7 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46311</v>
       </c>
       <c r="N61" t="s">
@@ -12929,7 +12903,7 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46341</v>
       </c>
       <c r="N62" t="s">
@@ -12973,7 +12947,7 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46341</v>
       </c>
       <c r="N63" t="s">
@@ -13017,7 +12991,7 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46356</v>
       </c>
       <c r="N64" t="s">
@@ -13061,7 +13035,7 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46341</v>
       </c>
       <c r="N65" t="s">
@@ -13105,7 +13079,7 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46341</v>
       </c>
       <c r="N66" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (02/09/2026 09:39)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,8 +1773,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1790,7 +1798,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1798,12 +1806,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2103,55 +2129,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2195,7 +2221,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2239,7 +2265,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2283,7 +2309,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2409,7 +2435,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2453,7 +2479,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2497,7 +2523,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2544,7 +2570,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2667,7 +2693,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2711,7 +2737,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2755,7 +2781,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2799,7 +2825,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2846,7 +2872,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2890,7 +2916,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3016,7 +3042,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3060,7 +3086,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3145,7 +3171,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3192,7 +3218,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3239,7 +3265,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3283,7 +3309,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3327,7 +3353,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3412,7 +3438,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3497,7 +3523,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3544,7 +3570,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3588,7 +3614,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3632,7 +3658,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3717,7 +3743,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3761,7 +3787,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3805,7 +3831,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3890,7 +3916,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3934,7 +3960,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3978,7 +4004,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4022,7 +4048,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4189,7 +4215,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4233,7 +4259,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4277,7 +4303,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4321,7 +4347,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4368,7 +4394,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4412,7 +4438,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4494,7 +4520,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4538,7 +4564,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4626,7 +4652,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4670,7 +4696,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4717,7 +4743,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4761,7 +4787,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4805,7 +4831,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4849,7 +4875,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4893,7 +4919,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4940,7 +4966,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4984,7 +5010,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5031,7 +5057,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5075,7 +5101,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5122,7 +5148,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5210,7 +5236,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5254,7 +5280,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5298,7 +5324,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5342,7 +5368,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5386,7 +5412,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5430,7 +5456,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5515,7 +5541,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5559,7 +5585,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5603,7 +5629,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5647,7 +5673,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5691,7 +5717,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5735,7 +5761,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5779,7 +5805,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5823,7 +5849,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5870,7 +5896,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5914,7 +5940,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5958,7 +5984,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6002,7 +6028,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6046,7 +6072,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6090,7 +6116,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6134,7 +6160,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6178,7 +6204,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6222,7 +6248,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6310,7 +6336,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6354,7 +6380,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6480,7 +6506,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6524,7 +6550,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6568,7 +6594,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6612,7 +6638,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6694,7 +6720,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6738,7 +6764,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6785,7 +6811,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6829,7 +6855,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6955,7 +6981,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6999,7 +7025,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7084,7 +7110,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7128,7 +7154,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7172,7 +7198,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7216,7 +7242,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7260,7 +7286,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7304,7 +7330,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7348,7 +7374,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7392,7 +7418,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7477,7 +7503,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7644,7 +7670,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7688,7 +7714,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7732,7 +7758,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7776,7 +7802,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7820,7 +7846,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7864,7 +7890,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7908,7 +7934,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7993,7 +8019,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8037,7 +8063,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8122,7 +8148,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8248,7 +8274,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8292,7 +8318,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8377,7 +8403,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8421,7 +8447,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8465,7 +8491,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8509,7 +8535,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8553,7 +8579,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8597,7 +8623,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8641,7 +8667,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8685,7 +8711,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8770,7 +8796,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8937,7 +8963,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8981,7 +9007,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9025,7 +9051,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9069,7 +9095,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9154,7 +9180,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9198,7 +9224,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9242,7 +9268,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9286,7 +9312,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9330,7 +9356,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9374,7 +9400,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9418,7 +9444,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9462,7 +9488,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9506,7 +9532,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9550,7 +9576,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9594,7 +9620,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9638,7 +9664,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9682,7 +9708,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9726,7 +9752,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9770,7 +9796,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9814,7 +9840,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9858,7 +9884,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9902,7 +9928,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9946,7 +9972,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9990,7 +10016,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10034,7 +10060,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10119,7 +10145,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10204,7 +10230,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10219,55 +10245,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10554,8 +10580,8 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="1">
-        <v>46296</v>
+      <c r="M8" s="2">
+        <v>46297</v>
       </c>
       <c r="N8" t="s">
         <v>582</v>
@@ -10639,8 +10665,8 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="1">
-        <v>46341</v>
+      <c r="M10" s="2">
+        <v>46342</v>
       </c>
       <c r="N10" t="s">
         <v>582</v>
@@ -10683,8 +10709,8 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="1">
-        <v>46341</v>
+      <c r="M11" s="2">
+        <v>46342</v>
       </c>
       <c r="N11" t="s">
         <v>582</v>
@@ -10850,8 +10876,8 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="1">
-        <v>46296</v>
+      <c r="M15" s="2">
+        <v>46297</v>
       </c>
       <c r="N15" t="s">
         <v>582</v>
@@ -10894,8 +10920,8 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="1">
-        <v>46341</v>
+      <c r="M16" s="2">
+        <v>46342</v>
       </c>
       <c r="N16" t="s">
         <v>582</v>
@@ -10938,8 +10964,8 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="1">
-        <v>46296</v>
+      <c r="M17" s="2">
+        <v>46297</v>
       </c>
       <c r="N17" t="s">
         <v>582</v>
@@ -10982,8 +11008,8 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="1">
-        <v>46341</v>
+      <c r="M18" s="2">
+        <v>46342</v>
       </c>
       <c r="N18" t="s">
         <v>582</v>
@@ -11026,8 +11052,8 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="1">
-        <v>46341</v>
+      <c r="M19" s="2">
+        <v>46342</v>
       </c>
       <c r="N19" t="s">
         <v>582</v>
@@ -11070,8 +11096,8 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="1">
-        <v>46341</v>
+      <c r="M20" s="2">
+        <v>46342</v>
       </c>
       <c r="N20" t="s">
         <v>582</v>
@@ -11114,8 +11140,8 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="1">
-        <v>46341</v>
+      <c r="M21" s="2">
+        <v>46342</v>
       </c>
       <c r="N21" t="s">
         <v>582</v>
@@ -11281,8 +11307,8 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="1">
-        <v>46341</v>
+      <c r="M25" s="2">
+        <v>46342</v>
       </c>
       <c r="N25" t="s">
         <v>582</v>
@@ -11366,8 +11392,8 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="1">
-        <v>46296</v>
+      <c r="M27" s="2">
+        <v>46297</v>
       </c>
       <c r="N27" t="s">
         <v>582</v>
@@ -11410,8 +11436,8 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="1">
-        <v>46341</v>
+      <c r="M28" s="2">
+        <v>46342</v>
       </c>
       <c r="N28" t="s">
         <v>582</v>
@@ -11454,8 +11480,8 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="1">
-        <v>46311</v>
+      <c r="M29" s="2">
+        <v>46312</v>
       </c>
       <c r="N29" t="s">
         <v>582</v>
@@ -11498,8 +11524,8 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="1">
-        <v>46341</v>
+      <c r="M30" s="2">
+        <v>46342</v>
       </c>
       <c r="N30" t="s">
         <v>582</v>
@@ -11542,8 +11568,8 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="1">
-        <v>46311</v>
+      <c r="M31" s="2">
+        <v>46312</v>
       </c>
       <c r="N31" t="s">
         <v>582</v>
@@ -11586,8 +11612,8 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="1">
-        <v>46296</v>
+      <c r="M32" s="2">
+        <v>46297</v>
       </c>
       <c r="N32" t="s">
         <v>582</v>
@@ -11630,8 +11656,8 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="1">
-        <v>46296</v>
+      <c r="M33" s="2">
+        <v>46297</v>
       </c>
       <c r="N33" t="s">
         <v>582</v>
@@ -11674,8 +11700,8 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="1">
-        <v>46296</v>
+      <c r="M34" s="2">
+        <v>46297</v>
       </c>
       <c r="N34" t="s">
         <v>582</v>
@@ -11718,8 +11744,8 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="1">
-        <v>46296</v>
+      <c r="M35" s="2">
+        <v>46297</v>
       </c>
       <c r="N35" t="s">
         <v>582</v>
@@ -11762,8 +11788,8 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="1">
-        <v>46296</v>
+      <c r="M36" s="2">
+        <v>46297</v>
       </c>
       <c r="N36" t="s">
         <v>582</v>
@@ -11806,8 +11832,8 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="1">
-        <v>46296</v>
+      <c r="M37" s="2">
+        <v>46297</v>
       </c>
       <c r="N37" t="s">
         <v>582</v>
@@ -11850,8 +11876,8 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="1">
-        <v>46296</v>
+      <c r="M38" s="2">
+        <v>46297</v>
       </c>
       <c r="N38" t="s">
         <v>582</v>
@@ -11935,8 +11961,8 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="1">
-        <v>46296</v>
+      <c r="M40" s="2">
+        <v>46297</v>
       </c>
       <c r="N40" t="s">
         <v>582</v>
@@ -11979,8 +12005,8 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="1">
-        <v>46341</v>
+      <c r="M41" s="2">
+        <v>46342</v>
       </c>
       <c r="N41" t="s">
         <v>582</v>
@@ -12023,8 +12049,8 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="1">
-        <v>46296</v>
+      <c r="M42" s="2">
+        <v>46297</v>
       </c>
       <c r="N42" t="s">
         <v>582</v>
@@ -12067,8 +12093,8 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="1">
-        <v>46356</v>
+      <c r="M43" s="2">
+        <v>46357</v>
       </c>
       <c r="N43" t="s">
         <v>582</v>
@@ -12111,8 +12137,8 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="1">
-        <v>46341</v>
+      <c r="M44" s="2">
+        <v>46342</v>
       </c>
       <c r="N44" t="s">
         <v>582</v>
@@ -12155,8 +12181,8 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="1">
-        <v>46341</v>
+      <c r="M45" s="2">
+        <v>46342</v>
       </c>
       <c r="N45" t="s">
         <v>582</v>
@@ -12199,8 +12225,8 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="1">
-        <v>46296</v>
+      <c r="M46" s="2">
+        <v>46297</v>
       </c>
       <c r="N46" t="s">
         <v>582</v>
@@ -12243,8 +12269,8 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="1">
-        <v>46296</v>
+      <c r="M47" s="2">
+        <v>46297</v>
       </c>
       <c r="N47" t="s">
         <v>582</v>
@@ -12287,8 +12313,8 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="1">
-        <v>46341</v>
+      <c r="M48" s="2">
+        <v>46342</v>
       </c>
       <c r="N48" t="s">
         <v>582</v>
@@ -12331,8 +12357,8 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="1">
-        <v>46311</v>
+      <c r="M49" s="2">
+        <v>46312</v>
       </c>
       <c r="N49" t="s">
         <v>582</v>
@@ -12375,8 +12401,8 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="1">
-        <v>46311</v>
+      <c r="M50" s="2">
+        <v>46312</v>
       </c>
       <c r="N50" t="s">
         <v>582</v>
@@ -12419,8 +12445,8 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="1">
-        <v>46341</v>
+      <c r="M51" s="2">
+        <v>46342</v>
       </c>
       <c r="N51" t="s">
         <v>582</v>
@@ -12463,8 +12489,8 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="1">
-        <v>46341</v>
+      <c r="M52" s="2">
+        <v>46342</v>
       </c>
       <c r="N52" t="s">
         <v>582</v>
@@ -12507,8 +12533,8 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="1">
-        <v>46341</v>
+      <c r="M53" s="2">
+        <v>46342</v>
       </c>
       <c r="N53" t="s">
         <v>582</v>
@@ -12551,8 +12577,8 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="1">
-        <v>46341</v>
+      <c r="M54" s="2">
+        <v>46342</v>
       </c>
       <c r="N54" t="s">
         <v>582</v>
@@ -12595,8 +12621,8 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="1">
-        <v>46341</v>
+      <c r="M55" s="2">
+        <v>46342</v>
       </c>
       <c r="N55" t="s">
         <v>582</v>
@@ -12639,8 +12665,8 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="1">
-        <v>46311</v>
+      <c r="M56" s="2">
+        <v>46312</v>
       </c>
       <c r="N56" t="s">
         <v>582</v>
@@ -12683,8 +12709,8 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="1">
-        <v>46311</v>
+      <c r="M57" s="2">
+        <v>46312</v>
       </c>
       <c r="N57" t="s">
         <v>582</v>
@@ -12727,8 +12753,8 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="1">
-        <v>46311</v>
+      <c r="M58" s="2">
+        <v>46312</v>
       </c>
       <c r="N58" t="s">
         <v>582</v>
@@ -12771,8 +12797,8 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="1">
-        <v>46341</v>
+      <c r="M59" s="2">
+        <v>46342</v>
       </c>
       <c r="N59" t="s">
         <v>582</v>
@@ -12815,8 +12841,8 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="1">
-        <v>46311</v>
+      <c r="M60" s="2">
+        <v>46312</v>
       </c>
       <c r="N60" t="s">
         <v>582</v>
@@ -12859,8 +12885,8 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="1">
-        <v>46311</v>
+      <c r="M61" s="2">
+        <v>46312</v>
       </c>
       <c r="N61" t="s">
         <v>582</v>
@@ -12903,8 +12929,8 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="1">
-        <v>46341</v>
+      <c r="M62" s="2">
+        <v>46342</v>
       </c>
       <c r="N62" t="s">
         <v>582</v>
@@ -12947,8 +12973,8 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="1">
-        <v>46341</v>
+      <c r="M63" s="2">
+        <v>46342</v>
       </c>
       <c r="N63" t="s">
         <v>582</v>
@@ -12991,8 +13017,8 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="1">
-        <v>46356</v>
+      <c r="M64" s="2">
+        <v>46357</v>
       </c>
       <c r="N64" t="s">
         <v>582</v>
@@ -13035,8 +13061,8 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="1">
-        <v>46341</v>
+      <c r="M65" s="2">
+        <v>46342</v>
       </c>
       <c r="N65" t="s">
         <v>582</v>
@@ -13079,8 +13105,8 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="1">
-        <v>46341</v>
+      <c r="M66" s="2">
+        <v>46342</v>
       </c>
       <c r="N66" t="s">
         <v>582</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (02/09/2026 12:05)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,16 +1773,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1798,7 +1790,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1806,30 +1798,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2129,55 +2103,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2221,7 +2195,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2265,7 +2239,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2309,7 +2283,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2435,7 +2409,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2479,7 +2453,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2523,7 +2497,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2570,7 +2544,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2693,7 +2667,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2737,7 +2711,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2781,7 +2755,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2825,7 +2799,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2872,7 +2846,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2916,7 +2890,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3042,7 +3016,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3086,7 +3060,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3171,7 +3145,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3218,7 +3192,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3265,7 +3239,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3309,7 +3283,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3353,7 +3327,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3438,7 +3412,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3523,7 +3497,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3570,7 +3544,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3614,7 +3588,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3658,7 +3632,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3743,7 +3717,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3787,7 +3761,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3831,7 +3805,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3916,7 +3890,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3960,7 +3934,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4004,7 +3978,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4048,7 +4022,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4215,7 +4189,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4259,7 +4233,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4303,7 +4277,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4347,7 +4321,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4394,7 +4368,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4438,7 +4412,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4520,7 +4494,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4564,7 +4538,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4696,7 +4670,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4743,7 +4717,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4787,7 +4761,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4831,7 +4805,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4875,7 +4849,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4919,7 +4893,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4966,7 +4940,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5010,7 +4984,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5057,7 +5031,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5101,7 +5075,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5148,7 +5122,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5236,7 +5210,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5280,7 +5254,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5324,7 +5298,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5368,7 +5342,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5412,7 +5386,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5456,7 +5430,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5541,7 +5515,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5585,7 +5559,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5629,7 +5603,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5673,7 +5647,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5717,7 +5691,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5761,7 +5735,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5805,7 +5779,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5849,7 +5823,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5896,7 +5870,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5940,7 +5914,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5984,7 +5958,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6028,7 +6002,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6072,7 +6046,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6116,7 +6090,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6160,7 +6134,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6204,7 +6178,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6248,7 +6222,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6336,7 +6310,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6380,7 +6354,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6506,7 +6480,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6550,7 +6524,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6594,7 +6568,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6638,7 +6612,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6720,7 +6694,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6764,7 +6738,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6811,7 +6785,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6855,7 +6829,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6981,7 +6955,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7025,7 +6999,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7110,7 +7084,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7154,7 +7128,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7198,7 +7172,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7242,7 +7216,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7286,7 +7260,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7330,7 +7304,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7374,7 +7348,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7418,7 +7392,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7503,7 +7477,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7670,7 +7644,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7714,7 +7688,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7758,7 +7732,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7802,7 +7776,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7846,7 +7820,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7890,7 +7864,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7934,7 +7908,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8019,7 +7993,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8063,7 +8037,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8148,7 +8122,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8274,7 +8248,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8318,7 +8292,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8403,7 +8377,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8447,7 +8421,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8491,7 +8465,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8535,7 +8509,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8579,7 +8553,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8623,7 +8597,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8667,7 +8641,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8711,7 +8685,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8796,7 +8770,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8963,7 +8937,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9007,7 +8981,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9051,7 +9025,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9095,7 +9069,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9180,7 +9154,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9224,7 +9198,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9268,7 +9242,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9312,7 +9286,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9356,7 +9330,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9400,7 +9374,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9444,7 +9418,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9488,7 +9462,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9532,7 +9506,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9576,7 +9550,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9620,7 +9594,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9664,7 +9638,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9708,7 +9682,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9752,7 +9726,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9796,7 +9770,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9840,7 +9814,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9884,7 +9858,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9928,7 +9902,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9972,7 +9946,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10016,7 +9990,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10060,7 +10034,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10145,7 +10119,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10230,7 +10204,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10245,55 +10219,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10580,7 +10554,7 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46297</v>
       </c>
       <c r="N8" t="s">
@@ -10665,7 +10639,7 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46342</v>
       </c>
       <c r="N10" t="s">
@@ -10709,7 +10683,7 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46342</v>
       </c>
       <c r="N11" t="s">
@@ -10876,7 +10850,7 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46297</v>
       </c>
       <c r="N15" t="s">
@@ -10920,7 +10894,7 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46342</v>
       </c>
       <c r="N16" t="s">
@@ -10964,7 +10938,7 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46297</v>
       </c>
       <c r="N17" t="s">
@@ -11008,7 +10982,7 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46342</v>
       </c>
       <c r="N18" t="s">
@@ -11052,7 +11026,7 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46342</v>
       </c>
       <c r="N19" t="s">
@@ -11096,7 +11070,7 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46342</v>
       </c>
       <c r="N20" t="s">
@@ -11140,7 +11114,7 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46342</v>
       </c>
       <c r="N21" t="s">
@@ -11307,7 +11281,7 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46342</v>
       </c>
       <c r="N25" t="s">
@@ -11392,7 +11366,7 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46297</v>
       </c>
       <c r="N27" t="s">
@@ -11436,7 +11410,7 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46342</v>
       </c>
       <c r="N28" t="s">
@@ -11480,7 +11454,7 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46312</v>
       </c>
       <c r="N29" t="s">
@@ -11524,7 +11498,7 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46342</v>
       </c>
       <c r="N30" t="s">
@@ -11568,7 +11542,7 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46312</v>
       </c>
       <c r="N31" t="s">
@@ -11612,7 +11586,7 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46297</v>
       </c>
       <c r="N32" t="s">
@@ -11656,7 +11630,7 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46297</v>
       </c>
       <c r="N33" t="s">
@@ -11700,7 +11674,7 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46297</v>
       </c>
       <c r="N34" t="s">
@@ -11744,7 +11718,7 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46297</v>
       </c>
       <c r="N35" t="s">
@@ -11788,7 +11762,7 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46297</v>
       </c>
       <c r="N36" t="s">
@@ -11832,7 +11806,7 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46297</v>
       </c>
       <c r="N37" t="s">
@@ -11876,7 +11850,7 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46297</v>
       </c>
       <c r="N38" t="s">
@@ -11961,7 +11935,7 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46297</v>
       </c>
       <c r="N40" t="s">
@@ -12005,7 +11979,7 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46342</v>
       </c>
       <c r="N41" t="s">
@@ -12049,7 +12023,7 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46297</v>
       </c>
       <c r="N42" t="s">
@@ -12093,7 +12067,7 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46357</v>
       </c>
       <c r="N43" t="s">
@@ -12137,7 +12111,7 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46342</v>
       </c>
       <c r="N44" t="s">
@@ -12181,7 +12155,7 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46342</v>
       </c>
       <c r="N45" t="s">
@@ -12225,7 +12199,7 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46297</v>
       </c>
       <c r="N46" t="s">
@@ -12269,7 +12243,7 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46297</v>
       </c>
       <c r="N47" t="s">
@@ -12313,7 +12287,7 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46342</v>
       </c>
       <c r="N48" t="s">
@@ -12357,7 +12331,7 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46312</v>
       </c>
       <c r="N49" t="s">
@@ -12401,7 +12375,7 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46312</v>
       </c>
       <c r="N50" t="s">
@@ -12445,7 +12419,7 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46342</v>
       </c>
       <c r="N51" t="s">
@@ -12489,7 +12463,7 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46342</v>
       </c>
       <c r="N52" t="s">
@@ -12533,7 +12507,7 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46342</v>
       </c>
       <c r="N53" t="s">
@@ -12577,7 +12551,7 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46342</v>
       </c>
       <c r="N54" t="s">
@@ -12621,7 +12595,7 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46342</v>
       </c>
       <c r="N55" t="s">
@@ -12665,7 +12639,7 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46312</v>
       </c>
       <c r="N56" t="s">
@@ -12709,7 +12683,7 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46312</v>
       </c>
       <c r="N57" t="s">
@@ -12753,7 +12727,7 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46312</v>
       </c>
       <c r="N58" t="s">
@@ -12797,7 +12771,7 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46342</v>
       </c>
       <c r="N59" t="s">
@@ -12841,7 +12815,7 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46312</v>
       </c>
       <c r="N60" t="s">
@@ -12885,7 +12859,7 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46312</v>
       </c>
       <c r="N61" t="s">
@@ -12929,7 +12903,7 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46342</v>
       </c>
       <c r="N62" t="s">
@@ -12973,7 +12947,7 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46342</v>
       </c>
       <c r="N63" t="s">
@@ -13017,7 +12991,7 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46357</v>
       </c>
       <c r="N64" t="s">
@@ -13061,7 +13035,7 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46342</v>
       </c>
       <c r="N65" t="s">
@@ -13105,7 +13079,7 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46342</v>
       </c>
       <c r="N66" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (03/09/2026 12:00)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10555,7 +10555,7 @@
         <v>577</v>
       </c>
       <c r="M8" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N8" t="s">
         <v>582</v>
@@ -10640,7 +10640,7 @@
         <v>578</v>
       </c>
       <c r="M10" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N10" t="s">
         <v>582</v>
@@ -10684,7 +10684,7 @@
         <v>578</v>
       </c>
       <c r="M11" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N11" t="s">
         <v>582</v>
@@ -10851,7 +10851,7 @@
         <v>577</v>
       </c>
       <c r="M15" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N15" t="s">
         <v>582</v>
@@ -10895,7 +10895,7 @@
         <v>578</v>
       </c>
       <c r="M16" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N16" t="s">
         <v>582</v>
@@ -10939,7 +10939,7 @@
         <v>577</v>
       </c>
       <c r="M17" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N17" t="s">
         <v>582</v>
@@ -10983,7 +10983,7 @@
         <v>578</v>
       </c>
       <c r="M18" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N18" t="s">
         <v>582</v>
@@ -11027,7 +11027,7 @@
         <v>578</v>
       </c>
       <c r="M19" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N19" t="s">
         <v>582</v>
@@ -11071,7 +11071,7 @@
         <v>578</v>
       </c>
       <c r="M20" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N20" t="s">
         <v>582</v>
@@ -11115,7 +11115,7 @@
         <v>578</v>
       </c>
       <c r="M21" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N21" t="s">
         <v>582</v>
@@ -11282,7 +11282,7 @@
         <v>578</v>
       </c>
       <c r="M25" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N25" t="s">
         <v>582</v>
@@ -11367,7 +11367,7 @@
         <v>577</v>
       </c>
       <c r="M27" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N27" t="s">
         <v>582</v>
@@ -11411,7 +11411,7 @@
         <v>578</v>
       </c>
       <c r="M28" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N28" t="s">
         <v>582</v>
@@ -11455,7 +11455,7 @@
         <v>581</v>
       </c>
       <c r="M29" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N29" t="s">
         <v>582</v>
@@ -11499,7 +11499,7 @@
         <v>578</v>
       </c>
       <c r="M30" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N30" t="s">
         <v>582</v>
@@ -11543,7 +11543,7 @@
         <v>581</v>
       </c>
       <c r="M31" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N31" t="s">
         <v>582</v>
@@ -11587,7 +11587,7 @@
         <v>577</v>
       </c>
       <c r="M32" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N32" t="s">
         <v>582</v>
@@ -11631,7 +11631,7 @@
         <v>577</v>
       </c>
       <c r="M33" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N33" t="s">
         <v>582</v>
@@ -11675,7 +11675,7 @@
         <v>577</v>
       </c>
       <c r="M34" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N34" t="s">
         <v>582</v>
@@ -11719,7 +11719,7 @@
         <v>577</v>
       </c>
       <c r="M35" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N35" t="s">
         <v>582</v>
@@ -11763,7 +11763,7 @@
         <v>577</v>
       </c>
       <c r="M36" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N36" t="s">
         <v>582</v>
@@ -11807,7 +11807,7 @@
         <v>577</v>
       </c>
       <c r="M37" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N37" t="s">
         <v>582</v>
@@ -11851,7 +11851,7 @@
         <v>577</v>
       </c>
       <c r="M38" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N38" t="s">
         <v>582</v>
@@ -11936,7 +11936,7 @@
         <v>577</v>
       </c>
       <c r="M40" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N40" t="s">
         <v>582</v>
@@ -11980,7 +11980,7 @@
         <v>578</v>
       </c>
       <c r="M41" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N41" t="s">
         <v>582</v>
@@ -12024,7 +12024,7 @@
         <v>577</v>
       </c>
       <c r="M42" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N42" t="s">
         <v>582</v>
@@ -12068,7 +12068,7 @@
         <v>580</v>
       </c>
       <c r="M43" s="1">
-        <v>46357</v>
+        <v>46358</v>
       </c>
       <c r="N43" t="s">
         <v>582</v>
@@ -12112,7 +12112,7 @@
         <v>578</v>
       </c>
       <c r="M44" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N44" t="s">
         <v>582</v>
@@ -12156,7 +12156,7 @@
         <v>578</v>
       </c>
       <c r="M45" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N45" t="s">
         <v>582</v>
@@ -12200,7 +12200,7 @@
         <v>577</v>
       </c>
       <c r="M46" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N46" t="s">
         <v>582</v>
@@ -12244,7 +12244,7 @@
         <v>577</v>
       </c>
       <c r="M47" s="1">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="N47" t="s">
         <v>582</v>
@@ -12288,7 +12288,7 @@
         <v>578</v>
       </c>
       <c r="M48" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N48" t="s">
         <v>582</v>
@@ -12332,7 +12332,7 @@
         <v>581</v>
       </c>
       <c r="M49" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N49" t="s">
         <v>582</v>
@@ -12376,7 +12376,7 @@
         <v>581</v>
       </c>
       <c r="M50" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N50" t="s">
         <v>582</v>
@@ -12420,7 +12420,7 @@
         <v>578</v>
       </c>
       <c r="M51" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N51" t="s">
         <v>582</v>
@@ -12464,7 +12464,7 @@
         <v>578</v>
       </c>
       <c r="M52" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N52" t="s">
         <v>582</v>
@@ -12508,7 +12508,7 @@
         <v>578</v>
       </c>
       <c r="M53" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N53" t="s">
         <v>582</v>
@@ -12552,7 +12552,7 @@
         <v>578</v>
       </c>
       <c r="M54" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N54" t="s">
         <v>582</v>
@@ -12596,7 +12596,7 @@
         <v>578</v>
       </c>
       <c r="M55" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N55" t="s">
         <v>582</v>
@@ -12640,7 +12640,7 @@
         <v>581</v>
       </c>
       <c r="M56" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N56" t="s">
         <v>582</v>
@@ -12684,7 +12684,7 @@
         <v>581</v>
       </c>
       <c r="M57" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N57" t="s">
         <v>582</v>
@@ -12728,7 +12728,7 @@
         <v>581</v>
       </c>
       <c r="M58" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N58" t="s">
         <v>582</v>
@@ -12772,7 +12772,7 @@
         <v>578</v>
       </c>
       <c r="M59" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N59" t="s">
         <v>582</v>
@@ -12816,7 +12816,7 @@
         <v>581</v>
       </c>
       <c r="M60" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N60" t="s">
         <v>582</v>
@@ -12860,7 +12860,7 @@
         <v>581</v>
       </c>
       <c r="M61" s="1">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="N61" t="s">
         <v>582</v>
@@ -12904,7 +12904,7 @@
         <v>578</v>
       </c>
       <c r="M62" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N62" t="s">
         <v>582</v>
@@ -12948,7 +12948,7 @@
         <v>578</v>
       </c>
       <c r="M63" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N63" t="s">
         <v>582</v>
@@ -12992,7 +12992,7 @@
         <v>580</v>
       </c>
       <c r="M64" s="1">
-        <v>46357</v>
+        <v>46358</v>
       </c>
       <c r="N64" t="s">
         <v>582</v>
@@ -13036,7 +13036,7 @@
         <v>578</v>
       </c>
       <c r="M65" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N65" t="s">
         <v>582</v>
@@ -13080,7 +13080,7 @@
         <v>578</v>
       </c>
       <c r="M66" s="1">
-        <v>46342</v>
+        <v>46343</v>
       </c>
       <c r="N66" t="s">
         <v>582</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (03/09/2026 13:43)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,8 +1773,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1790,7 +1798,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1798,12 +1806,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2103,55 +2129,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2195,7 +2221,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2239,7 +2265,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2283,7 +2309,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2409,7 +2435,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2453,7 +2479,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2497,7 +2523,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2544,7 +2570,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2667,7 +2693,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2711,7 +2737,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2755,7 +2781,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2799,7 +2825,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2846,7 +2872,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2890,7 +2916,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3016,7 +3042,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3060,7 +3086,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3145,7 +3171,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3192,7 +3218,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3239,7 +3265,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3283,7 +3309,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3327,7 +3353,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3412,7 +3438,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3497,7 +3523,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3544,7 +3570,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3588,7 +3614,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3632,7 +3658,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3717,7 +3743,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3761,7 +3787,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3805,7 +3831,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3890,7 +3916,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3934,7 +3960,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3978,7 +4004,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4022,7 +4048,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4189,7 +4215,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4233,7 +4259,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4277,7 +4303,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4321,7 +4347,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4368,7 +4394,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4412,7 +4438,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4494,7 +4520,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4538,7 +4564,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4626,7 +4652,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4670,7 +4696,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4717,7 +4743,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4761,7 +4787,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4805,7 +4831,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4849,7 +4875,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4893,7 +4919,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4940,7 +4966,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4984,7 +5010,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5031,7 +5057,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5075,7 +5101,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5122,7 +5148,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5210,7 +5236,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5254,7 +5280,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5298,7 +5324,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5342,7 +5368,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5386,7 +5412,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5430,7 +5456,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5515,7 +5541,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5559,7 +5585,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5603,7 +5629,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5647,7 +5673,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5691,7 +5717,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5735,7 +5761,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5779,7 +5805,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5823,7 +5849,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5870,7 +5896,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5914,7 +5940,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5958,7 +5984,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6002,7 +6028,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6046,7 +6072,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6090,7 +6116,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6134,7 +6160,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6178,7 +6204,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6222,7 +6248,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6310,7 +6336,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6354,7 +6380,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6480,7 +6506,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6524,7 +6550,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6568,7 +6594,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6612,7 +6638,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6694,7 +6720,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6738,7 +6764,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6785,7 +6811,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6829,7 +6855,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6955,7 +6981,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6999,7 +7025,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7084,7 +7110,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7128,7 +7154,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7172,7 +7198,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7216,7 +7242,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7260,7 +7286,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7304,7 +7330,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7348,7 +7374,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7392,7 +7418,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7477,7 +7503,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7644,7 +7670,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7688,7 +7714,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7732,7 +7758,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7776,7 +7802,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7820,7 +7846,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7864,7 +7890,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7908,7 +7934,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7993,7 +8019,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8037,7 +8063,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8122,7 +8148,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8248,7 +8274,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8292,7 +8318,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8377,7 +8403,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8421,7 +8447,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8465,7 +8491,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8509,7 +8535,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8553,7 +8579,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8597,7 +8623,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8641,7 +8667,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8685,7 +8711,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8770,7 +8796,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8937,7 +8963,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8981,7 +9007,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9025,7 +9051,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9069,7 +9095,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9154,7 +9180,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9198,7 +9224,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9242,7 +9268,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9286,7 +9312,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9330,7 +9356,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9374,7 +9400,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9418,7 +9444,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9462,7 +9488,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9506,7 +9532,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9550,7 +9576,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9594,7 +9620,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9638,7 +9664,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9682,7 +9708,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9726,7 +9752,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9770,7 +9796,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9814,7 +9840,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9858,7 +9884,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9902,7 +9928,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9946,7 +9972,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9990,7 +10016,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10034,7 +10060,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10119,7 +10145,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10204,7 +10230,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10219,55 +10245,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10554,7 +10580,7 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="2">
         <v>46298</v>
       </c>
       <c r="N8" t="s">
@@ -10639,7 +10665,7 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="2">
         <v>46343</v>
       </c>
       <c r="N10" t="s">
@@ -10683,7 +10709,7 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="2">
         <v>46343</v>
       </c>
       <c r="N11" t="s">
@@ -10850,7 +10876,7 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="2">
         <v>46298</v>
       </c>
       <c r="N15" t="s">
@@ -10894,7 +10920,7 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="1">
+      <c r="M16" s="2">
         <v>46343</v>
       </c>
       <c r="N16" t="s">
@@ -10938,7 +10964,7 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="1">
+      <c r="M17" s="2">
         <v>46298</v>
       </c>
       <c r="N17" t="s">
@@ -10982,7 +11008,7 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="1">
+      <c r="M18" s="2">
         <v>46343</v>
       </c>
       <c r="N18" t="s">
@@ -11026,7 +11052,7 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="1">
+      <c r="M19" s="2">
         <v>46343</v>
       </c>
       <c r="N19" t="s">
@@ -11070,7 +11096,7 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="1">
+      <c r="M20" s="2">
         <v>46343</v>
       </c>
       <c r="N20" t="s">
@@ -11114,7 +11140,7 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="2">
         <v>46343</v>
       </c>
       <c r="N21" t="s">
@@ -11281,7 +11307,7 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="2">
         <v>46343</v>
       </c>
       <c r="N25" t="s">
@@ -11366,7 +11392,7 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="1">
+      <c r="M27" s="2">
         <v>46298</v>
       </c>
       <c r="N27" t="s">
@@ -11410,7 +11436,7 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="1">
+      <c r="M28" s="2">
         <v>46343</v>
       </c>
       <c r="N28" t="s">
@@ -11454,7 +11480,7 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="2">
         <v>46313</v>
       </c>
       <c r="N29" t="s">
@@ -11498,7 +11524,7 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="2">
         <v>46343</v>
       </c>
       <c r="N30" t="s">
@@ -11542,7 +11568,7 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="1">
+      <c r="M31" s="2">
         <v>46313</v>
       </c>
       <c r="N31" t="s">
@@ -11586,7 +11612,7 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="1">
+      <c r="M32" s="2">
         <v>46298</v>
       </c>
       <c r="N32" t="s">
@@ -11630,7 +11656,7 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="1">
+      <c r="M33" s="2">
         <v>46298</v>
       </c>
       <c r="N33" t="s">
@@ -11674,7 +11700,7 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="1">
+      <c r="M34" s="2">
         <v>46298</v>
       </c>
       <c r="N34" t="s">
@@ -11718,7 +11744,7 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="1">
+      <c r="M35" s="2">
         <v>46298</v>
       </c>
       <c r="N35" t="s">
@@ -11762,7 +11788,7 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="1">
+      <c r="M36" s="2">
         <v>46298</v>
       </c>
       <c r="N36" t="s">
@@ -11806,7 +11832,7 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="1">
+      <c r="M37" s="2">
         <v>46298</v>
       </c>
       <c r="N37" t="s">
@@ -11850,7 +11876,7 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="1">
+      <c r="M38" s="2">
         <v>46298</v>
       </c>
       <c r="N38" t="s">
@@ -11935,7 +11961,7 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="1">
+      <c r="M40" s="2">
         <v>46298</v>
       </c>
       <c r="N40" t="s">
@@ -11979,7 +12005,7 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M41" s="2">
         <v>46343</v>
       </c>
       <c r="N41" t="s">
@@ -12023,7 +12049,7 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="2">
         <v>46298</v>
       </c>
       <c r="N42" t="s">
@@ -12067,7 +12093,7 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="1">
+      <c r="M43" s="2">
         <v>46358</v>
       </c>
       <c r="N43" t="s">
@@ -12111,7 +12137,7 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="1">
+      <c r="M44" s="2">
         <v>46343</v>
       </c>
       <c r="N44" t="s">
@@ -12155,7 +12181,7 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="1">
+      <c r="M45" s="2">
         <v>46343</v>
       </c>
       <c r="N45" t="s">
@@ -12199,7 +12225,7 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="2">
         <v>46298</v>
       </c>
       <c r="N46" t="s">
@@ -12243,7 +12269,7 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="1">
+      <c r="M47" s="2">
         <v>46298</v>
       </c>
       <c r="N47" t="s">
@@ -12287,7 +12313,7 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="1">
+      <c r="M48" s="2">
         <v>46343</v>
       </c>
       <c r="N48" t="s">
@@ -12331,7 +12357,7 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="1">
+      <c r="M49" s="2">
         <v>46313</v>
       </c>
       <c r="N49" t="s">
@@ -12375,7 +12401,7 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="1">
+      <c r="M50" s="2">
         <v>46313</v>
       </c>
       <c r="N50" t="s">
@@ -12419,7 +12445,7 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="1">
+      <c r="M51" s="2">
         <v>46343</v>
       </c>
       <c r="N51" t="s">
@@ -12463,7 +12489,7 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="1">
+      <c r="M52" s="2">
         <v>46343</v>
       </c>
       <c r="N52" t="s">
@@ -12507,7 +12533,7 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="1">
+      <c r="M53" s="2">
         <v>46343</v>
       </c>
       <c r="N53" t="s">
@@ -12551,7 +12577,7 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="1">
+      <c r="M54" s="2">
         <v>46343</v>
       </c>
       <c r="N54" t="s">
@@ -12595,7 +12621,7 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="1">
+      <c r="M55" s="2">
         <v>46343</v>
       </c>
       <c r="N55" t="s">
@@ -12639,7 +12665,7 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="1">
+      <c r="M56" s="2">
         <v>46313</v>
       </c>
       <c r="N56" t="s">
@@ -12683,7 +12709,7 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="1">
+      <c r="M57" s="2">
         <v>46313</v>
       </c>
       <c r="N57" t="s">
@@ -12727,7 +12753,7 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="1">
+      <c r="M58" s="2">
         <v>46313</v>
       </c>
       <c r="N58" t="s">
@@ -12771,7 +12797,7 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="1">
+      <c r="M59" s="2">
         <v>46343</v>
       </c>
       <c r="N59" t="s">
@@ -12815,7 +12841,7 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="1">
+      <c r="M60" s="2">
         <v>46313</v>
       </c>
       <c r="N60" t="s">
@@ -12859,7 +12885,7 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="1">
+      <c r="M61" s="2">
         <v>46313</v>
       </c>
       <c r="N61" t="s">
@@ -12903,7 +12929,7 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="1">
+      <c r="M62" s="2">
         <v>46343</v>
       </c>
       <c r="N62" t="s">
@@ -12947,7 +12973,7 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="1">
+      <c r="M63" s="2">
         <v>46343</v>
       </c>
       <c r="N63" t="s">
@@ -12991,7 +13017,7 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="1">
+      <c r="M64" s="2">
         <v>46358</v>
       </c>
       <c r="N64" t="s">
@@ -13035,7 +13061,7 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="1">
+      <c r="M65" s="2">
         <v>46343</v>
       </c>
       <c r="N65" t="s">
@@ -13079,7 +13105,7 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="1">
+      <c r="M66" s="2">
         <v>46343</v>
       </c>
       <c r="N66" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (04/09/2026 11:56)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,16 +1773,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1798,7 +1790,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1806,30 +1798,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2129,55 +2103,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2221,7 +2195,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2265,7 +2239,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2309,7 +2283,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2435,7 +2409,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2479,7 +2453,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2523,7 +2497,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2570,7 +2544,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2693,7 +2667,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2737,7 +2711,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2781,7 +2755,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2825,7 +2799,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2872,7 +2846,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2916,7 +2890,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3042,7 +3016,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3086,7 +3060,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3171,7 +3145,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3218,7 +3192,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3265,7 +3239,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3309,7 +3283,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3353,7 +3327,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3438,7 +3412,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3523,7 +3497,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3570,7 +3544,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3614,7 +3588,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3658,7 +3632,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3743,7 +3717,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3787,7 +3761,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3831,7 +3805,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3916,7 +3890,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3960,7 +3934,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4004,7 +3978,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4048,7 +4022,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4215,7 +4189,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4259,7 +4233,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4303,7 +4277,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4347,7 +4321,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4394,7 +4368,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4438,7 +4412,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4520,7 +4494,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4564,7 +4538,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4696,7 +4670,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4743,7 +4717,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4787,7 +4761,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4831,7 +4805,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4875,7 +4849,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4919,7 +4893,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4966,7 +4940,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5010,7 +4984,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5057,7 +5031,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5101,7 +5075,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5148,7 +5122,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5236,7 +5210,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5280,7 +5254,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5324,7 +5298,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5368,7 +5342,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5412,7 +5386,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5456,7 +5430,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5541,7 +5515,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5585,7 +5559,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5629,7 +5603,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5673,7 +5647,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5717,7 +5691,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5761,7 +5735,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5805,7 +5779,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5849,7 +5823,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5896,7 +5870,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5940,7 +5914,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5984,7 +5958,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6028,7 +6002,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6072,7 +6046,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6116,7 +6090,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6160,7 +6134,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6204,7 +6178,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6248,7 +6222,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6336,7 +6310,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6380,7 +6354,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6506,7 +6480,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6550,7 +6524,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6594,7 +6568,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6638,7 +6612,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6720,7 +6694,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6764,7 +6738,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6811,7 +6785,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6855,7 +6829,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6981,7 +6955,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7025,7 +6999,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7110,7 +7084,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7154,7 +7128,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7198,7 +7172,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7242,7 +7216,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7286,7 +7260,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7330,7 +7304,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7374,7 +7348,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7418,7 +7392,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7503,7 +7477,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7670,7 +7644,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7714,7 +7688,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7758,7 +7732,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7802,7 +7776,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7846,7 +7820,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7890,7 +7864,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7934,7 +7908,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8019,7 +7993,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8063,7 +8037,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8148,7 +8122,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8274,7 +8248,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8318,7 +8292,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8403,7 +8377,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8447,7 +8421,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8491,7 +8465,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8535,7 +8509,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8579,7 +8553,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8623,7 +8597,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8667,7 +8641,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8711,7 +8685,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8796,7 +8770,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8963,7 +8937,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9007,7 +8981,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9051,7 +9025,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9095,7 +9069,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9180,7 +9154,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9224,7 +9198,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9268,7 +9242,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9312,7 +9286,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9356,7 +9330,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9400,7 +9374,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9444,7 +9418,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9488,7 +9462,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9532,7 +9506,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9576,7 +9550,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9620,7 +9594,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9664,7 +9638,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9708,7 +9682,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9752,7 +9726,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9796,7 +9770,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9840,7 +9814,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9884,7 +9858,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9928,7 +9902,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9972,7 +9946,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10016,7 +9990,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10060,7 +10034,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10145,7 +10119,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10230,7 +10204,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10245,55 +10219,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10580,8 +10554,8 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="2">
-        <v>46298</v>
+      <c r="M8" s="1">
+        <v>46299</v>
       </c>
       <c r="N8" t="s">
         <v>582</v>
@@ -10665,8 +10639,8 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="2">
-        <v>46343</v>
+      <c r="M10" s="1">
+        <v>46344</v>
       </c>
       <c r="N10" t="s">
         <v>582</v>
@@ -10709,8 +10683,8 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="2">
-        <v>46343</v>
+      <c r="M11" s="1">
+        <v>46344</v>
       </c>
       <c r="N11" t="s">
         <v>582</v>
@@ -10876,8 +10850,8 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="2">
-        <v>46298</v>
+      <c r="M15" s="1">
+        <v>46299</v>
       </c>
       <c r="N15" t="s">
         <v>582</v>
@@ -10920,8 +10894,8 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="2">
-        <v>46343</v>
+      <c r="M16" s="1">
+        <v>46344</v>
       </c>
       <c r="N16" t="s">
         <v>582</v>
@@ -10964,8 +10938,8 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="2">
-        <v>46298</v>
+      <c r="M17" s="1">
+        <v>46299</v>
       </c>
       <c r="N17" t="s">
         <v>582</v>
@@ -11008,8 +10982,8 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="2">
-        <v>46343</v>
+      <c r="M18" s="1">
+        <v>46344</v>
       </c>
       <c r="N18" t="s">
         <v>582</v>
@@ -11052,8 +11026,8 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="2">
-        <v>46343</v>
+      <c r="M19" s="1">
+        <v>46344</v>
       </c>
       <c r="N19" t="s">
         <v>582</v>
@@ -11096,8 +11070,8 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="2">
-        <v>46343</v>
+      <c r="M20" s="1">
+        <v>46344</v>
       </c>
       <c r="N20" t="s">
         <v>582</v>
@@ -11140,8 +11114,8 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="2">
-        <v>46343</v>
+      <c r="M21" s="1">
+        <v>46344</v>
       </c>
       <c r="N21" t="s">
         <v>582</v>
@@ -11307,8 +11281,8 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="2">
-        <v>46343</v>
+      <c r="M25" s="1">
+        <v>46344</v>
       </c>
       <c r="N25" t="s">
         <v>582</v>
@@ -11392,8 +11366,8 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="2">
-        <v>46298</v>
+      <c r="M27" s="1">
+        <v>46299</v>
       </c>
       <c r="N27" t="s">
         <v>582</v>
@@ -11436,8 +11410,8 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="2">
-        <v>46343</v>
+      <c r="M28" s="1">
+        <v>46344</v>
       </c>
       <c r="N28" t="s">
         <v>582</v>
@@ -11480,8 +11454,8 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="2">
-        <v>46313</v>
+      <c r="M29" s="1">
+        <v>46314</v>
       </c>
       <c r="N29" t="s">
         <v>582</v>
@@ -11524,8 +11498,8 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="2">
-        <v>46343</v>
+      <c r="M30" s="1">
+        <v>46344</v>
       </c>
       <c r="N30" t="s">
         <v>582</v>
@@ -11568,8 +11542,8 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="2">
-        <v>46313</v>
+      <c r="M31" s="1">
+        <v>46314</v>
       </c>
       <c r="N31" t="s">
         <v>582</v>
@@ -11612,8 +11586,8 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="2">
-        <v>46298</v>
+      <c r="M32" s="1">
+        <v>46299</v>
       </c>
       <c r="N32" t="s">
         <v>582</v>
@@ -11656,8 +11630,8 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="2">
-        <v>46298</v>
+      <c r="M33" s="1">
+        <v>46299</v>
       </c>
       <c r="N33" t="s">
         <v>582</v>
@@ -11700,8 +11674,8 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="2">
-        <v>46298</v>
+      <c r="M34" s="1">
+        <v>46299</v>
       </c>
       <c r="N34" t="s">
         <v>582</v>
@@ -11744,8 +11718,8 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="2">
-        <v>46298</v>
+      <c r="M35" s="1">
+        <v>46299</v>
       </c>
       <c r="N35" t="s">
         <v>582</v>
@@ -11788,8 +11762,8 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="2">
-        <v>46298</v>
+      <c r="M36" s="1">
+        <v>46299</v>
       </c>
       <c r="N36" t="s">
         <v>582</v>
@@ -11832,8 +11806,8 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="2">
-        <v>46298</v>
+      <c r="M37" s="1">
+        <v>46299</v>
       </c>
       <c r="N37" t="s">
         <v>582</v>
@@ -11876,8 +11850,8 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="2">
-        <v>46298</v>
+      <c r="M38" s="1">
+        <v>46299</v>
       </c>
       <c r="N38" t="s">
         <v>582</v>
@@ -11961,8 +11935,8 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="2">
-        <v>46298</v>
+      <c r="M40" s="1">
+        <v>46299</v>
       </c>
       <c r="N40" t="s">
         <v>582</v>
@@ -12005,8 +11979,8 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="2">
-        <v>46343</v>
+      <c r="M41" s="1">
+        <v>46344</v>
       </c>
       <c r="N41" t="s">
         <v>582</v>
@@ -12049,8 +12023,8 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="2">
-        <v>46298</v>
+      <c r="M42" s="1">
+        <v>46299</v>
       </c>
       <c r="N42" t="s">
         <v>582</v>
@@ -12093,8 +12067,8 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="2">
-        <v>46358</v>
+      <c r="M43" s="1">
+        <v>46359</v>
       </c>
       <c r="N43" t="s">
         <v>582</v>
@@ -12137,8 +12111,8 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="2">
-        <v>46343</v>
+      <c r="M44" s="1">
+        <v>46344</v>
       </c>
       <c r="N44" t="s">
         <v>582</v>
@@ -12181,8 +12155,8 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="2">
-        <v>46343</v>
+      <c r="M45" s="1">
+        <v>46344</v>
       </c>
       <c r="N45" t="s">
         <v>582</v>
@@ -12225,8 +12199,8 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="2">
-        <v>46298</v>
+      <c r="M46" s="1">
+        <v>46299</v>
       </c>
       <c r="N46" t="s">
         <v>582</v>
@@ -12269,8 +12243,8 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="2">
-        <v>46298</v>
+      <c r="M47" s="1">
+        <v>46299</v>
       </c>
       <c r="N47" t="s">
         <v>582</v>
@@ -12313,8 +12287,8 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="2">
-        <v>46343</v>
+      <c r="M48" s="1">
+        <v>46344</v>
       </c>
       <c r="N48" t="s">
         <v>582</v>
@@ -12357,8 +12331,8 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="2">
-        <v>46313</v>
+      <c r="M49" s="1">
+        <v>46314</v>
       </c>
       <c r="N49" t="s">
         <v>582</v>
@@ -12401,8 +12375,8 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="2">
-        <v>46313</v>
+      <c r="M50" s="1">
+        <v>46314</v>
       </c>
       <c r="N50" t="s">
         <v>582</v>
@@ -12445,8 +12419,8 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="2">
-        <v>46343</v>
+      <c r="M51" s="1">
+        <v>46344</v>
       </c>
       <c r="N51" t="s">
         <v>582</v>
@@ -12489,8 +12463,8 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="2">
-        <v>46343</v>
+      <c r="M52" s="1">
+        <v>46344</v>
       </c>
       <c r="N52" t="s">
         <v>582</v>
@@ -12533,8 +12507,8 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="2">
-        <v>46343</v>
+      <c r="M53" s="1">
+        <v>46344</v>
       </c>
       <c r="N53" t="s">
         <v>582</v>
@@ -12577,8 +12551,8 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="2">
-        <v>46343</v>
+      <c r="M54" s="1">
+        <v>46344</v>
       </c>
       <c r="N54" t="s">
         <v>582</v>
@@ -12621,8 +12595,8 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="2">
-        <v>46343</v>
+      <c r="M55" s="1">
+        <v>46344</v>
       </c>
       <c r="N55" t="s">
         <v>582</v>
@@ -12665,8 +12639,8 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="2">
-        <v>46313</v>
+      <c r="M56" s="1">
+        <v>46314</v>
       </c>
       <c r="N56" t="s">
         <v>582</v>
@@ -12709,8 +12683,8 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="2">
-        <v>46313</v>
+      <c r="M57" s="1">
+        <v>46314</v>
       </c>
       <c r="N57" t="s">
         <v>582</v>
@@ -12753,8 +12727,8 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="2">
-        <v>46313</v>
+      <c r="M58" s="1">
+        <v>46314</v>
       </c>
       <c r="N58" t="s">
         <v>582</v>
@@ -12797,8 +12771,8 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="2">
-        <v>46343</v>
+      <c r="M59" s="1">
+        <v>46344</v>
       </c>
       <c r="N59" t="s">
         <v>582</v>
@@ -12841,8 +12815,8 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="2">
-        <v>46313</v>
+      <c r="M60" s="1">
+        <v>46314</v>
       </c>
       <c r="N60" t="s">
         <v>582</v>
@@ -12885,8 +12859,8 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="2">
-        <v>46313</v>
+      <c r="M61" s="1">
+        <v>46314</v>
       </c>
       <c r="N61" t="s">
         <v>582</v>
@@ -12929,8 +12903,8 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="2">
-        <v>46343</v>
+      <c r="M62" s="1">
+        <v>46344</v>
       </c>
       <c r="N62" t="s">
         <v>582</v>
@@ -12973,8 +12947,8 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="2">
-        <v>46343</v>
+      <c r="M63" s="1">
+        <v>46344</v>
       </c>
       <c r="N63" t="s">
         <v>582</v>
@@ -13017,8 +12991,8 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="2">
-        <v>46358</v>
+      <c r="M64" s="1">
+        <v>46359</v>
       </c>
       <c r="N64" t="s">
         <v>582</v>
@@ -13061,8 +13035,8 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="2">
-        <v>46343</v>
+      <c r="M65" s="1">
+        <v>46344</v>
       </c>
       <c r="N65" t="s">
         <v>582</v>
@@ -13105,8 +13079,8 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="2">
-        <v>46343</v>
+      <c r="M66" s="1">
+        <v>46344</v>
       </c>
       <c r="N66" t="s">
         <v>582</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (07/09/2026 13:25)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10555,7 +10555,7 @@
         <v>577</v>
       </c>
       <c r="M8" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N8" t="s">
         <v>582</v>
@@ -10640,7 +10640,7 @@
         <v>578</v>
       </c>
       <c r="M10" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N10" t="s">
         <v>582</v>
@@ -10684,7 +10684,7 @@
         <v>578</v>
       </c>
       <c r="M11" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N11" t="s">
         <v>582</v>
@@ -10851,7 +10851,7 @@
         <v>577</v>
       </c>
       <c r="M15" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N15" t="s">
         <v>582</v>
@@ -10895,7 +10895,7 @@
         <v>578</v>
       </c>
       <c r="M16" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N16" t="s">
         <v>582</v>
@@ -10939,7 +10939,7 @@
         <v>577</v>
       </c>
       <c r="M17" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N17" t="s">
         <v>582</v>
@@ -10983,7 +10983,7 @@
         <v>578</v>
       </c>
       <c r="M18" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N18" t="s">
         <v>582</v>
@@ -11027,7 +11027,7 @@
         <v>578</v>
       </c>
       <c r="M19" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N19" t="s">
         <v>582</v>
@@ -11071,7 +11071,7 @@
         <v>578</v>
       </c>
       <c r="M20" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N20" t="s">
         <v>582</v>
@@ -11115,7 +11115,7 @@
         <v>578</v>
       </c>
       <c r="M21" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N21" t="s">
         <v>582</v>
@@ -11282,7 +11282,7 @@
         <v>578</v>
       </c>
       <c r="M25" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N25" t="s">
         <v>582</v>
@@ -11367,7 +11367,7 @@
         <v>577</v>
       </c>
       <c r="M27" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N27" t="s">
         <v>582</v>
@@ -11411,7 +11411,7 @@
         <v>578</v>
       </c>
       <c r="M28" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N28" t="s">
         <v>582</v>
@@ -11455,7 +11455,7 @@
         <v>581</v>
       </c>
       <c r="M29" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N29" t="s">
         <v>582</v>
@@ -11499,7 +11499,7 @@
         <v>578</v>
       </c>
       <c r="M30" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N30" t="s">
         <v>582</v>
@@ -11543,7 +11543,7 @@
         <v>581</v>
       </c>
       <c r="M31" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N31" t="s">
         <v>582</v>
@@ -11587,7 +11587,7 @@
         <v>577</v>
       </c>
       <c r="M32" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N32" t="s">
         <v>582</v>
@@ -11631,7 +11631,7 @@
         <v>577</v>
       </c>
       <c r="M33" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N33" t="s">
         <v>582</v>
@@ -11675,7 +11675,7 @@
         <v>577</v>
       </c>
       <c r="M34" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N34" t="s">
         <v>582</v>
@@ -11719,7 +11719,7 @@
         <v>577</v>
       </c>
       <c r="M35" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N35" t="s">
         <v>582</v>
@@ -11763,7 +11763,7 @@
         <v>577</v>
       </c>
       <c r="M36" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N36" t="s">
         <v>582</v>
@@ -11807,7 +11807,7 @@
         <v>577</v>
       </c>
       <c r="M37" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N37" t="s">
         <v>582</v>
@@ -11851,7 +11851,7 @@
         <v>577</v>
       </c>
       <c r="M38" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N38" t="s">
         <v>582</v>
@@ -11936,7 +11936,7 @@
         <v>577</v>
       </c>
       <c r="M40" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N40" t="s">
         <v>582</v>
@@ -11980,7 +11980,7 @@
         <v>578</v>
       </c>
       <c r="M41" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N41" t="s">
         <v>582</v>
@@ -12024,7 +12024,7 @@
         <v>577</v>
       </c>
       <c r="M42" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N42" t="s">
         <v>582</v>
@@ -12068,7 +12068,7 @@
         <v>580</v>
       </c>
       <c r="M43" s="1">
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="N43" t="s">
         <v>582</v>
@@ -12112,7 +12112,7 @@
         <v>578</v>
       </c>
       <c r="M44" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N44" t="s">
         <v>582</v>
@@ -12156,7 +12156,7 @@
         <v>578</v>
       </c>
       <c r="M45" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N45" t="s">
         <v>582</v>
@@ -12200,7 +12200,7 @@
         <v>577</v>
       </c>
       <c r="M46" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N46" t="s">
         <v>582</v>
@@ -12244,7 +12244,7 @@
         <v>577</v>
       </c>
       <c r="M47" s="1">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="N47" t="s">
         <v>582</v>
@@ -12288,7 +12288,7 @@
         <v>578</v>
       </c>
       <c r="M48" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N48" t="s">
         <v>582</v>
@@ -12332,7 +12332,7 @@
         <v>581</v>
       </c>
       <c r="M49" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N49" t="s">
         <v>582</v>
@@ -12376,7 +12376,7 @@
         <v>581</v>
       </c>
       <c r="M50" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N50" t="s">
         <v>582</v>
@@ -12420,7 +12420,7 @@
         <v>578</v>
       </c>
       <c r="M51" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N51" t="s">
         <v>582</v>
@@ -12464,7 +12464,7 @@
         <v>578</v>
       </c>
       <c r="M52" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N52" t="s">
         <v>582</v>
@@ -12508,7 +12508,7 @@
         <v>578</v>
       </c>
       <c r="M53" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N53" t="s">
         <v>582</v>
@@ -12552,7 +12552,7 @@
         <v>578</v>
       </c>
       <c r="M54" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N54" t="s">
         <v>582</v>
@@ -12596,7 +12596,7 @@
         <v>578</v>
       </c>
       <c r="M55" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N55" t="s">
         <v>582</v>
@@ -12640,7 +12640,7 @@
         <v>581</v>
       </c>
       <c r="M56" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N56" t="s">
         <v>582</v>
@@ -12684,7 +12684,7 @@
         <v>581</v>
       </c>
       <c r="M57" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N57" t="s">
         <v>582</v>
@@ -12728,7 +12728,7 @@
         <v>581</v>
       </c>
       <c r="M58" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N58" t="s">
         <v>582</v>
@@ -12772,7 +12772,7 @@
         <v>578</v>
       </c>
       <c r="M59" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N59" t="s">
         <v>582</v>
@@ -12816,7 +12816,7 @@
         <v>581</v>
       </c>
       <c r="M60" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N60" t="s">
         <v>582</v>
@@ -12860,7 +12860,7 @@
         <v>581</v>
       </c>
       <c r="M61" s="1">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="N61" t="s">
         <v>582</v>
@@ -12904,7 +12904,7 @@
         <v>578</v>
       </c>
       <c r="M62" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N62" t="s">
         <v>582</v>
@@ -12948,7 +12948,7 @@
         <v>578</v>
       </c>
       <c r="M63" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N63" t="s">
         <v>582</v>
@@ -12992,7 +12992,7 @@
         <v>580</v>
       </c>
       <c r="M64" s="1">
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="N64" t="s">
         <v>582</v>
@@ -13036,7 +13036,7 @@
         <v>578</v>
       </c>
       <c r="M65" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N65" t="s">
         <v>582</v>
@@ -13080,7 +13080,7 @@
         <v>578</v>
       </c>
       <c r="M66" s="1">
-        <v>46344</v>
+        <v>46347</v>
       </c>
       <c r="N66" t="s">
         <v>582</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (08/09/2026 08:23)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,8 +1773,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1790,7 +1798,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1798,12 +1806,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2103,55 +2129,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2195,7 +2221,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>46104</v>
       </c>
     </row>
@@ -2239,7 +2265,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -2283,7 +2309,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -2409,7 +2435,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2453,7 +2479,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2497,7 +2523,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2544,7 +2570,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -2667,7 +2693,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -2711,7 +2737,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2755,7 +2781,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -2799,7 +2825,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2846,7 +2872,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -2890,7 +2916,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3016,7 +3042,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3060,7 +3086,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3145,7 +3171,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3192,7 +3218,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3239,7 +3265,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3283,7 +3309,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45964</v>
       </c>
     </row>
@@ -3327,7 +3353,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -3412,7 +3438,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -3497,7 +3523,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3544,7 +3570,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3588,7 +3614,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3632,7 +3658,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -3717,7 +3743,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -3761,7 +3787,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -3805,7 +3831,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3890,7 +3916,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3934,7 +3960,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -3978,7 +4004,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -4022,7 +4048,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4189,7 +4215,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="1">
+      <c r="P48" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4233,7 +4259,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="1">
+      <c r="P49" s="2">
         <v>45955</v>
       </c>
     </row>
@@ -4277,7 +4303,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="1">
+      <c r="P50" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4321,7 +4347,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="1">
+      <c r="P51" s="2">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4368,7 +4394,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="1">
+      <c r="P52" s="2">
         <v>46163</v>
       </c>
     </row>
@@ -4412,7 +4438,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="1">
+      <c r="P53" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4494,7 +4520,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="1">
+      <c r="P55" s="2">
         <v>46050</v>
       </c>
     </row>
@@ -4538,7 +4564,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="1">
+      <c r="P56" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4626,7 +4652,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="1">
+      <c r="P58" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -4670,7 +4696,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="1">
+      <c r="P59" s="2">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4717,7 +4743,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="1">
+      <c r="P60" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -4761,7 +4787,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="1">
+      <c r="P61" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -4805,7 +4831,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="1">
+      <c r="P62" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -4849,7 +4875,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="1">
+      <c r="P63" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4893,7 +4919,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="1">
+      <c r="P64" s="2">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4940,7 +4966,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="1">
+      <c r="P65" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -4984,7 +5010,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="1">
+      <c r="P66" s="2">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5031,7 +5057,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="1">
+      <c r="P67" s="2">
         <v>45916</v>
       </c>
     </row>
@@ -5075,7 +5101,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="1">
+      <c r="P68" s="2">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5122,7 +5148,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="1">
+      <c r="P69" s="2">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5210,7 +5236,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="1">
+      <c r="P71" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5254,7 +5280,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="1">
+      <c r="P72" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5298,7 +5324,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="1">
+      <c r="P73" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5342,7 +5368,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="1">
+      <c r="P74" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5386,7 +5412,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="1">
+      <c r="P75" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5430,7 +5456,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="1">
+      <c r="P76" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -5515,7 +5541,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="1">
+      <c r="P78" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -5559,7 +5585,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="1">
+      <c r="P79" s="2">
         <v>46140</v>
       </c>
     </row>
@@ -5603,7 +5629,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="1">
+      <c r="P80" s="2">
         <v>46095</v>
       </c>
     </row>
@@ -5647,7 +5673,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="1">
+      <c r="P81" s="2">
         <v>46040</v>
       </c>
     </row>
@@ -5691,7 +5717,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="1">
+      <c r="P82" s="2">
         <v>46060</v>
       </c>
     </row>
@@ -5735,7 +5761,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="1">
+      <c r="P83" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5779,7 +5805,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="1">
+      <c r="P84" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5823,7 +5849,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="1">
+      <c r="P85" s="2">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5870,7 +5896,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="1">
+      <c r="P86" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5914,7 +5940,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="1">
+      <c r="P87" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -5958,7 +5984,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="1">
+      <c r="P88" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6002,7 +6028,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="1">
+      <c r="P89" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6046,7 +6072,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="1">
+      <c r="P90" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6090,7 +6116,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="1">
+      <c r="P91" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6134,7 +6160,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="1">
+      <c r="P92" s="2">
         <v>46080</v>
       </c>
     </row>
@@ -6178,7 +6204,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="1">
+      <c r="P93" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -6222,7 +6248,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="1">
+      <c r="P94" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -6310,7 +6336,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="1">
+      <c r="P96" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6354,7 +6380,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="1">
+      <c r="P97" s="2">
         <v>46032</v>
       </c>
     </row>
@@ -6480,7 +6506,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="1">
+      <c r="P100" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -6524,7 +6550,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="1">
+      <c r="P101" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6568,7 +6594,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="1">
+      <c r="P102" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6612,7 +6638,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="1">
+      <c r="P103" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -6694,7 +6720,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="1">
+      <c r="P105" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -6738,7 +6764,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="1">
+      <c r="P106" s="2">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6785,7 +6811,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="1">
+      <c r="P107" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6829,7 +6855,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="1">
+      <c r="P108" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -6955,7 +6981,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="1">
+      <c r="P111" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -6999,7 +7025,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="1">
+      <c r="P112" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -7084,7 +7110,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="1">
+      <c r="P114" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -7128,7 +7154,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="1">
+      <c r="P115" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7172,7 +7198,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="1">
+      <c r="P116" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7216,7 +7242,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="1">
+      <c r="P117" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -7260,7 +7286,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="1">
+      <c r="P118" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -7304,7 +7330,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="1">
+      <c r="P119" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7348,7 +7374,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="1">
+      <c r="P120" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7392,7 +7418,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="1">
+      <c r="P121" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -7477,7 +7503,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="1">
+      <c r="P123" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -7644,7 +7670,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="1">
+      <c r="P127" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -7688,7 +7714,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="1">
+      <c r="P128" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -7732,7 +7758,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="1">
+      <c r="P129" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7776,7 +7802,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="1">
+      <c r="P130" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7820,7 +7846,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="1">
+      <c r="P131" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7864,7 +7890,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="1">
+      <c r="P132" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -7908,7 +7934,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="1">
+      <c r="P133" s="2">
         <v>46130</v>
       </c>
     </row>
@@ -7993,7 +8019,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="1">
+      <c r="P135" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8037,7 +8063,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="1">
+      <c r="P136" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8122,7 +8148,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="1">
+      <c r="P138" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8248,7 +8274,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="1">
+      <c r="P141" s="2">
         <v>46160</v>
       </c>
     </row>
@@ -8292,7 +8318,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="1">
+      <c r="P142" s="2">
         <v>46123</v>
       </c>
     </row>
@@ -8377,7 +8403,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="1">
+      <c r="P144" s="2">
         <v>46167</v>
       </c>
     </row>
@@ -8421,7 +8447,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="1">
+      <c r="P145" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8465,7 +8491,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="1">
+      <c r="P146" s="2">
         <v>46101</v>
       </c>
     </row>
@@ -8509,7 +8535,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="1">
+      <c r="P147" s="2">
         <v>46081</v>
       </c>
     </row>
@@ -8553,7 +8579,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="1">
+      <c r="P148" s="2">
         <v>45976</v>
       </c>
     </row>
@@ -8597,7 +8623,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="1">
+      <c r="P149" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8641,7 +8667,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="1">
+      <c r="P150" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8685,7 +8711,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="1">
+      <c r="P151" s="2">
         <v>45979</v>
       </c>
     </row>
@@ -8770,7 +8796,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="1">
+      <c r="P153" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -8937,7 +8963,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="1">
+      <c r="P157" s="2">
         <v>45959</v>
       </c>
     </row>
@@ -8981,7 +9007,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="1">
+      <c r="P158" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9025,7 +9051,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="1">
+      <c r="P159" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9069,7 +9095,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="1">
+      <c r="P160" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9154,7 +9180,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="1">
+      <c r="P162" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9198,7 +9224,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="1">
+      <c r="P163" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9242,7 +9268,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="1">
+      <c r="P164" s="2">
         <v>45984</v>
       </c>
     </row>
@@ -9286,7 +9312,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="1">
+      <c r="P165" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9330,7 +9356,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="1">
+      <c r="P166" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9374,7 +9400,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="1">
+      <c r="P167" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9418,7 +9444,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="1">
+      <c r="P168" s="2">
         <v>45994</v>
       </c>
     </row>
@@ -9462,7 +9488,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="1">
+      <c r="P169" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9506,7 +9532,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="1">
+      <c r="P170" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9550,7 +9576,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="1">
+      <c r="P171" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9594,7 +9620,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="1">
+      <c r="P172" s="2">
         <v>45954</v>
       </c>
     </row>
@@ -9638,7 +9664,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="1">
+      <c r="P173" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -9682,7 +9708,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="1">
+      <c r="P174" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -9726,7 +9752,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="1">
+      <c r="P175" s="2">
         <v>45911</v>
       </c>
     </row>
@@ -9770,7 +9796,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="1">
+      <c r="P176" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9814,7 +9840,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="1">
+      <c r="P177" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9858,7 +9884,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="1">
+      <c r="P178" s="2">
         <v>45908</v>
       </c>
     </row>
@@ -9902,7 +9928,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="1">
+      <c r="P179" s="2">
         <v>45835</v>
       </c>
     </row>
@@ -9946,7 +9972,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="1">
+      <c r="P180" s="2">
         <v>46025</v>
       </c>
     </row>
@@ -9990,7 +10016,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="1">
+      <c r="P181" s="2">
         <v>46024</v>
       </c>
     </row>
@@ -10034,7 +10060,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="1">
+      <c r="P182" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10119,7 +10145,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="1">
+      <c r="P184" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10204,7 +10230,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="1">
+      <c r="P186" s="2">
         <v>45904</v>
       </c>
     </row>
@@ -10219,55 +10245,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10554,8 +10580,8 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="1">
-        <v>46302</v>
+      <c r="M8" s="2">
+        <v>46303</v>
       </c>
       <c r="N8" t="s">
         <v>582</v>
@@ -10639,8 +10665,8 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="1">
-        <v>46347</v>
+      <c r="M10" s="2">
+        <v>46348</v>
       </c>
       <c r="N10" t="s">
         <v>582</v>
@@ -10683,8 +10709,8 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="1">
-        <v>46347</v>
+      <c r="M11" s="2">
+        <v>46348</v>
       </c>
       <c r="N11" t="s">
         <v>582</v>
@@ -10850,8 +10876,8 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="1">
-        <v>46302</v>
+      <c r="M15" s="2">
+        <v>46303</v>
       </c>
       <c r="N15" t="s">
         <v>582</v>
@@ -10894,8 +10920,8 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="1">
-        <v>46347</v>
+      <c r="M16" s="2">
+        <v>46348</v>
       </c>
       <c r="N16" t="s">
         <v>582</v>
@@ -10938,8 +10964,8 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="1">
-        <v>46302</v>
+      <c r="M17" s="2">
+        <v>46303</v>
       </c>
       <c r="N17" t="s">
         <v>582</v>
@@ -10982,8 +11008,8 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="1">
-        <v>46347</v>
+      <c r="M18" s="2">
+        <v>46348</v>
       </c>
       <c r="N18" t="s">
         <v>582</v>
@@ -11026,8 +11052,8 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="1">
-        <v>46347</v>
+      <c r="M19" s="2">
+        <v>46348</v>
       </c>
       <c r="N19" t="s">
         <v>582</v>
@@ -11070,8 +11096,8 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="1">
-        <v>46347</v>
+      <c r="M20" s="2">
+        <v>46348</v>
       </c>
       <c r="N20" t="s">
         <v>582</v>
@@ -11114,8 +11140,8 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="1">
-        <v>46347</v>
+      <c r="M21" s="2">
+        <v>46348</v>
       </c>
       <c r="N21" t="s">
         <v>582</v>
@@ -11281,8 +11307,8 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="1">
-        <v>46347</v>
+      <c r="M25" s="2">
+        <v>46348</v>
       </c>
       <c r="N25" t="s">
         <v>582</v>
@@ -11366,8 +11392,8 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="1">
-        <v>46302</v>
+      <c r="M27" s="2">
+        <v>46303</v>
       </c>
       <c r="N27" t="s">
         <v>582</v>
@@ -11410,8 +11436,8 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="1">
-        <v>46347</v>
+      <c r="M28" s="2">
+        <v>46348</v>
       </c>
       <c r="N28" t="s">
         <v>582</v>
@@ -11454,8 +11480,8 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="1">
-        <v>46317</v>
+      <c r="M29" s="2">
+        <v>46318</v>
       </c>
       <c r="N29" t="s">
         <v>582</v>
@@ -11498,8 +11524,8 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="1">
-        <v>46347</v>
+      <c r="M30" s="2">
+        <v>46348</v>
       </c>
       <c r="N30" t="s">
         <v>582</v>
@@ -11542,8 +11568,8 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="1">
-        <v>46317</v>
+      <c r="M31" s="2">
+        <v>46318</v>
       </c>
       <c r="N31" t="s">
         <v>582</v>
@@ -11586,8 +11612,8 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="1">
-        <v>46302</v>
+      <c r="M32" s="2">
+        <v>46303</v>
       </c>
       <c r="N32" t="s">
         <v>582</v>
@@ -11630,8 +11656,8 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="1">
-        <v>46302</v>
+      <c r="M33" s="2">
+        <v>46303</v>
       </c>
       <c r="N33" t="s">
         <v>582</v>
@@ -11674,8 +11700,8 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="1">
-        <v>46302</v>
+      <c r="M34" s="2">
+        <v>46303</v>
       </c>
       <c r="N34" t="s">
         <v>582</v>
@@ -11718,8 +11744,8 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="1">
-        <v>46302</v>
+      <c r="M35" s="2">
+        <v>46303</v>
       </c>
       <c r="N35" t="s">
         <v>582</v>
@@ -11762,8 +11788,8 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="1">
-        <v>46302</v>
+      <c r="M36" s="2">
+        <v>46303</v>
       </c>
       <c r="N36" t="s">
         <v>582</v>
@@ -11806,8 +11832,8 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="1">
-        <v>46302</v>
+      <c r="M37" s="2">
+        <v>46303</v>
       </c>
       <c r="N37" t="s">
         <v>582</v>
@@ -11850,8 +11876,8 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="1">
-        <v>46302</v>
+      <c r="M38" s="2">
+        <v>46303</v>
       </c>
       <c r="N38" t="s">
         <v>582</v>
@@ -11935,8 +11961,8 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="1">
-        <v>46302</v>
+      <c r="M40" s="2">
+        <v>46303</v>
       </c>
       <c r="N40" t="s">
         <v>582</v>
@@ -11979,8 +12005,8 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="1">
-        <v>46347</v>
+      <c r="M41" s="2">
+        <v>46348</v>
       </c>
       <c r="N41" t="s">
         <v>582</v>
@@ -12023,8 +12049,8 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="1">
-        <v>46302</v>
+      <c r="M42" s="2">
+        <v>46303</v>
       </c>
       <c r="N42" t="s">
         <v>582</v>
@@ -12067,8 +12093,8 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="1">
-        <v>46362</v>
+      <c r="M43" s="2">
+        <v>46363</v>
       </c>
       <c r="N43" t="s">
         <v>582</v>
@@ -12111,8 +12137,8 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="1">
-        <v>46347</v>
+      <c r="M44" s="2">
+        <v>46348</v>
       </c>
       <c r="N44" t="s">
         <v>582</v>
@@ -12155,8 +12181,8 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="1">
-        <v>46347</v>
+      <c r="M45" s="2">
+        <v>46348</v>
       </c>
       <c r="N45" t="s">
         <v>582</v>
@@ -12199,8 +12225,8 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="1">
-        <v>46302</v>
+      <c r="M46" s="2">
+        <v>46303</v>
       </c>
       <c r="N46" t="s">
         <v>582</v>
@@ -12243,8 +12269,8 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="1">
-        <v>46302</v>
+      <c r="M47" s="2">
+        <v>46303</v>
       </c>
       <c r="N47" t="s">
         <v>582</v>
@@ -12287,8 +12313,8 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="1">
-        <v>46347</v>
+      <c r="M48" s="2">
+        <v>46348</v>
       </c>
       <c r="N48" t="s">
         <v>582</v>
@@ -12331,8 +12357,8 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="1">
-        <v>46317</v>
+      <c r="M49" s="2">
+        <v>46318</v>
       </c>
       <c r="N49" t="s">
         <v>582</v>
@@ -12375,8 +12401,8 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="1">
-        <v>46317</v>
+      <c r="M50" s="2">
+        <v>46318</v>
       </c>
       <c r="N50" t="s">
         <v>582</v>
@@ -12419,8 +12445,8 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="1">
-        <v>46347</v>
+      <c r="M51" s="2">
+        <v>46348</v>
       </c>
       <c r="N51" t="s">
         <v>582</v>
@@ -12463,8 +12489,8 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="1">
-        <v>46347</v>
+      <c r="M52" s="2">
+        <v>46348</v>
       </c>
       <c r="N52" t="s">
         <v>582</v>
@@ -12507,8 +12533,8 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="1">
-        <v>46347</v>
+      <c r="M53" s="2">
+        <v>46348</v>
       </c>
       <c r="N53" t="s">
         <v>582</v>
@@ -12551,8 +12577,8 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="1">
-        <v>46347</v>
+      <c r="M54" s="2">
+        <v>46348</v>
       </c>
       <c r="N54" t="s">
         <v>582</v>
@@ -12595,8 +12621,8 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="1">
-        <v>46347</v>
+      <c r="M55" s="2">
+        <v>46348</v>
       </c>
       <c r="N55" t="s">
         <v>582</v>
@@ -12639,8 +12665,8 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="1">
-        <v>46317</v>
+      <c r="M56" s="2">
+        <v>46318</v>
       </c>
       <c r="N56" t="s">
         <v>582</v>
@@ -12683,8 +12709,8 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="1">
-        <v>46317</v>
+      <c r="M57" s="2">
+        <v>46318</v>
       </c>
       <c r="N57" t="s">
         <v>582</v>
@@ -12727,8 +12753,8 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="1">
-        <v>46317</v>
+      <c r="M58" s="2">
+        <v>46318</v>
       </c>
       <c r="N58" t="s">
         <v>582</v>
@@ -12771,8 +12797,8 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="1">
-        <v>46347</v>
+      <c r="M59" s="2">
+        <v>46348</v>
       </c>
       <c r="N59" t="s">
         <v>582</v>
@@ -12815,8 +12841,8 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="1">
-        <v>46317</v>
+      <c r="M60" s="2">
+        <v>46318</v>
       </c>
       <c r="N60" t="s">
         <v>582</v>
@@ -12859,8 +12885,8 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="1">
-        <v>46317</v>
+      <c r="M61" s="2">
+        <v>46318</v>
       </c>
       <c r="N61" t="s">
         <v>582</v>
@@ -12903,8 +12929,8 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="1">
-        <v>46347</v>
+      <c r="M62" s="2">
+        <v>46348</v>
       </c>
       <c r="N62" t="s">
         <v>582</v>
@@ -12947,8 +12973,8 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="1">
-        <v>46347</v>
+      <c r="M63" s="2">
+        <v>46348</v>
       </c>
       <c r="N63" t="s">
         <v>582</v>
@@ -12991,8 +13017,8 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="1">
-        <v>46362</v>
+      <c r="M64" s="2">
+        <v>46363</v>
       </c>
       <c r="N64" t="s">
         <v>582</v>
@@ -13035,8 +13061,8 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="1">
-        <v>46347</v>
+      <c r="M65" s="2">
+        <v>46348</v>
       </c>
       <c r="N65" t="s">
         <v>582</v>
@@ -13079,8 +13105,8 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="1">
-        <v>46347</v>
+      <c r="M66" s="2">
+        <v>46348</v>
       </c>
       <c r="N66" t="s">
         <v>582</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (08/09/2026 12:04)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -1773,16 +1773,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1798,7 +1790,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1806,30 +1798,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2129,55 +2103,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2221,7 +2195,7 @@
       <c r="N2" t="s">
         <v>395</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>46104</v>
       </c>
     </row>
@@ -2265,7 +2239,7 @@
       <c r="N3" t="s">
         <v>395</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -2309,7 +2283,7 @@
       <c r="N4" t="s">
         <v>395</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -2435,7 +2409,7 @@
       <c r="N7" t="s">
         <v>395</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2479,7 +2453,7 @@
       <c r="N8" t="s">
         <v>395</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2523,7 +2497,7 @@
       <c r="N9" t="s">
         <v>395</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>46032</v>
       </c>
       <c r="Q9" t="s">
@@ -2570,7 +2544,7 @@
       <c r="N10" t="s">
         <v>395</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -2693,7 +2667,7 @@
       <c r="N13" t="s">
         <v>395</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -2737,7 +2711,7 @@
       <c r="N14" t="s">
         <v>395</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2781,7 +2755,7 @@
       <c r="N15" t="s">
         <v>395</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -2825,7 +2799,7 @@
       <c r="N16" t="s">
         <v>395</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46101</v>
       </c>
       <c r="Q16" t="s">
@@ -2872,7 +2846,7 @@
       <c r="N17" t="s">
         <v>395</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -2916,7 +2890,7 @@
       <c r="N18" t="s">
         <v>395</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3042,7 +3016,7 @@
       <c r="N21" t="s">
         <v>395</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3086,7 +3060,7 @@
       <c r="N22" t="s">
         <v>395</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3171,7 +3145,7 @@
       <c r="N24" t="s">
         <v>395</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46160</v>
       </c>
       <c r="Q24" t="s">
@@ -3218,7 +3192,7 @@
       <c r="N25" t="s">
         <v>395</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>46101</v>
       </c>
       <c r="Q25" t="s">
@@ -3265,7 +3239,7 @@
       <c r="N26" t="s">
         <v>395</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3309,7 +3283,7 @@
       <c r="N27" t="s">
         <v>395</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45964</v>
       </c>
     </row>
@@ -3353,7 +3327,7 @@
       <c r="N28" t="s">
         <v>395</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -3438,7 +3412,7 @@
       <c r="N30" t="s">
         <v>395</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -3523,7 +3497,7 @@
       <c r="N32" t="s">
         <v>395</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>46101</v>
       </c>
       <c r="Q32" t="s">
@@ -3570,7 +3544,7 @@
       <c r="N33" t="s">
         <v>395</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3614,7 +3588,7 @@
       <c r="N34" t="s">
         <v>395</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3658,7 +3632,7 @@
       <c r="N35" t="s">
         <v>395</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -3743,7 +3717,7 @@
       <c r="N37" t="s">
         <v>395</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -3787,7 +3761,7 @@
       <c r="N38" t="s">
         <v>395</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -3831,7 +3805,7 @@
       <c r="N39" t="s">
         <v>395</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3916,7 +3890,7 @@
       <c r="N41" t="s">
         <v>395</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -3960,7 +3934,7 @@
       <c r="N42" t="s">
         <v>395</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4004,7 +3978,7 @@
       <c r="N43" t="s">
         <v>395</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -4048,7 +4022,7 @@
       <c r="N44" t="s">
         <v>395</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4215,7 +4189,7 @@
       <c r="N48" t="s">
         <v>395</v>
       </c>
-      <c r="P48" s="2">
+      <c r="P48" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4259,7 +4233,7 @@
       <c r="N49" t="s">
         <v>395</v>
       </c>
-      <c r="P49" s="2">
+      <c r="P49" s="1">
         <v>45955</v>
       </c>
     </row>
@@ -4303,7 +4277,7 @@
       <c r="N50" t="s">
         <v>395</v>
       </c>
-      <c r="P50" s="2">
+      <c r="P50" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4347,7 +4321,7 @@
       <c r="N51" t="s">
         <v>395</v>
       </c>
-      <c r="P51" s="2">
+      <c r="P51" s="1">
         <v>46050</v>
       </c>
       <c r="Q51" t="s">
@@ -4394,7 +4368,7 @@
       <c r="N52" t="s">
         <v>395</v>
       </c>
-      <c r="P52" s="2">
+      <c r="P52" s="1">
         <v>46163</v>
       </c>
     </row>
@@ -4438,7 +4412,7 @@
       <c r="N53" t="s">
         <v>395</v>
       </c>
-      <c r="P53" s="2">
+      <c r="P53" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4520,7 +4494,7 @@
       <c r="N55" t="s">
         <v>395</v>
       </c>
-      <c r="P55" s="2">
+      <c r="P55" s="1">
         <v>46050</v>
       </c>
     </row>
@@ -4564,7 +4538,7 @@
       <c r="N56" t="s">
         <v>395</v>
       </c>
-      <c r="P56" s="2">
+      <c r="P56" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4652,7 +4626,7 @@
       <c r="N58" t="s">
         <v>395</v>
       </c>
-      <c r="P58" s="2">
+      <c r="P58" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -4696,7 +4670,7 @@
       <c r="N59" t="s">
         <v>395</v>
       </c>
-      <c r="P59" s="2">
+      <c r="P59" s="1">
         <v>46050</v>
       </c>
       <c r="Q59" t="s">
@@ -4743,7 +4717,7 @@
       <c r="N60" t="s">
         <v>395</v>
       </c>
-      <c r="P60" s="2">
+      <c r="P60" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -4787,7 +4761,7 @@
       <c r="N61" t="s">
         <v>395</v>
       </c>
-      <c r="P61" s="2">
+      <c r="P61" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -4831,7 +4805,7 @@
       <c r="N62" t="s">
         <v>395</v>
       </c>
-      <c r="P62" s="2">
+      <c r="P62" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -4875,7 +4849,7 @@
       <c r="N63" t="s">
         <v>395</v>
       </c>
-      <c r="P63" s="2">
+      <c r="P63" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -4919,7 +4893,7 @@
       <c r="N64" t="s">
         <v>395</v>
       </c>
-      <c r="P64" s="2">
+      <c r="P64" s="1">
         <v>46101</v>
       </c>
       <c r="Q64" t="s">
@@ -4966,7 +4940,7 @@
       <c r="N65" t="s">
         <v>395</v>
       </c>
-      <c r="P65" s="2">
+      <c r="P65" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -5010,7 +4984,7 @@
       <c r="N66" t="s">
         <v>395</v>
       </c>
-      <c r="P66" s="2">
+      <c r="P66" s="1">
         <v>45946</v>
       </c>
       <c r="Q66" t="s">
@@ -5057,7 +5031,7 @@
       <c r="N67" t="s">
         <v>395</v>
       </c>
-      <c r="P67" s="2">
+      <c r="P67" s="1">
         <v>45916</v>
       </c>
     </row>
@@ -5101,7 +5075,7 @@
       <c r="N68" t="s">
         <v>395</v>
       </c>
-      <c r="P68" s="2">
+      <c r="P68" s="1">
         <v>46066</v>
       </c>
       <c r="Q68" t="s">
@@ -5148,7 +5122,7 @@
       <c r="N69" t="s">
         <v>395</v>
       </c>
-      <c r="P69" s="2">
+      <c r="P69" s="1">
         <v>45989</v>
       </c>
       <c r="Q69" t="s">
@@ -5236,7 +5210,7 @@
       <c r="N71" t="s">
         <v>395</v>
       </c>
-      <c r="P71" s="2">
+      <c r="P71" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5280,7 +5254,7 @@
       <c r="N72" t="s">
         <v>395</v>
       </c>
-      <c r="P72" s="2">
+      <c r="P72" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5324,7 +5298,7 @@
       <c r="N73" t="s">
         <v>395</v>
       </c>
-      <c r="P73" s="2">
+      <c r="P73" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5368,7 +5342,7 @@
       <c r="N74" t="s">
         <v>395</v>
       </c>
-      <c r="P74" s="2">
+      <c r="P74" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5412,7 +5386,7 @@
       <c r="N75" t="s">
         <v>395</v>
       </c>
-      <c r="P75" s="2">
+      <c r="P75" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5456,7 +5430,7 @@
       <c r="N76" t="s">
         <v>395</v>
       </c>
-      <c r="P76" s="2">
+      <c r="P76" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -5541,7 +5515,7 @@
       <c r="N78" t="s">
         <v>395</v>
       </c>
-      <c r="P78" s="2">
+      <c r="P78" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -5585,7 +5559,7 @@
       <c r="N79" t="s">
         <v>395</v>
       </c>
-      <c r="P79" s="2">
+      <c r="P79" s="1">
         <v>46140</v>
       </c>
     </row>
@@ -5629,7 +5603,7 @@
       <c r="N80" t="s">
         <v>395</v>
       </c>
-      <c r="P80" s="2">
+      <c r="P80" s="1">
         <v>46095</v>
       </c>
     </row>
@@ -5673,7 +5647,7 @@
       <c r="N81" t="s">
         <v>395</v>
       </c>
-      <c r="P81" s="2">
+      <c r="P81" s="1">
         <v>46040</v>
       </c>
     </row>
@@ -5717,7 +5691,7 @@
       <c r="N82" t="s">
         <v>395</v>
       </c>
-      <c r="P82" s="2">
+      <c r="P82" s="1">
         <v>46060</v>
       </c>
     </row>
@@ -5761,7 +5735,7 @@
       <c r="N83" t="s">
         <v>395</v>
       </c>
-      <c r="P83" s="2">
+      <c r="P83" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5805,7 +5779,7 @@
       <c r="N84" t="s">
         <v>395</v>
       </c>
-      <c r="P84" s="2">
+      <c r="P84" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5849,7 +5823,7 @@
       <c r="N85" t="s">
         <v>395</v>
       </c>
-      <c r="P85" s="2">
+      <c r="P85" s="1">
         <v>45976</v>
       </c>
       <c r="Q85" t="s">
@@ -5896,7 +5870,7 @@
       <c r="N86" t="s">
         <v>395</v>
       </c>
-      <c r="P86" s="2">
+      <c r="P86" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5940,7 +5914,7 @@
       <c r="N87" t="s">
         <v>395</v>
       </c>
-      <c r="P87" s="2">
+      <c r="P87" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -5984,7 +5958,7 @@
       <c r="N88" t="s">
         <v>395</v>
       </c>
-      <c r="P88" s="2">
+      <c r="P88" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6028,7 +6002,7 @@
       <c r="N89" t="s">
         <v>395</v>
       </c>
-      <c r="P89" s="2">
+      <c r="P89" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6072,7 +6046,7 @@
       <c r="N90" t="s">
         <v>395</v>
       </c>
-      <c r="P90" s="2">
+      <c r="P90" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6116,7 +6090,7 @@
       <c r="N91" t="s">
         <v>395</v>
       </c>
-      <c r="P91" s="2">
+      <c r="P91" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6160,7 +6134,7 @@
       <c r="N92" t="s">
         <v>395</v>
       </c>
-      <c r="P92" s="2">
+      <c r="P92" s="1">
         <v>46080</v>
       </c>
     </row>
@@ -6204,7 +6178,7 @@
       <c r="N93" t="s">
         <v>395</v>
       </c>
-      <c r="P93" s="2">
+      <c r="P93" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -6248,7 +6222,7 @@
       <c r="N94" t="s">
         <v>395</v>
       </c>
-      <c r="P94" s="2">
+      <c r="P94" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -6336,7 +6310,7 @@
       <c r="N96" t="s">
         <v>395</v>
       </c>
-      <c r="P96" s="2">
+      <c r="P96" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6380,7 +6354,7 @@
       <c r="N97" t="s">
         <v>395</v>
       </c>
-      <c r="P97" s="2">
+      <c r="P97" s="1">
         <v>46032</v>
       </c>
     </row>
@@ -6506,7 +6480,7 @@
       <c r="N100" t="s">
         <v>395</v>
       </c>
-      <c r="P100" s="2">
+      <c r="P100" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -6550,7 +6524,7 @@
       <c r="N101" t="s">
         <v>395</v>
       </c>
-      <c r="P101" s="2">
+      <c r="P101" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6594,7 +6568,7 @@
       <c r="N102" t="s">
         <v>395</v>
       </c>
-      <c r="P102" s="2">
+      <c r="P102" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6638,7 +6612,7 @@
       <c r="N103" t="s">
         <v>395</v>
       </c>
-      <c r="P103" s="2">
+      <c r="P103" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -6720,7 +6694,7 @@
       <c r="N105" t="s">
         <v>395</v>
       </c>
-      <c r="P105" s="2">
+      <c r="P105" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -6764,7 +6738,7 @@
       <c r="N106" t="s">
         <v>395</v>
       </c>
-      <c r="P106" s="2">
+      <c r="P106" s="1">
         <v>45911</v>
       </c>
       <c r="Q106" t="s">
@@ -6811,7 +6785,7 @@
       <c r="N107" t="s">
         <v>395</v>
       </c>
-      <c r="P107" s="2">
+      <c r="P107" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6855,7 +6829,7 @@
       <c r="N108" t="s">
         <v>395</v>
       </c>
-      <c r="P108" s="2">
+      <c r="P108" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -6981,7 +6955,7 @@
       <c r="N111" t="s">
         <v>395</v>
       </c>
-      <c r="P111" s="2">
+      <c r="P111" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -7025,7 +6999,7 @@
       <c r="N112" t="s">
         <v>395</v>
       </c>
-      <c r="P112" s="2">
+      <c r="P112" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -7110,7 +7084,7 @@
       <c r="N114" t="s">
         <v>395</v>
       </c>
-      <c r="P114" s="2">
+      <c r="P114" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -7154,7 +7128,7 @@
       <c r="N115" t="s">
         <v>395</v>
       </c>
-      <c r="P115" s="2">
+      <c r="P115" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7198,7 +7172,7 @@
       <c r="N116" t="s">
         <v>395</v>
       </c>
-      <c r="P116" s="2">
+      <c r="P116" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7242,7 +7216,7 @@
       <c r="N117" t="s">
         <v>395</v>
       </c>
-      <c r="P117" s="2">
+      <c r="P117" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -7286,7 +7260,7 @@
       <c r="N118" t="s">
         <v>395</v>
       </c>
-      <c r="P118" s="2">
+      <c r="P118" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -7330,7 +7304,7 @@
       <c r="N119" t="s">
         <v>395</v>
       </c>
-      <c r="P119" s="2">
+      <c r="P119" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7374,7 +7348,7 @@
       <c r="N120" t="s">
         <v>395</v>
       </c>
-      <c r="P120" s="2">
+      <c r="P120" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7418,7 +7392,7 @@
       <c r="N121" t="s">
         <v>395</v>
       </c>
-      <c r="P121" s="2">
+      <c r="P121" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -7503,7 +7477,7 @@
       <c r="N123" t="s">
         <v>395</v>
       </c>
-      <c r="P123" s="2">
+      <c r="P123" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -7670,7 +7644,7 @@
       <c r="N127" t="s">
         <v>395</v>
       </c>
-      <c r="P127" s="2">
+      <c r="P127" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -7714,7 +7688,7 @@
       <c r="N128" t="s">
         <v>395</v>
       </c>
-      <c r="P128" s="2">
+      <c r="P128" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -7758,7 +7732,7 @@
       <c r="N129" t="s">
         <v>395</v>
       </c>
-      <c r="P129" s="2">
+      <c r="P129" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7802,7 +7776,7 @@
       <c r="N130" t="s">
         <v>395</v>
       </c>
-      <c r="P130" s="2">
+      <c r="P130" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7846,7 +7820,7 @@
       <c r="N131" t="s">
         <v>395</v>
       </c>
-      <c r="P131" s="2">
+      <c r="P131" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7890,7 +7864,7 @@
       <c r="N132" t="s">
         <v>395</v>
       </c>
-      <c r="P132" s="2">
+      <c r="P132" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -7934,7 +7908,7 @@
       <c r="N133" t="s">
         <v>395</v>
       </c>
-      <c r="P133" s="2">
+      <c r="P133" s="1">
         <v>46130</v>
       </c>
     </row>
@@ -8019,7 +7993,7 @@
       <c r="N135" t="s">
         <v>395</v>
       </c>
-      <c r="P135" s="2">
+      <c r="P135" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8063,7 +8037,7 @@
       <c r="N136" t="s">
         <v>395</v>
       </c>
-      <c r="P136" s="2">
+      <c r="P136" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8148,7 +8122,7 @@
       <c r="N138" t="s">
         <v>395</v>
       </c>
-      <c r="P138" s="2">
+      <c r="P138" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8274,7 +8248,7 @@
       <c r="N141" t="s">
         <v>395</v>
       </c>
-      <c r="P141" s="2">
+      <c r="P141" s="1">
         <v>46160</v>
       </c>
     </row>
@@ -8318,7 +8292,7 @@
       <c r="N142" t="s">
         <v>395</v>
       </c>
-      <c r="P142" s="2">
+      <c r="P142" s="1">
         <v>46123</v>
       </c>
     </row>
@@ -8403,7 +8377,7 @@
       <c r="N144" t="s">
         <v>395</v>
       </c>
-      <c r="P144" s="2">
+      <c r="P144" s="1">
         <v>46167</v>
       </c>
     </row>
@@ -8447,7 +8421,7 @@
       <c r="N145" t="s">
         <v>395</v>
       </c>
-      <c r="P145" s="2">
+      <c r="P145" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8491,7 +8465,7 @@
       <c r="N146" t="s">
         <v>395</v>
       </c>
-      <c r="P146" s="2">
+      <c r="P146" s="1">
         <v>46101</v>
       </c>
     </row>
@@ -8535,7 +8509,7 @@
       <c r="N147" t="s">
         <v>395</v>
       </c>
-      <c r="P147" s="2">
+      <c r="P147" s="1">
         <v>46081</v>
       </c>
     </row>
@@ -8579,7 +8553,7 @@
       <c r="N148" t="s">
         <v>395</v>
       </c>
-      <c r="P148" s="2">
+      <c r="P148" s="1">
         <v>45976</v>
       </c>
     </row>
@@ -8623,7 +8597,7 @@
       <c r="N149" t="s">
         <v>395</v>
       </c>
-      <c r="P149" s="2">
+      <c r="P149" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8667,7 +8641,7 @@
       <c r="N150" t="s">
         <v>395</v>
       </c>
-      <c r="P150" s="2">
+      <c r="P150" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8711,7 +8685,7 @@
       <c r="N151" t="s">
         <v>395</v>
       </c>
-      <c r="P151" s="2">
+      <c r="P151" s="1">
         <v>45979</v>
       </c>
     </row>
@@ -8796,7 +8770,7 @@
       <c r="N153" t="s">
         <v>395</v>
       </c>
-      <c r="P153" s="2">
+      <c r="P153" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -8963,7 +8937,7 @@
       <c r="N157" t="s">
         <v>395</v>
       </c>
-      <c r="P157" s="2">
+      <c r="P157" s="1">
         <v>45959</v>
       </c>
     </row>
@@ -9007,7 +8981,7 @@
       <c r="N158" t="s">
         <v>395</v>
       </c>
-      <c r="P158" s="2">
+      <c r="P158" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9051,7 +9025,7 @@
       <c r="N159" t="s">
         <v>395</v>
       </c>
-      <c r="P159" s="2">
+      <c r="P159" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9095,7 +9069,7 @@
       <c r="N160" t="s">
         <v>395</v>
       </c>
-      <c r="P160" s="2">
+      <c r="P160" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9180,7 +9154,7 @@
       <c r="N162" t="s">
         <v>395</v>
       </c>
-      <c r="P162" s="2">
+      <c r="P162" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9224,7 +9198,7 @@
       <c r="N163" t="s">
         <v>395</v>
       </c>
-      <c r="P163" s="2">
+      <c r="P163" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9268,7 +9242,7 @@
       <c r="N164" t="s">
         <v>395</v>
       </c>
-      <c r="P164" s="2">
+      <c r="P164" s="1">
         <v>45984</v>
       </c>
     </row>
@@ -9312,7 +9286,7 @@
       <c r="N165" t="s">
         <v>395</v>
       </c>
-      <c r="P165" s="2">
+      <c r="P165" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9356,7 +9330,7 @@
       <c r="N166" t="s">
         <v>395</v>
       </c>
-      <c r="P166" s="2">
+      <c r="P166" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9400,7 +9374,7 @@
       <c r="N167" t="s">
         <v>395</v>
       </c>
-      <c r="P167" s="2">
+      <c r="P167" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9444,7 +9418,7 @@
       <c r="N168" t="s">
         <v>395</v>
       </c>
-      <c r="P168" s="2">
+      <c r="P168" s="1">
         <v>45994</v>
       </c>
     </row>
@@ -9488,7 +9462,7 @@
       <c r="N169" t="s">
         <v>395</v>
       </c>
-      <c r="P169" s="2">
+      <c r="P169" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9532,7 +9506,7 @@
       <c r="N170" t="s">
         <v>395</v>
       </c>
-      <c r="P170" s="2">
+      <c r="P170" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9576,7 +9550,7 @@
       <c r="N171" t="s">
         <v>395</v>
       </c>
-      <c r="P171" s="2">
+      <c r="P171" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9620,7 +9594,7 @@
       <c r="N172" t="s">
         <v>395</v>
       </c>
-      <c r="P172" s="2">
+      <c r="P172" s="1">
         <v>45954</v>
       </c>
     </row>
@@ -9664,7 +9638,7 @@
       <c r="N173" t="s">
         <v>395</v>
       </c>
-      <c r="P173" s="2">
+      <c r="P173" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -9708,7 +9682,7 @@
       <c r="N174" t="s">
         <v>395</v>
       </c>
-      <c r="P174" s="2">
+      <c r="P174" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -9752,7 +9726,7 @@
       <c r="N175" t="s">
         <v>395</v>
       </c>
-      <c r="P175" s="2">
+      <c r="P175" s="1">
         <v>45911</v>
       </c>
     </row>
@@ -9796,7 +9770,7 @@
       <c r="N176" t="s">
         <v>395</v>
       </c>
-      <c r="P176" s="2">
+      <c r="P176" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9840,7 +9814,7 @@
       <c r="N177" t="s">
         <v>395</v>
       </c>
-      <c r="P177" s="2">
+      <c r="P177" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9884,7 +9858,7 @@
       <c r="N178" t="s">
         <v>395</v>
       </c>
-      <c r="P178" s="2">
+      <c r="P178" s="1">
         <v>45908</v>
       </c>
     </row>
@@ -9928,7 +9902,7 @@
       <c r="N179" t="s">
         <v>395</v>
       </c>
-      <c r="P179" s="2">
+      <c r="P179" s="1">
         <v>45835</v>
       </c>
     </row>
@@ -9972,7 +9946,7 @@
       <c r="N180" t="s">
         <v>395</v>
       </c>
-      <c r="P180" s="2">
+      <c r="P180" s="1">
         <v>46025</v>
       </c>
     </row>
@@ -10016,7 +9990,7 @@
       <c r="N181" t="s">
         <v>395</v>
       </c>
-      <c r="P181" s="2">
+      <c r="P181" s="1">
         <v>46024</v>
       </c>
     </row>
@@ -10060,7 +10034,7 @@
       <c r="N182" t="s">
         <v>395</v>
       </c>
-      <c r="P182" s="2">
+      <c r="P182" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10145,7 +10119,7 @@
       <c r="N184" t="s">
         <v>395</v>
       </c>
-      <c r="P184" s="2">
+      <c r="P184" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10230,7 +10204,7 @@
       <c r="N186" t="s">
         <v>395</v>
       </c>
-      <c r="P186" s="2">
+      <c r="P186" s="1">
         <v>45904</v>
       </c>
     </row>
@@ -10245,55 +10219,55 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10580,7 +10554,7 @@
       <c r="L8" t="s">
         <v>577</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="1">
         <v>46303</v>
       </c>
       <c r="N8" t="s">
@@ -10665,7 +10639,7 @@
       <c r="L10" t="s">
         <v>578</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="1">
         <v>46348</v>
       </c>
       <c r="N10" t="s">
@@ -10709,7 +10683,7 @@
       <c r="L11" t="s">
         <v>578</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="1">
         <v>46348</v>
       </c>
       <c r="N11" t="s">
@@ -10876,7 +10850,7 @@
       <c r="L15" t="s">
         <v>577</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="1">
         <v>46303</v>
       </c>
       <c r="N15" t="s">
@@ -10920,7 +10894,7 @@
       <c r="L16" t="s">
         <v>578</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16" s="1">
         <v>46348</v>
       </c>
       <c r="N16" t="s">
@@ -10964,7 +10938,7 @@
       <c r="L17" t="s">
         <v>577</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17" s="1">
         <v>46303</v>
       </c>
       <c r="N17" t="s">
@@ -11008,7 +10982,7 @@
       <c r="L18" t="s">
         <v>578</v>
       </c>
-      <c r="M18" s="2">
+      <c r="M18" s="1">
         <v>46348</v>
       </c>
       <c r="N18" t="s">
@@ -11052,7 +11026,7 @@
       <c r="L19" t="s">
         <v>578</v>
       </c>
-      <c r="M19" s="2">
+      <c r="M19" s="1">
         <v>46348</v>
       </c>
       <c r="N19" t="s">
@@ -11096,7 +11070,7 @@
       <c r="L20" t="s">
         <v>578</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M20" s="1">
         <v>46348</v>
       </c>
       <c r="N20" t="s">
@@ -11140,7 +11114,7 @@
       <c r="L21" t="s">
         <v>578</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="1">
         <v>46348</v>
       </c>
       <c r="N21" t="s">
@@ -11307,7 +11281,7 @@
       <c r="L25" t="s">
         <v>578</v>
       </c>
-      <c r="M25" s="2">
+      <c r="M25" s="1">
         <v>46348</v>
       </c>
       <c r="N25" t="s">
@@ -11392,7 +11366,7 @@
       <c r="L27" t="s">
         <v>577</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="1">
         <v>46303</v>
       </c>
       <c r="N27" t="s">
@@ -11436,7 +11410,7 @@
       <c r="L28" t="s">
         <v>578</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="1">
         <v>46348</v>
       </c>
       <c r="N28" t="s">
@@ -11480,7 +11454,7 @@
       <c r="L29" t="s">
         <v>581</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="1">
         <v>46318</v>
       </c>
       <c r="N29" t="s">
@@ -11524,7 +11498,7 @@
       <c r="L30" t="s">
         <v>578</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="1">
         <v>46348</v>
       </c>
       <c r="N30" t="s">
@@ -11568,7 +11542,7 @@
       <c r="L31" t="s">
         <v>581</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="1">
         <v>46318</v>
       </c>
       <c r="N31" t="s">
@@ -11612,7 +11586,7 @@
       <c r="L32" t="s">
         <v>577</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="1">
         <v>46303</v>
       </c>
       <c r="N32" t="s">
@@ -11656,7 +11630,7 @@
       <c r="L33" t="s">
         <v>577</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="1">
         <v>46303</v>
       </c>
       <c r="N33" t="s">
@@ -11700,7 +11674,7 @@
       <c r="L34" t="s">
         <v>577</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="1">
         <v>46303</v>
       </c>
       <c r="N34" t="s">
@@ -11744,7 +11718,7 @@
       <c r="L35" t="s">
         <v>577</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="1">
         <v>46303</v>
       </c>
       <c r="N35" t="s">
@@ -11788,7 +11762,7 @@
       <c r="L36" t="s">
         <v>577</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="1">
         <v>46303</v>
       </c>
       <c r="N36" t="s">
@@ -11832,7 +11806,7 @@
       <c r="L37" t="s">
         <v>577</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="1">
         <v>46303</v>
       </c>
       <c r="N37" t="s">
@@ -11876,7 +11850,7 @@
       <c r="L38" t="s">
         <v>577</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="1">
         <v>46303</v>
       </c>
       <c r="N38" t="s">
@@ -11961,7 +11935,7 @@
       <c r="L40" t="s">
         <v>577</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="1">
         <v>46303</v>
       </c>
       <c r="N40" t="s">
@@ -12005,7 +11979,7 @@
       <c r="L41" t="s">
         <v>578</v>
       </c>
-      <c r="M41" s="2">
+      <c r="M41" s="1">
         <v>46348</v>
       </c>
       <c r="N41" t="s">
@@ -12049,7 +12023,7 @@
       <c r="L42" t="s">
         <v>577</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M42" s="1">
         <v>46303</v>
       </c>
       <c r="N42" t="s">
@@ -12093,7 +12067,7 @@
       <c r="L43" t="s">
         <v>580</v>
       </c>
-      <c r="M43" s="2">
+      <c r="M43" s="1">
         <v>46363</v>
       </c>
       <c r="N43" t="s">
@@ -12137,7 +12111,7 @@
       <c r="L44" t="s">
         <v>578</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="1">
         <v>46348</v>
       </c>
       <c r="N44" t="s">
@@ -12181,7 +12155,7 @@
       <c r="L45" t="s">
         <v>578</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="1">
         <v>46348</v>
       </c>
       <c r="N45" t="s">
@@ -12225,7 +12199,7 @@
       <c r="L46" t="s">
         <v>577</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="1">
         <v>46303</v>
       </c>
       <c r="N46" t="s">
@@ -12269,7 +12243,7 @@
       <c r="L47" t="s">
         <v>577</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="1">
         <v>46303</v>
       </c>
       <c r="N47" t="s">
@@ -12313,7 +12287,7 @@
       <c r="L48" t="s">
         <v>578</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="1">
         <v>46348</v>
       </c>
       <c r="N48" t="s">
@@ -12357,7 +12331,7 @@
       <c r="L49" t="s">
         <v>581</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="1">
         <v>46318</v>
       </c>
       <c r="N49" t="s">
@@ -12401,7 +12375,7 @@
       <c r="L50" t="s">
         <v>581</v>
       </c>
-      <c r="M50" s="2">
+      <c r="M50" s="1">
         <v>46318</v>
       </c>
       <c r="N50" t="s">
@@ -12445,7 +12419,7 @@
       <c r="L51" t="s">
         <v>578</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="1">
         <v>46348</v>
       </c>
       <c r="N51" t="s">
@@ -12489,7 +12463,7 @@
       <c r="L52" t="s">
         <v>578</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="1">
         <v>46348</v>
       </c>
       <c r="N52" t="s">
@@ -12533,7 +12507,7 @@
       <c r="L53" t="s">
         <v>578</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="1">
         <v>46348</v>
       </c>
       <c r="N53" t="s">
@@ -12577,7 +12551,7 @@
       <c r="L54" t="s">
         <v>578</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="1">
         <v>46348</v>
       </c>
       <c r="N54" t="s">
@@ -12621,7 +12595,7 @@
       <c r="L55" t="s">
         <v>578</v>
       </c>
-      <c r="M55" s="2">
+      <c r="M55" s="1">
         <v>46348</v>
       </c>
       <c r="N55" t="s">
@@ -12665,7 +12639,7 @@
       <c r="L56" t="s">
         <v>581</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M56" s="1">
         <v>46318</v>
       </c>
       <c r="N56" t="s">
@@ -12709,7 +12683,7 @@
       <c r="L57" t="s">
         <v>581</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="1">
         <v>46318</v>
       </c>
       <c r="N57" t="s">
@@ -12753,7 +12727,7 @@
       <c r="L58" t="s">
         <v>581</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="1">
         <v>46318</v>
       </c>
       <c r="N58" t="s">
@@ -12797,7 +12771,7 @@
       <c r="L59" t="s">
         <v>578</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="1">
         <v>46348</v>
       </c>
       <c r="N59" t="s">
@@ -12841,7 +12815,7 @@
       <c r="L60" t="s">
         <v>581</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="1">
         <v>46318</v>
       </c>
       <c r="N60" t="s">
@@ -12885,7 +12859,7 @@
       <c r="L61" t="s">
         <v>581</v>
       </c>
-      <c r="M61" s="2">
+      <c r="M61" s="1">
         <v>46318</v>
       </c>
       <c r="N61" t="s">
@@ -12929,7 +12903,7 @@
       <c r="L62" t="s">
         <v>578</v>
       </c>
-      <c r="M62" s="2">
+      <c r="M62" s="1">
         <v>46348</v>
       </c>
       <c r="N62" t="s">
@@ -12973,7 +12947,7 @@
       <c r="L63" t="s">
         <v>578</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="1">
         <v>46348</v>
       </c>
       <c r="N63" t="s">
@@ -13017,7 +12991,7 @@
       <c r="L64" t="s">
         <v>580</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="1">
         <v>46363</v>
       </c>
       <c r="N64" t="s">
@@ -13061,7 +13035,7 @@
       <c r="L65" t="s">
         <v>578</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="1">
         <v>46348</v>
       </c>
       <c r="N65" t="s">
@@ -13105,7 +13079,7 @@
       <c r="L66" t="s">
         <v>578</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="1">
         <v>46348</v>
       </c>
       <c r="N66" t="s">

</xml_diff>

<commit_message>
Atualização automática: tpjl (09/09/2026 12:06)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10555,7 +10555,7 @@
         <v>577</v>
       </c>
       <c r="M8" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N8" t="s">
         <v>582</v>
@@ -10640,7 +10640,7 @@
         <v>578</v>
       </c>
       <c r="M10" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N10" t="s">
         <v>582</v>
@@ -10684,7 +10684,7 @@
         <v>578</v>
       </c>
       <c r="M11" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N11" t="s">
         <v>582</v>
@@ -10851,7 +10851,7 @@
         <v>577</v>
       </c>
       <c r="M15" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N15" t="s">
         <v>582</v>
@@ -10895,7 +10895,7 @@
         <v>578</v>
       </c>
       <c r="M16" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N16" t="s">
         <v>582</v>
@@ -10939,7 +10939,7 @@
         <v>577</v>
       </c>
       <c r="M17" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N17" t="s">
         <v>582</v>
@@ -10983,7 +10983,7 @@
         <v>578</v>
       </c>
       <c r="M18" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N18" t="s">
         <v>582</v>
@@ -11027,7 +11027,7 @@
         <v>578</v>
       </c>
       <c r="M19" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N19" t="s">
         <v>582</v>
@@ -11071,7 +11071,7 @@
         <v>578</v>
       </c>
       <c r="M20" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N20" t="s">
         <v>582</v>
@@ -11115,7 +11115,7 @@
         <v>578</v>
       </c>
       <c r="M21" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N21" t="s">
         <v>582</v>
@@ -11282,7 +11282,7 @@
         <v>578</v>
       </c>
       <c r="M25" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N25" t="s">
         <v>582</v>
@@ -11367,7 +11367,7 @@
         <v>577</v>
       </c>
       <c r="M27" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N27" t="s">
         <v>582</v>
@@ -11411,7 +11411,7 @@
         <v>578</v>
       </c>
       <c r="M28" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N28" t="s">
         <v>582</v>
@@ -11455,7 +11455,7 @@
         <v>581</v>
       </c>
       <c r="M29" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N29" t="s">
         <v>582</v>
@@ -11499,7 +11499,7 @@
         <v>578</v>
       </c>
       <c r="M30" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N30" t="s">
         <v>582</v>
@@ -11543,7 +11543,7 @@
         <v>581</v>
       </c>
       <c r="M31" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N31" t="s">
         <v>582</v>
@@ -11587,7 +11587,7 @@
         <v>577</v>
       </c>
       <c r="M32" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N32" t="s">
         <v>582</v>
@@ -11631,7 +11631,7 @@
         <v>577</v>
       </c>
       <c r="M33" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N33" t="s">
         <v>582</v>
@@ -11675,7 +11675,7 @@
         <v>577</v>
       </c>
       <c r="M34" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N34" t="s">
         <v>582</v>
@@ -11719,7 +11719,7 @@
         <v>577</v>
       </c>
       <c r="M35" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N35" t="s">
         <v>582</v>
@@ -11763,7 +11763,7 @@
         <v>577</v>
       </c>
       <c r="M36" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N36" t="s">
         <v>582</v>
@@ -11807,7 +11807,7 @@
         <v>577</v>
       </c>
       <c r="M37" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N37" t="s">
         <v>582</v>
@@ -11851,7 +11851,7 @@
         <v>577</v>
       </c>
       <c r="M38" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N38" t="s">
         <v>582</v>
@@ -11936,7 +11936,7 @@
         <v>577</v>
       </c>
       <c r="M40" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N40" t="s">
         <v>582</v>
@@ -11980,7 +11980,7 @@
         <v>578</v>
       </c>
       <c r="M41" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N41" t="s">
         <v>582</v>
@@ -12024,7 +12024,7 @@
         <v>577</v>
       </c>
       <c r="M42" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N42" t="s">
         <v>582</v>
@@ -12068,7 +12068,7 @@
         <v>580</v>
       </c>
       <c r="M43" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N43" t="s">
         <v>582</v>
@@ -12112,7 +12112,7 @@
         <v>578</v>
       </c>
       <c r="M44" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N44" t="s">
         <v>582</v>
@@ -12156,7 +12156,7 @@
         <v>578</v>
       </c>
       <c r="M45" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N45" t="s">
         <v>582</v>
@@ -12200,7 +12200,7 @@
         <v>577</v>
       </c>
       <c r="M46" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N46" t="s">
         <v>582</v>
@@ -12244,7 +12244,7 @@
         <v>577</v>
       </c>
       <c r="M47" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="N47" t="s">
         <v>582</v>
@@ -12288,7 +12288,7 @@
         <v>578</v>
       </c>
       <c r="M48" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N48" t="s">
         <v>582</v>
@@ -12332,7 +12332,7 @@
         <v>581</v>
       </c>
       <c r="M49" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N49" t="s">
         <v>582</v>
@@ -12376,7 +12376,7 @@
         <v>581</v>
       </c>
       <c r="M50" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N50" t="s">
         <v>582</v>
@@ -12420,7 +12420,7 @@
         <v>578</v>
       </c>
       <c r="M51" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N51" t="s">
         <v>582</v>
@@ -12464,7 +12464,7 @@
         <v>578</v>
       </c>
       <c r="M52" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N52" t="s">
         <v>582</v>
@@ -12508,7 +12508,7 @@
         <v>578</v>
       </c>
       <c r="M53" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N53" t="s">
         <v>582</v>
@@ -12552,7 +12552,7 @@
         <v>578</v>
       </c>
       <c r="M54" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N54" t="s">
         <v>582</v>
@@ -12596,7 +12596,7 @@
         <v>578</v>
       </c>
       <c r="M55" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N55" t="s">
         <v>582</v>
@@ -12640,7 +12640,7 @@
         <v>581</v>
       </c>
       <c r="M56" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N56" t="s">
         <v>582</v>
@@ -12684,7 +12684,7 @@
         <v>581</v>
       </c>
       <c r="M57" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N57" t="s">
         <v>582</v>
@@ -12728,7 +12728,7 @@
         <v>581</v>
       </c>
       <c r="M58" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N58" t="s">
         <v>582</v>
@@ -12772,7 +12772,7 @@
         <v>578</v>
       </c>
       <c r="M59" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N59" t="s">
         <v>582</v>
@@ -12816,7 +12816,7 @@
         <v>581</v>
       </c>
       <c r="M60" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N60" t="s">
         <v>582</v>
@@ -12860,7 +12860,7 @@
         <v>581</v>
       </c>
       <c r="M61" s="1">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="N61" t="s">
         <v>582</v>
@@ -12904,7 +12904,7 @@
         <v>578</v>
       </c>
       <c r="M62" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N62" t="s">
         <v>582</v>
@@ -12948,7 +12948,7 @@
         <v>578</v>
       </c>
       <c r="M63" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N63" t="s">
         <v>582</v>
@@ -12992,7 +12992,7 @@
         <v>580</v>
       </c>
       <c r="M64" s="1">
-        <v>46363</v>
+        <v>46364</v>
       </c>
       <c r="N64" t="s">
         <v>582</v>
@@ -13036,7 +13036,7 @@
         <v>578</v>
       </c>
       <c r="M65" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N65" t="s">
         <v>582</v>
@@ -13080,7 +13080,7 @@
         <v>578</v>
       </c>
       <c r="M66" s="1">
-        <v>46348</v>
+        <v>46349</v>
       </c>
       <c r="N66" t="s">
         <v>582</v>

</xml_diff>

<commit_message>
Atualização automática: tpjl (10/09/2026 11:58)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2546" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2596" uniqueCount="597">
   <si>
     <t>numero_requisicao</t>
   </si>
@@ -1430,6 +1430,21 @@
     <t>LST243001U8</t>
   </si>
   <si>
+    <t>LST243004U8</t>
+  </si>
+  <si>
+    <t>LST243007U8</t>
+  </si>
+  <si>
+    <t>LST245013U8</t>
+  </si>
+  <si>
+    <t>LST245015U8</t>
+  </si>
+  <si>
+    <t>LST245019U8</t>
+  </si>
+  <si>
     <t>A-1636-32</t>
   </si>
   <si>
@@ -1598,6 +1613,21 @@
     <t>S3461-76</t>
   </si>
   <si>
+    <t>3074154-01</t>
+  </si>
+  <si>
+    <t>B-5417</t>
+  </si>
+  <si>
+    <t>A-1635-133</t>
+  </si>
+  <si>
+    <t>2654006-10</t>
+  </si>
+  <si>
+    <t>2622243-11</t>
+  </si>
+  <si>
     <t>BUSHING</t>
   </si>
   <si>
@@ -1745,22 +1775,34 @@
     <t>BOLT MPI</t>
   </si>
   <si>
+    <t>GOVERNOR PROPELLER</t>
+  </si>
+  <si>
+    <t>FLANGE ASSY-PRIMARY EXHAUST</t>
+  </si>
+  <si>
+    <t>ECCENTRIC-WING ASSY ATTACH</t>
+  </si>
+  <si>
     <t>Empenho Solicitado</t>
   </si>
   <si>
+    <t>Mapa Gerado</t>
+  </si>
+  <si>
+    <t>Aguardando Conferência do ACI</t>
+  </si>
+  <si>
+    <t>Validada</t>
+  </si>
+  <si>
     <t>Em Cotação</t>
   </si>
   <si>
-    <t>Validada</t>
-  </si>
-  <si>
-    <t>Selecionada para Cotação</t>
+    <t>Em Discrepância</t>
   </si>
   <si>
     <t>Análise do Pedido</t>
-  </si>
-  <si>
-    <t>Selecionada para cotação</t>
   </si>
   <si>
     <t>No prazo</t>
@@ -10215,7 +10257,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q66"/>
+  <dimension ref="A1:Q71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -10297,7 +10339,7 @@
         <v>516.34</v>
       </c>
       <c r="I2" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J2" t="s">
         <v>387</v>
@@ -10338,7 +10380,7 @@
         <v>191.04</v>
       </c>
       <c r="I3" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J3" t="s">
         <v>387</v>
@@ -10364,7 +10406,7 @@
         <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="E4" t="s">
         <v>297</v>
@@ -10379,7 +10421,7 @@
         <v>314.56</v>
       </c>
       <c r="I4" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J4" t="s">
         <v>387</v>
@@ -10405,10 +10447,10 @@
         <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="E5" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -10420,7 +10462,7 @@
         <v>1859.13</v>
       </c>
       <c r="I5" t="s">
-        <v>380</v>
+        <v>589</v>
       </c>
       <c r="J5" t="s">
         <v>380</v>
@@ -10461,7 +10503,7 @@
         <v>1572.48</v>
       </c>
       <c r="I6" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J6" t="s">
         <v>387</v>
@@ -10502,7 +10544,7 @@
         <v>1148.68</v>
       </c>
       <c r="I7" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J7" t="s">
         <v>387</v>
@@ -10543,22 +10585,22 @@
         <v>1250.4</v>
       </c>
       <c r="I8" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="J8" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K8" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L8" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M8" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N8" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -10572,7 +10614,7 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="E9" t="s">
         <v>298</v>
@@ -10587,7 +10629,7 @@
         <v>174</v>
       </c>
       <c r="I9" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J9" t="s">
         <v>387</v>
@@ -10613,10 +10655,10 @@
         <v>173</v>
       </c>
       <c r="D10" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="E10" t="s">
-        <v>528</v>
+        <v>538</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -10631,19 +10673,19 @@
         <v>382</v>
       </c>
       <c r="J10" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K10" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L10" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M10" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N10" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -10657,7 +10699,7 @@
         <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E11" t="s">
         <v>341</v>
@@ -10675,19 +10717,19 @@
         <v>382</v>
       </c>
       <c r="J11" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K11" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L11" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M11" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N11" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -10701,10 +10743,10 @@
         <v>173</v>
       </c>
       <c r="D12" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="E12" t="s">
-        <v>529</v>
+        <v>539</v>
       </c>
       <c r="F12">
         <v>2</v>
@@ -10757,7 +10799,7 @@
         <v>2292.34</v>
       </c>
       <c r="I13" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J13" t="s">
         <v>387</v>
@@ -10783,10 +10825,10 @@
         <v>173</v>
       </c>
       <c r="D14" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="E14" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="F14">
         <v>21</v>
@@ -10798,7 +10840,7 @@
         <v>10768.59</v>
       </c>
       <c r="I14" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J14" t="s">
         <v>387</v>
@@ -10824,10 +10866,10 @@
         <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="E15" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -10839,22 +10881,22 @@
         <v>11325.54</v>
       </c>
       <c r="I15" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J15" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K15" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L15" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M15" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N15" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -10868,10 +10910,10 @@
         <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="E16" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -10886,19 +10928,19 @@
         <v>382</v>
       </c>
       <c r="J16" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K16" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L16" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M16" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N16" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="17" spans="1:14">
@@ -10912,10 +10954,10 @@
         <v>173</v>
       </c>
       <c r="D17" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="E17" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -10927,22 +10969,22 @@
         <v>1076.62</v>
       </c>
       <c r="I17" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J17" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K17" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L17" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M17" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N17" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -10956,10 +10998,10 @@
         <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="E18" t="s">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -10974,19 +11016,19 @@
         <v>382</v>
       </c>
       <c r="J18" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K18" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L18" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M18" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N18" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -11000,37 +11042,37 @@
         <v>173</v>
       </c>
       <c r="D19" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="E19" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G19">
-        <v>226.41</v>
+        <v>132.39</v>
       </c>
       <c r="H19">
-        <v>905.64</v>
+        <v>1323.9</v>
       </c>
       <c r="I19" t="s">
-        <v>382</v>
+        <v>592</v>
       </c>
       <c r="J19" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K19" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L19" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M19" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -11044,10 +11086,10 @@
         <v>173</v>
       </c>
       <c r="D20" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="E20" t="s">
-        <v>536</v>
+        <v>546</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -11062,19 +11104,19 @@
         <v>382</v>
       </c>
       <c r="J20" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K20" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L20" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M20" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N20" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -11088,10 +11130,10 @@
         <v>173</v>
       </c>
       <c r="D21" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="E21" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -11106,19 +11148,19 @@
         <v>382</v>
       </c>
       <c r="J21" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K21" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L21" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M21" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N21" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -11132,10 +11174,10 @@
         <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="E22" t="s">
-        <v>538</v>
+        <v>548</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -11147,7 +11189,7 @@
         <v>285.3</v>
       </c>
       <c r="I22" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J22" t="s">
         <v>387</v>
@@ -11173,10 +11215,10 @@
         <v>173</v>
       </c>
       <c r="D23" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="E23" t="s">
-        <v>539</v>
+        <v>549</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -11188,7 +11230,7 @@
         <v>274.86</v>
       </c>
       <c r="I23" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J23" t="s">
         <v>387</v>
@@ -11214,7 +11256,7 @@
         <v>173</v>
       </c>
       <c r="D24" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="E24" t="s">
         <v>307</v>
@@ -11229,7 +11271,7 @@
         <v>245.6</v>
       </c>
       <c r="I24" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J24" t="s">
         <v>387</v>
@@ -11255,10 +11297,10 @@
         <v>173</v>
       </c>
       <c r="D25" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="E25" t="s">
-        <v>540</v>
+        <v>550</v>
       </c>
       <c r="F25">
         <v>5</v>
@@ -11270,22 +11312,22 @@
         <v>21612.9</v>
       </c>
       <c r="I25" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="J25" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K25" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L25" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M25" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N25" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -11299,10 +11341,10 @@
         <v>173</v>
       </c>
       <c r="D26" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="E26" t="s">
-        <v>541</v>
+        <v>551</v>
       </c>
       <c r="F26">
         <v>8</v>
@@ -11314,7 +11356,7 @@
         <v>8029.04</v>
       </c>
       <c r="I26" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="J26" t="s">
         <v>387</v>
@@ -11340,10 +11382,10 @@
         <v>173</v>
       </c>
       <c r="D27" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="E27" t="s">
-        <v>542</v>
+        <v>552</v>
       </c>
       <c r="F27">
         <v>7</v>
@@ -11355,22 +11397,22 @@
         <v>9269.4</v>
       </c>
       <c r="I27" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J27" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K27" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L27" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M27" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N27" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -11384,10 +11426,10 @@
         <v>173</v>
       </c>
       <c r="D28" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="E28" t="s">
-        <v>543</v>
+        <v>553</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -11402,19 +11444,19 @@
         <v>382</v>
       </c>
       <c r="J28" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K28" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L28" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M28" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N28" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -11428,10 +11470,10 @@
         <v>173</v>
       </c>
       <c r="D29" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="E29" t="s">
-        <v>544</v>
+        <v>554</v>
       </c>
       <c r="F29">
         <v>20</v>
@@ -11443,22 +11485,22 @@
         <v>24038.4</v>
       </c>
       <c r="I29" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J29" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K29" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L29" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M29" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N29" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -11472,10 +11514,10 @@
         <v>173</v>
       </c>
       <c r="D30" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="E30" t="s">
-        <v>545</v>
+        <v>555</v>
       </c>
       <c r="F30">
         <v>2</v>
@@ -11490,19 +11532,19 @@
         <v>382</v>
       </c>
       <c r="J30" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K30" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L30" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M30" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N30" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -11516,10 +11558,10 @@
         <v>173</v>
       </c>
       <c r="D31" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="E31" t="s">
-        <v>546</v>
+        <v>556</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -11531,22 +11573,22 @@
         <v>7890</v>
       </c>
       <c r="I31" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J31" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K31" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L31" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M31" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N31" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -11560,10 +11602,10 @@
         <v>173</v>
       </c>
       <c r="D32" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="E32" t="s">
-        <v>547</v>
+        <v>557</v>
       </c>
       <c r="F32">
         <v>1</v>
@@ -11575,22 +11617,22 @@
         <v>15090</v>
       </c>
       <c r="I32" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J32" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K32" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L32" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M32" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N32" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -11604,10 +11646,10 @@
         <v>173</v>
       </c>
       <c r="D33" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="E33" t="s">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="F33">
         <v>1</v>
@@ -11619,22 +11661,22 @@
         <v>1527.63</v>
       </c>
       <c r="I33" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J33" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K33" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L33" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M33" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N33" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -11648,10 +11690,10 @@
         <v>173</v>
       </c>
       <c r="D34" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="E34" t="s">
-        <v>549</v>
+        <v>559</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -11663,22 +11705,22 @@
         <v>5078.8</v>
       </c>
       <c r="I34" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J34" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K34" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L34" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M34" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N34" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -11692,10 +11734,10 @@
         <v>173</v>
       </c>
       <c r="D35" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="E35" t="s">
-        <v>550</v>
+        <v>560</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -11707,22 +11749,22 @@
         <v>828.12</v>
       </c>
       <c r="I35" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J35" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K35" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L35" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M35" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N35" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -11736,10 +11778,10 @@
         <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="E36" t="s">
-        <v>551</v>
+        <v>561</v>
       </c>
       <c r="F36">
         <v>36</v>
@@ -11751,22 +11793,22 @@
         <v>4016.16</v>
       </c>
       <c r="I36" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J36" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K36" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L36" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M36" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N36" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -11780,10 +11822,10 @@
         <v>173</v>
       </c>
       <c r="D37" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="E37" t="s">
-        <v>552</v>
+        <v>562</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -11795,22 +11837,22 @@
         <v>2270.92</v>
       </c>
       <c r="I37" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J37" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K37" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L37" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M37" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N37" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -11824,10 +11866,10 @@
         <v>173</v>
       </c>
       <c r="D38" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="E38" t="s">
-        <v>553</v>
+        <v>563</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -11839,22 +11881,22 @@
         <v>3100.05</v>
       </c>
       <c r="I38" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J38" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K38" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L38" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M38" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N38" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -11868,10 +11910,10 @@
         <v>173</v>
       </c>
       <c r="D39" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="E39" t="s">
-        <v>554</v>
+        <v>564</v>
       </c>
       <c r="F39">
         <v>4</v>
@@ -11909,10 +11951,10 @@
         <v>173</v>
       </c>
       <c r="D40" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="E40" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="F40">
         <v>2</v>
@@ -11924,22 +11966,22 @@
         <v>15180.86</v>
       </c>
       <c r="I40" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="J40" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K40" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L40" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M40" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N40" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -11953,10 +11995,10 @@
         <v>173</v>
       </c>
       <c r="D41" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="E41" t="s">
-        <v>556</v>
+        <v>566</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -11971,19 +12013,19 @@
         <v>382</v>
       </c>
       <c r="J41" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K41" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L41" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M41" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N41" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -12012,22 +12054,22 @@
         <v>210381.85</v>
       </c>
       <c r="I42" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="J42" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K42" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L42" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M42" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N42" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="43" spans="1:14">
@@ -12041,10 +12083,10 @@
         <v>173</v>
       </c>
       <c r="D43" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="E43" t="s">
-        <v>557</v>
+        <v>567</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -12056,22 +12098,22 @@
         <v>7890.58</v>
       </c>
       <c r="I43" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="J43" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="K43" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="L43" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="M43" s="1">
-        <v>46364</v>
+        <v>46350</v>
       </c>
       <c r="N43" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -12085,7 +12127,7 @@
         <v>173</v>
       </c>
       <c r="D44" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="E44" t="s">
         <v>296</v>
@@ -12100,22 +12142,22 @@
         <v>352.52</v>
       </c>
       <c r="I44" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="J44" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K44" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L44" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M44" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N44" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -12129,10 +12171,10 @@
         <v>173</v>
       </c>
       <c r="D45" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="E45" t="s">
-        <v>558</v>
+        <v>568</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -12144,22 +12186,22 @@
         <v>376.62</v>
       </c>
       <c r="I45" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="J45" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K45" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L45" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M45" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N45" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -12173,10 +12215,10 @@
         <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="E46" t="s">
-        <v>559</v>
+        <v>569</v>
       </c>
       <c r="F46">
         <v>2</v>
@@ -12188,22 +12230,22 @@
         <v>1721.52</v>
       </c>
       <c r="I46" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J46" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K46" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L46" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M46" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N46" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -12217,10 +12259,10 @@
         <v>173</v>
       </c>
       <c r="D47" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="E47" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="F47">
         <v>2</v>
@@ -12232,22 +12274,22 @@
         <v>2577.94</v>
       </c>
       <c r="I47" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J47" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="K47" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="L47" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="M47" s="1">
-        <v>46304</v>
+        <v>46285</v>
       </c>
       <c r="N47" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -12261,10 +12303,10 @@
         <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="E48" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="F48">
         <v>2</v>
@@ -12276,22 +12318,22 @@
         <v>3459.72</v>
       </c>
       <c r="I48" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="J48" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K48" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L48" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M48" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N48" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -12305,10 +12347,10 @@
         <v>173</v>
       </c>
       <c r="D49" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="E49" t="s">
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="F49">
         <v>9</v>
@@ -12320,22 +12362,22 @@
         <v>13757.4</v>
       </c>
       <c r="I49" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J49" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K49" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L49" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M49" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N49" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -12349,10 +12391,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="E50" t="s">
-        <v>562</v>
+        <v>572</v>
       </c>
       <c r="F50">
         <v>1</v>
@@ -12364,22 +12406,22 @@
         <v>4208.01</v>
       </c>
       <c r="I50" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J50" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K50" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L50" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M50" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N50" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -12393,10 +12435,10 @@
         <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="E51" t="s">
-        <v>563</v>
+        <v>573</v>
       </c>
       <c r="F51">
         <v>4</v>
@@ -12411,19 +12453,19 @@
         <v>382</v>
       </c>
       <c r="J51" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K51" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L51" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M51" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N51" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -12437,10 +12479,10 @@
         <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="E52" t="s">
-        <v>564</v>
+        <v>574</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -12455,19 +12497,19 @@
         <v>382</v>
       </c>
       <c r="J52" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K52" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L52" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M52" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N52" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -12481,10 +12523,10 @@
         <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="E53" t="s">
-        <v>565</v>
+        <v>575</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -12499,19 +12541,19 @@
         <v>382</v>
       </c>
       <c r="J53" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K53" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L53" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M53" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N53" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -12525,10 +12567,10 @@
         <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="E54" t="s">
-        <v>566</v>
+        <v>576</v>
       </c>
       <c r="F54">
         <v>4</v>
@@ -12540,22 +12582,22 @@
         <v>3875.24</v>
       </c>
       <c r="I54" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="J54" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K54" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L54" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M54" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N54" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -12569,10 +12611,10 @@
         <v>173</v>
       </c>
       <c r="D55" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
       <c r="E55" t="s">
-        <v>567</v>
+        <v>577</v>
       </c>
       <c r="F55">
         <v>1</v>
@@ -12587,19 +12629,19 @@
         <v>382</v>
       </c>
       <c r="J55" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K55" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L55" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M55" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N55" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -12613,10 +12655,10 @@
         <v>173</v>
       </c>
       <c r="D56" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="E56" t="s">
-        <v>568</v>
+        <v>578</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -12628,22 +12670,22 @@
         <v>3576.55</v>
       </c>
       <c r="I56" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J56" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K56" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L56" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M56" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N56" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -12657,10 +12699,10 @@
         <v>173</v>
       </c>
       <c r="D57" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="E57" t="s">
-        <v>569</v>
+        <v>579</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -12672,22 +12714,22 @@
         <v>908.11</v>
       </c>
       <c r="I57" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J57" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K57" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L57" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M57" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N57" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -12701,10 +12743,10 @@
         <v>173</v>
       </c>
       <c r="D58" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="E58" t="s">
-        <v>570</v>
+        <v>580</v>
       </c>
       <c r="F58">
         <v>4</v>
@@ -12716,22 +12758,22 @@
         <v>1500.8</v>
       </c>
       <c r="I58" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J58" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K58" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L58" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M58" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N58" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -12760,22 +12802,22 @@
         <v>869.98</v>
       </c>
       <c r="I59" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="J59" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K59" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L59" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M59" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N59" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -12789,10 +12831,10 @@
         <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="E60" t="s">
-        <v>571</v>
+        <v>581</v>
       </c>
       <c r="F60">
         <v>3</v>
@@ -12804,22 +12846,22 @@
         <v>1379.52</v>
       </c>
       <c r="I60" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J60" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K60" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L60" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M60" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N60" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="61" spans="1:14">
@@ -12833,10 +12875,10 @@
         <v>173</v>
       </c>
       <c r="D61" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="E61" t="s">
-        <v>572</v>
+        <v>582</v>
       </c>
       <c r="F61">
         <v>5</v>
@@ -12848,22 +12890,22 @@
         <v>5645.05</v>
       </c>
       <c r="I61" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="J61" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="K61" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="L61" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="M61" s="1">
-        <v>46319</v>
+        <v>46305</v>
       </c>
       <c r="N61" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -12877,10 +12919,10 @@
         <v>173</v>
       </c>
       <c r="D62" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="E62" t="s">
-        <v>573</v>
+        <v>583</v>
       </c>
       <c r="F62">
         <v>21</v>
@@ -12892,22 +12934,22 @@
         <v>204.96</v>
       </c>
       <c r="I62" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="J62" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K62" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L62" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M62" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N62" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -12939,19 +12981,19 @@
         <v>382</v>
       </c>
       <c r="J63" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K63" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L63" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M63" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N63" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -12965,7 +13007,7 @@
         <v>173</v>
       </c>
       <c r="D64" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="E64" t="s">
         <v>308</v>
@@ -12980,22 +13022,22 @@
         <v>1999.52</v>
       </c>
       <c r="I64" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="J64" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="K64" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="L64" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="M64" s="1">
-        <v>46364</v>
+        <v>46350</v>
       </c>
       <c r="N64" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -13009,37 +13051,37 @@
         <v>173</v>
       </c>
       <c r="D65" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="E65" t="s">
-        <v>574</v>
+        <v>584</v>
       </c>
       <c r="F65">
         <v>2</v>
       </c>
       <c r="G65">
-        <v>4742.74</v>
+        <v>4424.23</v>
       </c>
       <c r="H65">
-        <v>9485.48</v>
+        <v>8848.459999999999</v>
       </c>
       <c r="I65" t="s">
-        <v>382</v>
+        <v>592</v>
       </c>
       <c r="J65" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K65" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L65" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M65" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N65" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -13053,10 +13095,10 @@
         <v>173</v>
       </c>
       <c r="D66" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="E66" t="s">
-        <v>575</v>
+        <v>585</v>
       </c>
       <c r="F66">
         <v>2</v>
@@ -13068,22 +13110,239 @@
         <v>297.92</v>
       </c>
       <c r="I66" t="s">
-        <v>382</v>
+        <v>592</v>
       </c>
       <c r="J66" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="K66" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="L66" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="M66" s="1">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="N66" t="s">
-        <v>582</v>
+        <v>596</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14">
+      <c r="A67" t="s">
+        <v>471</v>
+      </c>
+      <c r="B67" t="s">
+        <v>172</v>
+      </c>
+      <c r="C67" t="s">
+        <v>173</v>
+      </c>
+      <c r="D67" t="s">
+        <v>532</v>
+      </c>
+      <c r="E67" t="s">
+        <v>586</v>
+      </c>
+      <c r="F67">
+        <v>1</v>
+      </c>
+      <c r="G67">
+        <v>27326.55</v>
+      </c>
+      <c r="H67">
+        <v>27326.55</v>
+      </c>
+      <c r="I67" t="s">
+        <v>592</v>
+      </c>
+      <c r="J67" t="s">
+        <v>592</v>
+      </c>
+      <c r="K67" t="s">
+        <v>592</v>
+      </c>
+      <c r="L67" t="s">
+        <v>592</v>
+      </c>
+      <c r="M67" s="1">
+        <v>46350</v>
+      </c>
+      <c r="N67" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
+      <c r="A68" t="s">
+        <v>472</v>
+      </c>
+      <c r="B68" t="s">
+        <v>172</v>
+      </c>
+      <c r="C68" t="s">
+        <v>173</v>
+      </c>
+      <c r="D68" t="s">
+        <v>533</v>
+      </c>
+      <c r="E68" t="s">
+        <v>298</v>
+      </c>
+      <c r="F68">
+        <v>16</v>
+      </c>
+      <c r="G68">
+        <v>50.39</v>
+      </c>
+      <c r="H68">
+        <v>806.24</v>
+      </c>
+      <c r="I68" t="s">
+        <v>592</v>
+      </c>
+      <c r="J68" t="s">
+        <v>592</v>
+      </c>
+      <c r="K68" t="s">
+        <v>592</v>
+      </c>
+      <c r="L68" t="s">
+        <v>592</v>
+      </c>
+      <c r="M68" s="1">
+        <v>46350</v>
+      </c>
+      <c r="N68" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
+      <c r="A69" t="s">
+        <v>473</v>
+      </c>
+      <c r="B69" t="s">
+        <v>172</v>
+      </c>
+      <c r="C69" t="s">
+        <v>173</v>
+      </c>
+      <c r="D69" t="s">
+        <v>534</v>
+      </c>
+      <c r="E69" t="s">
+        <v>294</v>
+      </c>
+      <c r="F69">
+        <v>100</v>
+      </c>
+      <c r="G69">
+        <v>4</v>
+      </c>
+      <c r="H69">
+        <v>400</v>
+      </c>
+      <c r="I69" t="s">
+        <v>592</v>
+      </c>
+      <c r="J69" t="s">
+        <v>592</v>
+      </c>
+      <c r="K69" t="s">
+        <v>592</v>
+      </c>
+      <c r="L69" t="s">
+        <v>592</v>
+      </c>
+      <c r="M69" s="1">
+        <v>46350</v>
+      </c>
+      <c r="N69" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
+      <c r="A70" t="s">
+        <v>474</v>
+      </c>
+      <c r="B70" t="s">
+        <v>172</v>
+      </c>
+      <c r="C70" t="s">
+        <v>173</v>
+      </c>
+      <c r="D70" t="s">
+        <v>535</v>
+      </c>
+      <c r="E70" t="s">
+        <v>587</v>
+      </c>
+      <c r="F70">
+        <v>2</v>
+      </c>
+      <c r="G70">
+        <v>1521.88</v>
+      </c>
+      <c r="H70">
+        <v>3043.76</v>
+      </c>
+      <c r="I70" t="s">
+        <v>594</v>
+      </c>
+      <c r="J70" t="s">
+        <v>594</v>
+      </c>
+      <c r="K70" t="s">
+        <v>594</v>
+      </c>
+      <c r="L70" t="s">
+        <v>594</v>
+      </c>
+      <c r="N70" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
+      <c r="A71" t="s">
+        <v>475</v>
+      </c>
+      <c r="B71" t="s">
+        <v>172</v>
+      </c>
+      <c r="C71" t="s">
+        <v>173</v>
+      </c>
+      <c r="D71" t="s">
+        <v>536</v>
+      </c>
+      <c r="E71" t="s">
+        <v>588</v>
+      </c>
+      <c r="F71">
+        <v>4</v>
+      </c>
+      <c r="G71">
+        <v>512.08</v>
+      </c>
+      <c r="H71">
+        <v>2048.32</v>
+      </c>
+      <c r="I71" t="s">
+        <v>595</v>
+      </c>
+      <c r="J71" t="s">
+        <v>595</v>
+      </c>
+      <c r="K71" t="s">
+        <v>595</v>
+      </c>
+      <c r="L71" t="s">
+        <v>595</v>
+      </c>
+      <c r="M71" s="1">
+        <v>46365</v>
+      </c>
+      <c r="N71" t="s">
+        <v>596</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: tpjl (11/09/2026 11:59)
</commit_message>
<xml_diff>
--- a/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
+++ b/Projetos/02_Dados_Tratados/base_tpjl_tratada.xlsx
@@ -10597,7 +10597,7 @@
         <v>590</v>
       </c>
       <c r="M8" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N8" t="s">
         <v>596</v>
@@ -10682,7 +10682,7 @@
         <v>592</v>
       </c>
       <c r="M10" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N10" t="s">
         <v>596</v>
@@ -10726,7 +10726,7 @@
         <v>592</v>
       </c>
       <c r="M11" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N11" t="s">
         <v>596</v>
@@ -10893,7 +10893,7 @@
         <v>590</v>
       </c>
       <c r="M15" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N15" t="s">
         <v>596</v>
@@ -10937,7 +10937,7 @@
         <v>592</v>
       </c>
       <c r="M16" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N16" t="s">
         <v>596</v>
@@ -10981,7 +10981,7 @@
         <v>590</v>
       </c>
       <c r="M17" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N17" t="s">
         <v>596</v>
@@ -11025,7 +11025,7 @@
         <v>592</v>
       </c>
       <c r="M18" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N18" t="s">
         <v>596</v>
@@ -11069,7 +11069,7 @@
         <v>592</v>
       </c>
       <c r="M19" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N19" t="s">
         <v>596</v>
@@ -11113,7 +11113,7 @@
         <v>592</v>
       </c>
       <c r="M20" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N20" t="s">
         <v>596</v>
@@ -11157,7 +11157,7 @@
         <v>592</v>
       </c>
       <c r="M21" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N21" t="s">
         <v>596</v>
@@ -11324,7 +11324,7 @@
         <v>592</v>
       </c>
       <c r="M25" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N25" t="s">
         <v>596</v>
@@ -11409,7 +11409,7 @@
         <v>590</v>
       </c>
       <c r="M27" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N27" t="s">
         <v>596</v>
@@ -11453,7 +11453,7 @@
         <v>592</v>
       </c>
       <c r="M28" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N28" t="s">
         <v>596</v>
@@ -11497,7 +11497,7 @@
         <v>593</v>
       </c>
       <c r="M29" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N29" t="s">
         <v>596</v>
@@ -11541,7 +11541,7 @@
         <v>592</v>
       </c>
       <c r="M30" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N30" t="s">
         <v>596</v>
@@ -11585,7 +11585,7 @@
         <v>593</v>
       </c>
       <c r="M31" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N31" t="s">
         <v>596</v>
@@ -11629,7 +11629,7 @@
         <v>590</v>
       </c>
       <c r="M32" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N32" t="s">
         <v>596</v>
@@ -11673,7 +11673,7 @@
         <v>590</v>
       </c>
       <c r="M33" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N33" t="s">
         <v>596</v>
@@ -11717,7 +11717,7 @@
         <v>590</v>
       </c>
       <c r="M34" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N34" t="s">
         <v>596</v>
@@ -11761,7 +11761,7 @@
         <v>590</v>
       </c>
       <c r="M35" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N35" t="s">
         <v>596</v>
@@ -11805,7 +11805,7 @@
         <v>590</v>
       </c>
       <c r="M36" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N36" t="s">
         <v>596</v>
@@ -11849,7 +11849,7 @@
         <v>590</v>
       </c>
       <c r="M37" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N37" t="s">
         <v>596</v>
@@ -11893,7 +11893,7 @@
         <v>590</v>
       </c>
       <c r="M38" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N38" t="s">
         <v>596</v>
@@ -11978,7 +11978,7 @@
         <v>590</v>
       </c>
       <c r="M40" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N40" t="s">
         <v>596</v>
@@ -12022,7 +12022,7 @@
         <v>592</v>
       </c>
       <c r="M41" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N41" t="s">
         <v>596</v>
@@ -12066,7 +12066,7 @@
         <v>590</v>
       </c>
       <c r="M42" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N42" t="s">
         <v>596</v>
@@ -12110,7 +12110,7 @@
         <v>592</v>
       </c>
       <c r="M43" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N43" t="s">
         <v>596</v>
@@ -12154,7 +12154,7 @@
         <v>592</v>
       </c>
       <c r="M44" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N44" t="s">
         <v>596</v>
@@ -12198,7 +12198,7 @@
         <v>592</v>
       </c>
       <c r="M45" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N45" t="s">
         <v>596</v>
@@ -12242,7 +12242,7 @@
         <v>590</v>
       </c>
       <c r="M46" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N46" t="s">
         <v>596</v>
@@ -12286,7 +12286,7 @@
         <v>590</v>
       </c>
       <c r="M47" s="1">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="N47" t="s">
         <v>596</v>
@@ -12330,7 +12330,7 @@
         <v>592</v>
       </c>
       <c r="M48" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N48" t="s">
         <v>596</v>
@@ -12374,7 +12374,7 @@
         <v>593</v>
       </c>
       <c r="M49" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N49" t="s">
         <v>596</v>
@@ -12418,7 +12418,7 @@
         <v>593</v>
       </c>
       <c r="M50" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N50" t="s">
         <v>596</v>
@@ -12462,7 +12462,7 @@
         <v>592</v>
       </c>
       <c r="M51" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N51" t="s">
         <v>596</v>
@@ -12506,7 +12506,7 @@
         <v>592</v>
       </c>
       <c r="M52" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N52" t="s">
         <v>596</v>
@@ -12550,7 +12550,7 @@
         <v>592</v>
       </c>
       <c r="M53" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N53" t="s">
         <v>596</v>
@@ -12594,7 +12594,7 @@
         <v>592</v>
       </c>
       <c r="M54" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N54" t="s">
         <v>596</v>
@@ -12638,7 +12638,7 @@
         <v>592</v>
       </c>
       <c r="M55" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N55" t="s">
         <v>596</v>
@@ -12682,7 +12682,7 @@
         <v>593</v>
       </c>
       <c r="M56" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N56" t="s">
         <v>596</v>
@@ -12726,7 +12726,7 @@
         <v>593</v>
       </c>
       <c r="M57" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N57" t="s">
         <v>596</v>
@@ -12770,7 +12770,7 @@
         <v>593</v>
       </c>
       <c r="M58" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N58" t="s">
         <v>596</v>
@@ -12814,7 +12814,7 @@
         <v>592</v>
       </c>
       <c r="M59" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N59" t="s">
         <v>596</v>
@@ -12858,7 +12858,7 @@
         <v>593</v>
       </c>
       <c r="M60" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N60" t="s">
         <v>596</v>
@@ -12902,7 +12902,7 @@
         <v>593</v>
       </c>
       <c r="M61" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="N61" t="s">
         <v>596</v>
@@ -12946,7 +12946,7 @@
         <v>592</v>
       </c>
       <c r="M62" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N62" t="s">
         <v>596</v>
@@ -12990,7 +12990,7 @@
         <v>592</v>
       </c>
       <c r="M63" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N63" t="s">
         <v>596</v>
@@ -13034,7 +13034,7 @@
         <v>592</v>
       </c>
       <c r="M64" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N64" t="s">
         <v>596</v>
@@ -13078,7 +13078,7 @@
         <v>592</v>
       </c>
       <c r="M65" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N65" t="s">
         <v>596</v>
@@ -13122,7 +13122,7 @@
         <v>592</v>
       </c>
       <c r="M66" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N66" t="s">
         <v>596</v>
@@ -13166,7 +13166,7 @@
         <v>592</v>
       </c>
       <c r="M67" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N67" t="s">
         <v>596</v>
@@ -13210,7 +13210,7 @@
         <v>592</v>
       </c>
       <c r="M68" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N68" t="s">
         <v>596</v>
@@ -13254,7 +13254,7 @@
         <v>592</v>
       </c>
       <c r="M69" s="1">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="N69" t="s">
         <v>596</v>
@@ -13339,7 +13339,7 @@
         <v>595</v>
       </c>
       <c r="M71" s="1">
-        <v>46365</v>
+        <v>46366</v>
       </c>
       <c r="N71" t="s">
         <v>596</v>

</xml_diff>